<commit_message>
Danimarca: foglio nel workbook (88 aziende), normalizzazione filiere e handoff aggiornato
- normalize_dk.py: allinea il campo Filiera alla tassonomia dei fogli IT/DE/FI
  e sposta i codici CVR dalla denominazione al campo Dimensione
- MyEUDR_Lead_Mapping.xlsx: 4 fogli, 364 righe (Danimarca 88)
- MyEUDR_CONTINUA.md: stato aggiornato + vincoli dell'ambiente web (egress
  bloccato su proff.dk/CVR, budget WebSearch) e piano di arricchimento contatti
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Italia" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Germania" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finlandia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Italia" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Germania" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Finlandia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Danimarca" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Italia'!$A$2:$J$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Germania'!$A$2:$J$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Finlandia'!$A$2:$J$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -90,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -109,6 +111,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13903,4 +13908,4209 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J90"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyEUDR — Lead mapping · Danimarca · aziende potenzialmente soggette all'EUDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Denominazione</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Filiera EUDR</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Dimensione (fatt./dip.)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Ruolo</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Email / PEC</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Sito web</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>GETAMA DANMARK A/S</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello/pelle</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo (bruttofortjeneste) 55,4 M DKK ≈ 7,4 M€ nel 2024 (era 19,8 M DKK nel 2023) / 21 dip. dichiarati (lasso.dk 2024); fatturato non pubblicato. ATTENZIONE: sul CVR 17871188 compaiono anche denominazioni/sedi diverse (JT Randers A/S, Randers SØ) – verificare l'assetto societario prima del contatto</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Jesper Temp</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.getama.dk/</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Gedsted (Vesthimmerland), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://lasso.dk/firmaer/17871188/getama-danmark-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>NIELAUS A/S</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute in legno e pelle</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>11 dip. (proff.dk, CVR 35480943, NACE 310000 Fremstilling af møbler); fatturato non pubblicato. Taglia sotto 5 M€ mantenuta per copertura del cluster Syddanmark; co-direttore Kim Nordentoft Frederiksen</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Jesper Nordentoft Frederiksen</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nielaus.dk/</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Vejrup, Bramming (Esbjerg), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/nielaus-as/bramming/producenter/GUJZBOI016D/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ONECOLLECTION A/S (House of Finn Juhl)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello/pelle</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>≈93 dip. su 4 unità (krak.dk/proff.dk 2025); risultato d'esercizio 4,14 M DKK nel 2025 (6,13 M DKK nel 2024); fatturato non pubblicato. Stima ricavi ~13-20 M€ sulla base degli addetti: da verificare. Ha acquisito nel 2024 un concorrente con 35 dipendenti</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Bo Nørgaard</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://onecollection.com/</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Ringkøbing (Ringkøbing-Skjern), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/onecollection-as/ringk%C3%B8bing/m%C3%B8bler/GXS757I015G</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>SØRENSEN LÆDER A/S (Sorensen Leather)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Pelle/Concia</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); bruttofortjeneste 23,85 mio DKK (~3,2 M EUR) nel 2022; ca. 20 dipendenti; commercio all'ingrosso di pelli e cuoio (engroshandel med huder, skind og læder). Fonte: proff.dk (CVR 50828514), anno 2022</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Louise Vesterskov Sørensen</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør (CEO)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/sorensen-leather</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://sorensenleather.com/</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Lystrup/Aarhus (Lægårdsvej 19, 8520), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/s%C3%B8rensen-l%C3%A6der-as/lystrup/skind-l%C3%A6der-og-pels/GKJEN4I07RD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>AUBO PRODUCTION A/S</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine e arredo bagno</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 116 M DKK ≈ 15,5 M€ (bilancio 2025, proff.dk/ownr) / 102 dip. – 74 FTE ott. 2025 (CVR 28854846); fatturato non pubblicato ma stimabile sopra 30 M€. AZIENDA DI CONFINE: controllata di TCM Group A/S (gruppo quotato danese, ricavi di gruppo ~1 mld DKK) – valutare l'approccio a livello di capogruppo</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Torben Andersen</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Aulum (Herning), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/aubo-production-as/aulum/producenter/GQ8037I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>BØJSØ DØRE &amp; VINDUER A/S</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — porte e finestre in legno</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>41 dipendenti (unità produttiva). Fatturato non pubblicato separatamente nelle fonti consultate. Con ~40 addetti in produzione i ricavi si collocano verosimilmente nella fascia bassa del target (stima non verificata). CVR 12224494, attività dal 01.01.1988 (fondata nel 1972 da Bøje Sørensen), sede Højagervej 5-7, 6623 Vorbasse. LEGAME DI GRUPPO IMPORTANTE: dal 2017 controllata da INWIDO DENMARK A/S, parte del gruppo quotato svedese Inwido — la due diligence EUDR potrebbe essere centralizzata a livello di gruppo, il che riduce la probabilità di acquisto autonomo del software. Lead da qualificare con cautela.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Lasse Sørensen</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/b%C3%B8js%C3%B8-d%C3%B8re-&amp;-vinduer-a-s</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>https://boejsoe.dk/</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Vorbasse (Billund), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/b%C3%B8js%C3%B8-d%C3%B8re-vinduer-as/vorbasse/producenter/GJL0QJI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>DANSK HÅRDTTRÆ SAVVÆRK A/S (DHS)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — segheria/import legni duri</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>12 dipendenti (9 ULA, ago. 2024). Bruttofortjeneste 2023: 6,849 M DKK (~0,92 M€), da 7,241 M DKK 2022; risultato 2023: 1,121 M DKK. SOTTO LA SOGLIA dei 5 M€ di fatturato: mantenuta per copertura della filiera perché segheria/importatore di legni duri, cioè operatore EUDR in senso stretto con obbligo di DDS anche a dimensioni ridotte (le PMI non sono esentate dagli obblighi sostanziali). CVR 15008792, costituita 01.11.1990, sede Stokkebrovej 2B, 6340 Kruså. Controllata da Holdbi Holding ApS; presidente del CdA Knud Mainusch.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Mikkel Søgaard Christiansen</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://dhs.as/</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Kruså (Aabenraa), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/dansk-h%C3%A5rdttr%C3%A6-savv%C3%A6rk-as/krus%C3%A5/savbrug-og-h%C3%B8vlerier/GJVKGKI01F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>DINESEN FLOORS A/S</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — segheria/pavimenti in tavole</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>109 dipendenti. Bilancio 2025: bruttofortjeneste 49,85 M DKK (~6,7 M€), risultato d'esercizio -11,14 M DKK. Fatturato non pubblicato singolarmente; con 109 addetti e questo margine lordo i ricavi sono verosimilmente nella parte alta della fascia tollerabile (stima non verificata, da confermare a bilancio). AZIENDA DI CONFINE per dimensione. CVR 33920717, costituita 1971, sede Klovtoftvej 2, Jels, 6630 Rødding. LEGAME DI GRUPPO: controllata da Jels Savværk Holding ApS; showroom a København K. Acquista legname di quercia principalmente da foreste dell'Europa centrale: operatore EUDR. NOTA: sito ufficiale non confermato da fonte verificata in questa sessione, quindi non riportato.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Tine Thorman Kaspersen</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Jels, 6630 Rødding (Vejen), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/dinesen-floors-as/r%C3%B8dding/savbrug-og-h%C3%B8vlerier/GWA6I7I01F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>FREDERICIA FURNITURE A/S</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello/imbottiti</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 60,4 M DKK ≈ 8,1 M€ nel 2024 (60,4 M DKK anche nel 2023) / 47 dip. nella sede di Fredericia (lasso.dk/proff.dk 2024); risultato ante imposte 6,5 M€ DKK; fatturato non pubblicato. Stima ricavi ~18-27 M€: da verificare. Capogruppo Thomas Graversen Holding ApS (gruppo indipendente danese)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Rasmus Lehmann Graversen</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør (dal 01.05.2024)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Fredericia, Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://lasso.dk/firmaer/45607313/fredericia-furniture-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Farstrup Furniture A/S</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute e imbottiti</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 19 M DKK ≈ 2,5 M€ / 43 dip. (bilancio 2025, proff.dk-lasso.dk); patrimonio netto 9,4 M DKK; fatturato non pubblicato. Azienda sotto soglia (stima ricavi ~6-8 M€) tenuta per copertura</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Steen Cederholm-Johansen</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>https://farstrup.dk/</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Søndersø (Nordfyn), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/farstrup-furniture-as/s%C3%B8nders%C3%B8/producenter/GKF1OMI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>GLOBAL TIMBER A/S</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import/export legname</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>29 dipendenti (27 ULA, dato CVR/proff). Fatturato record 317,8 M DKK (~42,6 M€) nell'anno di picco, con utile ante imposte 21,4 M DKK; esercizio 01.07.2023-30.06.2024 chiuso con utile 5,32 M DKK e fatturato successivamente in contrazione (perdita di 26 M DKK sulla bottom line in due anni secondo la stampa di settore). AZIENDA DI CONFINE sul valore di picco, sotto la soglia di esclusione ~50 M€. VERIFICATA COME ATTIVA (l'esclusione richiesta valeva solo in caso di cessata attività). CVR 29429774, sede Michael Drewsens Vej 1A, 8270 Højbjerg, costituita 28.03.2006. Importatore puro di legname = operatore EUDR in senso stretto, massima priorità.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Anders Bitzer</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://globaltimber.dk/</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Højbjerg (Aarhus), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/global-timber-as/h%C3%B8jbjerg/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GQM2S6I10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>GRAMRODE MØBELFABRIK A/S</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 18 M DKK ≈ 2,4 M€ (2024, proff.dk/lasso.dk) / 23 dip. (CVR 25777530); fatturato non pubblicato. Stima ricavi ~5-7 M€: da verificare</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Henning Oscar Jørgensen</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Juelsminde (Hedensted), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/gramrode-m%C3%B8belfabrik-as/juelsminde/producenter/GKHJSGI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>HAMMEL FURNITURE A/S</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sistemi contenitivi e sedute</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>38-55 dip. tra sede/produzione Hammel e stabilimento Skærbæk (proff.dk CVR 32559476 e sito aziendale); fatturato non pubblicato. Stima ricavi ~8-15 M€: da verificare</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Jens-Ole Staghøj</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/hammel-furniture-a-s</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hammel-furniture.dk/</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Hammel (Favrskov), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/hammel-furniture-as/hammel/producenter/GSOF1AI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>HVIDBJERG VINDUET A/S</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — finestre e porte in legno</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Circa 155 dipendenti complessivi (66 nell'unità di Thyholm + 106 nell'unità di Thisted secondo i registri; il totale aziendale dichiarato è ~155). Fatturato non pubblicato nelle banche dati consultate (campo vuoto su proff). AZIENDA DI CONFINE: con questo organico i ricavi potrebbero superare la fascia target — da verificare a bilancio prima del contatto. CVR 17010344, costituita 01.01.1993, capitale sociale 5.000.000 DKK. LEGAME DI GRUPPO: controllata da Hvidbjerg i A/S. Produce finestre e porte in legno/alluminio a Nors (Thy): soggetta a EUDR per il legname immesso sul mercato UE.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Claus Arberg</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Hvidbjerg, Thyholm (Struer) — secondo stabilimento a Nors, Thy (Thisted), Region Midtjylland / Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/hvidbjerg-vinduet-as/thyholm/producenter/GL4UY5I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>HØRNING PARKET A/S</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>22 dipendenti. Fatturato non pubblicato nelle fonti consultate; la stampa di settore riporta una crescita marcata dei ricavi (circa dieci volte in cinque anni al momento di un riconoscimento nel 2016) e una solida posizione di mercato. CVR 33965362, costituita 14.10.2011, sede Christiansmindevej 12, 8660 Skanderborg. Origine storica: Hørning Parket Fabrik, 1925. Produttore di parquet che acquista/importa legname di latifoglia: soggetto agli obblighi EUDR di due diligence e DDS. NOTA: sito ufficiale non confermato da fonte verificata in questa sessione, quindi non riportato.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Peter Mathiasen</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Skanderborg, Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/h%C3%B8rning-parket-as/skanderborg/producenter/GTM41UI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>HårdtTrælasten P/S</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legni nobili</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2 dipendenti nell'unità produttiva registrata. Fatturato non pubblicato. NETTAMENTE SOTTO LA SOGLIA dei 5 M€: inserita solo per copertura della filiera degli importatori di legni nobili (operatore EUDR in senso stretto). CVR 39719630, P/S costituita l'11.07.2018 ma attività avviata nel 2002; sede Islandsgade 40, 4690 Haslev (unità anche a Rysagervej 20, Haslev). NACE 468300 commercio all'ingrosso di legno e materiali da costruzione. Lead a bassa priorità per dimensione, ma pertinente per profilo di rischio EUDR (legni tropicali/nobili).</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Michael Kaasing Andersen</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>haardttrae@haardttrae.dk</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://haardttrae.dk/</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Haslev (Faxe), Region Sjælland</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/h%C3%A5rdttr%C3%A6lasten-ps/haslev/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GXJDCBI10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>INNOVATION LIVING A/S (già Innovation Randers A/S)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — divani letto</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 47,3 M DKK ≈ 6,3 M€ nel 2023 (49,9 M DKK nel 2022) / 57 dip. (proff.dk-lasso.dk, CVR 65699516); risultato 13,7 M DKK; fatturato non pubblicato. Stima ricavi ~15-25 M€: da verificare. Parte del gruppo INNOVATION HOLDING A/S (8 società, controllo familiare danese)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Morten Lind Mølgaard</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Randers NØ, Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/innovation-living-as/randers-n%C3%B8/m%C3%B8bler/13462KI015G</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>JKE DESIGN A/S</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 55,6 M DKK ≈ 7,5 M€ nel 2023 (58,7 M DKK nel 2022) / 102 dip. (proff.dk/estatistik, CVR 63271012); fatturato non pubblicato. Stima ricavi ~20-27 M€: da verificare. Controllata di BALLINGSLÖV INTERNATIONAL DANMARK A/S (gruppo svedese Stena Adactum)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Freddy Lauridsen</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Jerslev J (Brønderslev), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/jke-design-as/jerslev-j/producenter/GKNXIBI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>KEFLICO A/S</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname (hårdttræ/pannelli)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 349 M DKK 2024 (~46,8 M€, cambio 7,46), in calo dai 368 M DKK 2023; risultato d'esercizio 2,8 M DKK. 62 dipendenti (fonte proff.dk/CVR). AZIENDA DI CONFINE: sopra la fascia tollerabile 5-40 M€ ma sotto la soglia di esclusione ~50 M€; mantenuta perché importatore/grossista puro di legname (operatore EUDR in senso stretto) e quindi lead ad altissima priorità. CVR 23980010, sede Juelstrupparken 24, 9530 Støvring. Controllata da Direktør Erik Kauffeldts Fond. Ha acquisito un altro importatore danese di legname certificato.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Mads Tidemann Stenstrop</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/keflico-a-s</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://keflico.com/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Støvring (Rebild), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/keflico-as/st%C3%B8vring/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GKB2RFI10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>KRYDSFINER-HANDELEN A/S</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio pannelli (compensato/MDF)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>18 dipendenti. Bilancio 2024: bruttofortjeneste 30 M DKK (~4,0 M€), risultato ante imposte 14,5 M DKK, risultato netto 11,3 M DKK, patrimonio netto 27,1 M DKK. Fatturato non pubblicato; il livello di margine lordo è compatibile con ricavi nella fascia target per un grossista di pannelli. CVR 17948598, costituita 01.08.1994, sede Hobrovej 54, 2610 Rødovre. LEGAME DI GRUPPO: CdA con Björn Carl David Ljungberg e presidente Cato Ness (riconducibile a proprietà nordica/scandinava). Importatore di compensato (spesso da Asia/Baltico) = operatore EUDR in senso stretto, alta priorità.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Lars Langgaard</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://krydsfiner.dk/</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Rødovre, Region Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/krydsfiner-handelen-as/r%C3%B8dovre/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GK7DYBI10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>KVIST INDUSTRIES A/S</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — componenti e sedute (subfornitura)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>110 dip. (proff.dk, CVR 22629115); codice NACE 310900 Fremstilling af andre møbler; fatturato non pubblicato. Stima ~15-25 M€ sulla base degli addetti: da verificare</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Jesper Tordrup Andersen</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Årre (Varde/Esbjerg), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/kvist-industries-as/%C3%A5rre/producenter/GW40QBI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Klim Furniture A/S (già Klim Møbelfabrik)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imbottiti e sedute</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 8,6 M DKK ≈ 1,2 M€ (bilancio 2025, proff.dk/lasso.dk) / 15-23 dip. (CVR 39299011); fatturato non pubblicato. Taglia sotto 5 M€ tenuta per copertura; co-proprietario e direttore Kasper Høgenhaug (dal 2024)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Jan Middelboe</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://klim-furniture.dk/</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Fjerritslev (Jammerbugt), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/klim-furniture-as/fjerritslev/producenter/GX91UZI016D/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>LILLEHEDEN A/S</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — legno lamellare/glulam</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>89 dipendenti secondo proff/CVR (76 secondo altra fonte). Bruttofortjeneste 2023: 49,6 M DKK (~6,6 M€); risultato 15,5 M DKK. Fatturato non pubblicato singolarmente. CVR 24077713, sede Hovedvejen 114, 9850 Hirtshals. LEGAME DI GRUPPO: controllata da Nordic Wood Industries A/S (gruppo con oltre 550 dipendenti e oltre 800 M DKK di fatturato consolidato ~107 M€) — la compliance EUDR potrebbe essere gestita a livello di capogruppo. NOTA REFERENTE: le fonti riportano nomi discordanti (Hans Henrik von Platen-Hallermund vs Christian Grønbæk Esbensen), quindi il campo referente è lasciato vuoto in attesa di verifica diretta su CVR.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lilleheden.dk/</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Hirtshals (Hjørring), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/lilleheden-as/hirtshals/l%C3%A5se-og-beslag/GKB3IQI10PL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>MULTIFORM A/S</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine su misura</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 8,1 M DKK ≈ 1,1 M€ nel 2024, risultato -5,4 M DKK / 37 dip. (proff.dk-lasso.dk, CVR 18606488); fatturato non pubblicato. Taglia stimata sotto 10 M€, tenuta per copertura del cluster Herning. Controllata del gruppo svedese Ballingslöv International (che possiede anche JKE Design e Kvik)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Allan Meyer</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Kibæk (Herning), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/multiform-as/kib%C3%A6k/producenter/GLGFCDI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>N. EILERSEN A/S</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 16 M DKK ≈ 2,1 M€ (bilancio 2025, proff.dk/ownr) / 25 dip. in Danimarca; il gruppo familiare controlla inoltre 2 stabilimenti esteri (Europa e Asia) con ~300 addetti complessivi; fatturato non pubblicato. Taglia DK sotto 5 M€ tenuta per copertura</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Anders Juul Eilersen</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>https://eilersen.eu/</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Skamby (Nordfyn), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/n.-eilersen-as/skamby/producenter/GKEJPJI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>NPI (Nordic Panel Import)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import pannelli a base legno</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>9 dipendenti (dato dichiarato sul sito aziendale). Fatturato non pubblicato nelle fonti consultate: verosimilmente sotto o attorno alla soglia dei 5 M€, mantenuta per copertura in quanto importatore puro di pannelli a base legno da paesi extra-UE, cioè operatore EUDR in senso stretto ad alta priorità. Fondata nel settembre 2002 da Theis G. Larsen e Michael Schram; sede Helge Nielsens Alle 7, 1G, 8723 Løsning — STESSO INDIRIZZO di SOMMER-SAVEX A/S, possibile prossimità/legame tra le due realtà da verificare. ATTENZIONE: la ragione sociale esatta registrata al CVR (forma giuridica ApS/A/S) non è stata verificabile in questa sessione; verificato solo il numero CVR 37418730. I fondatori non risultano formalmente confermati come direttori in carica, quindi il campo referente è lasciato vuoto.</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.npi.dk/</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Løsning (Hedensted), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.npi.dk/about-npi/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>SIKA DESIGN A/S</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi in rattan/legno</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 29 M DKK ≈ 3,9 M€ (2021, proff.dk/lasso.dk) / 21 dip. (CVR 31476712); fatturato non pubblicato. Stima ricavi ~8-10 M€: da verificare</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Louise Andreasen</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>https://sika-design.dk/</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Rynkeby (Kerteminde), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/sika-design-as/rynkeby/interi%C3%B8r-og-interi%C3%B8rudstyr/0IQNL4I07ST</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SKOVBY MØBELFABRIK A/S</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello/pannelli</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>≈207 dip. su 3 unità in Midtjylland (krak.dk 2025); fatturato non pubblicato (bilancio classe B) – patrimonio netto 90,8 M DKK e risultato -9,5 M DKK nell'esercizio 01.09.23-31.08.24 (proff.dk/lasso.dk 2024). Stima ricavi ~25-35 M€ sulla base degli addetti: da verificare</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Preben Rasmussen</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>skovby@skovby.dk</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.skovby.dk/</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Galten (Skanderborg), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/skovby-m%C3%B8belfabrik-as/galten/producenter/GL6246I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>SOFTLINE A/S</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Utile lordo 40 M DKK ≈ 5,4 M€ (2023, proff.dk/erhvervplus) / 43 dip. in Danimarca (CVR 27266355); fatturato non pubblicato. Stima ricavi ~12-18 M€: da verificare</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Finn Herluf Sørensen</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/softline-furniture</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>https://softlinefurniture.com/</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Maribo (Lolland), Region Sjælland</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/softline-as/maribo/producenter/GPBT05I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SOMMER-SAVEX A/S</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname (hårdttræ/impiallacciature)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non verificato (dati di bilancio non accessibili in questa sessione). CVR 13923795, costituita 1990, sede Helge Nielsens Alle 7, 8723 Løsning. Oggetto sociale: produzione e commercio, incl. import/export, di legno e impiallacciature. Controllata da Line Hjort Holding ApS (acquisita da Line Hjort nel 2016). NOTA: l'indicazione di ~14 dipendenti e l'email info@sommer-savex.dk fornite nel lead di partenza NON sono state verificabili su fonte reale, quindi non riportate. Importatore puro di legname = operatore EUDR in senso stretto, massima priorità.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Line Hjort</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Direktør / proprietaria</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sommer-savex.dk/</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Løsning (Hedensted), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/sommer-savex-as/l%C3%B8sning/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GJREDHI10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>SUPERWOOD A/S</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — impregnazione legno/rivestimenti</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>28 dipendenti. Bruttofortjeneste 2024: 16,565 M DKK (~2,2 M€), in crescita dai 14,413 M DKK 2023; risultato netto 1,018 M DKK. Fatturato non pubblicato; per un impregnatore con questo margine i ricavi sono verosimilmente nella fascia bassa/media del target ma NON verificati. CVR 26434602, costituita 24.01.2002, sede Palsgårdvej 3, 7362 Hampen. Codice NACE: segheria e piallatura del legno. Acquista/importa legname di conifera nordico da trattare: soggetto EUDR con esigenza documentata di tracciabilità (l'azienda comunica pubblicamente l'impegno a documentare la propria sostenibilità).</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Ole Dalsgård Nielsen</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/superwood-a-s</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.superwood.dk/</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Hampen (Ikast-Brande), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/superwood-as/hampen/savbrug-og-h%C3%B8vlerier/0FQL2II01F8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Skagerak Denmark A/S</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi indoor/outdoor</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Utile lordo 53,7 M DKK ≈ 7,2 M€ nel 2021 (39,2 M DKK nel 2020) / 40 dip. – 33 FTE dic. 2022 (estatistik.dk, CVR 28855990); fatturato non pubblicato. Stima ricavi ~15-22 M€: da verificare</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Josef Theodor Kaiser</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg, Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>https://estatistik.dk/virksomhed/skagerak-denmark-as/28855990</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>TIMBERMAN DENMARK A/S</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>22 dipendenti. Fatturato non pubblicato nelle fonti consultate; ultimo esercizio 2025: risultato ante imposte 43,07 M DKK (~5,8 M€), risultato netto 33,6 M DKK, patrimonio netto 72,4 M DKK — indicatori coerenti con una fascia di ricavi nel target. CVR 25776380, costituita 01.12.2000, sede Havnevej 11, 9560 Hadsund. Codice NACE: commercio all'ingrosso di legno e materiali da costruzione. LEGAME DI GRUPPO: controllata da Timberman Holding ApS; nel CdA figurano Lovisa Märtha Maria Krantz e il presidente Fredrick John Sylva (azionariato nordico).</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Mogens Albæk Fisker</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.timberman.dk/</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Hadsund (Mariagerfjord), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/timberman-denmark-as/hadsund/t%C3%B8mmer-tr%C3%A6last-og-byggevarer-agentur-og-engros/GL4I5LI10LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>VERMUND LARSEN A/S (VELA / VERMUND)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute e tavoli (contract/healthcare)</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>≈150 dip. in 5 paesi (2026, da.wikipedia/azienda); utile d'esercizio 17,1 M DKK nel bilancio 2025 (lasso.dk); fatturato non pubblicato. Azienda di confine verso l'alto (stima ricavi ~25-40 M€) ma indipendente, di proprietà della famiglia Larsen</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Per Buus</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/vela-vermund-larsen</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://vermund.eu/</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg SV, Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>https://lasso.dk/firmaer/52796628/vermund-larsen-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>SKOVS KORN A/S. KORN- OG FODERSTOFAGENTUR</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — trading korn og foderstof</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>8 dipendenti; bruttofortjeneste 12 M DKK (2025) ≈ 1,6 M€. Fatturato non pubblicato (societa' di agenzia/intermediazione: il volume intermediato e' molto superiore al margine iscritto a bilancio). Presidente CdA: Hans Ove Skov. Fonte: proff.dk / lasso.dk, dati 2025. CVR 10309905. TAGLIA SOTTO IL TARGET sui dati pubblicati.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Christian Petersen</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Vejle, Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/skovs-korn-as.-korn-og-foderstofagentur/vejle/jordbrugsr%C3%A5varer-levende-dyr-tekstilr%C3%A5varer-og-indsatsvarer-agentur/064Z69I10OL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>ALL CREATIVE A/S</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>11-50 dipendenti (LinkedIn/proff.dk). CVR 21124796, NACE 172100 (fremstilling af bølgepap, pap og emballage af papir og pap), sede Islevdalvej 214, unità anche a Vejle e Havndal. Fatturato NON pubblicato su fonti verificabili: dato di fatturato da confermare su CVR/regnskab. ATTENZIONE: probabile fascia sotto i 10 M€ target.</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/allcreativedk</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://allcreative.dk/</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Rødovre (Hovedstaden)</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/all-creative-as/r%C3%B8dovre/papir-og-papirprodukter-produktion/GSG8C7I10K1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>BOXEN EMBALLAGE A/S</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>31 dipendenti; bruttofortjeneste (margine lordo) 17 mio DKK nel 2024 (~2,3 M€ di margine lordo, cambio 7,46). CVR 31155975, NACE 172100, Bøgildsmindevej 3. Fatturato non pubblicato (classe contabile B): stima fascia 5-15 M€ da confermare. Gruppo di 3 società, capogruppo CRHJ Holding ApS (controllo familiare, indipendente).</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Christian Rune Passer Jørgensen</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Administrerende direktør</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.boxenemballage.dk/</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Nørresundby (Nordjylland)</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/boxen-emballage-as/n%C3%B8rresundby/producenter/GQAW39I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>BUCHS A/S</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>27 specialisti in Buchs A/S; il gruppo (Buchs + Buchs Labels, Randers/Silkeborg/Ho Chi Minh City) si avvicina a 100 dipendenti. CVR 29845646. Produzione interna oggi all'80% imballaggi; dal 2023 nuova tipografia di etichette (Buchs Labels A/S). Fatturato non pubblicato: DA VERIFICARE su regnskab; fascia stimata 5-15 M€ a livello di gruppo.</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Henrik Olesen</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/buchs-a-s</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://buchs.dk/</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Randers SV (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/buchs-as/randers-sv/trykeritjenester/GKN0O3I07QV</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>COLOR LABEL A/S</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>13 dipendenti; bruttofortjeneste 14,756 mio DKK nel 2024 (~2,0 M€ di margine lordo), risultato ante imposte 5,169 mio DKK. CVR 15136901, Vejlbjergvej 14, fondata 1991. Produzione di etichette autoadesive. SOTTO SOGLIA: fatturato stimato ben sotto i 10 M€, probabilmente vicino o sotto i 5 M€. Capogruppo Color Label Holding ApS.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Erik Grønning</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Fondatore e direttore</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.colorlabel.dk/</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Risskov, Aarhus (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/color-label-as/risskov/b%C3%B8ger-aviser-og-blader-engros/090FPHI10MF</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>EMBALLAGEFABRIKKEN THY PAP</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>n.d. - nessun dato di fatturato o addetti reperito su fonte verificabile. Produttore di imballaggi in cartone e astucci con oltre 25 anni di attività, lavora anche come terzista per tipografie; sede Industrivej 19 B, 7700 Thisted. DA VERIFICARE su CVR: ragione sociale esatta, dimensione e referente.</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://thy-pap.dk/</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Thisted (Nordjylland)</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>https://thy-pap.dk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>H. EMBALLAGE ApS</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>21 dipendenti; ricavi/margine lordo dichiarati 9,211 mio DKK (~1,2 M€). CVR 38528742, NACE 172100, Højrupvej 11. SOTTO SOGLIA: ampiamente al di sotto della fascia minima 5 M€ - lead marginale, incluso solo perché già segnalato come lead parziale da verificare.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Glamsbjerg, Assens (Syddanmark)</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/h.-emballage-aps/glamsbjerg/papir-og-papirprodukter/GWNSLZI0ZDH</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>IKAST ETIKET A/S</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>12 dipendenti; risultato netto 7,62 mio DKK nell'ultimo bilancio (prec. 8,3 mio DKK), patrimonio netto 10,9 mio DKK. CVR 10402980, Neptunvej 6, fondata 1986. SOTTO SOGLIA: fatturato non pubblicato ma dimensione ampiamente sotto i 5 M€ - lead piccolo. Consiglio amministrazione: Benny Nørmark Nyborg, Ulrik Lauritsen, Henning Hausted (nessun adm. direktør pubblicato).</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ikastetiket.dk/</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Ikast, Ikast-Brande (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/ikast-etiket-as/ikast/engroshandel-annet/GJF022I10N6</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>JOHNSEN GRAPHIC SOLUTIONS A/S (oggi anche Johnsen Print &amp; Digital Media A/S)</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>92 dipendenti. CVR 18624141, Bakkehegnet 3, fondata 1995. Capogruppo Johnsen + Holding A/S (controllo familiare danese, indipendente). Fatturato non pubblicato su fonte verificabile: con 92 addetti nel settore grafico la fascia stimata è 10-20 M€, DA CONFERMARE su regnskab. NB: sotto la stessa CVR compare anche la denominazione Johnsen Print &amp; Digital Media A/S.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/johnsen-offset-a-s</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>https://johnsen.dk/</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Grenaa, Norddjurs (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/johnsen-graphic-solutions-as/grenaa/trykeritjenester/0B36H9I07QV</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>KAILOW A/S</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>28 dipendenti; bruttofortjeneste 18 mio DKK nel 2024 (~2,4 M€ di margine lordo). CVR 15945672, Floras Allé 11, fondata 1992. Capogruppo KAILOW GRUPPEN A/S (indipendente, familiare). Fatturato non pubblicato: stima fascia 5-10 M€ - AZIENDA DI CONFINE, al di sotto del target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Jørgen Kailow</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Direktør (capogruppo KAILOW GRUPPEN A/S)</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Vanløse, København (Hovedstaden)</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/kailow-as/vanl%C3%B8se/trykeritjenester/09HRRCI07QV</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>KLS PUREPRINT A/S</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>41 dipendenti. CVR 13918783, Jernholmen 42A. Tipografia certificata Cradle2Cradle, storica azienda familiare (ex K. Larsen &amp; Søn). LEGAME DI GRUPPO: capogruppo F. E. BORDING A/S (gruppo grafico danese quotato) - la decisione di acquisto potrebbe essere centralizzata. Fatturato non pubblicato a livello di controllata.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/klspureprint</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://klspureprint.dk/</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Hvidovre (Hovedstaden)</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/kls-pureprint-as/hvidovre/trykeritjenester/GJRDH3I07QV</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>MC EMBALLAGE A/S</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>79-87 dipendenti; bruttofortjeneste 110 mio DKK (~14,7 M€ di margine lordo). CVR 10887194, Delta 3, fondata 1987, engroshandel di imballaggi (incl. carta/cartone). Azienda a proprietà dei dipendenti (medarbejdereje), indipendente. AZIENDA DI CONFINE: essendo distributore, il fatturato è verosimilmente &gt;40 M€ - verificare regnskab prima di classificarla nel target.</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Peder Kristian Eriksen</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mcemballage.dk/</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Hinnerup, Favrskov (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/mc-emballage-as/hinnerup/grossister/06HCM2I10NS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>ODENSE SEGLMÆRKEFABRIK A/S</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>15 dipendenti (unità produttiva). CVR 17620487, Cikorievej 8, fondata 1964, settore papir og papirprodukter (sigilli/etichette in carta). SOTTO SOGLIA: dimensione ampiamente sotto i 5 M€ - lead piccolo, incluso per completezza della filiera etichette/carta.</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Odense SØ (Syddanmark)</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/odense-seglm%C3%A6rkefabrik-as/odense-s%C3%B8/papir-og-papirprodukter/GKEKGVI0ZDH</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>SCANLUX PACKAGING A/S</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>28-38 dipendenti (fonti divergenti); bruttofortjeneste 22,0 mio DKK 2023 vs 19,4 mio DKK 2022 (~2,9 M€ di margine lordo). CVR 71051218, Kratbjerg 308, attività registrata come engroshandel/imballaggi. Capogruppo Kornelius II ApS. DA VERIFICARE: quota effettiva di imballaggi in carta/cartone rispetto ad altri materiali; fatturato non pubblicato.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Jan Kornelius Pedersen</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Administrerende direktør</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Fredensborg (Hovedstaden)</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/scanlux-packaging-as/fredensborg/engroshandel-annet/16AVGYI10N6</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>SKJERN PAPER A/S (già Skjern Papirfabrik A/S)</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartiera</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>75 dipendenti; produzione ~70.000 t/anno di carta (dato 2021). Proprietà Buur Invest A/S + dirigenti operativi (indipendente danese dal 2005). Fatturato non reperito su fonte verificabile: con questi volumi è AZIENDA DI CONFINE, plausibilmente sopra i 40 M€ - verificare regnskab prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/skjern-papirfabrik-a-s</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Skjern, Ringkøbing-Skjern (Midtjylland)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://energiforskning.dk/medlemmer/skjern-papirfabrik-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>STIBO COMPLETE A/S (già Rosendahls A/S - Print Design Media)</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>150 dipendenti; fatturato ~200 mio DKK (~26,8 M€, cambio 7,46). CVR 37120928, Oddesundvej 1. AZIENDA DI CONFINE: sopra la fascia 10-20 M€ ma dentro il tollerabile 5-40 M€. LEGAME DI GRUPPO: ex Rosendahls, acquisita e ridenominata Stibo Complete A/S nel 2022 (gruppo Stibo, danese, fondazione).</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Søren Schønberg Henriksen</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Administrerende direktør</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Esbjerg N (Syddanmark)</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/rosendahls-as-print-design-media/esbjerg-n/trykeritjenester/GKF0WAI07QV/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>STOK EMBALLAGE K/S</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>100-200 dipendenti complessivi (62 a Langeskov, 10 a Vejle); bruttofortjeneste 146 mio DKK nel 2024 (~19,6 M€ di solo margine lordo). CVR 16427284, NACE 172100, Erik Stoks Allé 4. Capogruppo STOK Denmark ApS. AZIENDA DI CONFINE / SOPRA FASCIA: il fatturato è verosimilmente &gt;50 M€ - da verificare prima del contatto, potenzialmente da escludere.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Martin Frederiksen</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Administrerende direktør</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.stok.dk/</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Langeskov, Kerteminde (Syddanmark); stabilimento bølgepap a Middelfart</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/stok-emballage-ks/langeskov/papir-og-papirprodukter/09S3DGI0ZDH</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>CAFÉU DENMARK ApS</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — engros B2B</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Bruttofortjeneste 7,3 mio. DKK nell'ultimo bilancio disponibile (+421% in 5 anni); dipendenti non pubblicati. Fonte: food-supply.dk / proff.dk. SOTTO IL TARGET. · CVR 33243537</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Esbjerg N (Storstrømsvej 42, 6715), Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/caf%C3%A9u-denmark-aps/esbjerg-n/kaffe-og-te-agentur-og-engros/GT4AIYI0Z8T</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Copenhagen Coffee Lab ApS</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione/engros B2B</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>16 dipendenti; risultato ante imposte ~4,7 mio. DKK es. 2024; utile 2023 1,3 mio. DKK (2 mio. DKK nel 2022). Fatturato non pubblicato. Fonte: proff.dk. SOTTO IL TARGET. · CVR 40207929</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Allan Krogsgaard Nielsen</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>https://copenhagencoffeelab.com/en</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>København SV (Bådehavnsgade 44F, 2450), Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/copenhagen-coffee-lab-aps/k%C3%B8benhavn-sv/producenter/GXVBRXI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>DANSK KAFFE ApS</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — import/export caffè verde</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Micro-impresa: capitale sociale 80 t.DKK; dipendenti e fatturato non pubblicati nelle fonti consultate. Codice NACE 463700 (engros di caffè, tè, cacao e spezie); oggetto sociale: import/export di caffè. Fonte: proff.dk. SOTTO IL TARGET ma importatore puro. · CVR 25081544</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Jens Erik Nielsen</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Odense C (Filosofgangen 9, 5000), Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>https://proff.dk/firma/dansk-kaffe-aps/odense-c/kaffe-og-te-agentur-og-engros/0EXL1KI0Z8T</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Estate Coffee Copenhagen A/S</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + cacao/cioccolato</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>10-20 dipendenti; bruttofortjeneste 10 mio. DKK (bilancio 2021); fatturato non pubblicato. Costituita nel 1994. Fonte: paqle.dk / proff.dk / retailnews.dk. SOTTO IL TARGET ma doppia commodity EUDR (caffè + cacao). · CVR 18179407</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Anders Laursen</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Administrerende direktør (subentrato a Steen Aalund Olsen)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr"/>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Haarby (Assens), Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/roller/estate-coffee-copenhagen-as/haarby/producenter/GLOZ6AI016D/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>I.M. FRELLSEN K/S (Frellsen Kaffe &amp; Te / Frellsen Chokoladefabrik)</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde + cacao/cioccolato</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato aggregato ~300 mio. DKK (~40 M€) nel 2022; dipendenti riportati tra 476 e 550 a seconda della fonte (include rete retail). Fonte: proff.dk / sn.dk. AL LIMITE SUPERIORE del range tollerabile; doppia commodity EUDR (caffè verde + cacao) - lead ad alta priorità. · CVR 25340604</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Peter Muldorff Frellsen</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Direktør (con Henrik Muldorff Frellsen)</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Roskilde (Industrivej 14, 4000), Regione Sjælland</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/i-m-frellsen-kaffe-te/roskilde/n%C3%A6rings-og-nydelsesmidler-produktion/GM5KIDI10JW</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Just Coffee</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde bio + torrefazione</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>n.d. - impresa familiare, torrefazione propria; importa direttamente caffè verde certificato bio e sostenibile. Fatturato e dipendenti non pubblicati nelle fonti consultate. Fonte: sito aziendale / drypdryp.dk. Probabilmente SOTTO IL TARGET; operatore EUDR (import diretto). · ragione sociale CVR non verificata</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.justcoffee.dk/</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Jyllinge (Roskilde), Regione Sjælland</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.justcoffee.dk/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Kontra A/S (KONTRA Coffee)</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione/engros (import caffè verde)</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>28-29 dipendenti nell'unità produttiva di Hvidovre + 8 nel punto vendita di København Ø; fatturato non pubblicato nelle fonti consultate. Attiva dal 2005. Fonte: proff.dk. SOTTO IL TARGET (stima &lt;10 M€) ma torrefattore/importatore strutturato. · CVR 56312412</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/kontra-coffee</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>https://www.kontracoffee.com/</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Hvidovre (Jernholmen 45E, 2650) - punto vendita København Ø, Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/kontra-as/hvidovre/kaffe-og-te-agentur-og-engros/H0B8BKI0Z8T</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>La Cabra Risteri ApS (gruppo La Cabra)</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Unità risteri: 59 dipendenti (CVR 43681176, costituita 01/11/2022). Fatturato di gruppo La Cabra 150 mio. DKK (~20 M€) es. 2023/24, raddoppiato sull'anno precedente (33 mio. DKK a marzo 2022); ~50% del fatturato da USA. Fonte: fodevarewatch.dk + proff.dk. IN TARGET.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Esben Hageneier Piper</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Direktør / co-fondatore e comproprietario del gruppo La Cabra</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Nordhavn, København (Århusgade 118X, 2150), Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/la-cabra-risteri-aps/nordhavn/producenter/0Q08M0I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Nordic Coffee House ApS</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — engros e import</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>n.d. - fatturato e dipendenti non pubblicati nelle fonti consultate. Registrata nella categoria 'Kaffe og te - agentur og engros'. Fonte: proff.dk. Taglia probabilmente sotto il target: da verificare. · CVR 39807122</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Kolding, Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/nordic-coffee-house-aps/kolding/kaffe-og-te-agentur-og-engros/GXLJKUI0Z8T</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>The Coffee Collective A/S</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Nettoomsætning 81,1 mio. DKK (~10,9 M€) es. 2023/24, +14,2% su 71,1 mio. DKK; risultato ante imposte 1,8 mio. DKK. Dipendenti n.d. Fonte dati di bilancio 2023/24 (find-virksomhed.dk / proff.dk). IN TARGET. · CVR 30706595</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="3" t="inlineStr"/>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr"/>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Frederiksberg / København, Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://find-virksomhed.dk/firma/the-coffee-collective-a-s-30706595</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>AALBORG CHOKOLADEN ApS</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>32 dipendenti; bruttofortjeneste 7,37 mio. DKK e risultato ante imposte 0,25 mio. DKK (2024). Fatturato non pubblicato. Capogruppo: ASLAK COMPANY ApS. Fonte: proff.dk. SOTTO IL TARGET (micro/piccola). · CVR 29842957</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>John Aslak Jensen</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg Øst (Troensevej 4M, 9220), Regione Nordjylland</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/aalborg-chokoladen-aps/aalborg-%C3%B8st/n%C3%A6rings-og-nydelsesmidler/GQUFGRI116S</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>COPENHAGEN CHOCOLATE FACTORY ApS</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 48,3 mio. DKK (~6,5 M€) nell'ultimo esercizio disponibile; 20-50 dipendenti. Costituita nel 2010. Fonte: vainu.com (dati CVR) / paqle.dk / proff.dk. Nel range tollerabile inferiore.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Kastrup (Tårnby), Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>https://search.vainu.com/company/copenhagen-chocolate-factory-aps-omsaetning-og-noegletal/DK32761844/virksomhedsoplysninger</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>PETER BEIER CHOKOLADE A/S</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>64 dipendenti medi (dato di bilancio riportato, in crescita da 56); risultato netto 1,96 mio. DKK (+25% a/a) e patrimonio netto 13,4 mio. DKK nel bilancio citato dalle fonti. Fatturato non pubblicato. Fonte: proff.dk / sn.dk / food-supply.dk. Probabilmente sotto il target. · CVR 26058007</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Peter Beier</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Direktør / fondatore</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr"/>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Helsingør (Ørsholtvej 35A, 3000), Regione Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/peter-beier-chokolade-as/helsing%C3%B8r/udleje/0FIIHJI01TD</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>PR CHOKOLADE A/S</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione ed engros</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>46 dipendenti; bruttofortjeneste 17 mio. DKK (2024). Fatturato non pubblicato. Costituita 29/05/2000; NACE 463600 (engros zucchero/cioccolato) + 108200 (fabbricazione cacao e cioccolato). Fonte: proff.dk / lasso.dk. Sotto il target. · CVR 25391462</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Kim Lund Bennedbæk Clausen</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Kolding (Kokbjerg 29A, 6000), Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/pr-chokolade-as/kolding/producenter/GLUG9CI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>SPANGSBERG CHOKOLADE A/S / Spangsberg Chokoladefabrik A/S</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>100-200 dipendenti (di cui 38 nell'unità produttiva di Taastrup); bruttofortjeneste 38 mio. DKK (2024) e 34 mio. DKK (2023); fatturato non pubblicato ma coerente con il target 10-20 M€. Presidente CdA: Peter Ernst Wengler-Jørgensen. Produzione e commercio di flødeboller, cioccolato e dolciumi. Fonte: proff.dk / paqle.dk. · CVR 26458005</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Michael Spangsberg</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Taastrup (Taastrupgårdsvej 16-22, 2630), Regione Hovedstaden - unità anche a Esbjerg N</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/spangsberg-chokoladefabrik-as/taastrup/producenter/GSWDT2I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Summerbird A/S</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>193-221 dipendenti a seconda della fonte; bruttofortjeneste 63,7 mio. DKK (2022) e 79,0 mio. DKK (2021); risultato 2024 8,0 mio. DKK (7,3 mio. DKK nel 2023). Fatturato non pubblicato: stimabile ~150-200 mio. DKK (~20-27 M€) sulla base di margine e organico, ma NON verificato. Presidente CdA: Peter Eriksen Jensen. Fonte: proff.dk / estatistik.dk / fyens.dk. · CVR 24209644</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Mikael Grønlykke</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Administrerende direktør (dal 03/08/2009)</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Assens (Fyn), Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/summerbird-as/assens/producenter/GN6UXHI016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Xocolatl Christiansfeld ApS</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione ed engros</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>56 dipendenti (fonte paqle: 50-100); bruttofortjeneste 15 mio. DKK (2024), 14,5 mio. DKK (2023), 12,7 mio. DKK (2022). Fatturato non pubblicato. Capogruppo: MINKO INVEST ApS. Fonte: proff.dk. Sotto il target ma con produzione propria da cacao. · CVR 34458375</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Gitte Kohls</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Administrerende direktør</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr"/>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Haderslev (Storegade 11A, 6100) - produzione a Hejls, Regione Syddanmark</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/xocolatl-christiansfeld-aps/haderslev/producenter/0KIK93I016D</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>AVK GUMMI A/S</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); bruttofortjeneste 105 mio DKK (~14,1 M EUR) nel 2023; 231 dipendenti. ATTENZIONE: dimensione possibilmente sopra la fascia target. Fonti: proff.dk (CVR 55375313), paqle.dk, anno 2023</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Peter Lorentzen</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr"/>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.avkgummi.dk/</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Låsby (area Galten/Skanderborg), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/avk-gummi-as/l%C3%A5sby/gummi-og-plastprodukter/GKL15SI10NU</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>DANSK GUMMI INDUSTRI A/S</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato nelle fonti consultate (n.d.); ca. 40-62 dipendenti; utile 2025 ca. 16 mio DKK (~2,1 M EUR). Fonti: proff.dk (CVR 35405909) e jv.dk, anno 2025</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr"/>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/dansk-gummi-industri</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>https://danskgummi.com/</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Kolding (Profilvej 18, 6000), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/dansk-gummi-industri-as/kolding/gummi-og-plastprodukter/GUH82GI10NU</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>H.C. JACOBSEN A/S</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); bruttofortjeneste 3,2 mio DKK (~0,4 M EUR) nel 2025. ATTENZIONE: sotto la fascia target. Fonte: proff.dk (CVR 75144911), anno 2025</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Bjarni Engelhardt Andersen</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr"/>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>https://hcemballage.dk/</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Ganløse/Stenløse (Sandbakken 5, 3660), Region Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/h.c.-jacobsen-as/stenl%C3%B8se/gummi-og-plastprodukter/GKU06AI10NU</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>RG ROM GUMMI A/S</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); bruttofortjeneste 53 mio DKK (~7,1 M EUR) nel 2023; 71-80 dipendenti. Fonti: proff.dk (CVR 76653313), romgummi.dk, anno 2023</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Jesper Berg Kristensen</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør (CEO)</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://romgummi.dk/</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Lemvig, Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/rg-rom-gummi-as/lemvig/gummi-og-plastprodukter/19MY2PI10NU</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Rubberproff ApS</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato e dipendenti non pubblicati nelle fonti accessibili); societa attiva dal 2019. Fonte: proff.dk (CVR 40465790)</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="inlineStr"/>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>https://rubberproff.dk/</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Hals (Ulstedvej 36, 9370), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/rubberproff-aps/n%C3%B8rresundby/engroshandel-annet/GY1KTSI10N6</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>SKANDINAVISK DÆK IMPORT A/S</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Gomma</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato e dipendenti non pubblicati nelle fonti accessibili). Fonte: proff.dk (CVR 87222810)</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør/ejer</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>mg@sdi.dk</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>https://sdi.dk/</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Havdrup (Industrivænget 14, 4622), Region Sjælland</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>https://sdi.dk/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>A-ONE DANMARK ApS</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e numero dipendenti non pubblicati (ApS, bilancio in forma ridotta). Fonte: proff.dk (consultato 2026). CVR 33390971. Mangimi per scrofe e suinetti fino a 30 kg; parte del gruppo nordirlandese Devenish (quindi NON indipendente, ma entita' danese di taglia PMI).</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Jesper Skjøtt</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>http://www.a-one-danmark.dk/</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Skive, Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/a-one-danmark-aps/skive/korn-r%C3%A5tobak-s%C3%A5varer-og-fodervarer-engros/GT8V6GI10P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>AB NEO A/S (già AGRO KORN A/S)</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>57 dipendenti (fonte proff.dk/erhvervplus.dk, 2025; altre fonti 50-100). Fatturato non pubblicato; risultato negativo -13 M DKK (es. 01/09/2023-31/08/2024) e -57 M DKK (es. 01/09/2024-31/08/2025). CVR 37404241. Produzione di mangimi completi per animali da allevamento. ATTENZIONE: controllata del gruppo britannico AB Agri/ABF - entita' danese di taglia PMI ma non indipendente.</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Jesper Riisgaard Nielsen</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Videbæk (Ringkøbing-Skjern), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/ab-neo-as/videb%C3%A6k/foder/0M9PAPI00FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>CEBECO FOURAGE A/S</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — kraftfoder bovini da latte</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 10,8 M DKK ≈ 1,4 M€ (ultimo esercizio disponibile); 1 dipendente. TAGLIA MOLTO SOTTO IL TARGET (micro-impresa commerciale). Presidente CdA: Meindert Tjoelker. Fonte: proff.dk / Vainu. CVR 19628841. Commercio all'ingrosso di cereali e materie prime per mangimi; mangimi concentrati per vacche da latte.</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Johannes Josef Westenbroek</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr"/>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>https://cebeco.dk/</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Kibæk (Herning), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/cebeco-fourage-as/kib%C3%A6k/korn-r%C3%A5tobak-s%C3%A5varer-og-fodervarer-engros/0BOPPLI10P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>COMPEX ApS</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — minerali/premix zootecnici</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato e numero dipendenti non pubblicati (ApS, bilancio in forma ridotta). Presidente CdA: Steen Jørgensen. Fonte: proff.dk (consultato 2026). CVR 33748450. Registrata NACE 46210 (ingrosso cereali/sementi/mangimi); importa minerali per zootecnia dalla Germania - rilevanza EUDR-soia da verificare (piu' orientata a minerali e attrezzature per bovini da latte).</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Jonni Drost Hahn</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>https://compex.dk/</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Bolderslev (Aabenraa), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/compex-aps/bolderslev/n%C3%A6rings-og-nydelsesmidler/0K3CGYI116S/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>CR FODERSERVICE K/S</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>16 dipendenti (2025); bruttofortjeneste 8,94 M DKK (2024) ≈ 1,2 M€, era 10,21 M DKK (2023); risultato 0,53 M DKK. Fatturato NON pubblicato (K/S, bilancio ridotto): la dimensione effettiva del giro d'affari e' verosimilmente superiore ma non documentabile. Fonte: proff.dk / lasso.dk, dati 2024. CVR 33078366. Miscelazione mangimi con unita' mobili presso l'allevamento (hjemmeblanding), acquisto di soia/materie prime proteiche.</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Niels Frost Rasmussen</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Direktør (fondatore)</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>https://cr-f.dk/</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Bogense (Nordfyn), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/cr-foderservice-ks/bogense/jordbrug/GT1OQ7I10OF/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>NORDVEST FODER A/S</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (su proff.dk il campo omsaetning risulta '-'); numero dipendenti n.d. Societa' controllata da Jysk Agri Holding A/S. Fonte: proff.dk (consultato 2026). CVR 14333045. Commercio all'ingrosso di cereali, sementi e materie prime per mangimi (NACE 46210) - operatore EUDR potenziale su soia.</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr"/>
+      <c r="E82" s="5" t="inlineStr"/>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/nordvest-foder-a-s</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nordvestfoder.dk/</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Vestervig (Thisted, Thy), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/nordvest-foder-as/vestervig/n%C3%A6rings-og-nydelsesmidler/GJSZAMI116S</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>NUTRIMIN A/S</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>66 dipendenti; bruttofortjeneste 41,98 M DKK (2022, era 55,31 M DKK nel 2021), risultato netto 8,82 M DKK (2022). Fatturato non pubblicato (bilancio in forma ridotta) - taglia stimata nella fascia PMI ma DA VERIFICARE. Fonte: proff.dk, dati 2022. CVR 28513518. Terzo fornitore danese di premix vitaminico-minerali, concentrati, mangimi per suinetti e latte per vitelli (uso di soia/proteine vegetali).</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Torben Jensen</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/nutrimin-a-s</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nutrimin.dk/</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Ans By (Silkeborg), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/nutrimin-as/ans-by/foder/0GZ566I00FB</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>DRAGSBÆK A/S</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato non pubblicato nelle fonti accessibili); produttore di margarina, oli vegetali e grassi speciali; controllata di Orkla Food Ingredients Denmark A/S. ATTENZIONE: dimensione probabilmente sopra la fascia target. Fonte: proff.dk (CVR 89318718)</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Christian Munk</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Adm. direktør</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>https://dragsbaek.dk/</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Thisted (Tilstedvej 73, 7700), Region Nordjylland</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/dragsb%C3%A6k-as/thisted/mejerivarer-%C3%A6g-madolie-og-fedt/1H6ERII10PV</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Naturli' Foods</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Olio di palma</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato e dipendenti non pubblicati nelle fonti accessibili); produttore plant-based che dichiara l'uso di olio di palma certificato RSPO in parte della gamma; parte del gruppo Dragsbæk</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.naturli-foods.dk/</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Vejen, Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.naturli-foods.com/faq/oils/</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>TBC INGREDIENTS ApS</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); bruttofortjeneste 10,27 mio DKK (~1,4 M EUR); 4-5 dipendenti; importatore/rivenditore di oli vegetali con l'olio di palma come componente principale. Fonti: proff.dk (CVR 28119666) e piano d'azione palma su etiskhandel.dk (2021)</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Jens Aksel Christensen</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>Odder (Knudsminde 3B, 8300), Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>https://etiskhandel.dk/wp-content/uploads/Palmeoliehandlingsplan-tbc-ingredients-2021.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>BØJE KØD ENGROS ApS (Bøje &amp; David Kød Engros)</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato e dipendenti non pubblicati nelle fonti accessibili); grossista di carne per ristorazione/mense dal 2000. Fonte: proff.dk (CVR 25588037)</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bojekod.dk/</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>Kastrup (Kirstinehøj 75, 2770), Region Hovedstaden</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.proff.dk/firma/b%C3%B8je-k%C3%B8d-engros-aps/kastrup/k%C3%B8d-og-vildt-engros/GO2BIII10OV</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Grambogård</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 45 mio DKK (~6,0 M EUR); macello/lavorazione carni con linea bovina da manze e manzi. Fonte: effektivtlandbrug.landbrugnet.dk, articolo 2023</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Niels Beier</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Direktør</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>https://grambogaard.dk/</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Tommerup (Fyn), Region Syddanmark</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>https://effektivtlandbrug.landbrugnet.dk/artikler/svin/85640/-det-handler-om-smag-og-kvalitet</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>JN Meat International</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (n.d.); 70 dipendenti; sezionamento proprio di carne bovina e di vitello (marchio SASHI). Fonti: jnmeat.dk e LinkedIn aziendale</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>John Nielsen</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Stifter (fondatore)</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/jnmeat</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>https://jnmeat.dk/</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Slagelse, Region Sjælland</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>https://jnmeat.dk/en</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Randers Kød Engros ApS</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>n.d. (fatturato e dipendenti non pubblicati nelle fonti accessibili); grossista di carne dal 1976, gamma con oksekød/kalvekød</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr"/>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>https://randerskoed.dk/</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Randers, Region Midtjylland</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>https://randerskoed.dk/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J90"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId74"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Svezia: foglio nel workbook (89 aziende, email 71/89)
- arricchimento contatti: email da 33 a 71 su 89, sito 87/89, LinkedIn 48/89
- workbook: 5 fogli, 454 righe (IT 95, DE 97, FI 84, DK 89, SE 89)
- MyEUDR_CONTINUA.md: stato Svezia, rifiniture aperte e lezioni operative
  (lanciare 2-3 agenti per volta, salvataggio incrementale, insidia KSEK/MSEK)
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -11,12 +11,14 @@
     <sheet name="Germania" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Finlandia" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Danimarca" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Svezia" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Italia'!$A$2:$J$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Germania'!$A$2:$J$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Finlandia'!$A$2:$J$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18627,4 +18629,4641 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J91"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyEUDR — Lead mapping · Svezia · aziende potenzialmente soggette all'EUDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Denominazione</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Filiera EUDR</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Dimensione (fatt./dip.)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Ruolo</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Email / PEC</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Sito web</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tärnsjö Garveri Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — conceria al vegetale di pelli bovine, pelletteria</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 51.898 KSEK (~4,6 M€) e 43 dipendenti — bilancio 2024 (fonte bolagsfakta/allabolag); org.nr 556474-7797. Sotto la soglia minima ideale: in Svezia le concerie sono pochissime e questa è la principale conceria indipendente attiva.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Ulrika Andersson</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>info@tarnsjogarveri.se</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://tarnsjogarveri.com/</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Tärnsjö (Heby), Uppsala län</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5564747797-Tarnsjo_Garveri_Aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Abstracta AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi acustici per ufficio</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 254 028 KSEK = 254,0 MSEK ≈ 22,5 M€ (2024); 63 dipendenti (2024; 67 nel 2023); org.nr 556046-3852 – fonte allabolag.se. Azienda di confine: sopra il target ideale ma entro la fascia tollerabile. Legame di gruppo: controllata del gruppo quotato Lammhults Design Group AB (564 MSEK consolidati, 160 addetti)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Yngvi Fridriksson</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/abstracta-ab</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>info@abstracta.se</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>https://abstracta.se/</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Lammhult (Växjö), Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hitta.se/verksamhet/abstracta-ab-llpyjcouv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Karlaträ</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria di conifere</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>≈7,9 M€ / 12 dip. (allabolag: 89 711 KSEK) · org.nr 556081-8782 · sotto la fascia target 10-20 M€, tenuta per copertura · produzione ~40 000 m³/anno</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>info@karlatra.se</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://karlatra.se/</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Bottnaryd (Jönköping), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5560818782/aktiebolaget-karlatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Balungstrands Sågverk AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e trävaror</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>≈10,1 M€ / 38 dip. (allabolag 2025: 114 525 KSEK) · org.nr 556637-7171 · legame di gruppo: controllata di Green Wood Sverige AB (stessa proprietà di Bäckebrons e Nordanå Trä) · calo -70,1% sul 2024, verificare durata esercizio</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Stefan Gillberg</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>VD (extern VD)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/balungstrands-s%C3%A5gverk-ab</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>info@balung.se</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://balung.se/</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Enviken (Falun), Dalarnas län</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/balungstrands-s%C3%A5gverk-ab/enviken/s%C3%A5gverk/2K22S43I5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Baseco Golv Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 110.032 KSEK (~9,7 M€) e 31 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556295-1953. Al limite inferiore del target. Produzione di pavimenti in legno, pannelli a parete e casette in legno.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>info@baseco.se</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.baseco.se</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Sorsele, Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/baseco-golv-aktiebolag/sorsele/tr%C3%A4varor/2K01D75I5YI6G</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Blå Station Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute e arredi contract</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 152 046 KSEK = 152,0 MSEK ≈ 13,5 M€ (2024); risultato 10 284 KSEK; 26 dipendenti (2024); org.nr 556272-1091 – fonte allabolag.se. Pienamente in target. Legame di gruppo: capogruppo Blå AB (2 società)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Jens Johan Lindau</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/blastation</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>info@blastation.se</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.blastation.se/</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Åhus (Kristianstad), Skåne län</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/bl%C3%A5-station-aktiebolag/%C3%A5hus/m%C3%B6bler/2JZWF2BI5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Brattby Sågverks AB</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria di conifere</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>≈12,7 M€ / 32 dip. (allabolag/bolagsfakta 2024: 143 413 KSEK, +25,6%) · org.nr 556415-5066 · membro SÅGAB-Sågverken Norrland · target ideale</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Marie Bergstrand</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/brattby-s-gverks-ab</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>info@brattbysagverk.se</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.brattbysagverk.se/</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Vännäs, Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5564155066/brattby-sagverks-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Brännfors Träförädling Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e lavorazione legno</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>≈7,0 M€ / 17 dip. (allabolag 2025: 79 011 KSEK; 2024: 53 348 KSEK con 15 dip.) · org.nr 556103-8695 · sotto la fascia target 10-20 M€, tenuta per copertura · membro SÅGAB</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>https://brannforstraforadling.se/</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Ostvik/Kåge (Skellefteå), Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/br%C3%A4nnfors-tr%C3%A4f%C3%B6r%C3%A4dling-aktiebolag/k%C3%A5ge/s%C3%A5gverk/2JYWCX3I5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Bröderna Anderssons Industrier i Ekenässjön Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 92 224 KSEK = 92,2 MSEK ≈ 8,2 M€ (2024, +10,4%); risultato 3 599 KSEK; 52 dipendenti (2024); org.nr 556066-4129 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile. Legame di gruppo: capogruppo Ekenäs Design AB. Rilevante EUDR su due commodity (legno struttura + pelle rivestimenti)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Jan Sven Inge Andersson</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/br%C3%B6derna-anderssons-m%C3%B6bler</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>shop@brodernaanderssons.se</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://brodernaanderssons.se/</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Ekenässjön (Vetlanda), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/br%C3%B6derna-anderssons-industrier-i-eken%C3%A4ssj%C3%B6n-aktiebolag/eken%C3%A4ssj%C3%B6n/m%C3%B6bler-produktion/2JYOBWHI63IJF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Bäckebrons Sågverk Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e piallatura</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>≈12,6 M€ / 39 dip. (allabolag 2025: 142 474 KSEK) · org.nr 556099-7008 · NOTA: nel 2023 il fatturato era 326 MSEK (≈29 M€), calo -66,7% nel 2025 (possibile esercizio ridotto) · legame di gruppo: controllata di Green Wood Sverige AB, capogruppo Ziegler Holding GmbH</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Stefan Gillberg</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/b%C3%A4ckebrons-s%C3%A5gverk-ab</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>stefan.gillberg@backebronssagverk.se</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.backebronssagverk.se/</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Västra Ämtervik (Sunne), Värmlands län</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/b%C3%A4ckebrons-s%C3%A5gverk-aktiebolag/v%C3%A4stra-%C3%A4mtervik/s%C3%A5gverk/2JYVGR4I5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Drömtrappor AB</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — scale in legno per edilizia</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 83.213 KSEK (~7,4 M€) e 74 dipendenti nel 2025 (fonte allabolag.se). Org.nr 556309-7038 (ex Trätrappor Norsjö AB). Sotto il target 10-20 M€ ma dentro la fascia tollerata.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Johan Jonsson</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>johan.jonsson@dromtrappor.se</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dromtrappor.se</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Norsjö, Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/dr%C3%B6mtrappor-ab/norsj%C3%B6/tr%C3%A4varor/2K04H5AI5YI6G</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Ekstrands Dörrar &amp; Fönster AB</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — finestre e porte in legno</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 167.769 KSEK (~14,8 M€) e 84 dipendenti nel 2025 (fonte allabolag.se). Org.nr 556570-0621. Pienamente in target. Capogruppo: Ekstrand &amp; Son Aktiebolag (gruppo di 6 società).</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Heidi Ekstrand</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>info@ekstrands.com</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ekstrands.com</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Osby, Skåne län</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5565700621/ekstrands-dorrar-fonster-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Fegens Sågverk AB</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e piallatura</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>≈16,8 M€ / 28 dip. (allabolag 2025: 189 377 KSEK) · org.nr 556080-4857 · produzione ~65 000 m³/anno · target ideale</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Johan Andersson</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://ca.linkedin.com/company/fegens-s%C3%A5gverk-ab</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>info@fegenssag.se</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://fegenssag.se/</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Smålandsstenar (Gislaved), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://allabolag.se/5560804857/fegens-sagverk-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Fogia Collection Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili e imbottiti di design</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 108 304 KSEK = 108,3 MSEK ≈ 9,6 M€ (2024); risultato 15 276 KSEK; 18 dipendenti (2024; 21 nel 2023); org.nr 556204-6218 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile. Operatore di brand/immissione sul mercato (SNI commercio all'ingrosso mobili): tipico soggetto EUDR come 'operatore'. Legame di gruppo: capogruppo Scandinavian Design Partners AB</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Franz Marcus Huber</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/fogia</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>info@fogia.se</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fogia.com/</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Nacka, Stockholms län</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/fogia-collection-aktiebolag/nacka/belysningsarmatur-komponenter/2JZHYBUI5YCO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Glimakra of Sweden AB</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi acustici per ufficio</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 165 564 KSEK = 165,6 MSEK ≈ 14,7 M€ (2024, -6,4%); 78 dipendenti (2024); org.nr 556120-7837 – fonte allabolag.se. Pienamente in target. Legame di gruppo: controllata di Garpco AB, con 2 sub-controllate; ha acquisito Fanerami Sweden (impiallacciature)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Anders Barrklint</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/glimakra-of-sweden-ab</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>info@glimakra.com</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>https://glimakra.com/</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Glimåkra (Östra Göinge), Skåne län</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/glimakra-of-sweden-ab/glim%C3%A5kra/m%C3%B6bler/2JYZZFHI5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Gyllsjö Träindustri AB</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imballaggi in legno/pallet</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 303.142 KSEK (~26,8 M€) e 82 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556083-9671. Sopra il target ideale ma dentro la fascia tollerata 5-40 M€. Gruppo di 4 società (85 addetti, 352 MSEK).</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Björn Olsson Lissner</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>info@gyllsjo.se</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://gyllsjo.se</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Klippan, Skåne län</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/gyllsj%C3%B6-tr%C3%A4industri-ab/klippan/lastpallar-lastmateriel/2JYS3CNI5YFTZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Gärsnäs Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute in legno massello</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 81 448 KSEK = 81,4 MSEK ≈ 7,2 M€ (2024); 29 dipendenti (2024; 37 dip. e 80 711 KSEK nel 2023); org.nr 556044-4746 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile. Legame di gruppo: controllata di Bordet i Stockholm AB. Nota: discordanza VD risolta – il sito ufficiale garsnas.se ('Ny vd på Gärsnäs') annuncia Magnus Eriksson VD dal 1/1/2023, subentrato a Dag Klockby (ora presidente del CdA); il registro riporta il nome completo Karl Johan Magnus Leifsson Eriksson</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Magnus Eriksson</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör dal 1° gennaio 2023, annuncio ufficiale garsnas.se)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/g%C3%A4rsn%C3%A4s</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>info@garsnas.se</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>https://garsnas.se/</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Gärsnäs (Simrishamn), Skåne län</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/g%C3%A4rsn%C3%A4s-aktiebolag/g%C3%A4rsn%C3%A4s/m%C3%B6bler/2JYJMMII5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Hjältevadshus AB</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — case in legno prefabbricate</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 140.766 KSEK (~12,5 M€) e 86 dipendenti nel 2025 (fonte allabolag.se). Org.nr 556232-9135. Pienamente in target. Azionista di controllo: gruppo Pulsen (dal 2011).</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Johan Bynell</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>johan.bynell@hjaltevadshus.se</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hjaltevadshus.se</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Hjältevad (Eksjö), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/hj%C3%A4ltevadshus-ab/hj%C3%A4ltevad/tr%C3%A4varor/2JZO0MNI5YI6G</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Horreds Möbel Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi contract e per ufficio</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 103 MSEK ≈ 9,1 M€ (esercizio 2022, +77% sul 2021); 50 dipendenti (2022, +11 sull'anno precedente); org.nr 556365-1974 – fonte allabolag.se / Mark-Posten. ATTENZIONE: dato non aggiornato al 2024, da riverificare. Fa parte di un gruppo di 3 società</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Per Ola Johansson</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/horreds-m-bel-ab</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>info@horreds.se</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.horreds.se/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Horred (Mark), Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/horreds-m%C3%B6bel-aktiebolag/horred/butiksinredningar-butiksutrustningar/2K0GDC6I5YDBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Johanson Design Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute e arredi contract</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 251 117 KSEK = 251,1 MSEK ≈ 22,2 M€ (2024); 70 dipendenti (2024; 80 a marzo 2025); org.nr 556358-5206 – fonte allabolag.se. Azienda di confine: leggermente sopra il target ideale 10-20 M€ ma entro la fascia tollerabile 5-40 M€</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Dan Mikael Johansson</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör) e presidente del CdA</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/johanson-design-ab/</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>info@johansondesign.se</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://johansondesign.com/</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Markaryd, Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/johanson-design-aktiebolag/markaryd/m%C3%B6bler/2K0EXTII5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Kvänum Kök AB</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 297 420 KSEK = 297,4 MSEK ≈ 26,3 M€ (ultimo esercizio disponibile); EBITDA 39 520 KSEK; 127 dipendenti; org.nr 556202-3159 – fonte allabolag.se. Azienda di confine: sopra il target ideale ma entro la fascia tollerabile 5-40 M€. Legame di gruppo: capogruppo Vedena AB</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Johan Niklas Efraimsson</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/kvanum</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>info@kvanum.com</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kvanum.com/se/</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Kvänum (Vara), Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/kv%C3%A4num-k%C3%B6k-ab/kv%C3%A4num/m%C3%B6bler/2JZHGJBI5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Lammhults Möbel Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili per ufficio e contract</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 95 362 KSEK = 95,4 MSEK ≈ 8,4 M€ (2024, -19,2%); risultato -31 368 KSEK; 41 dipendenti (2024; 45 nel 2023); org.nr 556058-2602 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile. Legame di gruppo: controllata del gruppo quotato Lammhults Design Group AB</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Beatrice Kortner Henriksson</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/lammhults-m-bel-ab</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>info@lammhults.se</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.lammhults.se/</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Lammhult (Växjö), Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/lammhults-m%C3%B6bel-aktiebolag/lammhult/m%C3%B6bler/2JYMKZUI5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Lars Carlsson Trävaru Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e commercio legname</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>≈6,2 M€ / 14 dip. (allabolag 2024: 70 552 KSEK) · org.nr 556093-1734 · sotto la fascia target 10-20 M€, tenuta per copertura · azienda familiare dal 1901</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>info@carlssontra.se</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.carlssontra.se/</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Älmeboda (Tingsryd), Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/lars-carlsson-tr%C3%A4varu-aktiebolag/%C3%A4lmeboda/s%C3%A5gverk/2JYU2DYI5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Leksandsdörren AB</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — porte in legno</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 69.543 KSEK (~6,2 M€) e 30 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556651-7891. Sotto il target 10-20 M€ ma dentro la fascia tollerata 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Per Anders Jäderberg</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>info@leksandsdorren.se</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>https://www.leksandsdorren.se</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Leksand, Dalarnas län</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5566517891/leksandsdorren-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>N K Lundströms Trävaror Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e trävaror</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>≈18,6 M€ / 34 dip. (allabolag 2024: 210 533 KSEK, +3,9%) · org.nr 556107-8154 · capogruppo KGL Trä Aktiebolag · membro SÅGAB · azienda familiare dal 1931 · target ideale</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Karl Ulf Peter Lundström</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/nkltra</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>info@nkltra.se</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nkltra.se/</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Tväråbäck (Vännäs), Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5561078154/n-k-lundstroms-travaror-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>NC Nordic Care AB</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi per strutture sanitarie</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 79 707 KSEK = 79,7 MSEK ≈ 7,1 M€ (2025); risultato 166 KSEK; 14 dipendenti; org.nr 556249-9177 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile. Attività di produzione mobili ufficio + commercio all'ingrosso (SNI 46471): rilevante come operatore EUDR</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Jörgen Johannesson</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör) e styrelseledamot</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/nc-nordic-care-ab</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>info@ncnordiccare.se</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ncnordiccare.se/</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Tranås, Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/bokslut/nc-nordic-care-ab/tran%C3%A5s/m%C3%B6bler/2JZRNU1I5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Nissabo AB</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — pannelli lamellari/limfog</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 80,4 MSEK (~7,1 M€) nel 2024 e ~18 addetti (fonte woodnet.se/allabolag.se; 64.874 KSEK e 7 dipendenti registrati nel 2023). Org.nr 556959-4681. Sotto il target ma dentro la fascia tollerata; azienda in forte crescita.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Folke Åkesson</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>offert@nissabo.se</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>https://nissabo.se</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Broaryd (Gislaved), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/nissabo-ab/broaryd/tr%C3%A4varor/2K3ZQRDI5YI6G</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Nola Industrier AB</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredo urbano e outdoor</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 86 155 KSEK = 86,2 MSEK ≈ 7,6 M€ (2024, -2,6%); risultato 2 629 KSEK; 22 dipendenti; org.nr 556207-4442 – fonte allabolag.se. Sotto il target ideale ma entro la fascia tollerabile</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Claes Henrik Edlund</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/nola-industrier</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>info@nola.se</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nola.se/</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Stockholm, Stockholms län</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/nola-industrier-ab/stockholm/kontorsinredningar/2JZIK3UI5YF48</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Nordanå Trä Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e selvicoltura</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>≈10,4 M€ / 25 dip. (allabolag 2025: 117 660 KSEK) · org.nr 556134-5751 · legame di gruppo: controllata di Green Wood Sverige AB (come Bäckebrons e Balungstrands) · calo -52,2%, verificare durata esercizio</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Patrik Siljemark</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>VD (extern VD)</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/nordan%C3%A5-tr%C3%A4-ab</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>patrik@nordanatra.se</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>https://nordanatra.se/</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Alfta (Ovanåker), Gävleborgs län</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/nordan%C3%A5-tr%C3%A4-aktiebolag/alfta/s%C3%A5gverk/2JZ2XUFI5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Norrgavel AB</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 127 986 KSEK = 128,0 MSEK ≈ 11,3 M€ (2024, +22,9%); risultato -8 606 KSEK; 62 dipendenti (2024); org.nr 556491-3381 – fonte allabolag.se. Pienamente in target. Produzione affidata a falegnamerie in Småland, Skåne, Baltico e Bosnia: catena di fornitura legno estesa, alto interesse EUDR</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Sofie Richter</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, in condivisione con David Richter – david.richter@norrgavel.se)</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/norrgavel-ab</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>sofie.richter@norrgavel.se</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>https://norrgavel.se/</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Malmö, Skåne län (assemblaggio e finitura a Lammhult)</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/norrgavel-ab/malm%C3%B6/m%C3%B6bler/2K17EN9I5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Norrlands Trä Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — piallatura e pannelli</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>≈24,3 M€ / 41 dip. (allabolag 2025: 275 049 KSEK; 44 dip. nel 2024) · org.nr 556092-4077 · membro SÅGAB · fascia alta del range tollerabile</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Jan Anders Nivfors</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/norrlands-tra</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>order@norrlandstra.com</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.norrlandstra.com/</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Älandsbro (Härnösand), Västernorrlands län</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5560924077/norrlands-tra-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Nydala Trävaru Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e piallatura</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>≈28,6 M€ / 41 dip. (allabolag 2023: 323 425 KSEK; 2022: 364 MSEK) · org.nr 556075-2825 · azienda di confine sulla fascia alta del range tollerabile · segheria familiare dal 1908, ~100 000 m³/anno</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Karl Ingemar Lindman</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>https://dk.linkedin.com/company/nydala-tr%C3%A4varu-ab</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>mail@nydalatra.se</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://nydalatravaru.se/</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Vrigstad (Sävsjö), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/nydala-tr%C3%A4varu-aktiebolag/vrigstad/s%C3%A5gverk/2JYQ8C9I5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Olle Dahl Såg Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e lavorazione legno</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>≈11,6 M€ / 16 dip. (allabolag 2025: 131 298 KSEK, -8,0%) · org.nr 556139-2910 · target ideale</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Jonas Dahl</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>info@olledahlsaw.se</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.olledahlsaw.se/</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Hästveda (Hässleholm), Skåne län</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5561392910/olle-dahl-sag-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Rödins Trä AB</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e trävaror</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>≈33,7 M€ / 37 dip. (allabolag 2025: 380 291 KSEK, +2,7%) · org.nr 556331-1801 · azienda di confine sulla fascia alta del range tollerabile · membro SÅGAB · 1 controllata</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Lars Gunnar Markus Rödin</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/r%C3%B6dins-tr%C3%A4-ab</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>info@rodinstra.se</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.rodinstra.se/</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Svenstavik (Berg), Jämtlands län</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/r%C3%B6dins-tr%C3%A4-ab/svenstavik/s%C3%A5gverk/2K092UXI5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Rörvikshus Sweden AB</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — case in legno prefabbricate</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 154.918 KSEK (~13,7 M€) e 49 dipendenti (fonte allabolag.se, ultimo bilancio disponibile). Org.nr 556622-0926. Pienamente in target. Capogruppo: Munio Sweden Aktiebolag.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Carl Johan Michael Svensson</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör esterno)</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>info@rorvikshus.se</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>https://rorvikshus.se</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Rörvik (Sävsjö), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/r%C3%B6rvikshus-sweden-ab/r%C3%B6rvik/hus/2K1ZFJYI5YF6Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Sjöbergs Workbenches AB</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — banchi da lavoro e componenti</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 67 063 KSEK = 67,1 MSEK ≈ 5,9 M€ (2024; 60 142 KSEK nel 2023); 27-29 dipendenti; org.nr 556085-1825 – fonte allabolag.se. Azienda di confine: appena sopra la soglia minima di 5 M€. Legame di gruppo: capogruppo Idun Woodcraft AB; controllata Svenska Hyvelbänkar. Produzione di banchi, mobili e componenti in legno massello</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Anders Olsson</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/sj%C3%B6bergs-workbenches-ab</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>office@sjobergs.se</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://sjobergs.se/</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Stockaryd (Sävsjö), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/sj%C3%B6bergs-workbenches-ab/stockaryd/tr%C3%A4varor/2JYSCQ9I5YI6G</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Skaraborgs Träförädling Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e piallatura</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>≈30,2 M€ / 29 dip. (allabolag 2023: 341 232 KSEK, -12,4%; 28 dip. dato aziendale) · org.nr 556261-5657 · azienda di confine sulla fascia alta del range tollerabile · hyvleri familiare dal 1985</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Per-Anders Lennart Andersson</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/skaraborgs-tr%C3%A4f%C3%B6r%C3%A4dling-ab</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>per@traforadling.se</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>https://traforadling.se/</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Töreboda, Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5562615657/skaraborgs-traforadling-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Småland Timber AB</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e lavorazione legno</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>≈14,6 M€ / 26 dip. (allabolag 2023: 164 742 KSEK; 2022: 187 418 KSEK con 31 dip.) · org.nr 556136-0248 · ex Rydaholms Träförädling AB · target ideale</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Bernt Göte Martinsson</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>bernt.martinsson@smalandtimber.se</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://smalandtimber.se/</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Rydaholm (Värnamo), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/sm%C3%A5land-timber-ab/rydaholm/s%C3%A5gverk/2JZ3914I5YHTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Stockhult Glommers Timber AB</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e essiccazione</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>≈26 M€ / 15 dip. (fatturato 296,6 MSEK, riconoscimento Gasell Dagens Industri; allabolag 2020: 98 352 KSEK) · org.nr 556579-8435 · crescita +269% in 4 anni, azienda di confine sulla fascia alta · produzione ~70 000 m³/anno</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Paul Björnsson</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/glommers-timber-ab</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>info@glommerstimber.se</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.glommerstimber.se/</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Glommersträsk (Arvidsjaur), Norrbottens län</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5565798435/glommers-timber-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Stolab Möbel AB</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — sedute e tavoli in massello</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 83,3 MSEK ≈ 7,4 M€ (2024; risultato -5,6 MSEK); 50 dipendenti (2024); org.nr 556182-5224 – fonte allabolag.se / proff.se. Sotto il target ideale ma entro la fascia tollerabile. Ha acquisito Albin i Hyssna (produzione svedese)</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Anders Martin Johansson</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/stolab</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>info@stolab.se</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.stolab.se/</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Smålandsstenar (Gislaved), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/stolab-m%C3%B6bel-ab/sm%C3%A5landsstenar/m%C3%B6bler/2JZD7T4I5YGJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Sunnerbo Fönster AB</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — finestre e porte in legno</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 101.636 KSEK (~9,0 M€) e 40 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556708-7282. Di poco sotto il target 10-20 M€, dentro la fascia tollerata.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Peter Mikael Karlsson</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>info@sunnerbofonster.se</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>https://sunnerbofonster.se</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Nybro, Kalmar län</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/sunnerbo-f%C3%B6nster-ab/nybro/tr%C3%A4varor-produktion/2K2I01EI63IL3</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Swedese Möbler Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno curvato</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 165 761 KSEK = 165,8 MSEK ≈ 14,7 M€ (2024, -1,3%); risultato 4 153 KSEK; 87 dipendenti (2024); org.nr 556280-1323 – fonte allabolag.se. Pienamente in target 10-20 M€</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Julio Patino Suaznabar</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/swedese-m%C3%B6bler-ab</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>info@swedese.se</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.swedese.se/</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Vaggeryd, Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/swedese-m%C3%B6bler-aktiebolag/vaggeryd/m%C3%B6bler-produktion/2JZY4YZI63IJF</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>VårgårdaHus AB</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — case in legno prefabbricate</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 151.086 KSEK (~13,4 M€) e 53 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556477-6911. Pienamente in target. Fa parte del gruppo SVENSKA HUSCOMPAGNIET AB (7 società).</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Martin Ravn-Nielsen</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>info@vargardahus.se</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vargardahus.se</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Vårgårda, Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/v%C3%A5rg%C3%A5rdahus-ab/v%C3%A5rg%C3%A5rda/tr%C3%A4varor-produktion/2K14HCFI63IL3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Willa Nordic AB</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — case in legno prefabbricate</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 208.856 KSEK (~18,5 M€) e 63 dipendenti nel 2024 (fonte allabolag.se). Org.nr 556361-9161. Pienamente in target.</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Klas Fridsäll</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>klas.fridsall@willanordic.se</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>https://willanordic.se</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Stockaryd (Sävsjö), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/willa-nordic-ab/stockaryd/tr%C3%A4-och-byggvaror-grossist/2K0FO0PI63IL2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Woodsafe Timber Protection AB</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — legno ignifugo per edilizia</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 76.742 KSEK (~6,8 M€) e 24-29 dipendenti nel 2024 (fonte allabolag.se/bolagsfakta.se). Org.nr 556630-5321. Sotto il target 10-20 M€ ma dentro la fascia tollerata.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/woodsafe-timber-protection</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>kundtjanst@woodsafe.com</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.woodsafe.se</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Västerås, Västmanlands län</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5566305321/woodsafe-timber-protection-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>ZilenZio AB</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — pannelli e pareti acustiche</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 123,4 MSEK ≈ 10,9 M€ (esercizio 2025; 106 963 KSEK nel 2023); risultato operativo 9,1 MSEK; 20 dipendenti (2023), 28 a livello di gruppo; org.nr 556651-5689 – fonte allabolag.se/proff.se. Pienamente in target</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Hans Robert Bergström</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/zilenzio-ab</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>info@zilenzio.se</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://zilenzio.com/</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Örebro, Örebro län</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/zilenzio-ab/%C3%B6rebro/kontorsinredningar/2K25QZTI5YF48</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Älgsjö Såg AB</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria di conifere</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>≈12,2 M€ / 12 dip. (allabolag 2025: 137 399 KSEK, +13,1%) · org.nr 556341-1577 · capogruppo Älgsjö Invest AB · membro SÅGAB · target ideale · VD non pubblicato (Jörgen Törnqvist risulta styrelseledamot)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>info@algsjosag.se</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>http://www.algsjosag.se/</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Ullånger (Kramfors), Västernorrlands län</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5563411577/algsjo-sag-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Åsljunga Pallen Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — pallet e imballaggi legno</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>≈22,6 M€ / 80 dip. (allabolag 2024: 255 909 KSEK) · org.nr 556093-5156 · maggior produttore svedese di pallet (HS 4415, Allegato I EUDR) · fascia alta del range tollerabile</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Lars Stefan Nilsson</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/%C3%A5sljunga-pallen-ab</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>info@asljungapallen.se</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.asljungapallen.se/</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Örkelljunga, Skåne län</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/%C3%A5sljunga-pallen-aktiebolag/%C3%B6rkelljunga/tr%C3%A4varor-produktion/2JYU510I63IL3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Halmstads Gummifabrik</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — stampaggio articoli tecnici in gomma (industria, marine, mining, tenute)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 282.998 KSEK (~25,0 M€) e 81 dipendenti — bilancio 2024 (fonte allabolag/bolagsfakta); org.nr 556051-6188. Sopra la fascia ideale ma entro il tollerabile.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Christian Kiks</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ab-halmstads-gummifabrik</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>info@hgf.se</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hgf.se/</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Halmstad, Hallands län</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5560516188/aktiebolaget-halmstads-gummifabrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Däckteam i Sverige Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — catena/centrale acquisti pneumatici e cerchi (oltre 160 officine affiliate)</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 172.964 KSEK (~15,3 M€) e 6 dipendenti — bilancio 2024 (fonte bolagsfakta/allabolag); org.nr 556390-4837. In pieno target di fatturato; struttura centrale snella (rete di officine affiliate).</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Martin Tillsten</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/d-ckteam-i-sverige-ab</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>info@dackteam.se</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>https://www.dackteam.se/</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Malmö, Skåne län</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5563904837-Dackteam_i_Sverige_Aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Puratos Sweden AB</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import e distribuzione cioccolato/cacao per panificazione e pasticceria</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 121,5 MSEK (~10,8 M€) 2024 (+9,1%); 9 dipendenti (fonte: allabolag.se / bolagsfakta.se, bilancio 2024). Org.nr 556842-9715. Filiale svedese del gruppo Puratos (BE); fornisce cioccolato (Belcolade) e cacao a bagerier/konditorier.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.puratos.se/</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Vellinge / Malmö (Skåne län)</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/puratos-sweden-ab/vellinge/livsmedel/2K3ARV7I5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Rubber Company, R. Holmquist Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — distribuzione e lavorazione articoli industriali in gomma (tubi, trasmissioni, vulcanizzazione)</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 118.377 KSEK (~10,5 M€) e 39-42 dipendenti — ultimo esercizio disponibile 2024/2025 (fonte allabolag/bolagsfakta); org.nr 556068-0448. In pieno target.</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Per Holmqvist</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/rubber-company-ab</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>rubber@rubberco.se</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>https://www.rubberco.se/</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Vallentuna, Stockholms län</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5560680448/rubber-company-r-holmquist-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Billes Tryckeri AB</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 248.036 KSEK (~22,0 M€) e 99 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 559063-9349. AZIENDA DI CONFINE: appena sopra il target 10-20 M€, ben dentro la fascia tollerabile. Tipografia indipendente a controllo familiare (collegata a Billes Tryckeri Förvaltning AB, org.nr 556259-9034). E-mail diretta VD pubblicata nelle fonti: niklas.bille@billes.se.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Niklas Wilhelm Bille</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>info@billes.se</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.billes.se/</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Mölndal, Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/billes-tryckeri-ab/m%C3%B6lndal/tryckerier/2KGISXHI5YI3L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Bording AB</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 91.326 KSEK (~8,1 M€) e 42 dipendenti — fonte allabolag/bolagsfakta, es. 2023. Org.nr 556239-7090. AZIENDA DI CONFINE: sotto il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Nota: la stessa entità compare anche come Bording PurePrint AB; legame con il gruppo danese Bording.</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Björn Andersson</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>info@bording.se</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>https://bording.se/</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Borås, Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/bording-ab/bor%C3%A5s/tryckerier/2JZPH2AI5YI3L</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Econopack Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 127.623 KSEK (~11,3 M€) e 10 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556262-9211. IN TARGET per fatturato, ma organico ridotto (modello distributivo/commerciale su soluzioni di imballaggio). Nota legame di gruppo: capogruppo S-Pack AB.</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Per Marcus Liljevall</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>VD (extern verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/econopack</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.econopack.se/</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Mölndal, Västra Götalands län</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5562629211/econopack-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Jinnestål Etikett AB</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 68.020 KSEK (~6,0 M€) e 24 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556654-3418. AZIENDA DI CONFINE: sotto il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Etichettificio (etikettryckeri) indipendente, presidenza Peter Klingberg.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Gustav Klingberg</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>https://www.jinnestal.se/</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Helsingborg, Skåne län</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5566543418/jinnestal-etikett-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Kartongbolaget i Hälsingborg Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi cartone</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 137.281 KSEK (~12,1 M€) e 46 dipendenti — fonte allabolag/bolagsfakta, es. 2025. Org.nr 556075-7071. IN TARGET. Produzione di imballaggi in carta e cartone, con e senza stampa. Nota legame di gruppo: gruppo di 3 società, capogruppo Joliwa i Allerum AB.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Torsten Joakim Johansson</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>info@kartongbolaget.se</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>https://kartongbolaget.se/</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Helsingborg, Skåne län</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/kartongbolaget-i-h%C3%A4lsingborg-aktiebolag/helsingborg/pappersvaror/2JYQBM7I5YG1W</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Klippans Bruk AB</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartiera</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 264.323 KSEK (~23,4 M€) e 54 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556530-3228. AZIENDA DI CONFINE: sopra il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Cartiera (produzione di carta e locazione immobili), sede Bruksallén 9, Klippan, tel. 0435-291 00; presidente Stefan Uno Sundh, VD attuale non pubblicato nelle fonti consultate. Il sito web non è stato confermato dalle fonti consultate (lo stabilimento opera storicamente anche sotto l'insegna Svenska Pappersbruket AB).</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Klippan, Skåne län</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/klippans-bruk-ab/klippan/producenter/2K1FRGCI63IK3</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Lenanders Grafiska AB</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 122.940 KSEK (~10,9 M€) e 42 dipendenti — fonte allabolag/bolagssoket, es. 2024. Org.nr 556323-6776 (da riverificare: fonti aggregate riportano numerazioni divergenti). IN TARGET. Nota legame di gruppo: collegata a Scandinavian Print Group (proprietà danese); VD non pubblicato nelle fonti consultate — in cda risultano Henrik Corvenius Frydendahl ed Esben Mols Kabell.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/lenanders-grafiska-ab</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>info@lenanders.se</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lenanders.se/</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Kalmar, Kalmar län</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bolagssoket.se/foretag/lenanders-grafiska-ab/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Lessebo Paper AB</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartiera</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 376.018 KSEK (~33,3 M€) e 91 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556955-1616. AZIENDA DI CONFINE: sopra il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Cartiera indipendente (carta e pasta di carta). Nota legame di gruppo: capogruppo Lessebo Finance AB; presidente Karl Göran Johansson.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Jens Olsson</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>VD (extern verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>https://lessebopaper.com/</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Lessebo, Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5569551616/lessebo-paper-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Ljungbergs Tryckeri i Klippan AB</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 144.190 KSEK (~12,8 M€) e 32 dipendenti — fonte allabolag/bolagsfakta, es. 2025. Org.nr 556884-2511. IN TARGET. Nota legame di gruppo: gruppo grafico di 9 società con capogruppo Scanner Colour i Klippan AB (con Norra Skåne Offset AB, Klippans Bokbinderi AB, RST Klippan AB; ~80 addetti complessivi).</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Sofia Ljungberg Igbe</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/ljungbergs-tryckeri-ab</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ljungbergs.se/</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Klippan, Skåne län</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/ljungbergs-tryckeri-i-klippan-ab/klippan/tryckerier/2K3JMDRI5YI3L</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>NPA Nordiskt Papper AB</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — sacchetti carta</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 95.602 KSEK (~8,5 M€) e 29 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556963-0683. AZIENDA DI CONFINE: sotto il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Attività: conversione e vendita di prodotti in carta e politene (sacchetti e borse di carta). Nota legame di gruppo: gruppo di 6 società, capogruppo NPA Gruppen AB.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Mats Werner Lidbeck</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>https://nordisktpapper.se/</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Ljungby, Kronobergs län</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5569630683/npa-nordiskt-papper-ab</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Norbag AB</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — sacchetti carta</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 357.159 KSEK (~31,6 M€) e 121 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556656-1782. AZIENDA DI CONFINE: sopra il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Produttore nordico di shopper e sacchetti di carta per pane e rifiuti organici. Nota legame di gruppo: gruppo di 18 società, capogruppo Tingstad Group AB, capogruppo ultima Danti Invest AB; presidente Dan Paul Jigberg.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Torbjörn Rodhe</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>VD (extern verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.norbag.com/</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Töcksfors (Årjäng), Värmlands län</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/norbag-ab/t%C3%B6cksfors/pappersvaror-produktion/2K26QK6I63IJV</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Pappersgrossisten i Jönköping Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — grossista carta</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 80.655 KSEK (~7,1 M€) e 14 dipendenti — fonte allabolag/bolagsfakta, es. 2024. Org.nr 556323-1132. AZIENDA DI CONFINE: sotto il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Nota legame di gruppo: capogruppo LOLAB Förvaltnings AB.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Jan Olof Helge Larsson</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>https://pg24.se/</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Jönköping, Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5563231132/pappersgrossisten-i-jonkoping-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Svensk Emballageteknik Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi wellpapp</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 158.400 KSEK (~14,0 M€) es. 2025 (156.002 KSEK nel 2024) e 36 dipendenti — fonte allabolag/merinfo. Org.nr 556324-8250. IN TARGET. Attività: progettazione, produzione e vendita di imballaggi in wellpapp (cartone ondulato), polistirolo espanso, legno, flightcases. Nota legame di gruppo: controllata di Team ET AB (8 società, 66 addetti, 263,0 MSEK).</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Göran Rune Forsmark</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>https://et.se/</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Järfälla, Stockholms län</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/svensk-emballageteknik-aktiebolag/j%C3%A4rf%C3%A4lla/f%C3%B6rpackningar-industrin/2K07PTMI5YEN2</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>TMG Tabergs AB</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 101.130 KSEK (~8,9 M€) e 38 dipendenti — fonte allabolag/krafman, es. 2023. Org.nr 556288-4113. AZIENDA DI CONFINE: poco sotto il target 10-20 M€, dentro la fascia tollerabile. Nota legame di gruppo: controllata di Taberg Media Group AB (org.nr 556600-6648, gruppo di 5 società, ~118-130 addetti, ~269 MSEK ≈ 23,8 M€ — il gruppo nel suo insieme è a target).</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Anders Nyström</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>VD (extern verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tmg-tabergs</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>https://tabergmediagroup.se/</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Taberg (Jönköping), Jönköpings län</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/tmg-tabergs-ab/taberg/tryckerier/2JZZWUPI5YI3L</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Bergman &amp; Bergstrand Aktiebolag (Bergstrands Kafferosteri)</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 91,2 MSEK (~8,1 M€) 2024 (+18,5%); 16 dipendenti (fonte: allabolag.se, bilancio 2024). Org.nr 556027-6528. SNI 10830 framställning av te och kaffe. Sotto il target ideale, dentro la fascia tollerabile.</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Fannie Myrén</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bergstrands-kafferosteri</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>info@bergstrands.se</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>https://bergstrands.se/</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Göteborg (Västra Götalands län)</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/bergman-bergstrand-aktiebolag/g%C3%B6teborg/livsmedel/2JYG0TSI5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Johan &amp; Nyström Kafferostare &amp; Tehandlare AB</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde (specialty)</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 196,8 MSEK (~17,4 M€) 2024 (-2,9%); 54 dipendenti (fonte: allabolag.se, bilancio 2024). Org.nr 556657-9446. Nota: dal 2016 controllata da Espresso House (EH Group AB).</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Johan Morén</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/johanochnystrom</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>info@johanochnystrom.se</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>https://johanochnystrom.se/</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Skogås / Huddinge (Stockholms län)</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/johan-nystr%C3%B6m-kafferostare-tehandlare-ab/skog%C3%A5s/kaffe-och-te-agenturer/2K2746UI63IHV</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Kaffekompaniet Din Pauspartner AB</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — engros/wholesale caffè e servizio caffè B2B</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 70,9 MSEK (~6,3 M€) esercizio 2022 (+32,8%); 28 dipendenti (fonte: allabolag.se / hitta.se, bilancio 2022). Org.nr 556317-9554. Gruppo: Miko Koffie NV (Belgio).</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Anders Sjögren</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/kaffekompaniet-din-partner-ab</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>info.goteborg@kaffekompaniet.se</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://kaffekompaniet.se/</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Askim / Göteborg (Västra Götalands län)</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5563179554/bokslut</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Kahls Kaffe Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale (kaffe, te, kakao)</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 344,8 MSEK (~30,5 M€) esercizio 2025 (+32,6%); 47 dipendenti (fonte: allabolag.se). Org.nr 556117-4920. Gruppo: Kahls Holding AB. Sopra il target ideale ma entro la fascia tollerabile (5-40 M€).</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Peter Goodman</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, esterno)</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>info@kahls.se</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>https://www.kahls.se/</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Västra Frölunda / Göteborg (Västra Götalands län)</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/kahls-kaffe-aktiebolag/v%C3%A4stra-fr%C3%B6lunda/kaffe-och-te-agenturer/2JYZA14I63IHV</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Lindvalls Kaffe Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 192,6 MSEK (~17,0 M€) 2024; 181 MSEK 2023; 19 dipendenti (fonte: allabolag.se / bolagsfakta.se, bilanci 2023-2024). Org.nr 556049-5284. Nota: la torrefazione di Uppsala deve lasciare l'immobile entro il 2026 (esproprio Trafikverket).</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Ulf Lindvall</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/lindvalls-kaffe-ab</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>https://lindvallskaffe.se/</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Uppsala (Uppsala län)</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/lindvalls-kaffe-aktiebolag/uppsala/livsmedel/2JYKPMCI5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Lykke Coffee Farms AB</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — coltivazione, import caffè verde + torrefazione</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 57,8 MSEK (~5,1 M€) 2024 (+28,7%); 13 dipendenti (gruppo di 4 società: 23 dipendenti, 55,0 MSEK) (fonte: allabolag.se / bolagsfakta.se, bilancio 2024). Org.nr 556764-1575.</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>https://sv.linkedin.com/company/lykke-coffee-farms</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>oj@lykkegardar.se</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://www.lykkegardar.se/</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Farsta / Stockholm (Stockholms län)</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/lykke-coffee-farms-ab/farsta/jordbruk/2K2TVQFI63IHJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Nordiska Kaffebolaget H. Hansson &amp; Co Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import/agenzia caffè e tè, engros</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 54,7 MSEK (~4,8 M€) 2024 (+8,4%); 17 dipendenti (14 nel 2023) (fonte: allabolag.se, bilancio 2024). Org.nr 556083-2379. SNI 46370 kaffe/te agenturer. Taglia appena sotto la fascia tollerabile ma importatore/agente puro.</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>info@sibyllans.se</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>https://sibyllans.se/</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Stockholm (Stockholms län)</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/nordiska-kaffebolaget-h.-hansson-co-aktiebolag/stockholm/kaffe-och-te-agenturer/2JYRXQ3I63IHV</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Tehuset Java Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — import e commercio caffè e tè (engros + retail)</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 62,4 MSEK (~5,5 M€); 26 dipendenti (fonte: allabolag.se / merinfo.se, ultimo bilancio disponibile). Org.nr 556311-4957. Controllata da Javaimporten i Sverige AB (org.nr 556779-5033, SNI 46370, VD Fredrik August Skeppstedt).</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/tehuset-java</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>order@tehusetjava.se</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>https://www.tehusetjava.se/</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Lund (Skåne län)</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/tehuset-java-aktiebolag/lund/livsmedel/2K04UZ1I5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Cool &amp; Candy</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — engros/wholesale zucchero, cioccolato e confetteria</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 196,7 MSEK (~17,4 M€) esercizio 2022 (+9,0%); 19-22 dipendenti (fonte: allabolag.se / bolagsfakta.se). Org.nr 556330-4137. SNI 46360 partihandel med socker, choklad och sockerkonfektyrer. Fa parte del gruppo Humble Group AB.</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Jens Peter Thomas Persson</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, esterno)</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Ystad (Skåne län)</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/aktiebolaget-cool-candy/ystad/livsmedel-agenturer-och-grossister/2K08WY1I63IIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Candy People AB</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/export ed engros di confetteria e cioccolato</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 251,2 MSEK (~22,2 M€) 2024; 10 dipendenti nella società AB (fonte: allabolag.se / bolagsfakta.se, bilancio 2024). Org.nr 556696-8375. Gruppo di 5 società, capogruppo J &amp; J Holding AB.</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Anna Youssef Bebinno</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/candy-people-ab</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>info@candypeople.com</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>https://candypeople.se/</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Malmö (Skåne län)</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/candy-people-ab/malm%C3%B6/livsmedel/2K2FGAFI5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Delicato Bakverk Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione dolciaria con cioccolato e cacao</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 396,6 MSEK (~35,1 M€) esercizio 2025 (+12,2%); 125 dipendenti (fonte: allabolag.se / bolagsfakta.se). Org.nr 556119-4720. Gruppo di 8 società, capogruppo Belvéns Bageri AB. Entro la fascia tollerabile (5-40 M€).</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Johan Berg</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, esterno)</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/delicato-bakverk-ab</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>info@delicato.se</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.delicato.se/</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Segeltorp / Huddinge (Stockholms län)</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/delicato-bakverk-aktiebolag/segeltorp/livsmedel-tillverkning/2JYZPB4I63IIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Grahns Konfektyr AB</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione confetteria e prodotti di cioccolato</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 259,7 MSEK (~23,0 M€) 2024; 208,6 MSEK 2023; 60-65 dipendenti (fonte: allabolag.se / bolagsfakta.se). Org.nr 556724-8884.</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Eric Jesper Lööw</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, esterno)</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/grahns-konfektyr-ab</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>info@grahns.se</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.grahns.se/</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Skövde (Västra Götalands län)</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/grahns-konfektyr-ab/sk%C3%B6vde/konfektyrer-choklad-/2K2LGQCI5YF14</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Malmö Chokladfabrik AB</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — bean-to-bar, tostatura propria di fave di cacao</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 42,6 MSEK (~3,8 M€) esercizio 2025 (+31,6%); 16 dipendenti (fonte: allabolag.se / bolagsfakta.se). Org.nr 556664-6286. Sotto la fascia tollerabile ma importatore diretto di fave di cacao (tostatura interna) e in forte crescita.</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Roger Stenfeldt</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör, esterno)</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/malm%C3%B6-chokladfabrik-ab</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>order@malmochokladfabrik.se</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>https://malmochokladfabrik.se/</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Oxie / Malmö (Skåne län)</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/malm%C3%B6-chokladfabrik-ab/oxie/livsmedel/2K28JRII5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Svenska Gummihuset Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — commercio all'ingrosso di pneumatici e cerchi (däck och fälg)</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 146.493 KSEK (~13,0 M€) e 12 dipendenti — bilancio 2025 (fonte allabolag/bolagsfakta); org.nr 556750-7297. In pieno target come fatturato; distributore, quindi organico ridotto.</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Joakim Granath</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gummihuset.se/</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Eskilstuna, Södermanlands län</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/5567507297/svenska-gummihuset-aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Tretorn Sweden AB</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — stivali in gomma (gummistövlar), palline da tennis e accessori</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 322.415 KSEK (~28,5 M€) e 48 dipendenti — bilancio 2024 (fonte allabolag/bolagsfakta); org.nr 559012-5695. Sopra la fascia ideale ma entro il tollerabile; capogruppo Thevea Brands Group AB (svedese).</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Vasko Markovski</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>https://se.tretorn.com/</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Helsingborg, Skåne län</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/tretorn-sweden-ab/helsingborg/konfektion/2KG7SLBI63II4</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Johan Hansson</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — produzione mangimi (EDELfoder) e commercio cereali/materie prime proteiche</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 191.871 KSEK (~17,0 M€) e 13 dipendenti — bilancio 2025 (fonte bolagsfakta/allabolag); org.nr 556037-8746. In pieno target di fatturato; organico ridotto tipico del settore mangimi/cereali.</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Jessica Anlér</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>kontakt@johanhansson.se</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>https://johanhansson.se/</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Uppsala, Uppsala län</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5560378746-Aktiebolaget_Johan_Hansson</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Västerbottens Fodercentral</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — fabbrica mangimi composti per bovini/suini, cereali e materie prime</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 170.138 KSEK (~15,1 M€) e 14 dipendenti — bilancio 2022 (fonte bolagsfakta/allabolag); org.nr 556061-1765. In pieno target di fatturato; organico ridotto tipico del settore mangimi.</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>info@fodercentralen.se</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>https://fodercentralen.se/</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Holmsund (Umeå), Västerbottens län</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5560611765-Aktiebolaget_Vasterbottens_Fodercentral</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Forsbecks Eftr. Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — commercio all'ingrosso di cereali, sementi e mangimi per zootecnia</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>ATTENZIONE TAGLIA: fatturato 589.951 KSEK (~52,2 M€) con soli 31-35 dipendenti — bilancio 2022 (fonte allabolag/bolagsfakta); org.nr 556002-3417. Sopra la soglia dei 40 M€ ma è PMI indipendente (famiglia Johansson dal 1953) con fatturato gonfiato dal costo della materia prima (ca. 100.000 t di cereali/anno).</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Per Magnus Johansson</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>per-magnus.johansson@forsbecks.com</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>https://www.forsbecks.se/</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>Skänninge (Mjölby), Östergötlands län</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/forsbecks-eftr.-aktiebolag/sk%C3%A4nninge/grossister/2JYALIXI63IGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Hönryds Kvarn Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — molino e produzione mangimi composti, stoccaggio e commercio cereali</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 198.432 KSEK (~17,6 M€) e 9-11 dipendenti — bilancio 2023 (11 dipendenti nel 2024) (fonte bolagsfakta/allabolag); org.nr 556421-9284. In pieno target di fatturato; organico ridotto tipico del settore mangimi.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>erika@honrydskvarn.se</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.honrydskvarn.se/</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>Morup (Falkenberg), Hallands län</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5564219284-Honryds_Kvarn_Aktiebolag</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Liljeholmens Stearinfabriks AB</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — candele in stearina (stearina di origine vegetale/palma), produzione a Oskarshamn</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 346.300 KSEK (~30,6 M€) nel 2024 e 93-98 dipendenti (93 nel 2023, fatturato 375.373 KSEK) (fonte bolagsfakta/allabolag); org.nr 556041-6348. Sopra la fascia ideale ma entro il tollerabile.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Anna Lundqvist</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>https://se.linkedin.com/company/liljeholmens-stearinfabriks-ab</t>
+        </is>
+      </c>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>anna.lundqvist@liljeholmens.se</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>https://liljeholmens.se/</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Oskarshamn, Kalmar län</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5560416348-Liljeholmens_Stearinfabriks_AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Aktiebolaget Ginsten Slakteri</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macello indipendente (bovini, suini, ovini) e commercio carni</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 227.210 KSEK (~20,1 M€) — bilancio 2024, +18,2% (fonte allabolag/bolagsfakta); org.nr 556257-9861. Nella società capofila risultano 0 dipendenti registrati (personale in società del gruppo). In pieno target di fatturato.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr"/>
+      <c r="F89" s="3" t="inlineStr"/>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ginsten.se/</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Harplinge (Halmstad), Hallands län</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.allabolag.se/foretag/aktiebolaget-ginsten-slakteri/harplinge/livsmedel/2JZTE39I5YFWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Nya Siljans Chark AB</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macello e salumificio (bovini, suini, selvaggina)</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 222.064 KSEK (~19,7 M€) e 81 dipendenti — bilancio 2024 (fonte bolagsfakta/allabolag); org.nr 559256-8256. In pieno target.</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Jonas Björ</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>https://siljanschark.se/</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Mora, Dalarnas län</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5592568256-Nya_Siljans_Chark_AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Närkes Slakteri i Gällersta Aktiebolag</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macello e sezionamento bovini, suini e ovini, intermediazione capi vivi</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 209.054 KSEK (~18,5 M€) e 27 dipendenti — bilancio 2024 (fonte bolagsfakta/allabolag); org.nr 556514-4861. In pieno target.</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Lars Mats Larsson</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>VD (verkställande direktör)</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>info@narkesslakteri.se</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>https://narkesslakteri.se/</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Örebro (Attersta/Gällersta), Örebro län</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bolagsfakta.se/5565144861-Narkes_Slakteri_i_Gallersta_Aktiebolag</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J91"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId206"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Olanda: foglio nel workbook (73 aziende, email 54/73)
- cacao 19, caffe 17, legno 17, carta 11, gomma 4, mangimi/soia 3, palma 2
- workbook: 6 fogli, 527 righe
- 3 filoni interrotti dal limite di quota, da completare (sezione 13 handoff)
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Finlandia" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Danimarca" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Svezia" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Olanda" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Italia'!$A$2:$J$97</definedName>
@@ -19,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Finlandia'!$A$2:$J$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23266,4 +23268,3685 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyEUDR — Lead mapping · Olanda · aziende potenzialmente soggette all'EUDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Denominazione</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Filiera EUDR</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Dimensione (fatt./dip.)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Ruolo</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Email / PEC</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Sito web</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>B.V. Houthandel F. Habraken</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 2-10 dipendenti dichiarati (fonte LinkedIn, 2025). KVK 17047540, BV costituita nel 1951 (attività Habraken Houtimport dal 1952). AZIENDA DI CONFINE: organico piccolo, probabile fatturato sotto i 10 M€. Importatore/grossista voorraadhoudend di hardhout e legname lavorato; dal 2016 sede e magazzino a Vroomshoop (in origine Valkenswaard). Membro VVNH e IKVO.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Frank Habraken</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Eigenaar/directeur</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/habrakenhoutimport</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>info@habrakenhout.nl</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.habrakenhout.nl</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Vroomshoop (Twenterand), Overijssel</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/vroomshoop/000017387744/bv-houthandel-f-habraken.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>BeBo Parket B.V.</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 20 M€ e ca. 90 dipendenti nel gruppo (NL, Belgio, Francia, Germania) — fonte profilo aziendale beboparket.nl, 2024. KVK 08169467. Pienamente in target. Nato come houthandel, oggi tra i maggiori fornitori di parquet dei Paesi Bassi; legame di gruppo con BeBo Groep B.V. (KVK 84481269).</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Frans Bolier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Directeur / mede-eigenaar</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/in/frans-bolier-b64b394a</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>info@beboparket.nl</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.beboparket.nl</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Vriezenveen, Overijssel</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/winkels-in-parket-laminaat-en-kurkvloeren/bebo-parket-b-v-vriezenveen-08169467-000019232209</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Beijleveld Houtimport B.V.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — pannelli/compensato</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 4 dipendenti (fonte company.info / creditsafe, 2025). KVK 24136531. AZIENDA DI CONFINE: organico molto ridotto ma import-trading puro nel porto di Rotterdam (Sluisjesdijk) — importa multiplex/compensato di betulla e conifera, segati e hardboard, produce anche pallet ed imballaggi in legno. Direttore statutario: persona giuridica Beyleveld Groep B.V. (dal 2006), nessun nome fisico pubblicato.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>info@beyleveld.com</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.beyleveldhoutimport.com</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Rotterdam, Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/beijleveld-houtimport-b-v-rotterdam-24136531-000016457986</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>GWW Houtimport B.V.</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato nei registri olandesi (BV con bilancio abbreviato); stima esterna ca. 5 M$ (fonte rocketreach, 2025 — dato non ufficiale, da verificare). 11 dipendenti (fonte rocketreach/creditsafe, 2025). KVK 29051274. TAGLIA SOTTO I 5-10 M€, azienda di confine. Fondata nel 1999, fornitore esclusivamente FSC/PEFC di hardhout tropicale per il settore GWW (opere stradali/idrauliche). Dal 01/01/2026 nello stesso holding (Van den Berg Houtgroep) di Van den Berg Hardhout e GWW Agency. Secondo direttore citato: John Hoogendoorn.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Arjan de Jong</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/gwwhoutimport</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>info@gwwhoutimport.nl</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gwwhoutimport.nl</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Lopik, Utrecht</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/lopik/6368980/gww-houtimport-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Gras Wood Wide B.V.</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 15 dipendenti (fonte sito aziendale / regiobedrijf.nl, 2025). KVK 35015522 (Amsterdam). Fondata nel 1921, sesta generazione familiare; importatore di naaldhout (conifere) certificato, ex 'Houtimport Gras' / 'Houthandel v/h F. &amp; G. Gras', ridenominata nel 2017-2018. Divisioni di vendita Houtimport Gras e NE-Hout (Noord-Europese Houtimport).</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Sven Gras</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Directeur-eigenaar</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>info@graswoodwide.com</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.graswoodwide.com</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Zaandam, Noord-Holland</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.graswoodwide.com/contact/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Hardhouthandel Hotim B.V.</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 2-10 dipendenti dichiarati (fonte LinkedIn / werkenindekempen.nl, 2025). AZIENDA DI CONFINE: organico piccolo, probabile fatturato sotto i 10 M€; n. KVK non reperito nelle fonti consultate. Importatore diretto voorraadhoudend di hardhout africano (import proprio, spedizione, essiccazione, stoccaggio); membro ATIBT.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/hardhouthandel-hotim</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>verkoop@hotim.nl</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hotim.nl</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Middelbeers (Oirschot), Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.atibt.org/en/news/1059/welcome-to-our-new-member-hotim-the-netherlands</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Houthandel Jos Dennebos B.V.</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Numero dipendenti discordante fra le fonti: 20-49 secondo 12build.com (2025), 2-5 secondo oozo.nl — dato da verificare. KVK 05073894, P.IVA NL812769272B01. Opera con il marchio Dennebos Flooring: produttore di parquet multistrato in rovere con stabilimento proprio a Raalte, export in 19 paesi. Socio unico: Jos Dennebos Exploitatie B.V.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>info@dennebosflooring.com</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dennebosflooring.com</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Raalte, Overijssel</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/houthandel-jos-dennebos-b-v-raalte-05073894-000016548884</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Houthandel Wicherson B.V.</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Numero dipendenti non pubblicato nelle fonti consultate (company.info/bedrijvenregister.nl, 2025). KVK 05007831. Attiva dal 1853/1854; dispone di segheria, piallatura, cabina di verniciatura e celle di essiccazione proprie — quindi trasformatore oltre che importatore. Membro VVNH.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Erik Lukas</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>info@wicherson.nl</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.wicherson.nl</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Steenwijk (Steenwijkerland), Overijssel</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/houthandel-wicherson-b-v-steenwijk-05007831-000019069103</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Houtimport Best B.V.</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Numero dipendenti non pubblicato nei registri consultati; team di vendita/acquisti strutturato (fonte sito aziendale, 2025). KVK 74687972. Specialista dal 1960 in import di hardhout, wood specials e plaatmateriaal; Luciën Arends ha rilevato l'azienda nell'aprile 2019 rendendola indipendente. Membro VVNH (Noord-Brabant).</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Luciën Arends</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Directeur/eigenaar</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/houtimportbest</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>info@houtimportbest.nl</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.houtimportbest.nl</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Best, Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/houtimport-best-b-v-best-74687972</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Houtimport Lekkerkerker B.V.</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Numero dipendenti non pubblicato nelle fonti consultate (creditsafe / drimble.nl, 2025). KVK 30147004, BV iscritta dal 1998 (attività dal 2000 con il fondatore Theo Lekkerkerker). Azienda familiare che importa/esporta legname da giardino centro-europeo: ca. 200.000 m³/anno (pino, abete, larice, douglas) — volume compatibile con la fascia 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Guido Lekkerkerker</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Directeur (2a generazione)</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/houtimport-lekkerkerker-b.v</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>houtimportlekkerkerker@planet.nl</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.houtimportlekkerkerker.nl</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Benschop (Lopik), Utrecht</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/benschop/17948002/houtimport-lekkerkerker-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Houtimport Reuver B.V.</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — pannelli/compensato</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 14 dipendenti (fonte company.info / creditsafe, 2025). KVK 12024480, P.IVA NL008890043B01. Fondata nel 1987. Fornitore di plaatmateriaal in legno per interior building, stand, cantieristica da diporto. Algemeen directeur è la persona giuridica Gebrs. Schoolmeesters Holding B.V. (nessun nome fisico pubblicato).</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/hout-import-reuver-bv</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>verkoop@hireuver.nl</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.houtimportreuver.nl</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Reuver (Beesel), Limburg</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/houtimport-reuver-b-v-reuver-12024480-000019946104</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Houtplex B.V.</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Ca. 16 dipendenti (fonte sito aziendale / houtwereld.nl, 2025). KVK 06040971. Importatore di hardhout tropicale da oltre 45 anni (fondata 1977); membro VVNH nella categoria import hardhout e plaatmateriaal. Fa parte del gruppo Wood United.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/houtplex-b.v.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>info@houtplex.nl</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>https://www.houtplex.nl</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Haaksbergen, Overijssel</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.vvnh.nl/vvnh_leden/208</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>L. Verhoeven's Emballagefabriek en Houthandel B.V.</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imballaggi in legno/pallet</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Numero dipendenti non pubblicato nelle fonti consultate; l'azienda si autodefinisce produttore di pallet di media dimensione (fonte sito aziendale, 2025). KVK 24247802. Azienda familiare dagli anni '50, oggi guidata da Leander Jonkers, nipote del fondatore L. Verhoeven. Produce pallet CP, block e stringer pallet e imballaggi su misura.</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Leander Jonkers</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/l.-verhoeven's-emballagefabr.-en-houth.-b.v.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>info@verhoeven-emballage.nl</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://verhoeven-emballage.nl</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Ridderkerk, Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/ridderkerk/18094449/l-verhoeven-s-emballagefabriek-en-houthandel-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>M.S. Pallets B.V.</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imballaggi in legno/pallet</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 6-10 dipendenti (fonte company.info / bedrijvenregister.nl, 2025). KVK 05049728, P.IVA NL808384119B01, costituita nel 1991. TAGLIA PROBABILMENTE SOTTO I 5 M€ — azienda di confine. Produzione/riparazione di pallet in legno e casse per patate, commercio di pallet nuovi e usati. Direttore statutario: persona giuridica Maso Onroerend (nessun nome fisico pubblicato).</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>info@mspallets.nl</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mspallets.nl</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Den Ham (Twenterand), Overijssel</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-houten-emballage/m-s-pallets-b-v-den-ham-05049728-000016563247</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Van Ierssel Houtimport B.V.</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 6-10 dipendenti (fonte oozo.nl / drimble.nl, 2025). KVK 20047459 (BV costituita il 21/09/1984; attività dal 1880). AZIENDA DI CONFINE per organico. Import, groothandel e lavorazione di legname; fa parte della Koninklijke Boogaerdt Groep (legame di gruppo con Boogaerdt Hout, Krimpen aan de Lek). Membro VVNH.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Fred Verver</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-ierssel-houtimport</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>info@vanierssel.nl</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vaniersselhoutimport.nl</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Etten-Leur, Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/etten-leur/000052043266/van-ierssel-houtimport.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Van de Stadt Houtimport B.V.</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Ca. 9 dipendenti (fonte company.info / drimble.nl, 2024). KVK 35004749. Importatore diretto di hardhout tropicale, attivo dal 1936 (radici Zaandam 1694), sede portuale Noorder IJ- en Zeeweg. Trading company: fatturato per addetto elevato, possibile target — organico ridotto, azienda di confine.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>F.B. Gast</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-de-stadt-houtimport-bv</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>info@vandestadt.nl</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vandestadt.nl</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Zaandam, Noord-Holland</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-hout-en-plaatmateriaal/van-de-stadt-houtimport-b-v-zaandam-35004749</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Van den Berg Hardhout B.V.</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 6-8 dipendenti (fonte drimble.nl / bedrijvenregister.nl, 2024). KVK 51971984. AZIENDA DI CONFINE: organico piccolo, probabile fatturato sotto i 10 M€. Dal 01/01/2026 nello stesso holding (Van den Berg Houtgroep) di GWW Houtimport e GWW Agency — legame di gruppo.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Albert Oudenaarden</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/vandenberghardhout</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>info@vandenberghardhout.nl</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vandenberghardhout.com</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Lopik, Utrecht</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/lopik/21946124/van-den-berg-hardhout-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Ascot Amsterdam B.V.</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/trading cacao Ghana</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; numero dipendenti e numero KVK non reperiti da fonti pubbliche accessibili via ricerca. Membro FCC (Federation of Cocoa Commerce). Sede Weteringschans 26, Amsterdam. Ufficio vendite dedicato della Cocoa Abrabopa Association (cooperativa di coltivatori ghanesi): importatore diretto di cacao = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ascot-amsterdam</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>info@ascot-amsterdam.com</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>https://ascot-amsterdam.com/</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cocoafederation.com/the-fcc/fcc-members/ascot-amsterdam-bv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>CocoaSupply B.V.</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/distribuzione semilavorati</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato; numero KVK non reperito da fonte pubblica accessibile via ricerca. Sede Van Nelleweg 1, unit 1.H8A, Rotterdam. Azienda familiare che produce, importa e distribuisce cacao in polvere, burro di cacao, nibs, massa di cacao e couverture industriali; certificazione bio NL-BIO-01. Importatore diretto = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>info@cocoasupply.eu</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://cocoasupply.eu/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Rotterdam (Zuid-Holland)</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://cocoasupply.eu/pages/contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Daarnhouwer &amp; Co B.V.</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/trading cacao</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato: company.info espone solo totale attivo 2024). Trader indipendente di cacao, caffè e frutta secca dal 1908; membro votante FCC (Federation of Cocoa Commerce). KVK 35026025. SBI 46219 / 46370. Operatore EUDR in senso stretto (import cacao da Africa/Asia/America Latina).</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/daarnhouwer-&amp;-co.</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://daarnhouwer.com/</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Zaandam / Zaanstad (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-overige-akkerbouwproducten/daarnhouwer-co-b-v-zaandam-35026025-000017718805</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Dietz Cacao Trading B.V.</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/trading cacao fine</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (deposito abbreviato). 5 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 14046399. Fondata 1992. SBI groothandel in koffie, thee, cacao en specerijen. Trader/broker indipendente di cacao fine per produttori di cioccolato: operatore/commerciante EUDR. Sotto la fascia ideale per organico, ma rilevante per volumi importati.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Jordy Kuijpers</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Sales Director</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>info@dietzcacao.nl</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dietzcacao.nl/</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Heerlen (Limburg)</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/heerlen/heerlen-centrum/heerlen-centrum/171578/dietz-cacao-trading-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Facta International B.V.</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/trading cacao e semilavorati</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). 6-10 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 32119985. Trader di fave di cacao, semilavorati del cacao e caffè; membro FCC. Sede Korte Hogendijk 12, Zaandam (+ ufficio Amsterdam). Organico piccolo ma volumi di trading elevati: operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Ben Dekker</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/facta-international-bv</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://facta-international.com/</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Zaandam / Zaanstad (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/zaanstad/zaandam-west/spoorbuurt/146088/facta-international-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Gaia Cacao B.V.</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/trading fave di cacao</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV giovane, deposito abbreviato); n. dipendenti non pubblicato. KVK 78049636. Attività: acquisto, vendita, import/export, distribuzione e trading di fave di cacao e derivati. Sede Damrak 349, Amsterdam. Azienda piccola/in crescita (sotto la fascia 5-40 M€) ma operatore EUDR diretto in quanto importatore di fave.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/gaia-cacao</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>sales@gaiacacao.com</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gaiacacao.com/</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam / Duivendrecht (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://us.kompass.com/c/gaia-cacao-b-v/nlc0730826/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Kargro Banden B.V.</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — pneumatici e ricostruzione</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (bilancio abbreviato). KVK 30041379, costituita 1968. Sede Heeswijk 135, 3417 GP Montfoort. Raccolta, selezione e lavorazione circolare di carcasse di pneumatici per autocarro/bus, destinate alla ricostruzione (cold retreading) in stabilimenti in NL e BE - filiera gomma naturale Allegato I. LEGAME DI GRUPPO: fa parte di Kargro Group (con Kargro International B.V. e Lintire). Numero dipendenti non pubblicato nelle fonti aperte. Lubertus Gerbrand van Straten risulta gevolmachtigde (procuratore) dal 01/07/2023 secondo Drimble, non 'directeur' - quindi non riportato come referente.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>info@kargro.nl</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>https://kargrobanden.nl</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Montfoort, Utrecht</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/montfoort/17047978/kargro.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Nijsen company B.V.</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — trading granaglie e mangimificio</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 30 M€ con ca. 100 addetti (fonte: Pigbusiness.nl, intervista aziendale 2013; dato più recente non pubblicato — bilancio abbreviato). Il sito aziendale indica oggi un team di oltre 100-125 persone. KVK 14015971. SBI 1091 (vervaardiging van veevoeders). Ex Nijsen/Granico B.V., azienda familiare dal 1938: import/export di granaglie, farine e materie prime (inclusa soia) per mengvoeders + produzione mangimi da flussi residui alimentari. Taglia leggermente sopra il target ma indipendente.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>John Geurts</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/nijsencompany</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>info@nijsen.co</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>https://nijsen.co/</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Veulen / Venray (Limburg)</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-veevoeders/nijsen-company-b-v-veulen-14015971-000015817172</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>PaBrEm B.V.</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — ingrosso/distribuzione prodotti cacao</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato; numero KVK non reperito da fonte pubblica accessibile via ricerca. Fondata nel 2013, sede Rollemastate 11, Leeuwarden. Grossista/distributore internazionale di prodotti a base di cacao e ortofrutta fresca, con attività di export. Azienda piccola: tenuta per copertura del segmento distribuzione cacao fuori dal cluster Amsterdam/Zaanstad.</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>info@pabrem.com</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>https://pabrem.com/</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Leeuwarden (Fryslân)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.europages.co.uk/companies/netherlands/cocoa.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Speerstra Feed Ingredients B.V.</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — import/trading ingredienti mangimistici</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; company.info espone i dati 2024 solo a pagamento). 2-5 dipendenti registrati KVK (fonte: oozo.nl, 2025); ca. 10 persone secondo i profili aziendali. KVK 01085923. Micro-impresa: fatturato verosimilmente sotto i 5 M€ — segnalata come taglia di confine inferiore. Società di trading e import internazionale di ingredienti per mangimi (soia e derivati proteici, cereali): operatore/commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Jan Speerstra</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Directeur / eigenaar</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/speerstra-feed-ingredients-bv</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>mail@speerstra.com</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>https://speerstra.com/</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Eesterga / De Fryske Marren (Friesland)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-akkerbouwproducten-en-veevoeder-algemeen-assortiment/speerstra-feed-ingredients-b-v-eesterga-01085923-000019415834</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Akarton B.V.</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). Oltre 65 dipendenti secondo il sito aziendale; company.info indica 21-50 (fonti karton.nl / company.info, 2025). KVK 12029719. Produttore di imballaggi in cartone ondulato industriale e commerciale, mercati Benelux/Germania/Austria/Islanda; fondata 1988, produzione propria dal 1992. LEGAME DI GRUPPO: amministratore statutario è Atlas Packaging Group B.V. (dal 2007). Nessun direttore persona fisica pubblicato (solo procuratori E.H. Aelen e C.H.A. Verhaegh).</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/akarton-bv</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>info@karton.nl</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://karton.nl</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Venlo, Limburg</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-golfpapier-en-karton/akarton-b-v-venlo-12029719</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Bangma Verpakking B.V.</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 32 dipendenti (fonte company.info / rocketreach.co, 2025). KVK 39027421. Fornitore e progettista di imballaggi industriali (carta, cartone, cartone ondulato) dal 1975, sede Cellebroederspoort 8. Membro NVC. ATTENZIONE: dal 2025 risulta amministratore 'A. Kalliomäki' — possibile passaggio a gruppo estero, da verificare. Nessun direttore persona fisica confermato come 'directeur/eigenaar' sulle fonti pubbliche.</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>sales@bangma.nl</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bangma.nl</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Dronten, Flevoland</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-emballage-voor-industrieel-gebruik/bangma-verpakking-b-v-dronten-39027421-000017208963</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>De Groot Drukkerij B.V.</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 121 dipendenti nella sede (164 nel gruppo, 115 FTE secondo GOC) (fonti drukkerij-gids.nl / goc.nl, 2024). KVK 23018002. Stamperia di libri e riviste, familiare di terza generazione, attiva dal 1913/1965. AZIENDA DI CONFINE VERSO L'ALTO: con oltre 120 addetti il fatturato può avvicinarsi o superare i 40 M€ — verificare prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Anton de Groot</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>https://grootsgedrukt.nl</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Goudriaan (Molenlanden), Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>https://drukkerij-gids.nl/goudriaan/de-groot-drukkerij-bv/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Drukkerij Van der Eems B.V.</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 65 dipendenti su due sedi, Easterein e Heerenveen (fonte vandereems.nl / regiobedrijf.nl, 2024-2025). KVK 01010712. Tipografia offset e digitale, familiare dal 1906, oggi alla quarta generazione. Membro KVGO. Nessun nome pubblicato con la qualifica esplicita di 'directeur': referente lasciato vuoto.</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/grafische-groep-van-der-eems</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>sjoukje@vandereems.nl</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vandereems.nl</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Easterein (Súdwest-Fryslân), Friesland</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goudengids.nl/nl/bedrijf/Easterein/L120000030/Drukkerij+Van+der+Eems/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Dutch Boxx Golfkarton B.V.</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 28 dipendenti (fonte transfirm.nl / drimble.nl, 2025). KVK 01099519 - BTW NL819667316B01. Produttore indipendente di scatole in cartone ondulato su misura, sede Mars 33; fondata nel 2008. Certificazioni FSSC 22000 e FSC. AZIENDA DI CONFINE: con 28 addetti il fatturato è probabilmente nella fascia 5-12 M€.</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Piet Stilma</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/dutchboxx-golfkarton-bv</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>golfkarton@dutchboxx.nl</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://dutchboxx.nl</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Heerenveen, Friesland</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/heerenveen/20219695/dutch-boxx-golfkarton-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Fris Karton B.V.</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 18-20 dipendenti (fonte kompass.nl / rocketreach.co, 2025). KVK 17059632. Produttore indipendente di scatole in cartone ondulato di tutti i formati, sede Hallenstraat 25, attiva dal 1984. SOTTO SOGLIA: con ~20 addetti il fatturato è verosimilmente intorno o sotto i 5 M€.</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Moniek van Steensel</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Eigenaar</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/fris-karton</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>verkoop@friskarton.nl</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.friskarton.nl</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Bladel, Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://graydongo.nl/nl/nl-grafisch-fris-karton-bv-bladel-17059632</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Papierfabriek Schut B.V.</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartiera</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 43-45 dipendenti (fonte drimble.nl / stagemarkt.nl, 2024-2025). KVK 09001229. Cartiera indipendente attiva dal 1618, specialità: carta per belle arti, acquerello, carta filigranata e carta circolare da residui del cliente. Membro Koninklijke VNP. Stima fatturato in fascia bassa del target (specialty paper, alto valore unitario).</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>René Kort</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/schut-papierfabriek-b-v-</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>info@schutpapier.com</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://schutpapier.nl</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Heelsum (Renkum), Gelderland</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/heelsum/000019015402/papierfabriek-schut-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Veldhuis Media B.V.</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 15,5 M€ (fonte bedrijvenregister.nl, dato 2017 - ultimo pubblicato; bilanci recenti depositati in forma abbreviata). 21-50 dipendenti (fonte bedrijvenregister.nl / drukkerij-gids.nl, 2024). KVK 05071502. Tipografia offset e legatoria (brochure, riviste, cataloghi, libri). Direzione condivisa con Erwin de Lange dal 2002. Partecipazione di minoranza della società di investimento Wadinko NV — legame di gruppo parziale.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Oscar Jager</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.veldhuismedia.nl</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Meppel, Drenthe (già Raalte, Overijssel)</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bedrijvenregister.nl/raalte/veldhuis-media-bv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Vermijs Kartonnage B.V.</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — astucci pieghevoli</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato in bilancio (BV con deposito abbreviato); stima terza parte ca. 5-6 M€ (RocketReach, 2026 - dato NON ufficiale). 22 dipendenti (fonte rocketreach.co / company.info, 2025-2026). KVK 20054190. Fondata nel 1970, sede Beneluxweg 33. Membro KVGO. SOTTO SOGLIA: dimensione al limite inferiore della fascia tollerabile (~5 M€).</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Merel Vermijs</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/vermijs-kartonnage-bv</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>info@vermijskartonnage.nl</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://vermijskartonnage.nl</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Oosterhout, Noord-Brabant</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-verpakkingsmiddelen-van-papier-en-karton/vermijs-kartonnage-b-v-oosterhout-20054190-000020066678</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Zaadhof's Cartonnage Fabrieken B.V.</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone e stampa</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 6 M€/anno (fonte RTV Noord, reportage 'Made in Grunn' sul familiebedrijf di Winschoten). 11-50 dipendenti (fonte LinkedIn company page / drimble.nl, 2025). KVK 02317727 - BTW NL001615294B01. Cartotecnica e tipografia da imballaggio indipendente, familiare, attiva dal 1951. Sede Industrieweg 5-18. SOTTO SOGLIA rispetto al target 10-20 M€, ma dentro la fascia tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Jan Zaadhof</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Eigenaar</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/zaadhof-cartonnagefabrieken-bv</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>info@zaadhof.nl</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.zaadhof.nl</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Winschoten, Groningen</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rtvnoord.nl/economie/1416341/made-in-grunn-winschoter-familiebedrijf-maakt-jaarlijks-tientallen-miljoenen-verpakkingen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Zalsman B.V.</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 50 dipendenti nella sede di Steinfurtstraat 1 (fonte drukkerij-gids.nl / company.info, 2024-2025). KVK 05044422. Tipografia indipendente fondata nel 1857; offset + digitale (installata Ricoh Pro VC80000 nel 2024). Ha rilevato Drukkerij van den Berg (Kampen). Soci: Zalcom B.V. e IMpact Sociale Media B.V. NESSUN legame con Zalsman Groningen (fallita 2024, società distinta).</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Herman Verlind</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>info@zalsman.nl</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://www.zalsman.nl</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Zwolle, Overijssel</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/overige-activiteiten-op-het-gebied-van-drukwerk-rest/zalsman-b-v-zwolle-05044422-000017223881</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Blanche Dael B.V. (Maison Blanche Dael)</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato); n. dipendenti non pubblicato nelle fonti consultate. KVK 76979229, Aan de Brikkebouw 10 Maastricht (entità costituita nel 2019), P.IVA NL860860814B01. Koffiebranderij + theepakkerij familiare dal 1878, SBI groothandel in koffie, thee, cacao en specerijen. Verosimilmente sotto la fascia 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Albert Berghof</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Directeur / eigenaar</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.blanchedael.nl/</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Maastricht (Limburg)</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.creditsafe.com/business-index/en-us/company/blanche-dael-bv-nl05333583</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Bocca Coffee B.V.</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ~4,8 M€ con 40 dipendenti (fonte: New10, articolo aziendale). Sede Kerkstraat 96 Amsterdam, torrefazione a Dronten; primo specialty roaster olandese, B Corp. SOTTO la fascia 5-40 M€ (borderline). Nota legame: il fondatore Menno Simons è anche fondatore dell'importatore di caffè verde Trabocca B.V.</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Menno Simons</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Oprichter / directeur</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bocca-coffee/</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>info@bocca.nl</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://bocca.nl/</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland) — torrefazione a Dronten (Flevoland)</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>https://new10.com/blog/bocca-coffee-bliksemstart-verandering-groei</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Brandsma Koffie B.V.</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato e n. dipendenti non pubblicato nelle fonti consultate (bilancio abbreviato). Numero KVK non reperito con le sole fonti aperte. Azienda familiare dal 1893 a Bolsward, torrefazione propria, fornitore nazionale per horeca, aziende e privati. Verosimilmente sotto la fascia 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Menno Brandsma</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Directeur (4a generazione)</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/brandsma-koffie</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.brandsmakoffie.nl/</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Bolsward (Friesland)</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://grachtenbeans.nl/koffiebrander/brandsma-koffie/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Fleur de Café B.V.</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato e n. dipendenti non pubblicato nelle fonti consultate (bilancio abbreviato). Numero KVK non reperito; P.IVA NL854149879B01. Hamburgweg 10, Deventer. Groothandel koffie/thee + koffiebranderij per horeca, retail e privati; fornisce anche impianti a chi vuole avviare una propria torrefazione. Verosimilmente piccola impresa sotto i 5 M€.</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>info@fleurdecafe.nl</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fleurdecafe.nl/</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Deventer (Overijssel)</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fleurdecafe.nl/klantenservice</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>G. Bijdendijk B.V. (Koffiehandelshuis G. Bijdendijk)</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato). 2-5 dipendenti registrati alla sede (fonte: Oozo.nl / registro KVK, 2025); il team pubblicato sul sito conta ~9 persone. KVK 08022494, Laan 57 Nunspeet. Casa commerciale di caffè verde attiva dal 1843 (175 anni nel 2018): volumi d'import elevati rispetto all'organico — operatore EUDR in senso stretto.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Mark Bouw</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Managing Director (con Robbert Bouw)</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/bijdendijk</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>info@bijdendijk.nl</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bijdendijk.nl/</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Nunspeet (Gelderland)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/nunspeet/nunspeet/hulshorst/145458/g-bijdendijk-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Giraffe Coffee B.V.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato e n. dipendenti non pubblicati nelle fonti consultate; numero KVK non reperito con le sole fonti aperte. Torrefazione specialty aperta nel 2013 a Rotterdam, con Coffee Bar &amp; Academy in Hoogstraat 46a; acquisto diretto con premio extra ai produttori, consegna a ristoranti e negozi in tutta NL. Micro-impresa, ben sotto i 5 M€ — segnalata per la componente di acquisto diretto di caffè verde.</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Maarten van der Jagt</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Oprichter (con Mark Jordaan)</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/giraffe-coffee-bv</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>https://giraffecoffee.com/</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Rotterdam (Zuid-Holland)</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>https://giraffecoffee.com/en/pages/over</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Greencof B.V.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV con bilancio abbreviato). KVK 37123582 (su company.info registrata a Zaandam; sede operativa Grote Oost 53, Hoorn), P.IVA NL820866702B01, fondata 2006. Importatore/esportatore di caffè verde specialty (fairtrade, bio, Rainforest Alliance) con stoccaggio ad Anversa e Amburgo. Operatore EUDR in senso stretto; taglia probabilmente sotto i 10 M€ — da verificare.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Leon Zaal</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>info@greencof.com</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://greencof.com/</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Hoorn (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-koffie-thee-cacao-en-specerijen/greencof-b-v-zaandam-37123582</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Hesselink Koffiesystemen B.V.</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato). 11-20 dipendenti (fonte: Oozo.nl / registro KVK, 2025). KVK 08049402, Rondweg Zuid 95 Winterswijk. Groothandel in koffie, thee, cacao en specerijen. Fa capo a Hesselink Koffie Groep B.V. (KVK 59575492, holding). Torrefazione familiare dal 1885. Probabilmente sotto la fascia 5-40 M€ — segnalata per rilevanza settoriale.</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>info@hesselinkkoffie.eu</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://hesselinkkoffie.nl/</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Winterswijk (Gelderland)</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/winterswijk/stad/winterswijk-zuidwest/171483/hesselink-koffiesystemen-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Kaldi Koffie en Thee B.V.</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato). KVK 24310514, Popovstraat 70 Zwolle, costituita nel 2000. Formula in franchising con oltre 30 negozi specializzati koffie &amp; thee in NL + canale B2B; marchi propri con caffè da diversi continenti. Numero di dipendenti della BV non pubblicato nelle fonti consultate.</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Martijn Bas</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Directeur (dagelijkse leiding)</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/kaldikoffieenthee</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>https://kaldi.nl/</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Zwolle (Overijssel)</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.creditsafe.com/business-index/en-us/company/kaldi-koffie-en-thee-bv-nl01235350</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Koffiebranderij G. Peeze B.V.</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato). ~55 dipendenti (fonte: GraydonGo / TransFirm, 2025). KVK 09026526, Ringoven 36 Arnhem, attiva dal 1971. ATTENZIONE LEGAME DI GRUPPO: da maggio 2025 le azioni sono state acquisite dal fondo Berk Partners e Peeze è confluita in Coffee Growth Group (direzione Myriam Lufting / Wouter Jansen van Velsen). Torrefazione B Corp, acquisto diretto di caffè verde all'origine.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>info@peeze.nl</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>https://peeze.nl/</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Arnhem (Gelderland)</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.transfirm.nl/nl/organisatie/090265260000-koffiebranderij-g.-peeze-b.v.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Moyee Nederland B.V.</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato); una fonte terza (rocketreach) riporta ~45 addetti — dato non ufficiale. KVK 61730556, Elementenstraat 10 Amsterdam, fondata 2014. Groothandel in koffie, thee, cacao en specerijen; modello 'FairChain' con torrefazione in Etiopia e importazione in NL. Micro/piccola impresa, verosimilmente sotto i 5 M€.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Guido van Staveren van Dijk</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Managing director / oprichter</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>b2b@moyeecoffee.com</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.moyeecoffee.com/</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-koffie-thee-cacao-en-specerijen/moyee-nederland-b-v-amsterdam-61730556-000030807255</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Neuteboom Koffiebranders B.V.</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato); n. dipendenti non pubblicato nelle fonti consultate. Capacità produttiva 10.000 t/anno su due impianti di torrefazione (fonte: Wikipedia NL / Mister Barish). Indicata tra le cinque maggiori torrefazioni olandesi (dato 2013). Aadijk 41, Almelo, attiva dal 1891. Specialista private label per l'Europa occidentale: probabile fascia alta del target o superiore — da verificare.</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Gilbert Willemsen</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Directeur / eigenaar</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/neuteboom-koffiebrander</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>https://neuteboom.nl/</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Almelo (Overijssel)</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Neuteboom_koffiebranders</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Origin Bridge (Barchem)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e n. dipendenti non pubblicati. KVK 70878315, P.IVA NL001587917B24 — la struttura del numero IVA indica una ditta individuale/eenmanszaak, NON una B.V.: la forma giuridica va verificata prima del contatto. Heidehoflaan 2B, Barchem. Importatore di caffè verde specialty dalla Colombia (micro-lotti e volumi da produzione) per torrefattori professionali in Europa. Micro-impresa, sotto i 5 M€, ma operatore EUDR in senso stretto.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="3" t="inlineStr"/>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>info@bridgetoorigin.com</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>https://originbridge.coffee/</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Barchem, gem. Lochem (Gelderland)</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>https://originbridge.coffee/legal-information/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Simon Levelt B.V.</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato della BV non pubblicato (accesso premium su company.info). Riferimenti di stampa: 11,5 M€ di fatturato nel 2011; fatturato al consumo della catena oltre 20 M€ nel 2016 (fonte: MT/Sprout, Fonk Magazine). 77 dipendenti (fonte: company.info / OpenKvK, 2025). KVK 34093465, A. Hofmanweg 3 Haarlem. Torrefazione + confezionamento tè + catena in franchising dal 1826. BORDERLINE: potrebbe superare i 40 M€ di giro d'affari di insegna — da verificare prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Mikkel Levelt</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Directeur (6a generazione, con Rob Sikkema)</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>https://www.simonlevelt.nl/</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Haarlem (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/gespecialiseerde-detailhandel-in-overige-voedings-en-genotmiddelen-rest/simon-levelt-b-v-haarlem-34093465-000020025106</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Smit &amp; Dorlas Koffiebranders B.V.</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato nei registri (bilancio abbreviato); stima di terze parti ~12,4 M$ (rocketreach — non ufficiale, da verificare). 94 dipendenti dichiarati dall'azienda (2025). KVK 31022124, costituita 28-03-1978 (marchi Smit e Dorlas dal 1822). Torrefazione artigianale per l'horeca. Se la stima regge, rientra nel target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/smit-&amp;-dorlas-koffiebranders-b.v.</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>info@smitdorlas.nl</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.smitdorlas.nl/</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Mijdrecht (Utrecht)</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.smitdorlas.nl/bedrijfsinformatie/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>TSU Trade B.V. (This Side Up Coffees)</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV con bilancio abbreviato). KVK 59161167 (Amsterdam), fondata 2013. Importatore di caffè verde specialty: container via porto di Rotterdam, rivendita a torrefattori specialty in tutta Europa. Micro/piccola impresa — verosimilmente sotto la fascia 5-40 M€, ma operatore EUDR in senso stretto (prima immissione di caffè verde sul mercato UE).</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Lennart Clerkx</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Oprichter / directeur</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/thissideupcoffees</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>order@thissideup.coffee</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>https://thissideup.coffee/</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>https://thissideup.coffee/contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Van Duijnen Koffie B.V.</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + engros/wholesale</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (bilancio abbreviato). 21-50 dipendenti (fonte: Oozo.nl / registro KVK, 2025). KVK 39086536, Rondebeltweg 34 Almere. Groothandel in koffie, thee, cacao en specerijen. Premiata 'Onderneming van het Jaar 2025-2026' ad Almere. Taglia stimata intorno o sotto la soglia inferiore del target.</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Paul Kragten</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-duijnen-koffie</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>customercare@vanduijnen.nl</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>https://vanduijnen.nl/</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Almere (Flevoland)</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/almere/almere-stad/gooisekant/171540/van-duijnen-koffie-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Chocolade- en Suikerwerkfabriek Marandi B.V.</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — lavorazione cacao e cioccolato</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. 21-50 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 09065319. Sede Klomperweg 69, Lunteren. Attività registrata: verwerking van cacao + vervaardiging van chocolade en suikerwerk (lavorazione diretta del cacao, quindi rilevante EUDR).</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Lunteren / Ede (Gelderland)</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/ede/lunteren/centrum-lunteren/365228/chocolade-en-suikerwerkfabriek-marandi-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Chocoladefabriek "De Beemster" B.V.</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolato e frutta secca ricoperta</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; stime terze indicano meno di 5 M$ e 11-50 dipendenti (fonte: ZoomInfo / company.info, 2025). KVK 37109862. Membro VBZ. Nota: sotto la soglia ideale 10-20 M€, tenuta per copertura del segmento produzione cioccolato.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Jos Klijnsma</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Algemeen directeur (general manager)</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/chocoladefabriek-'de-beemster'-b.v.</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.chocobeemster.nl/</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Middenbeemster / Purmerend (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/chocoladefabriek-de-beemster-b-v-middenbeemster-37109862-000020449763</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Chocolatemakers B.V.</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolato bean-to-bar</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ~4 M€ (fonte: MT/Sprout, articolo sulla fusione con Hands Off, 2025). KVK 57652066. SBI verwerking van cacao. Fabbrica bean-to-bar nel porto di Amsterdam, importa direttamente fave da Congo, Perù e Rep. Dominicana: operatore EUDR. Nota: sotto la fascia 5-40 M€, tenuta per copertura del segmento bean-to-bar.</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Enver Loke</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Oprichter (co-fondatore)</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>info@chocolatemakers.nl</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>https://www.chocolatemakers.com/</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/verwerking-van-cacao/chocolatemakers-b-v-amsterdam-57652066-000022805583</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Continental Chocolate B.V.</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. 20-49 dipendenti (fonte: transfirm.nl / Dun &amp; Bradstreet, dati KVK 2025). KVK 34146292. Costituita nel 2000. Sede Galvanistraat 10, Rotterdam. Produzione di cioccolato e prodotti dolciari a base di cacao.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Johannes M.C.G. van Logtestijn</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Bestuurder / key principal</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr"/>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Rotterdam (Zuid-Holland)</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://transfirm.nl/nl/organisatie/341462920000-continental-chocolate-b.v.?lang=en</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>De Chocoladefabriek B.V.</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione cioccolato retail</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; ~30 dipendenti (fonte: Het Ondernemersbelang, articolo sull'emissione NPEX di max 3 M€ in certificati di azioni preferenziali cumulative). KVK 37032938. Produttore di cioccolato per il retail olandese (HEMA, catene di supermercati). Probabilmente sotto la fascia ideale ma rilevante come operatore EUDR sul cioccolato.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Hans Neef</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Directeur / eigenaar</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/dechocoladefabriek</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>info@dechocoladefabriek.nl</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>https://www.dechocoladefabriek.nl/</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Heerhugowaard / Dijk en Waard (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.ondernemersbelang.nl/nieuws/de-chocoladefabriek-naar-npex-beurs-met-certificaten/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>De Euforij Chocolade B.V.</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolato da semilavorati cacao</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 61954578. Costituita nel 2014, sede Zaandijkerweg 1, Wormerveer (cluster cacao Zaanstreek). Produce cioccolato partendo da massa di cacao, burro di cacao e cacao in polvere (semilavorati Allegato I EUDR). Nota: micro/piccola impresa, sotto la fascia 5-40 M€, tenuta per copertura del cluster Zaanstreek.</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/de-euforij-chocolade-b-v-</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>chocolade@euforij.nl</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euforij.nl/</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Wormerveer / Zaanstad (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bedrijvenregister.nl/wormerveer/de-euforij-chocolade-bv</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Martinez Chocolade B.V.</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — bonbon e cioccolato</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. 8 dipendenti (6-10 secondo KVK) (fonte: transfirm.nl / oozo.nl, dati KVK 2025). KVK 34128566. Membro VBZ. Nota: nettamente sotto la fascia 5-40 M€, tenuta per copertura del segmento cioccolateria.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>X. Stam</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>https://www.martinezchocolade.nl/</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Amstelveen (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.transfirm.nl/nl/organisatie/341285660000-martinez-chocolade-b.v.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Original Beans B.V.</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cacao fine e cioccolato premium</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 50770764. Sede Mauritskade 64, Amsterdam. Attività registrata: acquisto di fave di cacao per la produzione di cioccolato (in conto terzi), rivendita e commercio all'ingrosso di cioccolato — quindi operatore EUDR sull'import di cacao. Dimensione presumibilmente sotto la fascia 5-40 M€: tenuta per copertura del segmento cacao fine.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>https://originalbeans.com/</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bedrijvenregister.nl/amsterdam/original-beans</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Ringers' Import B.V.</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import/ingrosso cioccolato</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. 11-20 dipendenti (fonte: oozo.nl / graydongo.nl, dati KVK, 2025). KVK 18049029. Sede Ir. Lelyweg 49, Haarlem. Attività: groothandel in suiker, chocolade en suikerwerk — importatore/commerciante di cioccolato, quindi soggetto EUDR come operatore o trader.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>http://www.ringersimport.nl/</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Haarlem (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/haarlem/waarder-en-veerpolder/waarderpolder/171566/ringers-import-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Rousseau Chocolade B.V.</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione cioccolato e praline</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. 54 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 14002870. Costituita nel 1955. SBI vervaardiging van chocolade en suikerwerk. Sede Langs de Heij 11, Sittard. Per organico plausibilmente nella fascia 10-20 M€, ma il fatturato non è depositato pubblicamente.</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr"/>
+      <c r="E67" s="3" t="inlineStr"/>
+      <c r="F67" s="3" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Sittard / Sittard-Geleen (Limburg)</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oozo.nl/bedrijven/sittard-geleen/overhoven/industrieterrein-noord/365188/rousseau-chocolade-b-v</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Steenland Chocolate B.V.</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione cioccolato (monete/medaglie)</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (deposito abbreviato). 51-100 dipendenti, indicati 55-67 fissi e fino a ~150 in alta stagione (fonte: oozo.nl / graydongo.nl, dati KVK 2025). KVK 24354029. Produttore leader mondiale di monete e medaglioni di cioccolato personalizzati, export in oltre 50 paesi. Nota gruppo: dal 2017 controllata da Sino-Pacific Trading Co. Ltd. Per organico si colloca nella fascia alta del target.</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/steenland-chocolate</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>https://www.steenland.nl/</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Gouda (Zuid-Holland)</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/steenland-chocolate-b-v-gouda-24354029-000018029809</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Trianon Chocolatiers B.V.</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato. La consociata operativa Trianon Productie B.V. (KVK 17146078) dichiara 21-50 dipendenti (fonte: oozo.nl, dati KVK). KVK 17198255 (Trianon Chocolatiers B.V.). Legame di gruppo: Trianon Holding B.V., Oss (KVK 17151352). Azienda familiare, fabbrica di cioccolato e caramelle; acquirente di cioccolato e semilavorati di cacao.</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>trianon@trianon.nl</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.trianon.nl/</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Oss (Noord-Brabant)</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>https://nl.kompass.com/c/trianon-chocolatiers-b-v/nl196607/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>RIS Rubber N.V.</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — articoli tecnici e mescole</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato. 180 dipendenti (fonte sito aziendale risrubber.com / pagina 'Over RIS', 2025). KVK 39067356. Sede Pekstraat 7, 8211 AB Lelystad. Attiva dal 1955, fabbrica di gomma con laboratorio di R&amp;S e impianti di prova propri. Membro NVR-TRA. Ragione sociale N.V. (non B.V.). Con 180 addetti stima fatturato in fascia alta/di confine del target (indicativamente 25-40 M€). E-mail: contatto commerciale pubblicato (Bianca Westmaas, Sales Manager); non risulta pubblicata una casella info@ generica.</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/ris-rubber-nv</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>bwestmaas@risrubber.com</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>https://www.risrubber.com</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Lelystad, Flevoland</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.risrubber.com/over-ris/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Rubber Design B.V.</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — antivibranti gomma-metallo</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 101-200 dipendenti (fonte Drimble.nl / Company.info, 2024-2025). KVK 23044439. Sede Industrieweg 21, 2995 BE Heerjansdam. Fondata 1979-1980; progetta, calcola e produce articoli tecnici in gomma e gomma-metallo antivibranti e antirumore per cantieristica navale, yacht e industria. Con 100-200 addetti il fatturato stimato si colloca nella fascia alta del target (indicativamente 20-40 M€).</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>info@rubberdesign.nl</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rubberdesign.nl</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Heerjansdam (Zwijndrecht), Zuid-Holland</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>https://drimble.nl/bedrijf/heerjansdam/1084011/rubber-design-bv.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Ruma Rubber B.V.</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — articoli tecnici in elastomeri</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 15 M$ (~14 M€) e 90 dipendenti (fonte Dun &amp; Bradstreet business directory, profilo aggiornato 2024-2025). KVK 04033678. Sede Lindberghstraat 49, 7903 BM Hoogeveen. Fondata 1937, specialista in tecnologia degli elastomeri; stabilimenti anche a Olkusz (PL) e Dubai (UAE). Membro NVR-TRA (Nederlandse Vereniging van Rubberfabrikanten). Fatturato esatto NON depositato pubblicamente (BV con bilancio abbreviato) - dato D&amp;B stimato. IN TARGET.</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Johannes C. van Haaren</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Key principal / Directeur</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/ruma-rubber-bv/</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>info@rumarubber.com</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>https://rumarubber.com</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Hoogeveen, Drenthe</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.dnb.com/business-directory/company-profiles.ruma_rubber_bv.8b91dcdabf64a6f6e9fbc7005f6b7b30.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Van Benthem Diervoeders Vollenhove B.V.</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimificio (rundvee/paarden)</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). Ca. 20-21 dipendenti (fonte: vbvoer.nl e drimble.nl, 2025). KVK 05044357. Mangimificio familiare attivo dal 1780, produttore di mengvoeder di taglia medio-piccola; dal 2025 collaborazione con P. Bos Veevoeders. Utilizzatore di sojaschroot: operatore/commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Ed van Benthem</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Eigenaar / directeur</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-benthem-veevoeders-en-kunstmest-b.v.</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>info@vanbenthemvollenhove.nl</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vbvoer.nl/</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Vollenhove / Steenwijkerland (Overijssel)</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vbvoer.nl/van-benthem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>S.R.C. (Special Refining Company) B.V.</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — raffinazione conto terzi oli vegetali</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (toll refiner: non acquista né vende olio, fattura solo il servizio di raffinazione — fatturato strutturalmente sotto la soglia dei trader). Capacità di raffinazione oltre 40.000 t/anno; organico ridotto e specializzato (numero esatto non pubblicato). Fondata nel 1996, parte del gruppo Pieter Bon. Circa 60% degli oli e grassi lavorati è biologico. Membro MVO. Raffinatore di palma e altri oli vegetali sul Noordzeekanaal.</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/src-b-v-</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://refinery.nl/</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Zaandam / Zaanstad (Noord-Holland)</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>https://mvo.nl/organisatie/leden/src</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Spack B.V.</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Olio di palma — produzione/confezionamento oli vegetali bio</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (company.info espone solo profilo, dati finanziari a pagamento). 10-24 dipendenti (fonte: regiobedrijf.nl su dati KVK, 2025). KVK 24225423. PMI probabilmente sotto i 10 M€ di fatturato: segnalata come taglia di confine inferiore. Nata a Rotterdam nel 1977 come trading di oli e grassi vegetali, oggi produttore/confezionatore di oli vegetali biologici (incl. palma e cocco): operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>info@spackbv.com</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.spack.nl/</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Nieuwe-Tonge / Goeree-Overflakkee (Zuid-Holland)</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>https://regiobedrijf.nl/groothandel-in-ruwe-plantaardige-en-dierlijke-olien-en-vetten-en-oliehoudende-grondstoffen/spack-bv-74891.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J75"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId166"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Belgio: CONSEGNATO - 90 aziende (email 65/90), workbook a 7 fogli / 644 righe
- carne/pelle completato (12), ripartizione: legno 25, cacao 18, carta 16,
  carne 9, gomma 5, caffe 5, mangimi 5, palma 4, pelle 3
- handoff: sezione 14 con esclusioni di merito (Pacorini logistica pura,
  Immobra olio di lino non Allegato I) e note di filiera
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Danimarca" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Svezia" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Olanda" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Belgio" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Italia'!$A$2:$J$97</definedName>
@@ -21,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28351,4 +28353,4368 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyEUDR — Lead mapping · Belgio · aziende potenzialmente soggette all'EUDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Denominazione</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Filiera EUDR</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Dimensione (fatt./dip.)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Ruolo</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Email / PEC</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Sito web</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Hulpiau Hides BV</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — commercio pelli bovine salate</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>6,1 FTE (ultimo bilancio depositato NBB, via Companyweb); fatturato NON pubblicato (schema abbreviato) - la collegata storica Hulpiau BV (BE 0429.082.864) dichiara un margine lordo di 2.284.726 EUR; n. impresa BE 0777.875.662. SOTTO la fascia target per dimensione, ma pienamente in scope EUDR: raccoglie pelli bovine wet-salted dai macelli belgi e le esporta nel mondo.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>info@hulpiauhides.com</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hulpiauhides.com/</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Dendermonde (Oost-Vlaanderen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0777875662/hulpiau-hides</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Radermecker SRL</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — conceria cuoio da selleria</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>9,1 FTE (ultimo bilancio depositato BNB, via Companyweb); fatturato NON pubblicato (schema abbreviato); n. impresa BE 0649.971.462 (societa' costituita il 16/03/2016, attivita' di conceria dal 1870, trasferita da Warneton a Comines nel 2019). MICROIMPRESA molto sotto la fascia target, inclusa perche' e' una delle ultime due concerie ancora attive in Belgio.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/radermecker</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.radermecker.com/</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Comines-Warneton (Hainaut, Vallonia)</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0649971462/radermecker</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Tannerie Masure SA</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — concia vegetale cuoio bovino</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 17.158.424 EUR (bilancio depositato BNB, via Trends Top/Pappers.be) - 3a azienda del settore cuoio/calzatura in Belgio; n. impresa BE 0401.249.606. Nel cuore della fascia target. Concia esclusivamente vegetale di groppe e collo bovini di provenienza europea; fa capo al Groupe Saturne (Tannerie Fortier Beaulieu + Masure).</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Olivier Lesage</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.masure.be/</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Estaimpuis / Estaimbourg (Hainaut, Vallonia)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/fr/company/tannerie-masure-0401249606</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Belignum NV</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname e pannelli</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 14.746.642 (ultimo bilancio depositato NBB; fonte trendstop, 40ª nel settore 'houthandel'). Impresa BE 0405.348.449. Sede: Boulevard Industriel / Industriëlaan 97B, 7700 Mouscron. Importatore di legni duri e teneri per commercianti di legname, grande distribuzione e carrozzerie; importatore esclusivo per il Belgio dei pannelli 'Tilly Naturholzplatten'. Legata al gruppo Lagae Hout NV (stesso indirizzo/LEI). Fatturato in pieno target; unico record vallone della filiera legno.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>info@belignum.be</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://www.belignum.be/</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Mouscron / Moeskroen (Vallonia, prov. Hainaut)</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/405348449/belignum.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Bulo NV</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili per ufficio</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 13.748.349 € (fonte jaarrekening.be, bilancio depositato NBB 02-10-2024); altra fonte (trendstop.knack.be) riporta 16.190.827 €. 29,0 FTE (2023). N. impresa BE 0459.905.605. Produttore di mobili per ufficio di design (scrivanie, armadi, pannelli in legno/melaminico), sede Blarenberglaan 6, 2800 Mechelen. IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Dirk Busschop</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bulo</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>info@bulo.be</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://bulo.com</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Mechelen, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://jaarrekening.be/en/bulo/0459.905.605</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Buzzispace NV</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi acustici per ufficio</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 26.116.920 € - 34,9 FTE (fonte companyweb.be / trendstop.knack.be, bilancio depositato NBB luglio 2025). N. impresa BE 0459.565.412. Sede sociale Italielei 8, 2000 Antwerpen; produzione in Kempen. Fondata nel 2007, arredi e pannelli acustici per ufficio con strutture e pannelli in legno. Capogruppo: Buzzispace Group NV (BE 0508.916.141) - segnalare il legame di gruppo. Sopra la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Tommaso Baldini</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>CEO e Managing Director (dal 01-10-2023)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/buzzispace</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.buzzi.space</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Anversa (Antwerpen), Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/459565412/buzzispace.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Callens NV (Callens African Woods)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato € 32.340.788 e 34,7 FTE (ultimo bilancio depositato NBB, deposito 24-12-2025; fonte trendstop/companyweb). Impresa BE 0425.280.365. Sede: Waterstraat 25, 8930 Menen. 19ª nel settore 'houthandel' per fatturato. Gestore forestale, produttore e importatore di legno tropicale africano (~165 persone in Camerun + ~45 in Belgio). Fascia alta del range tollerabile (32 M€) ma operatore EUDR in senso stretto: massima priorità.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Thierry Maelfait</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder / bestuurder</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>info@houtcallens.be</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://houtcallens.be/</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Menen (Fiandre, prov. West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/425280365/callens.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Carlens NV</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 14.868.112 e 26 FTE (ultimo bilancio depositato NBB; fonte trendstop, 39ª nel settore 'houthandel'). Impresa BE 0405.592.236. Sede: Gaston Geenslaan 1, 3200 Aarschot. Azienda familiare dal 1934, ~30 addetti, stock &gt;20.000 m³. Grossista di legname e pannelli verso rivenditori e imprese: fatturato in pieno target.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>info@carlenshout.be</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>https://carlenshout.be/</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Aarschot (Fiandre, prov. Vlaams-Brabant)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/405592236/carlens.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Confortluxe NV</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 17.317.401 € - 40,6 FTE (fonte trendstop.knack.be / companyweb.be, bilancio depositato NBB 27-07-2024). 19a nel settore Meubelindustrie. N. impresa BE 0412.863.078. Costituita 29-12-1972, sede Menensesteenweg 40, 8940 Wervik. Produce divani, relax e boxspring (telai in legno, rivestimenti in pelle). Amministratori attuali secondo FinCheck: Jimmy Ollevier, Heidi Ollevier, Jacqueline Pauwels (ruolo di gedelegeerd bestuurder non pubblicato in modo univoco). Legame di gruppo: holding familiare Telinfra, stessa proprieta di Meubelfabriek Lievens NV. IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>info@confortluxe.com</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.confortluxe.com</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Wervik, Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/412863078/confortluxe.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Decadt Houthandel NV</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 13.460.408 e 16,9 FTE (ultimo bilancio depositato NBB; fonte trendstop, 43ª nel settore 'houthandel'). Impresa BE 0415.284.714, fondata 01-01-1975. Sede: Rodenbachstraat 19, 8908 Vlamertinge (Ieper); seconda sede nella zona industriale di Veurne. Grossista/dettagliante di legname: stock di legni tropicali e commerciali (iroko, padouk, afzelia, cedro, rovere, Douglas, thermowood) + parquet e laminati. Fatturato in pieno target.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Stefaan Decadt</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>decadt.hout@telenet.be</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>https://decadt-hout.be/</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Vlamertinge / Ieper (Fiandre, prov. West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/415284714/decadt-houthandel.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Decolvenaere BV</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato annuo dichiarato 'oltre 10 milioni di euro' (fonte: reportage Sterck Magazine); presente nel ranking settoriale 'houthandel' di Trends Top. Impresa BE 0400.079.171, fondata 01-07-1959. Sede: Singel 140, 9000 Gent. Organico snello (6-9 addetti secondo Kompass) rispetto ai volumi: tipico importatore/commerciante. Importatore diretto di legname tropicale (azobé, iroko, sapelli, wengé, afrormosia...) — operatore EUDR in senso stretto. Fatturato esatto da confermare su NBB.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Daphné Decolvenaere</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder (5ª generazione)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>info@decolvenaere.be</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://decolvenaere.be/</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Gent (Fiandre, prov. Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/400079171/decolvenaere-houtimport.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Denderwood NV</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — import legname tropicale</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Impresa BE 0423.826.652. Sede: Joseph Cardijnstraat 3, 9420 Erpe-Mere. Margine lordo € 1.153.745 e 8,9 FTE (ultimo bilancio depositato NBB, deposito 06-03-2025); NON pubblica il fatturato (schema abbreviato → ricavi presumibilmente sotto ~11 M€): TAGLIA DA VERIFICARE, possibile fascia bassa/sotto i 5 M€. Azienda familiare D'Haeseleer, importatore diretto di legname duro asiatico e africano (rubberwood, meranti, ipé, materiale lamellare) dagli anni '60: profilo di operatore EUDR in senso stretto, prioritario nonostante il fatturato non pubblicato.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>https://denderwood.com/</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Erpe-Mere (Fiandre, prov. Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/423826652/denderwood.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Ethnicraft NV</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 39.757.392 € - 95,1 FTE (fonte companyweb.be, bilancio depositato NBB 30-07-2025); trendstop.knack.be riporta 40.887.490 € e la 4a posizione nel settore Meubelindustrie. N. impresa BE 0458.213.251. Fondata 07-06-1996, sede Scheldeweg 5, 2850 Boom. Mobili in teak e rovere massello prodotti in Asia (Indonesia/Vietnam) e importati nell'UE: rischio EUDR elevato su legname tropicale. Legame di gruppo con Studio Ethnicraft NV (BE 0846.804.654). AL LIMITE ALTO della fascia tollerabile 5-40 M€ (sopra la fascia ideale 10-20 M€).</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Benoît Loos</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>CEO Ethnicraft Europe (cofondatore)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>info@ethnicraft.com</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://ethnicraft.com</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Boom, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/458213251/ethnicraft.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Extremis NV</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili da esterno</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 12.900.125 € - 24,8 FTE (fonte trendstop.knack.be / companyweb.be, ultimo bilancio depositato NBB). 25a nel settore Meubelindustrie. N. impresa BE 0434.625.128. Sede Couthoflaan 20B, 8972 Poperinge (Proven). Designer e produttore di arredi da esterno (tavoli e panche con piani in legno duro tropicale e iroko, oltre ad acciaio e alluminio). Legame di gruppo: Groep Extremis (BE 0501.740.121). PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Dirk Wynants</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Fondatore e proprietario</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/extremis</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>info@extremis.com</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.extremis.com</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Poperinge (Proven), Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/434625128/extremis.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Hanssens Hout NV</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname e pannelli</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato € 15.493.557 (trendstop, 38ª nel settore 'houthandel'); ultimo fatturato riportato da pappers.be € 16.469.428. Impresa BE 0400.089.663. Sede: Port Arthurlaan 90, 9000 Gent (zona portuale). Grossista di legname, pannelli e materiali derivati. Fatturato in pieno target 10-20 M€. Amministratore anche tramite NV Port Arthur Invest (rappr. permanente Frederic Hanssens).</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Frederic Hanssens</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Bestuurder</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>info@hanssenshout.be</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hanssenshout.be/</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Gent (Fiandre, prov. Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/nl/company/hanssens-hout-0400.089.663</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Houthandel Denis Luyten NV</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 16.097.197 (trendstop, 35ª nel settore 'houthandel'); € 16.134.848 e 34,8 FTE secondo companyweb (ultimo bilancio depositato NBB). Impresa BE 0403.778.831, fondata 01-01-1968. Sede: Molenstraat 62, 2200 Morkhoven (Herentals). Commercio di legname, listelli, soffitti, parquet e legno da esterni; certificata FSC (elencata su ikzoekfsc.be). Fatturato in pieno target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>info@houtluyten.be</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://houtluyten.be/</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Morkhoven / Herentals (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/403778831/houthandel-denis-luyten.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Jori NV</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 16.143.273 € - 106,8 FTE (fonte companyweb.be / trendstop.levif.be, ultimo bilancio depositato NBB, deposito 21-07-2025). N. impresa BE 0888.984.313 (sul sito aziendale compare anche BE 0405.975.286, entita storica del gruppo). Fabbrica di divani e poltrone in pelle e tessuto con struttura in legno, sede Hoogweg 52, 8940 Wervik. Divisione contract JORI-care. PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jori</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>jori@jori.com</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jori.com</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Wervik, Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/nl/detail/888984313/jori.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Keukenontwerpers NV</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 16.033.016 € (fonte trendstop.knack.be, ultimo bilancio depositato NBB): 7a nel settore Vervaardiging en verkoop van keukenmeubelen. N. impresa BE 0472.648.534, costituita 09-08-2000. Sede Antwerpseweg 88, 2440 Geel (circa 20 addetti nella sede principale, piu showroom). ATTENZIONE: opera come distributore/installatore di cucine su misura (insegna SieMatic Keukenontwerpers) piu che come fabbricante: rilevante come trader EUDR di mobili in pannelli a base legno. IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>geel@keukenontwerpers.com</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>https://www.keukenontwerpers.com</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Geel, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/472648534/keukenontwerpers.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Lavrijsen Houtbedrijf NV</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio e lavorazione legname</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato € 12.763.339 (ultimo bilancio depositato NBB; fonte trendstop, 46ª nel settore 'houthandel'). Impresa BE 0407.106.030, fondata 13-05-1970. Sede: Koning-Albertstraat 68, 2440 Geel. 20-49 addetti. Commercio di legname + piallatura/segheria (houtschaverij). Fatturato in pieno target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Jan Lavrijsen e Bert Lavrijsen</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerders</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>info@lavrijsen-geel.be</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://lavrijsen.be/</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Geel (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/407106030/lavrijsen-houtbedrijf.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Manutti BV</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili da esterno</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 15.340.098 € - 27,4 FTE in Belgio (fonte companyweb.be / jaarrekening.be, bilancio depositato NBB 17-06-2024). N. impresa BE 0476.263.070. Fondata 03-12-2001, sede Beverenstraat 13-17, 8540 Deerlijk. Mobili da esterno di lusso con teak e legni tropicali; stabilimento produttivo in Indonesia (circa 140 addetti) - importazione diretta di legname, rischio EUDR alto. Legame di gruppo con Manutti Invest BV (BE 0478.148.434); finanziamento PMV. PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Stephane De Winter</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/manutti_official</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>info@manutti.com</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.manutti.com</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Deerlijk, Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/476263070/manutti.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Mecam NV</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 32.145.268 € - 111,6 FTE (fonte trendstop.knack.be / companyweb.be, bilancio depositato NBB 28-06-2025). 6a nel settore Meubelindustrie. N. impresa BE 0418.633.291. Sede Vilvertstraat 11, 3650 Dilsen-Stokkem (Lanklaar). Presentata come il maggior produttore di zitmeubelen del Benelux: divani e poltrone con telai in legno e rivestimenti in pelle (marchi Mecam e Neo-Style, sotto l'ombrello Mecam Group). Sopra la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Inge Meers</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>CFO e amministratrice (co-gestione con Luc Meers)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>info@mecamgroup.be</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mecamgroup.be</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Dilsen-Stokkem (Lanklaar), Limburgo (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/418633291/mecam.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Meubelfabriek Lievens NV</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in legno massello</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 19.952.978 € - 53,5 FTE (fonte trendstop.knack.be / companyweb.be, ultimo bilancio depositato NBB). 14a nel settore Meubelindustrie. N. impresa BE 0413.666.990. Fondata 24-08-1973, sede Kanegemstraat 11, 8700 Tielt. Produce mobili per sala da pranzo, soggiorno, camera e bagno in legno massello e pannelli melamminici. Appartiene alla holding familiare Telinfra (famiglia Ollevier) insieme a Confortluxe NV. IN TARGET (limite alto della fascia 10-20 M€).</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Lieven Decoene</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>info@lievensnv.be</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.lievensnv.be</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Tielt, Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/413666990/meubelfabriek-lievens.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Passe Partout NV</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 15.783.321 € - 11,3 FTE (fonte companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0464.204.485. Sede Wilfordkaai 10/B/C, 9140 Temse. Produttore e distributore B2B di mobili europei fatti a mano (divani, poltrone, panche, tavoli) con strutture in legno e rivestimenti in pelle/tessuto; vendita solo a rivenditori professionali. Espositore Meubelbeurs/Furniture Fair Brussels. PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Dirk Steenbeke</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder (amministratore)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/passe-partout-nv</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>info@passepartoutnv.be</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>https://passepartoutnv.be</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Temse, Fiandre Orientali (Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/464204485/passe-partout.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Royal Botania NV</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili da giardino in teak</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 21.667.220 € - 42,4 FTE (fonte trendstop.knack.be / companyweb.be, bilancio depositato NBB 15-04-2024). 14a nel settore Meubelindustrie. N. impresa BE 0447.099.427. Sede Elsendonkstraat 146, 2560 Nijlen. Arredi da esterno di alta gamma in teak e altri legni duri (oltre ad alluminio e inox): uso diretto di legname tropicale coperto dall'Allegato I EUDR. Filiale commerciale a New York. Leggermente sopra la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Kris Van Puyvelde</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>CEO e cofondatore</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>info@royalbotania.com</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>https://www.royalbotania.com</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Nijlen, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/447099427/royal-botania.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>VC Wood Zottegem NV</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato € 26.791.183 (ultimo bilancio depositato NBB; fonte trendstop, 23ª nel settore 'houthandel'). Impresa BE 0407.925.778, sede a 9620 Zottegem. Grossista di legname. BORDERLINE ALTO rispetto al target ideale 10-20 M€ ma entro il range tollerabile. Contatti (e-mail, referente) non reperiti in fonti pubbliche: da completare prima del contatto commerciale.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Zottegem (Fiandre, prov. Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/407925778/vc-wood-zottegem.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Vanerum België NV</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi scolastici contract</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 18.208.808 € - 74,5 FTE (fonte companyweb.be, bilancio depositato NBB 16-07-2024); trendstop.knack.be riporta 18.095.255 € e la 17a posizione nel settore Meubelindustrie. N. impresa BE 0421.014.939. Sede Kleine Schaluinweg 7, 3290 Diest. Dal 1968 progetta e produce arredi scolastici e per uffici (banchi, armadi, lavagne) con pannelli a base legno; azienda certificata FSC (elenco ikzoekfsc.be) - forte esposizione alle regole EUDR sui pannelli. Parte del gruppo internazionale Vanerum/i3-Group. IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Gert Van Erum</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>CEO / gedelegeerd bestuurder (tramite i3-Group Holding NV)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>info@vanerum.be</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vanerum.be</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Diest, Brabante Fiammingo (Vlaams-Brabant)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/421014939/vanerum-belgie.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Vincent Sheppard NV</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili in fibra e legno</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 20.832.726 € - 36,3 FTE in Belgio (fonte trendstop.knack.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0456.646.801. 14a nel settore Meubelindustrie per fatturato. Produttore di mobili Lloyd Loom e arredi indoor/outdoor con telai in legno massello e rattan; sede Industriepark 5, 8587 Spiere-Helkijn; produzione anche in Indonesia (rischio EUDR su legno e fibre importate). Leggermente sopra la fascia ideale ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Brendan McCarthy</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/vincent-sheppard</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>info@vincentsheppard.com</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vincentsheppard.com</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Spiere-Helkijn, Fiandre Occidentali (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/456646801/vincent-sheppard.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Woodtex NV</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — legname e pannelli</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 11.778.466 e 35,4 FTE (ultimo bilancio depositato NBB, deposito 23-06-2025; fonte trendstop, 50ª nel settore 'houthandel'). Impresa BE 0413.744.194. Sede: Boomsesteenweg (A12) 680-682, 2610 Wilrijk. Azienda familiare dal 1966 (3ª generazione: Bert e Karolien Van der Auwera), commercio di legname e plaatmateriaal + bouwmarkt. Fatturato in pieno target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/woodtex-nv</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>woodtex@woodtex.be</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://woodtex.be/</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Wilrijk / Antwerpen (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/413744194/woodtex.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Klingele Chocolade NV</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolato bio, fairtrade, senza zucchero</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ~8 M€ con ~40 dipendenti (fonte: UNIZO, KMO van het Jaar 2025); 32,7 FTE da ultimo bilancio depositato NBB (companyweb.be), che non pubblica la cifra d'affari. N. impresa BE 0479.916.606. Fondata 1995, export in oltre 40 paesi; cioccolato bio e Fairtrade — acquista fave/semilavorati certificati, operatore EUDR. Taglia sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Koen Klingele</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Managing director / gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/in/koen-klingele-a0b0509</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>info@klingelechocolade.be</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>https://klingelechocolade.be/</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Evergem (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.unizo.be/berichten/pers/klingele-chocolade-de-nationale-kmo-van-het-jaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Le Cercle du Cacao SRL</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — sourcing e trading fave</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>N. impresa BE 0843.535.556. Micro-impresa (fatturato non pubblicato nei conti depositati NBB, ben sotto i 5 M€: fuori dal target dimensionale). Inserita perché è un importatore/trader diretto di fave di cacao verso il porto di Anversa per i produttori bean-to-bar — operatore EUDR in senso stretto. Fondata nel 2012; sourcing da India, Colombia, Messico.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Nico Regout</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Fondatrice / Gérante</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/in/nico-regout-543a1350</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>info@lecercleducacao.be</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>http://lecercleducacao.be/</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Bruxelles (Schaerbeek, 1030) — Regione di Bruxelles-Capitale</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0843535556/le-cercle-du-cacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Van De Wiele Rubber NV</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — estrusione e stampaggio gomma</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato in bilancio; margine lordo 3.331.259 EUR e 28,4 FTE (Trends Top/NBB); n. impresa BE 0405.713.386</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/van-de-wiele-rubber</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>info@vandewiele-rubber.be</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vandewiele-rubber.be/</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Kluisbergen (Berchem, Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/405713386/van-de-wiele-rubber.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Accent NV</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 33.126.981 € (fonte derijkstebelgen.be su dati bilanci NBB; 17 M€ nel 2018). N. impresa BE 0428.014.379. Sede Westlaan 2, 8560 Gullegem (Wevelgem). Etichettificio fondato nel 1985 da Daniël Declerck, specializzato in etichette per food e non-food. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. LEGAME DI GRUPPO: capofila storica del gruppo Asteria (partecipato dal fondo Waterland), ca. 850 dipendenti in 7 paesi. Certificata FSC.</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Ives Declerck</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder / CEO</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/accent-etiketten</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>info@accent-etiketten.be</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://www.accent-etiketten.be</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Gullegem (Wevelgem), Provincia di Fiandre Occidentali (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/428014379/accent.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Allbox NV</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 35.733.025 € - 36,2 FTE (fonte trendstop.knack.be / staatsbladmonitor.be, bilancio depositato NBB il 19-07-2024). N. impresa BE 0417.348.339. Produttore integrato di cartone ondulato e imballaggi (design, ondulatore, trasformazione, trasporto in proprio), sede Venetiëlaan 28-30, 8530 Harelbeke. Azienda familiare con oltre 30 anni di attività. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€; società collegata: Verkoopkantoor Allbox en Desouter NV (BE 0419.278.540). Certificata FSC.</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>info@allbox.be</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>https://allboxnetwork.be</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Harelbeke, Provincia di Fiandre Occidentali (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/417348339/allbox.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Antilope De Bie NV</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 15.593.574 € - 72,1 FTE (fonte companyweb.be / trendstop.knack.be, ultimo bilancio depositato NBB, 2024). N. impresa BE 0414.535.339. Drukkerij familiare di 4a generazione attiva dal 1922, sede Nijverheidsstraat 6, 2570 Duffel. Cresciuta per acquisizioni (Antilope Printing 2017, Bema Graphics). PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Bart De Bie</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>CEO / Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/bartdebie-antilopedebie/</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>info@antilopedebie.be</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://antilopedebie.be</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Duffel, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0414535339/antilope-de-bie</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Autajon Packaging Belgium SA</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — astucci in cartone</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 30.789.352 € - 179,3 FTE (fonte fincheck.be / companyweb.be, bilancio depositato NBB il 17-07-2025). N. impresa BE 0402.682.929. Astucci pieghevoli e packaging premium in cartone per cosmetica, cioccolato e lusso; sede Boulevard Industriel 115, 1070 Anderlecht. Fondata nel 1968. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. LEGAME DI GRUPPO: filiale del gruppo francese Autajon. Membro ECMA.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>contact@autajon.com</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.autajon.com</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Anderlecht, Regione di Bruxelles-Capitale</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://fincheck.be/en/autajon-packaging-belgium/0402.682.929/Anderlecht/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Cartonnages Delsaux SA</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — astucci di lusso</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato nell'ultimo bilancio depositato NBB (schema abbreviato); margine lordo 2.828.246 € e 113° posto nel settore Emballage secondo trendstop.levif.be; organico dichiarato 20-49 collaboratori. N. impresa BE 0401.231.293, società costituita il 29-06-1963 con know-how risalente al 1885. Sede Boulevard du Textile 13, 7700 Mouscron. Trasformazione di cartone compatto in astucci rivestiti, cofanetti e packaging di lusso per cioccolato, vini e spiriti, cosmetica ed editoria. AZIENDA DI CONFINE: dimensione stimata sotto il target 10-20 M€, probabilmente vicina o inferiore ai 5 M€ di fatturato — da verificare sul bilancio integrale NBB.</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Christophe Delsaux</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Amministratore (direzione familiare con Charles e Sylvie Delsaux)</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/company/cartonnages-delsaux</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.cartonnagesdelsaux.com</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Mouscron, Provincia di Hainaut (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/401231293/cartonnages-delsaux.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Corpack NV</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>DATO DI FATTURATO NON REPERITO su fonti pubbliche accessibili (bilancio NBB da consultare direttamente). Produttore indipendente di imballaggi in cartone ondulato su misura (scatole americane stampate e imballaggi industriali pesanti), fondato nel 1994, rivolto specificamente alle PMI; stabilimento di 10.000 m² dal 2000. Sede Doornpark 20, 9120 Beveren-Waas. Certificata FSC. DA QUALIFICARE: dimensione presumibilmente nella fascia bassa 5-15 M€, da verificare.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr"/>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>info@corpack.be</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>https://corpack.be</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Beveren-Waas, Provincia di Fiandre Orientali (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bsearch.be/companyinfo/2/9083706359453121/G10/SE/corpack-beveren-waas-en.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Covera Packaging NV</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato nella fascia 10.000.000-25.000.000 € - 9,3 FTE (fonte companyweb.be / fincheck.be, ultimo bilancio depositato NBB; l'azienda deposita in schema abbreviato e non pubblica la cifra d'affari esatta). N. impresa BE 0462.810.754. Produzione e distribuzione di imballaggi in cartone ondulato e materiali d'imballaggio; sede Smallandlaan 37, 2660 Hoboken (Antwerpen). Origine familiare come Comptoir Verrier Anversois. IN TARGET stimato ma verificare il fatturato esatto.</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Johan Stouten</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/covera-packaging</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>sales@covera.be</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://covera.be</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Hoboken (Anversa), Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://fincheck.be/nl/covera-packaging/0462.810.754/Antwerpen/overzicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Desmedt Labels BV</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 6.500.000 € con 32 dipendenti secondo l'ultimo dato pubblicato (fonte made-in.be / Voka Ondernemers); organico più recente indicato in ca. 21 persone a Bornem. Azienda familiare fondata nel 1889 da François Desmedt, oggi alla quinta generazione (Henri Kökler); trasferita da Bruxelles a Bornem nel 2012. Etichette autoadesive prodotte in modo CO2-neutro. SOTTO il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€; dato di fatturato non recentissimo, da riverificare sul bilancio NBB.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Henri Kökler</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/desmedt</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.desmedt.be</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Bornem, Provincia di Anversa (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.made-in.be/antwerpen/desmedt-labels-neemt-nieuwe-start/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Emballages Gruselle SRL</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — imballaggi cartone</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>DATO DI FATTURATO NON PUBBLICATO sulle fonti accessibili (companyweb/fincheck/pappers riportano la scheda ma non la cifra d'affari; l'azienda deposita in schema abbreviato). N. impresa BE 0448.350.331, costituita nel 1992. Azienda familiare, fabbricazione di scatole in cartone e articoli d'imballaggio e protezione; officina nel parco industriale di Martinrou, Rue de Rabiseau 12, 6220 Fleurus. AZIENDA DI CONFINE: taglia stimata SOTTO i 5 M€ — inserita per copertura della filiera in Vallonia, da qualificare prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>gruselle@skynet.be</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.emballagesgruselle.eu</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Fleurus, Provincia di Hainaut (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/448350331/gruselle-emballages.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Etilux SA</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato consolidato ca. 16.000.000 € e 50 dipendenti (fonte ccimag.be, gennaio 2024; l'articolo ccimag di giugno 2023 indicava ca. 18 M€). 42 FTE nell'ultimo bilancio depositato NBB; la società deposita in schema abbreviato e non pubblica la cifra d'affari (fonte pappers.be / companyweb.be). N. impresa BE 0412.681.550. Sede Rue de l'Espérance 42, 4000 Liegi. Azienda familiare fondata nel 1972: etichette adesive, tracciabilità/RFID, adesivi tecnici e imballaggi; filiale in Lussemburgo. IN TARGET 10-20 M€. Secondo amministratore delegato: Olivier Bronne.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Quentin Gemoets</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>info@etilux.be</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.etilux.com</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Liegi, Provincia di Liegi (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://ccimag.be/2024/01/05/la-transition-generationnelle-se-finalise-chez-etilux/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Imprimerie Bietlot SA</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 6.970.646 € - 33,5 FTE (fonte companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0473.613.485. Imprimerie industriale offset (magazine, edizione, stampati amministrativi), sede Rue du Rond-Point 185, 6060 Gilly (Charleroi). SOTTO IL TARGET 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Partecipata storica di Sambrinvest.</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>info@bietlot.be</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.bietlot.be</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Gilly (Charleroi), Provincia di Hainaut (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/fr/0473613485/imprimerie-bietlot</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Kartonnage Lefevere-Beel NV</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 26.865.930 € - 69,2 FTE (fonte pappers.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0413.759.339. Trasformazione di cartone ondulato in imballaggi su misura, sede Driekoningenstraat 7, 8710 Wielsbeke. Amministratori: Didier Lefevere, Marieke Lannoo e la società BellRock. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Didier Lefevere</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>CEO / Bestuurder</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/kartonnage-lefevere-beel</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>info@lefeverebeel.be</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lefeverebeel.be</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Wielsbeke, Provincia di Fiandre Occidentali (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/nl/company/kartonnage-lefevere-beel-0413759339</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Label-Pak-Int'l Co SA</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato NON pubblicato nell'ultimo bilancio depositato NBB (schema abbreviato, deposito 01-07-2023); margine lordo 1.920.400 € e 27,2 FTE (fonte companyweb.be / fincheck.be). N. impresa BE 0402.690.550. Sede Avenue Galilée 8, 1300 Wavre. Azienda familiare fondata nel 1968, oltre 50 anni di stampa di etichette personalizzate in carta. AZIENDA DI CONFINE: dimensione stimata SOTTO il target 10-20 M€ e probabilmente sotto i 5 M€ — da verificare sul bilancio integrale NBB.</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Wavre, Provincia del Brabante Vallone (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0402690550/label-pak-int-l-co</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Snel Grafics SA</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 11.822.115 € (fonte trendstop.levif.be / companyweb, ultimo bilancio depositato NBB). Ca. 65 dipendenti (fonte ccimag.be / RTBF). N. impresa BE 0440.957.842. Imprimerie offset e digitale (libri, brochure) rilevata in MBO nel 1995 da Roland Soubras e Flavio De Beni. Sede Rue du Fond des Fourches 21, 4041 Vottem. IN TARGET.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Roland Soubras</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/in/roland-soubras-63aa1560</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>info@snel.be</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.snel.be</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Vottem (Herstal), Provincia di Liegi (Vallonia)</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/440957842/snel-grafics.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Van de Velde Packaging NV</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 15.032.194 € - 52,3 FTE (fonte fincheck.be / pappers.be, ultimo bilancio depositato NBB). N. impresa BE 0444.255.050. Produzione di imballaggi in carta e cartone ondulato, sede Industrielaan 22, 8810 Lichtervelde. PERFETTAMENTE IN TARGET 10-20 M€. LEGAME DI GRUPPO: società del gruppo belga P. Van de Velde / Van de Velde Packaging (quartier generale a Wetteren, ca. 1.300 addetti e 309 M€ di fatturato di gruppo nel 2023, sedi in 8 paesi europei; aumento di capitale 2025 sottoscritto da Kartesia); il gedelegeerd bestuurder iscritto in KBO è la persona giuridica P. Van de Velde NV.</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Carl Mourisse</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Bestuurder</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>info.lichtervelde@vandeveldepackaging.com</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vandeveldepackaging.com</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Lichtervelde, Provincia di Fiandre Occidentali (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>https://fincheck.be/en/van-de-velde-packaging/0444.255.050/Lichtervelde/overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Varia-Pack NV</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — commercio imballaggi carta</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 23.056.460 € - 36,1 FTE (fonte fincheck.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0407.977.446. Grossista/distributore di articoli di carta e cartone e materiali d'imballaggio (NACE commercio all'ingrosso di carta e cartone), sede Aarschotsesteenweg 114, 3012 Wilsele-Leuven. Fondata il 18-01-1971. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. LEGAME DI GRUPPO: appartiene al gruppo britannico Bunzl.</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
+      <c r="F49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.variapack.com</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Wilsele (Leuven), Provincia del Brabante Fiammingo (Fiandre)</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://fincheck.be/nl/varia-pack/0407.977.446/Leuven/overzicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Belmoca NV</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — capsule e private label</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 13.137.013 (ultimo bilancio depositato NBB; fonte trendstop, 19ª nel settore 'koffie en thee'). Impresa BE 0842.626.627. Sede: Weversstraat 24, 1840 Londerzeel. Produttore di capsule di caffè compatibili (marchio proprio Belmio, lanciato nel 2016) e private label per terzi: acquista e immette caffè sul mercato UE = operatore EUDR. Fatturato in pieno target 10-20 M€. Altro dirigente pubblicato: Alain Adler, Managing Director.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Bruno van Den Branden</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>https://belmoca.com/</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Londerzeel (Fiandre, prov. Vlaams-Brabant)</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/842626627/belmoca.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Koffie St.-Michel NV</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione e private label</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Impresa BE 0406.919.552, fondata nel 1880. Sede: Asiadok 28A, 2030 Antwerpen (porto di Anversa). Margine lordo € 686.005 e 43ª posizione nel settore 'koffie en thee' (trendstop); NON pubblica il fatturato nell'ultimo bilancio depositato (schema abbreviato NBB → ricavi presumibilmente sotto la soglia delle piccole società, ~11 M€): TAGLIA DA VERIFICARE, possibile sotto i 5 M€. Torrefazione familiare, indicata come la più antica e la più grande di Anversa (fornisce ~60% del mercato locale) e private-label roaster per marchi terzi. Contatto alternativo pubblicato: stmichel@skynet.be. Tel. 03 234 34 70.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Hendrik Hanssens</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Bedrijfsleider (5ª generazione)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>info@stmichel.be</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>https://stmichel.be/</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/406919552/koffie-st-michel.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Rucquoy Frères NV</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 17.021.444 (ultimo bilancio depositato NBB, deposito 04-06-2025; fonte companyweb/trendstop). Impresa BE 0404.850.383. Sede: Van Meterenkaai 4 bus 14, 2000 Antwerpen (sede sociale registrata anche a Brasschaat). Azienda familiare dal 1919, import/export di caffè verde. TARGET IDEALE: importatore = operatore EUDR in senso stretto, fatturato in pieno range.</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Steven De Punt</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/rucquoy-fr%C3%A8res</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>trade@rucquoy.com</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>https://rucquoy.com/</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0404850383/rucquoy-freres</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Sas NV (Sas Coffee)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione e private label</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato € 37.126.839 (ultimo bilancio depositato NBB; fonte trendstop, 14ª nel settore 'koffie en thee'). Impresa BE 0404.190.783. Sede: Dennenlaan 10, 2340 Beerse. Azienda familiare dal 1947, torrefazione + confezionamento private label; fatturato triplicato in 10 anni. BORDERLINE ALTO: 37 M€, entro il range tollerabile (max 40) ma sopra il target ideale 10-20 M€. Torrefattore = importa/immette caffè sul mercato UE, operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Herman Sas</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>info@sas-koffie.be</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>https://sas-coffee.com/</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Beerse (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/404190783/sas.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Silco NV</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — commercio caffè verde</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato € 8.358.215 (ultimo bilancio depositato NBB, deposito 14-06-2024; fonte trendstop, 23ª nel settore 'koffie en thee'). Impresa BE 0715.792.692. Sede: Italiëlei 181, 2000 Antwerpen. Attività principale: groothandel in koffie, thee, cacao en specerijen (NACE 46370). SOTTO IL TARGET IDEALE (8,4 M€, entro il minimo tollerabile) e struttura molto snella (1 FTE dichiarato): tipica trading house di caffè verde. Da verificare la sostanza operativa prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/715792692/silco.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>A &amp; A Chocolaterie NV</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — figure stagionali e tavolette</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 22.087.972 € (ultimo bilancio depositato NBB, deposito 22-10-2025; 25.604.502 € e 31° posto di settore su trendstop.knack.be). N. impresa BE 0892.388.320. Sede Mosten 16, 9160 Lokeren; lavora ~15 t di cioccolato al giorno. Nella parte alta del target ma dentro il range. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), insieme alla consociata Pralinart NV.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hamlet.be/</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0892388320/a-a-chocolaterie</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Belvas SA</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline bio equosolidali</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 10.258.810 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0472.516.692. Cioccolateria industriale bio e Fairtrade: importa fave/semilavorati di cacao certificati — operatore EUDR. Perfettamente in target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Thierry Noesen</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Fondatore / Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>info@belvas.be</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>https://www.chocolaterie-belvas.be/</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Ghislenghien / Meslin-l'Évêque (Ath), Hainaut — Vallonia</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/fr/company/belvas-0472516692</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Bruyerre Chocolates SA</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 6.140.610 € (fonte: trendstop.levif.be, ultimo bilancio depositato NBB). N. impresa BE 0688.794.525. Cioccolatiere dal 1909, oltre 80 varietà di praline. Sotto la fascia ottimale ma nel range tollerabile 5-40 M€. Legame di gruppo: entità distinta da Bruyerre SA (BE 0431.703.151, distribuzione alimentare, ~179,6 M€ — quest'ultima fuori target).</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>contact@bruyerre.eu</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>https://bruyerre.eu/</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Gosselies (Charleroi), Hainaut — Vallonia</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/688794525/bruyerre-chocolates.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Chocolaterie Ickx NV</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 32.746.626 € e 139,7 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-03-2026). N. impresa BE 0421.359.189. Fondata 1981; forte export (Cina, Asia). Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI indipendente.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/chocolaterie-ickx</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>avangastel@choc-ickx.be</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ickx.be/</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Essen (Anversa) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0421359189/chocolaterie-ickx</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Confiserie De Bie - L'Abeille - Trefin NV</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolato e confetteria</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 11.404.101 € e 34,4 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 08-06-2026). N. impresa BE 0400.120.050. Sede Waaslandlaan 5, 9160 Lokeren. Produttore di cioccolato e caramelle (marchio Trefin). In pieno target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>info@trefin.com</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.trefin.com/</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0400120050/confiserie-de-bie-l-abeille-trefin</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Confiserie Vandenbulcke NV</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e tavolette</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 13.332.120 € e 31,5 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-12-2024). N. impresa BE 0417.738.319. Fondata 1949; export in oltre 50 paesi. In pieno target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/chocolatiervandenbulcke</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>info@vandenbulcke.com</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vandenbulcke.com/</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Heule, Kortrijk (West-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0417738319/confiserie-vandenbulcke</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Corné Port-Royal Chocolatier SA</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline artigianali</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 8.796.906 € (ultimo bilancio depositato NBB, deposito 26-06-2025; 8.421.952 € e 54° posto di settore su trendstop.knack.be). N. impresa BE 0433.283.558. Sede Avenue Vésale 12, 1300 Wavre; maison storica (marchio dal 1932), rete di ~20 boutique in Belgio e 15 in Francia. Sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/corn-port-royal</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.corneportroyal.com/</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Wavre (Brabant wallon) — Vallonia</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0433283558/corne-port-royal-chocolatier</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Delafaille NV</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 14.244.468 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB, deposito 17-06-2025); 43° nel settore cioccolato e dolciumi. N. impresa BE 0467.502.683. In pieno target 10-20 M€. Legame di gruppo: acquisita dallo svizzero Maestrani Schweizer Schokoladen (con la controllata Ostrapack); resta però PMI belga autonoma con obblighi EUDR propri.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Paul Daems</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>CEO / gedelegeerd bestuurder (uscente, transizione dopo l'acquisizione Maestrani 2025)</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>https://www.delafaille.be/</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Melsele, Beveren-Kruibeke-Zwijndrecht (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/467502683/delafaille.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Dolfin SA</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — tavolette premium</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>33,2 FTE da ultimo bilancio depositato NBB (deposito 20-01-2026, cifra d'affari non pubblicata); fatturato ~6 M€ secondo la stampa economica (L'Avenir/RTBF, ~385 t di cioccolato/anno). N. impresa BE 0437.332.220. Sede Avenue Robert Schuman 172, 1401 Baulers (Nivelles). Prima cioccolateria belga certificata carbon neutral (2008); programma di sostenibilità cacao proprio 'Cocoa Act 4'. Taglia sotto la fascia ottimale, nel range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/dolfin-sa</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dolfin.be/</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Baulers, Nivelles (Brabant wallon) — Vallonia</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0437332220/dolfin</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Gudrun Commercial NV</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e tartufi</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 43.457.280 € e 138,6 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 15-07-2026). N. impresa BE 0476.530.118. Sede Industriestraat 18, 2500 Lier. Firmataria di Beyond Chocolate. AZIENDA DI CONFINE: fatturato sopra la fascia tollerabile 5-40 M€ (ma sotto la soglia di esclusione ~50 M€). Legame di gruppo: acquisita dal gruppo spagnolo Natra (che controlla anche Natra Chocolate Belgium NV, ~93 M€, fuori target).</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Sofie De Lathouwer</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/gudrun-commercial-nv</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>info@chocolates.be</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>https://gudrungroup.be/</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Lier (Anversa) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0476530118/gudrun-commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>La Chocolaterie Galler SA</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — tavolette e praline</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 29.502.986 € (fonte: pappers.be/trendstop, bilancio NBB); dato più recente ~32 M€ con perdita netta 1,7 M€ nel 2024; 194 dipendenti. N. impresa BE 0416.169.689. Azienda di confine nella parte alta del range tollerabile (5-40 M€). Nota: nell'aprile 2026 rilevata da un consorzio vallone con piano di ristrutturazione (~70 licenziamenti su 170).</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.galler.com/</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Vaux-sous-Chèvremont (Chaudfontaine), Liegi — Vallonia</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/fr/company/la-chocolaterie-galler-0416169689</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Libeert NV</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — figure e tavolette di cioccolato</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ~35 M€ e 136,8 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 13-11-2025). N. impresa BE 0407.026.747. Azienda familiare, oltre 5.000 t di cioccolato all'anno, gamma bio. Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Lily Libeert</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Co-directrice (4a generazione della famiglia Libeert)</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>contact@libeert.com</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>https://www.libeert.com/</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Comines-Warneton (Komen-Waasten), Hainaut — Vallonia</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0407026747/libeert</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Manufacture Belge de Chocolats SRL</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e private label</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 25.731.148 € e 175,1 FTE (fonte: trendstop.levif.be / companyweb.be, ultimo bilancio depositato NBB, deposito 08-07-2025); 30° posto nel settore cioccolato e dolciumi. N. impresa BE 0722.764.519. Firmataria di Beyond Chocolate (impegni su deforestazione e tracciabilità del cacao). Nella parte alta del range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Arnaud Verwilghen</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>info@mbcchocolates.be</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mbcchocolates.be/</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Koekelberg, Bruxelles (1081) — Regione di Bruxelles-Capitale</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/722764519/manufacture-belge-de-chocolats.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Oxfam Fair Trade CV</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — import equosolidale cacao</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 17.446.343 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB); 81° posto nel settore alimentare/commercio. N. impresa BE 0453.066.016. Importatore equosolidale: acquista cacao (e caffè) direttamente dalle cooperative dei paesi produttori e immette i prodotti sul mercato UE — operatore EUDR in senso stretto. Firmataria di Beyond Chocolate. In pieno target 10-20 M€. Nota: struttura cooperativa legata a Oxfam-Wereldwinkels.</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>info@oft.be</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>https://www.oxfamfairtrade.be/</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Gent (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/453066016/oxfam-fairtrade.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Pierre Marcolini Group SA</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — bean-to-bar e praline</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 19.300.806 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0461.740.982. Maison bean-to-bar: acquista e importa direttamente fave di cacao dai paesi d'origine (Vietnam, Madagascar, Ecuador, Perù) — operatore EUDR in senso stretto. In pieno target 10-20 M€. Legame di gruppo: entità collegata Pierre Marcolini Belgium SA (BE 0460.046.551, ~11,3 M€, rete retail).</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>https://eu.marcolini.com/</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Bruxelles (Haren, 1130) — Regione di Bruxelles-Capitale</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pappers.be/fr/company/pierre-marcolini-group-0461740982</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Pralinart NV</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 18.427.020 € e 34 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 02-11-2023). N. impresa BE 0450.589.051. Sede Waaslandlaan 32, 9160 Lokeren; fino a 10 t di praline al giorno. In pieno target 10-20 M€. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), consociata di A &amp; A Chocolaterie NV.</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hamlet.be/</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0450589051/pralinart</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Hannecard Benelux NV</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — rivestimenti in gomma per rulli</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 16.954.714 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 83,3 FTE; n. impresa BE 0694.906.812</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/hannecard-nv</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>contact@hannecard.com</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hannecard.com/</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Ronse / Renaix (Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/694906812/hannecard-benelux.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Helvoet Rubber &amp; Plastic Technologies NV</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — articoli tecnici in gomma stampata</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 17,48 M EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0867.662.822</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr"/>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>info.lommel@helvoet.com</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>https://www.helvoet.com/</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Lommel (Limburg, Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/867662822/helvoet-rubber-plastic-technolog-.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Hercorub NV</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — rubbercompounds, technische rubberartikelen</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 15.240.806 EUR (Trends Top/NBB, ultimo esercizio pubblicato); ca. 67-95 dipendenti (fonte aziendale); n. impresa BE 0421.767.381</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Patrick Lenaerts</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Afgevaardigd bestuurder (gedelegeerd bestuurder)</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/hercorub-nv</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>info@hercorub.com</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hercorub.be/</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Lanaken (Limburg, Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/421767381/hercorub.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Hexpol Compounding BV</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — mescole di gomma (rubber compounding)</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 31.327.285 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0430.105.126</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hexpol.com/rubber/plant-locations/hexpol-compounding-sprl/</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Eupen (Liège, Wallonie – Ostbelgien)</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/430105126/hexpol-compounding.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Baert Mengvoeders NV</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi composti bovini, suini, pollame</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 38.875.690 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti — taglia gonfiata dal costo materia prima; n. impresa BE 0455.400.845</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Eric Baert</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/baert-mengvoeders</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>info@baertmengvoeders.be</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.baertmengvoeders.be/</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Zele (Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/455400845/baert-mengvoeders.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Vanrobaeys Granen &amp; Zaden NV</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — granaglie e semi per mangimi</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 19.714.376 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti; n. impresa BE 0452.220.037</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>info@vanrobaeysbelgium.com</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vanrobaeysbelgium.com/</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Menen-Rekkem (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/452220037/vanrobaeys-granen-zaden.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Voeders Debaillie NV</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi composti per bestiame</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 11.114.628 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0405.174.839</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Philippe Debaillie</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/voeders-debaillie---aliments-debaillie</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>info@debaillie.be</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>https://debaillie.be/</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Roeselare (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/405174839/voeders-debaillie.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Voeders Mellaerts NV</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi e materie prime</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 33.531.211 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 11,5 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0455.669.079</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/voeders-mellaerts</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>order@voedersmellaerts.eu</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>https://voedersmellaerts.eu/</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Tielt-Winge (Sint-Joris-Winge, Vlaams-Brabant)</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/455669079/voeders-mellaerts.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Voeders Scherrens NV</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi composti su misura</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 36.374.114 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0421.626.732</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Geert Scherrens</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/scherrensvoeders</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>info@scherrensvoeders.be</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.scherrensvoeders.be/</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Wingene (West-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/421626732/voeders-scherrens.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Vandeputte Oleochemicals SA</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — raffinazione oli vegetali (soia, lino)</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 34.266.885 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 18 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0471.546.593</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr"/>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.vandeputte.com/en/oleochemicals/</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Mouscron (Hainaut, Wallonie)</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/471546593/vandeputte-oleochemicals.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Baeten &amp; Co NV</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Olio di palma — raffinazione oli e grassi vegetali/animali</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 42.810.588 EUR (bilancio NBB depositato 15-07-2025) — taglia gonfiata dal costo materia prima: solo 13,7 FTE; n. impresa BE 0447.081.908</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr"/>
+      <c r="E81" s="3" t="inlineStr"/>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>info@baetennv.be</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>https://baetennv.be/</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Berlare (Overmere, Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0447081908/baeten-co</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Repro NV</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — raffinazione oli e grassi vegetali</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 14.157.353 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 1-5 dipendenti (societa' di raffinazione del Group Vandamme); n. impresa BE 0439.000.818</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr"/>
+      <c r="E82" s="5" t="inlineStr"/>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>https://www.groupvandamme.com/</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Deinze (Oost-Vlaanderen)</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/439000818/repro.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Royale Lacroix SA</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Olio di palma — margarine e grassi alimentari</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 49.349.520 EUR (bilancio NBB, ultimo esercizio pubblicato) — taglia gonfiata dal costo materia prima: solo 18,6 FTE; n. impresa BE 0404.423.583</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Patrice Lacroix</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/royale-lacroix</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>info@royalelacroix.be</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.royalelacroix.com/</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Flémalle (Liège, Wallonie)</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0404423583/royale-lacroix</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Ameloot BV</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macellazione e ingrosso</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 49.298.205 EUR (Trends Top/NBB, ultimo esercizio); n. impresa BE 0413.029.562. AZIENDA DI CONFINE: sopra i 40 M€ ma PMI familiare indipendente (3a generazione) con macello integrato SGL; dal 2024 controlla Slachtgroep Leieland BV; fatturato gonfiato dal costo materia prima.</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr"/>
+      <c r="E84" s="5" t="inlineStr"/>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>petra@ameloot.org</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>https://omerameloot.com/nl</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Harelbeke (West-Vlaanderen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/413029562/ameloot.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Dierickx NV</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — sezionamento carne bovina</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 40.843.828 EUR (ultimo bilancio depositato NBB, via Trends Top/Companyweb); azienda familiare indipendente alla 5a generazione; n. impresa BE 0422.204.673. Al limite alto della fascia: nella carne il fatturato e' gonfiato dal costo della materia prima.</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Cis van den Broeck</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>info@dierickxnv.be</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>https://dierickxnv.be/</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Zele (Oost-Vlaanderen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/422204673/dierickx.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Euro Meat Group NV</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macellazione bovini</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 11 milioni EUR (VILT, stampa settoriale agroalimentare belga); organico ca. 50 persone (40 operai + 10 impiegati); capacita' 75.000 bovini ed equini/anno, ca. 125.000 bovini macellati per conto terzi. Numero d'impresa BE non verificato su fonte pubblica. Fa parte del gruppo Cadus NV (macelli in Belgio) ed e' socio Febev.</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr"/>
+      <c r="E86" s="5" t="inlineStr"/>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>http://www.euromeatgroup.be/nl/home/</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>Moeskroen / Mouscron (Hainaut, Vallonia)</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>https://vilt.be/nl/nieuws/vijf-vleesspecialisten-nemen-familiebedrijf-derwa-over</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Jos Leemput BV</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — commercio all'ingrosso e sezionamento</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 44.954.796 EUR e 16,2 FTE (ultimo bilancio depositato NBB, via Companyweb/FinCheck); n. impresa BE 0424.110.724. AZIENDA DI CONFINE: sopra 40 M€ ma con soli 16 dipendenti - caso tipico di fatturato gonfiato dal costo della materia prima; PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Jos Leemput</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Titolare, responsabile acquisto e selezione bestiame (sito aziendale)</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.leemput.be/</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>Tienen / Hakendover (Vlaams-Brabant, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/424110724/leemput-jos.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Slachthuis Swaegers NV</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macellazione e sezionamento bovini</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 4.287.787 EUR e 4,8 FTE nella societa' di macellazione (ultimo bilancio NBB, via Companyweb/Trends Top); n. impresa BE 0436.764.571. SOTTO LA SOGLIA dei 5 M€ come singola entita': il fatturato riflette solo i servizi di macellazione: il gruppo familiare Swaegers &amp; Co dichiara 70.000 bovini/anno e 22.000 t di capacita' annua, quindi volumi EUDR molto superiori al fatturato contabile.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr"/>
+      <c r="E88" s="5" t="inlineStr"/>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>info@swaegers.be</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>https://www.swaegers.be/</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Hoogstraten (Antwerpen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/nl/detail/436764571/swaegers-slachthuis.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Slachthuis Velzeke BV</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macellazione bovini</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>50-99 dipendenti (Companyweb, dati piu' recenti); capacita' 2.000 bovini/settimana, uno dei maggiori macelli bovini del Belgio; n. impresa BE 1018.071.121. Fatturato NON disponibile: entita' costituita il 30/12/2024 (cambio di proprieta' nel 2025), nessun bilancio con cifra d'affari ancora depositato. Altri amministratori indicati: Guy De Bruycker, Johan Castelein.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Wouter Cokelaere</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Bestuurder</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr"/>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Velzeke-Ruddershove, Zottegem (Oost-Vlaanderen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/nl/1018071121/slachthuis-velzeke</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Sopraco NV</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — fornitura e ingrosso carni</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 8.889.508 EUR e 45,5 FTE (ultimo bilancio depositato NBB, via Companyweb/Trends Top); n. impresa BE 0507.988.901. Nella fascia bassa tollerata (5-40 M€). Capofila del gruppo familiare Sopraco, che dal 2017 controlla anche Rompa Leder (filiera pelle): doppia esposizione EUDR bovini + pelle.</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr"/>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>info@sopraco.eu</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sopraco.eu/</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Geel (Antwerpen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>https://trendstop.knack.be/en/detail/507988901/sopraco.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Van De Walle SRL</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — commercio all'ingrosso</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>n. impresa BE 0893.625.564 (Trends Top). Fatturato e organico NON pubblicati in forma accessibile (schema abbreviato NBB): azienda familiare fondata nel 1954, filiera verticalizzata dall'allevamento alla consegna con flotta frigo propria, clientela di macellerie e GDO. Dimensione stimabile come PMI, da verificare sul bilancio NBB.</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="3" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>info@vdw-grossisteenviande.be</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>https://vdw-grossisteenviande.be/</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Wayaux / Villers-Perwin, Les Bons Villers (Hainaut, Vallonia)</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>https://trendstop.levif.be/fr/detail/893625564/van-de-walle.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Vleeshandel Vens NV</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — ingrosso e sezionamento</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>32 FTE in bilancio (oltre 40 collaboratori secondo il sito aziendale); fatturato NON pubblicato (schema abbreviato NBB), margine lordo dichiarato 1.950.416 EUR; n. impresa BE 0468.329.064. Azienda familiare dal 1975; tratta rundsvlees, kalfsvlees, varkensvlees e lamsvlees.</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr"/>
+      <c r="E92" s="5" t="inlineStr"/>
+      <c r="F92" s="5" t="inlineStr"/>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>https://vleeshandelvens.be/</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Lendelede (West-Vlaanderen, Fiandre)</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>https://www.companyweb.be/en/0468329064/vleeshandel-vens</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J92"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId185"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Austria: CONSEGNATA - 93 aziende (email 90/93, referente 92/93)
PROGETTO COMPLETO: 8 fogli, 737 righe, 0 entita HTML, 0 anomalie su email e
LinkedIn. IT 95, DE 97, FI 84, DK 89, SE 89, NL 100, BE 90, AT 93.
Handoff: sezione 15 con esclusioni (filiali di gruppi esteri, aziende in
insolvenza, oli fuori Allegato I) e note di filiera.
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Svezia" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Olanda" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Belgio" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Austria" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Italia'!$A$2:$J$97</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32717,4 +32719,4863 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MyEUDR — Lead mapping · Austria · aziende potenzialmente soggette all'EUDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Denominazione</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Filiera EUDR</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Dimensione (fatt./dip.)</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Referente</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Ruolo</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Email / PEC</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Sito web</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>Sede</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Ludwig Reiter Schuhmanufaktur GmbH</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — calzature e pelletteria in cuoio</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ca. 15 Mio. € fatturato annuo, ca. 60 dipendenti, ca. 30.000 paia/anno (Wikipedia/AustriaWiki, dati 2019-2023). Secondo GF: Mag. Richard Reiter. Firmenbuch FN 242908v</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Ludwig Potyka-Reiter</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>office@ludwig-reiter.com</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ludwig-reiter.com/</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Wien (Süßenbrunn, 22. Bezirk), Wien</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/ludwig-reiter-schuhmanufaktur-gmbh_aJD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Tschurtschenthaler Gerberei GmbH</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — conceria e commercio pelli</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ca. 70.000 m² di pelli conciate/anno (firmenabc.at / meinbezirk.at); fatturato e organico non pubblicati. NOTA: conceria artigianale attiva dal 1890, sotto la soglia target di fatturato</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Alexander Tschurtschenthaler</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>St. Stefan im Gailtal, Kärnten</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/tschurtschenthaler-gerberei-gmbh_meb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Waldviertler Werkstätten GmbH</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Pelle/Concia — calzature e pelletteria in cuoio</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ca. 17,5-19 Mio. € fatturato (2016-2019, noe.ORF.at / NÖN); ca. 200-300 dipendenti (firmenabc.at). Secondo GF: Paul Tritscher</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Heinrich Staudinger</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>gea@gea.at</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>https://gea-waldviertler.at/</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Schrems, Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/waldviertler-werkstaetten-gmbh_jTd</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ANREI-Reisinger Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili massello</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>100-249 dipendenti (Kompass/karriere.at, 2024); fatturato non pubblicato. Produttore di mobili in legno massello (soggiorno, zona notte, sala da pranzo).</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Kurt Reisinger</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>anrei@anrei.at</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>https://anrei.at</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Pabneukirchen, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/anrei-reisinger-gesellschaft-m-b-h_DId</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>BRAUN LOCKENHAUS GmbH</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi contract</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>53-58 dipendenti (firmenabc.at / WKO, 2024-2025); fatturato non pubblicato - bilancio 5,0 M€ di totale attivo (firmenabc.at, es. 2024). Stima di fatturato plausibile sotto i 15 M€ ma NON confermata. Fa parte del gruppo SCHNEEWEISS interior / SCHNEEWEISS AG.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Jochen Joachims</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/braun-lockenhaus</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>info@braunlockenhaus.at</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.braunlockenhaus.at</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Lockenhaus (Hammerteich), Burgenland</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/braun-lockenhaus-gmbh_Foy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Breitschopf Gesellschaft mbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>ca. 30 M€ di fatturato annuo e 150 dipendenti; ca. 1.600 cucine su misura/anno (weekend.at/chefinfo + breitschopf.at, 2024). Produzione a Dietach. Co-Geschäftsführer: Johannes Breitschopf e Johann Breitschopf.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Martin Breitschopf</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/breitschopf-kuechen</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>info@breitschopf.at</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.breitschopf.at</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Dietach, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.breitschopf.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CONFORM Badmöbel GmbH</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili da bagno</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 9,0 M€ (stima Die Deutsche Wirtschaft, 2024); dipendenti: ca. 80 (LinkedIn) / 30 (WKO). AZIENDA DI CONFINE: leggermente sotto la soglia di 10 M€. Ragione sociale a Firmenbuch: Conform Badmöbel Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Herbert Schwingenschuh</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/conform-badm%C3%B6bel-gmbh</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>office@conformbad.at</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.conformbad.at</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Imst, Tirol</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/conform-badmoebel-gesellschaft-m-b-h_GrLx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>HOLZBAU MAIER GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — costruzioni in legno/Holzbau</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 35,0 Mio EUR (stima DDW, ranking imprese familiari austriache n. 917); oltre 140 dipendenti (sito aziendale). FN 525501x, LG Salzburg. Co-GF: Hildegund Maier. Fascia alta del target</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Birgit Maier</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>holzbau@maier.at</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>https://www.maier.at</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Bramberg am Wildkogel (Salzburg)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>https://die-deutsche-wirtschaft.de/famu_top/oesterreich-holzbau-maier-gmbh-co-kg-bramberg-umsatz-mitarbeiterzahl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Holzindustrie Kaml &amp; Huber Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria, legname di abete essiccato</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>30 dipendenti; taglio annuo ca. 100.000 fm; 9 celle di essiccazione da 1.200 m3 (sito aziendale). Fatturato non pubblicato, fascia stimata 15-20 Mio EUR. FN 79141i. Altri GF: Rupert Kaml, Petra Huber</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Rupert Huber</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>office@kaml-huber.com</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kaml-huber.com</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Rottenmann (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kaml-huber.com/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Holzindustrie Schafler GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imballaggi in legno/pallet</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>ca. 90 dipendenti (Industrielandkarte Steiermark); fatturato non pubblicato. Fra i maggiori produttori austriaci di imballaggi in legno (pallet, telai, tavole da cassero, bobine per cavi)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Bernd Christoph Schafler</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>info@schafler-holz.at</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.schafler-holz.at</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Hirnsdorf (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>https://holzindustrie-steiermark.industrielandkarte.com/betriebe/holzindustrie-schafler</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Hrachowina Fenster &amp; Türen GmbH</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — finestre e porte in legno</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato stimato ca. 25 Mio EUR (die-deutsche-wirtschaft.de, stima non ufficiale); FN 364952w. Socio/gerente storico Ing. Peter Hrachowina. Azienda familiare dal 1908</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Bert Ortner</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>office@hrachowina.at</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hrachowina.at</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Wien (Wien)</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/hrachowina-fenster-tueren-gmbh_Gzxo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>J.C. Bawart &amp; Söhne GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Volume ca. 200.000 m2 di parquet venduti/anno; fatturato e organico non pubblicati. FN 613429b, LG Feldkirch. Ultimo produttore di parquet del Vorarlberg</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Christoph Bawart</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>bawart@bawart.at</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>https://www.bawart.at</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Sulz (Vorarlberg)</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bawart.at/willkommen/firmenprofil/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Jannach Lärchenholz GmbH</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e piallatura larice</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>ca. 40 dipendenti (sito aziendale); fatturato non pubblicato. FN 220460g (Jannach Lärchenholz GmbH, piallatura) - collegata Jannach Ges.m.b.H. FN 80442y (segheria), stesso GF. E-mail non riportabile: nell'Impressum e offuscata anti-spam</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Mag. (FH) Helmut Jannach</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jannach.com</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Thalheim (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://jannach.com/kontakt/impressum.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Josef Speckner GmbH</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — imballaggi in legno/pallet</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>ca. 30 dipendenti; produzione ca. 1 mln di pallet + 10.000 imballaggi speciali/anno; fatturato non pubblicato, verosimilmente sotto i 10 Mio EUR (azienda di confine). Co-GF: Christoph Speckner. FN 114101x, LG Ried im Innkreis</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Josef Speckner</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>speckner@speckner.at</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>https://www.speckner.at</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Schwand im Innkreis (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.speckner.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Kager Fenster GmbH</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — finestre e porte in legno</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato; inserita al n. 1877 del ranking DDW delle maggiori imprese familiari austriache (fascia stimata sotto i 15 Mio EUR). FN 383552y. Azienda familiare dal 1933, finestre legno e legno-alluminio</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Ing. Helmut Kager</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>vorau@kager.at</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kager.at</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Vorau (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://die-deutsche-wirtschaft.de/famu_top/oesterreich-kager-fenster-gmbh-vorau-umsatz-mitarbeiterzahl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Karnische Massiv Möbel GmbH</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili e cucine massello</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>ca. 40 dipendenti (km-moebel.at / meinbezirk.at, 2024); fatturato non pubblicato. AZIENDA DI CONFINE: taglia probabilmente sotto i 10 M€. Produce cucine, mobili in massello, imbottiti e porte interne.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Werner Hohenwarter</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>info@km-moebel.at</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>https://km-moebel.at</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Kirchbach, Kärnten</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gewerbeverzeichnis-oesterreich.at/karnische_massiv_moebel_gmbh/2225.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Kienpointner GmbH</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi contract alberghieri</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>ca. 100 dipendenti (firmenabc.at / wlw.at, 2024); fatturato non pubblicato. Falegnameria industriale per arredi di hotel e ristorazione, 5a generazione familiare; opera anche come general contractor in AT/DE/IT/CH.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Gerhard Kienpointner</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>verkauf@kienpointner.com</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kienpointner.com</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Waidring, Tirol</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/kienpointner-gmbh_KKyx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>MAFI Naturholzboden GmbH</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 22,3 Mio EUR (2017, creditreform); ca. 100 dipendenti (2020). FN 116654a, BG Ried im Innkreis. Altri GF: Christiane Lindner, Heidrun Zerbs</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Florian Fillafer</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>office@mafi.com</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>https://mafi.com</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Schneegattern, Lengau (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/mafi-naturholzboden-gmbh_aTw</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Mayr - Schulmöbel Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi scolastici</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 39,0 M€ (stima Die Deutsche Wirtschaft, ranking imprese familiari austriache) e 150 dipendenti nella sede di Scharnstein (tips.at, 2024). AZIENDA DI CONFINE: vicino al limite superiore della fascia tollerata. Secondo Geschäftsführer: Ing. Florian Huemer. Leader di mercato austriaco negli arredi scolastici.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Franz Wiener</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/mayr-schulm%C3%B6bel</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>office@mayrschulmoebel.at</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mayrschulmoebel.at</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Scharnstein, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/mayr-schulmoebel-gesellschaft-m-b-h_cOe</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Meiberger Holzbau GmbH</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — costruzioni in legno/Holzbau</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Totale di bilancio 11,33 Mio EUR (bilancio al 31.01.2025, firmenabc.at); fatturato non pubblicato, PMI familiare stimabile nella fascia 10-15 Mio EUR</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Walter Meiberger</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/meiberger-holzbau</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>office@holzbau-meiberger.at</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.holzbau-meiberger.at</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Lofer (Salzburg)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/meiberger-holzbau-gmbh_cXK</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Meyer Parkett GmbH</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato stimato 6,2 Mio EUR e 31 dipendenti (die-deutsche-wirtschaft.de); sotto la fascia target (azienda di confine, &lt;10 Mio). FN 226133z</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Stefan Meyer</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>office@meyer.at</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.meyer.at</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Kalsdorf bei Graz (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>https://die-deutsche-wirtschaft.de/famu_top/oesterreich-meyer-parkett-gmbh-kalsdorf-bei-graz-umsatz-mitarbeiterzahl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Mühlbauer Holz GmbH</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 20,1 Mio EUR (2024) e 20,2 Mio EUR (2023) - firmenabc.at; ca. 42 dipendenti (Holzkurier 2018). Azienda familiare dal 1903</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>DI Joe Mühlbauer-Elbl</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>office@muehlbauerholz.com</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>https://www.muehlbauerholz.com</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Himberg (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/muehlbauer-holz-gmbh_NJFw</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Pußwald Holz GmbH</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e commercio all'ingrosso di legname</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e organico non pubblicati (dati riservati su firmenabc/northdata); PMI familiare, segheria + commercio all'ingrosso. FN 571568t</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Ing. Rainer Alexander Pußwald</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>office@pusswald-holz.at</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>https://pusswald-holz.at</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Sinabelkirchen (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>https://pusswald-holz.at/kontakt/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>RELAX Natürlich Wohnen GmbH</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — letti in massello</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Oltre 50 addetti impiegati nelle officine di premontaggio/assemblaggio (relax.eco, 2024); fatturato non pubblicato. Produce letti in legno massello, reti a doghe, materassi e prodotti in cirmolo. Seconda Geschäftsführerin: Adelheid Sigl. Possibile taglia sotto i 10 M€.</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Herbert Sigl</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>info@relax.eco</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>https://relax.eco</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Obertrum am See, Salzburg</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/relax-natuerlich-wohnen-gmbh_DcBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Rauchenzauner Möbel GmbH</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine e mobili bagno</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato stimato 18,8 M€ e 75 dipendenti (Die Deutsche Wirtschaft / firmenabc.at, 2024). Produzione industriale di cucine e mobili da bagno di fascia alta.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Gerhard Rauchenzauner</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>office@rauchenzauner.at</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rauchenzauner.at</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Frankenmarkt, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/rauchenzauner-moebel-gmbh_BBBnb</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SAMINA Produktions- und Handels GmbH</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — letti e sistemi letto</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>20-49 dipendenti (firmenabc.at, 2024); fatturato non pubblicato. AZIENDA DI CONFINE: taglia probabilmente sotto i 10 M€. Manifattura di sistemi letto con telai/doghe in legno massello non trattato, lattice naturale e lana; fondatore Günther W. Amann-Jennson.</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Philipp Amann</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>samina@samina.com</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>https://samina.com</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Frastanz, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/samina-produktions-und-handels-gmbh_iqg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>SCHAFFER SÄGEWERK-HOLZEXPORT GmbH</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria ed export legname</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>66 dipendenti in sede (80 worldwide) e taglio annuo ca. 115.000 fm (Industrielandkarte Steiermark); fatturato non pubblicato, fascia stimata 20-30 Mio EUR. FN 137937z. Azienda familiare guidata da Hans Schaffer</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Markus Johannes Schaffer</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>office@schafferholz.com</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.schafferholz.com</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Eppenstein, Weißkirchen in Steiermark (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>https://holzindustrie-steiermark.industrielandkarte.com/betriebe/schaffer-sagewerk-holzexport-gmbh</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Schösswender Möbel Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili e tavoli</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>ca. 180 dipendenti nello stabilimento mobili di Franking (schoesswender.at/schoesswender.com, 2024); gruppo Schösswender ca. 430 dipendenti e 28 M€ di fatturato di gruppo (2012, ultimo dato pubblico). Azienda mobili = societa piu grande del gruppo; fatturato singolo stimabile 15-25 M€ ma NON confermato. Legame di gruppo: Schösswender Holding (siti Franking, Litschau, Anras + produzione in Romania).</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Alfred Weiß</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/sch%C3%B6sswender-m%C3%B6bel</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>office@schoesswender.com</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>https://www.schoesswender.com</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Franking, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/schoesswender-moebel-gesellschaft-m-b-h_jQF</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Sohm HolzBautechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — costruzioni in legno/Holzbau</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>ca. 100 dipendenti (wirtschaftsforum.de); fatturato non pubblicato. Altri GF: Andreas Kempf, Christian Milz (Impressum). Azienda collegata: Sohm Objektbau GmbH</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Kilian Sohm</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/sohm-holzbautechnik</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>office@sohm-holzbau.at</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sohm-holzbau.at</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Alberschwende (Vorarlberg)</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sohm-holzbau.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Speedmaster GmbH</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — componenti per mobili</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato e dipendenti non pubblicati (firmenabc.at / WKO, 2024). Produttore industriale di parti e semilavorati per mobili (pannelli, frontali, corpi) che rifornisce oltre 8.700 falegnamerie in AT/DE/Alto Adige/CH. Forte consumo di pannelli a base legno -&gt; soggetto EUDR. Rilevata una divisione da Schweiger GmbH.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Hermann Huber</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>office@speedmaster.at</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>https://www.speedmaster.at</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Eberstalzell, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/speedmaster-gmbh_kRv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Storebest Ladeneinrichtungen GmbH</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — arredi negozi</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>50-60 dipendenti (firmenabc.at / herold.at, 2024); fatturato non pubblicato. Grande falegnameria industriale interna per arredi negozi e retail; fondata 1960.</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Gernot Karlsböck</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>office@storebest.at</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.storebest.at</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Aschach an der Steyr, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/storebest-ladeneinrichtungen-gesellschaft-m-b-h_um</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Troger-Holz Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria e pannelli per casseforme</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 24,0 Mio EUR (stima DDW); FN 54795g, BG Schwaz. Azienda familiare dal 1820, sedi Vomp e Stans</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Helmut Troger</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>office@trogerholz.at</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>https://www.trogerholz.at</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Vomp (Tirol)</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>https://die-deutsche-wirtschaft.de/famu_top/oesterreich-troger-holz-gmbh-vomp-umsatz-mitarbeiterzahl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Wallner Holzhandel GmbH</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>80 dipendenti (WKO/herold); fatturato non pubblicato, fascia stimata 20-30 Mio EUR. FN 267061m. Azienda familiare dal 1938, due sedi a St. Pölten e St. Pölten-Harland</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Gerhard Wallner</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>office@holz-wallner.at</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.holz-wallner.at</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Sankt Pölten (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.herold.at/gelbe-seiten/st-p%C3%B6lten/MDPKZ/wallner-holzhandel-gmbh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Weissengruber Möbelmanufaktur GmbH</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili e arredi hotel</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>ca. 60 dipendenti (weissengruber.at, 2024); fatturato non pubblicato. Produzione di mobili di alta gamma per rivenditori specializzati e per l'ospitalità. Possibile taglia sotto i 10 M€.</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Klaus Weissengruber</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>office@weissengruber.at</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>https://www.weissengruber.at</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Ried in der Riedmark, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/weissengruber-moebelmanufaktur-gmbh_BBdYe</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Wittmann Möbelwerkstätten GmbH</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — mobili imbottiti</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>120 dipendenti (firmenabc.at, 2024); totale attivo di bilancio 9,6 M€ al 31.12.2024. Fatturato non pubblicato: 23,5 M€ nel 2005 (MÖBELMARKT); una stima Die Deutsche Wirtschaft indica 45 M€ ma appare incoerente con il bilancio. AZIENDA DI CONFINE sul lato alto. Imbottiti di alta gamma in legno + pelle (doppia rilevanza EUDR), export ca. 70%.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Heinz Hofer-Wittmann</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/wittmann-moebelwerkstaetten-gmbh</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>info@wittmann.at</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wittmann.at</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Etsdorf am Kamp, Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/wittmann-moebelwerkstaetten-gmbh_NVdS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Zöchling-Holz GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — commercio legname</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato e organico non pubblicati; superficie operativa ca. 8.500 m2 con showroom 3.000-3.500 m2. FN 392997m. Azienda familiare dal 1904 (origine segheria), oggi commercio legname/parquet/porte</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Ing. Stefan Zöchling</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>mail@zoechling-holz.at</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>https://www.zoechling-holz.at</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Gerasdorf bei Wien (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>https://firmen.wko.at/z%C3%B6chling-holz-gmbh---co-kg-der-holzfachmarkt/nieder%C3%B6sterreich/?firmaid=6dae60ea-74f3-4abe-b47c-6d66fe0f4ef6</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>steininger.designers gmbh</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Legno/Arredo — cucine</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>ca. 44 dipendenti (firmenabc.at, 2025); totale attivo di bilancio 4,0 M€ (es. 2025). AZIENDA DI CONFINE: fatturato probabilmente sotto i 10 M€, non pubblicato.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Martin Steininger</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/steininger-designers</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>office@steiningerdesigners.com</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.steiningerdesigners.com</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>St. Martin im Mühlkreis, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/steininger-designers-gmbh_Eqjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>weinberger-holz gmbh</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Legno/Segheria — segheria, legname da costruzione e profilati</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Totale di bilancio 16,77 Mio EUR (bilancio al 31.12.2024, firmenabc.at); FN 119447h, LG Wolfsberg. Gruppo: collegata weinberger-trading gmbh</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Johann Alfred Weinberger</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>info@weinberger-holz.at</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>https://www.weinberger-holz.at</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Reichenfels (Kärnten)</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/weinberger-holz-gmbh_IPdi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Alvorada Kaffeerösterei GmbH</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione e distribuzione</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e dipendenti non pubblicati (Jahresabschluss non accessibile su firmenabc.at/wirtschaft.at) - VERIFICARE; probabile fascia medio-piccola. Firmenbuch FN 507244y, HG Wien; capitale 35.000 €; società iscritta il 02.03.2019 e attualmente ATTIVA. ATTENZIONE: il precedente gruppo Alvorada (marchio di caffè per la gastronomia viennese dal 1957) è finito in insolvenza nel 2018; l'attuale GmbH è la società subentrata, controllata al 100% da Minges Kaffeerösterei GmbH, con GF Ulli Minges. Oggetto sociale: commercio e distribuzione di caffè tostato, prodotti solubili e tè, esercizio di torrefazione e produzione.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Ulli Minges</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>sales@alvorada.com</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>http://alvorada.wien</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Vienna (Wien), Leopoldstadt</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/alvorada-kaffeeroesterei-gmbh_OibN</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>BAG Ölmühle BetriebsgmbH</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — olio di soia e farina di estrazione</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 33-35 Mio. € - ca. 22-25 dipendenti (fonte firmenabc.at / Creditreform e meinbezirk.at, dati 2019-2024). Firmenbuch FN 276013b, LG Eisenstadt, UID ATU62383316. È il PIÙ GRANDE oleificio di soia dell'Austria: dal 2011 lavora esclusivamente soia non-OGM di origine europea producendo Sojaöl e Sojaextraktionsschrot per l'industria mangimistica. CASO TIPICO di PMI con fatturato gonfiato dal costo materia prima (35 M€ con soli ~25 addetti): resta nella forbice tollerata 5-40 M€. Lead EUDR primario (soia = Allegato I, obbligo DDS come operatore).</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Josef Willim</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>bagoffice@bagoil.at</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>https://www.bagoil.at</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Güssing, Burgenland</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bagoil.at/en/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Franz Hauswirth Ges.m.b.H.</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — cioccolateria industriale</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 14,6 Mio. € nell'esercizio 2022/23 - ca. 70 dipendenti oggi (in precedenza 120) (fonte burgenland.ORF.at / falstaff.com / t-online.de, 2024-2025). Firmenbuch FN 122377t, LG Eisenstadt. ATTENZIONE: insolvenza a fine 2024 (prezzi cacao ed energia); procedura chiusa e AZIENDA RISANATA E ATTIVA - nel marzo 2025 il 100% delle quote è stato rilevato da Landgarten (Bruck an der Leitha), i vecchi GF Peter e Roman Hauswirth sono usciti e i nuovi GF sono Florian Kühbacher e Herbert Stava; i ca. 70 posti a Kittsee sono stati mantenuti. Produce figure di cioccolato, praline, banane al cioccolato: forte consumo di cacao = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Florian Kühbacher</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (con Herbert Stava)</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/hauswirth-schokobananen</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>office@chocolate-austria.com</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.chocolate-austria.com</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Kittsee, Burgenland</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/franz-hauswirth-ges-m-b-h_EukA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>KUK-Austria GmbH</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — distribuzione materie prime food/pharma</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>PMI di distribuzione (Großhandel materie prime alimentari e farmaceutiche) attiva dal 1945, con ca. 30-40 rappresentanze/agenzie generali e rete in Europa centro-orientale; fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at, WKO Firmen A-Z, northdata.com, 2024-2025). Firmenbuch FN 278142h, LG Ried im Innkreis. MEMBRO RSPO dall'11.09.2014 come Supply Chain Associate: prova documentale che tratta olio di palma / derivati del palma nel proprio portafoglio (oltre a pectine, gelatine, addensanti, cacao in polvere).</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Mag. Claudia Luzia Neuhold</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Gewerberechtliche Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>office@kuk.com</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>https://www.kuk.com</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Ried im Innkreis (Auleiten 4), Alta Austria (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.rspo.org/members/3170/kuk-austria-gmbh</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Soy Austria Produktions GmbH</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — trasformazione soia (farine, texturati)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e organico non pubblicati nelle fonti aperte (fonti herold.at, WKO Firmen A-Z, northdata.com, 2024-2025). Firmenbuch FN 99559k, LG St. Pölten (iscritta dal 1994). Impianto per prodotti di soia full-fat dal 1989 e secondo stabilimento dal 2017 per farine di soia sgrassate e texturati di soia; materia prima = soia austriaca e UE non-OGM, vendita all'industria alimentare mondiale. Dal 01.10.2025 assorbe l'operativo di J. u. H. Bamberger GmbH. Distribuzione tramite la consociata SOJA AUSTRIA Vertriebs GmbH (sede commerciale: Ares Tower, Donau-City-Straße 11, 1220 Wien). Secondo Geschäftsführer: Ing. Josef Bamberger.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Georg Bamberger</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/soy-austria-gmbh</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>produktion@soyaustria.com</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>https://soyaustria.com</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Uttendorf / Prinzersdorf (Bezirk St. Pölten-Land), Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>https://soyaustria.com/de/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>TEGUM Technische Gummiwaren Gesellschaft m.b.H. &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — nastri trasportatori e rivestimenti</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>fatturato e organico non pubblicati (firmenabc.at, 2025); produzione e commercio all'ingrosso di articoli tecnici in gomma, nastri trasportatori e gomma antiusura. Firmenbuch FN 27638w</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Ing. Walter Antosch</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>office@tegum.at</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>https://tegum.at/</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Hallein, Salzburg</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/tegum-technische-gummiwaren-gesellschaft-m-b-h-co_lgH</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Bayer Kartonagen GmbH</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartotecnica</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 12 Mio. € con 80 dipendenti (fonte Vorarlberger Nachrichten VN.at, intervista 08.11.2019); stima successiva 27,3 Mio. € (die-deutsche-wirtschaft.de ranking, dato stimato). Firmenbuch FN 388412w. Impresa familiare di 3a generazione, Schillerstraße 16. IN TARGET 10-20 M€ secondo il dato pubblicato. ATTENZIONE LEGAME DI GRUPPO: la produzione è stata rilevata da Schwarzach Packaging (Schwarzach, Vorarlberg) con effetto retroattivo dal 1° gennaio - verificare l'assetto attuale prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Josef Andreas Bayer</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/bayer-kartonagen-gmbh</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>office@bayer-kartonagen.com</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bayer-kartonagen.com</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Lustenau, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/bayer-kartonagen-gmbh_IPzn</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Bösmüller Print Management GesmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa e imballaggi</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Ca. 65 dipendenti su 3 sedi (Wien, Stockerau, Krems), di cui ca. 50 nello stabilimento di Stockerau (fonte sito aziendale/lehrlingsportal.at, dato 2023-2024). Fatturato non pubblicato: n.d. Firmenbuch FN 276051h, HG Wien. Sede legale Obere Augartenstraße 32, 1020 Wien; stabilimento Josef-Sandhofer-Straße 3, 2000 Stockerau. STIMA SOTTO LA FASCIA IDEALE: con ~65 addetti il fatturato è verosimilmente vicino o inferiore alla soglia dei 10 M€ - da verificare. Impresa familiare (2a generazione); secondo Geschäftsführer: Markus Purker. Attiva anche nel Verpackungsdruck (astucci e packaging in cartoncino).</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Ing. Doris Wallner-Bösmüller</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>office@boesmueller.at</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>https://boesmueller.at</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Stockerau, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>https://boesmueller.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>CARINI GmbH</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 5,2 Mio. USD (~4,8 Mio. €) - 33 dipendenti (fonte profilo RocketReach, dato stimato). Firmenbuch FN 205435k. Sede Industrie Nord, Bildgasse 42, 6890 Lustenau. AZIENDA SOTTO LA SOGLIA MINIMA 5 M€ secondo la stima disponibile: dimensione DA VERIFICARE prima del contatto (l'azienda si presenta come una delle principali etichettifici dell'area di lingua tedesca, quindi il dato stimato potrebbe essere sottostimato). Impresa familiare fondata nel 1939, 4a generazione (Simon Sohm in direzione, tecnica applicativa e vendite).</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Edgar Sohm</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/carini-gmbh</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>welcome@carini.at</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.carini.at</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Lustenau, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.carini.at/unternehmen-karriere/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Flatz GmbH</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato stimato ca. 18,4 Mio. USD (~17 Mio. €) - 96 dipendenti (fonte profilo RocketReach, dato stimato); azienda attiva dal 1935, uno dei principali produttori austriaci di imballaggi in cartone ondulato. Firmenbuch FN 136639s, LG Feldkirch. IN TARGET 10-20 M€. 4 stabilimenti a Lauterach (Funkenstraße 6/11, Scheibenstraße 20). Impresa familiare indipendente; Hans-Peter Flatz indicato come co-Geschäftsführer in fonti di stampa.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Mag. Stefan Flatz</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/flatz-gmbh</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>office@flatz.com</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.flatz.com</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Lauterach, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.flatz.com/de/karriere/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Gruber Karton Kreativ GmbH</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartotecnica e imballaggi</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e numero di dipendenti non pubblicati nelle fonti consultate: n.d. (fonte WKO Firmen A-Z / firmennetzwerk.at, 2025). Firmenbuch FN 643739a, Ried im Innkreis. Sede Frankenburger Straße 17, 4910 Ried im Innkreis. Impresa familiare con oltre 120 anni di attività, produce cartonaggi, imballaggi in cartone teso e ondulato, scatole per spedizione. DIMENSIONE DA VERIFICARE: probabilmente sotto la fascia ideale 10-20 M€. Gewerberechtlicher Geschäftsführer: Christian Magoč. Società collegata: Gruber Immo GmbH.</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Janin Simader, BSc</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>office@gruber-karton-kreativ.at</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>https://gruber-kartonagen.at</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Ried im Innkreis, Alta Austria (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>https://firmen.wko.at/gruber-karton-kreativ-gmbh-hersteller-von-kartonagen-karton-und-wellpappverpackungen/ober%C3%B6sterreich/?firmaid=d38297c8-65cd-4957-b852-3e53194f9fbd</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Kliemstein Papierverarbeitungs GmbH</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — lavorazione carta</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 7 Mio. USD (~6,5 Mio. €) - 24 dipendenti nella sede (fonte Dun &amp; Bradstreet business directory, dato stimato). Firmenbuch FN 229062g. Sede Bahnhofstraße 6, 8330 Feldbach. AZIENDA SOTTO LA FASCIA IDEALE 10-20 M€: rientra solo nel margine basso del range tollerabile 5-40 M€. Impresa familiare che lavora industrialmente carta e cartone (quaderni, blocchi, rilegature, cartelline, blocchi flipchart). Membro del Fachverband PROPAK.</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Mag. Thomas Kliemstein</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>office@kliemstein.co.at</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>https://www.kliemstein.co.at</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Feldbach, Stiria (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.kliemstein.co.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Margarethner Verpackungsgesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato e display</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Oltre 30 dipendenti (fonte WKO Firmen A-Z / karriere.at, dato 2024-2025). Fatturato non pubblicato: n.d.; con ~30 addetti la stima è verosimilmente sotto i 10 M€ - DA VERIFICARE. Firmenbuch FN 39371z, BG Korneuburg. Sede Heidestraße 17, 2433 Margarethen am Moos. Produce imballaggi speciali e display in cartone ondulato e teso (POS). Membro del Forum Wellpappe Austria. ATTENZIONE LEGAME DI GRUPPO: 100% Inter Carton Gesellschaft m.b.H. (Wien), che detiene anche il 34% di DONAUWELL Wellpappe.</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>DI Richard Höfer</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>office@mvg.co.at</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>https://mvg.co.at</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Margarethen am Moos, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>https://mvg.co.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>MÜROLL GmbH</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — rotoli carta ed etichette</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Ca. 140 dipendenti (fonte sito aziendale / WKO Firmen A-Z, dato 2024). Fatturato non pubblicato: n.d.; con 140 addetti la fascia stimata è ~25-40 M€, quindi al limite superiore del range tollerabile - DA VERIFICARE. Firmenbuch FN 68918a, LG Feldkirch. Sede Satteinser Straße 12, 6820 Frastanz. Produce rotoli di carta, banderole, etichette stampate e nastri adesivi (unico produttore austriaco di nastri adesivi): quota rilevante ma non esclusiva di prodotti a base carta. ASSETTO: 99,5% Johann und Oswald Müller Privatstiftung. Altri Geschäftsführer: Uwe Müller, Kurt Pichler.</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Michael Müller</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>office@mueroll.com</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mueroll.com</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Frastanz, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>https://www.mueroll.com/en/imprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Print Alliance HAV Produktions GmbH</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa offset</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Oltre 180 dipendenti (fonte sito aziendale / leitbetriebe.at, dato 2024). Fatturato non pubblicato: n.d.; con oltre 180 addetti la stima si colloca nella fascia alta del range tollerabile (~30-40 M€) - DA VERIFICARE prima del contatto. Firmenbuch FN 426711t, LG Wiener Neustadt. Sede Druckhausstraße 1, 2540 Bad Vöslau. Definita la più grande tipografia offset a foglio dell'Austria, attiva 24h; forte consumo di carta e cartoncino (rilevanza EUDR Allegato I). Membro Leitbetriebe Austria.</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Christoph Preitler</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>office@printalliance.at</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>https://printalliance.at</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Bad Vöslau, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>https://printalliance.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Salzer Papier GmbH</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartiera</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato stimato ca. 42 Mio. € (fonte die-deutsche-wirtschaft.de, stima su dati 2023) - 51-200 dipendenti (fonte LinkedIn/firmenabc); nel 2007 24,5 Mio. € con 95 dipendenti (noe.ORF.at). Produzione ca. 30.000 t di carta/anno. Firmenbuch FN 312367p, LG St. Pölten. AZIENDA DI CONFINE: la stima 42 Mio. € supera di poco la fascia tollerabile 5-40 M€ ma resta ben sotto la soglia di esclusione ~50 M€. Impresa familiare all'8a generazione, parte della Salzer Gruppe (Papier, Industrie-Service, Holz). Co-Geschäftsführer citato in stampa: Dr. Harald Egger. Membro Austropapier.</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Salzer</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/salzer-papier-gmbh</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>office@salzer.at</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>https://www.salzer.at</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>St. Pölten (Stattersdorf), Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>https://www.salzer.at/en/gruppe/kontakt/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Samson-Druck Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato oltre 18 Mio. € - ca. 120 dipendenti (fonte salzburg.wirtschaftszeit.at / die-salzburger-industrie.at, dato pubblicato 2023-2024). Firmenbuch FN 66316z, LG Salzburg. Azienda familiare di 3a generazione (Ramsbacher/Valentin/Frost), una delle maggiori tipografie offset austriache. PERFETTAMENTE IN TARGET 10-20 M€. Secondo Geschäftsführer: Tibor Valentin. Nota: 100% detenuta da Aichhorn Beteiligungs GmbH (holding familiare, non gruppo multinazionale).</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Markus Ramsbacher</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/samson-druck</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>office@samsondruck.at</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.samsondruck.at</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>St. Margarethen im Lungau, Salisburgo (Salzburg)</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.samsondruck.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Steirerpack GmbH</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato: n.d. Dipendenti non pubblicati nelle fonti consultate (fonte firmenabc.at / WKO Firmen A-Z / propak.at). Firmenbuch FN 79280p, LG Leoben (Handelsgericht). Sede Hauptstraße 21, 8763 Pölstal. Azienda fondata nel 1902, produce cartone ondulato, astucci, imballaggi fustellati, display e cartoni per vino. Membro del Forum Wellpappe Austria: i 7 produttori del forum occupano complessivamente ca. 1.600 addetti, il che colloca Steirerpack tra le realtà medie del settore. DIMENSIONE DA VERIFICARE. Co-Geschäftsführer: Franz Grafendorfer.</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Mag. Wolfgang Habenberger</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/steirerpack</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>office@steirerpack.at</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>https://steirerpack.at</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Pölstal (Möderbrugg), Stiria (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>https://steirerpack.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Ulrich Etiketten Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — etichette</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 33 Mio. € (+4% sull'anno precedente) - ca. 200 dipendenti (fonte labelpack.de / profili aziendali, 2023). Firmenbuch FN 89306h, BG Korneuburg. Sede produttiva Betriebsstraße 3, 2011 Höbersdorf; 3 uffici vendita in Germania. Azienda familiare indipendente. SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€. Co-Geschäftsführer: Florian Ulrich.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Rainer Ulrich</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>ulrich@ulrich.at</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>https://ulrich.at</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Höbersdorf (Sierndorf), Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>https://ulrich.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Wellpappenfabrik TEWA Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 12,5 Mio. € - ca. 50 dipendenti (fonte meinbezirk.at, articolo sulla successione familiare; fatturato riferito al 2012, organico aggiornato). IN TARGET 10-20 M€ secondo il dato pubblicato, ma il fatturato è un dato datato - DA VERIFICARE. Sede Buscheiden 9, 9560 Feldkirchen. Sito produttivo attivo dal 1846, impresa familiare. Membro del Forum Wellpappe Austria (7 produttori austriaci di cartone ondulato). Geschäftsführender Gesellschafter: KommR Franz Ronge.</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Felix Ronge</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>wirmachendas@tewa.com</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>https://www.tewa.com</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Feldkirchen in Kärnten, Carinzia (Kärnten)</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.tewa.com/team-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Wograndl Druck GmbH</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — stampa</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Ca. 48 dipendenti (fonte meinbezirk.at, articolo 2020-2021); descritta come la maggiore tipografia del Burgenland e tra le prime dieci in Austria; 26 gruppi stampa/verniciatura su tre turni. Fatturato non pubblicato: n.d. Firmenbuch FN 272989f, LG Eisenstadt. Sede Druckweg 1, 7210 Walbersdorf/Mattersburg. STIMA SOTTO LA FASCIA IDEALE: con ~48 addetti il fatturato è verosimilmente sotto i 10 M€ - da verificare. Impresa familiare fondata nel 1956 da Josef Wograndl.</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Jochen Wograndl</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/wograndl-druck-gmbh</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>print@wograndl.com</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wograndl.com</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Mattersburg (Walbersdorf), Burgenland</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wograndl.com/kontakt</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>pack it! Verpackungen GmbH</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato offset</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato 25,5 Mio. € (+15% sui ca. 23 Mio. € dell'anno precedente) - 63 dipendenti su produzione a quattro turni (fonte meinbezirk.at / packreport.de, dato riferito al bilancio successivo al 2011; investimento di 15 Mio. € nel nuovo impianto di cartone ondulato). SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€; dato non recente, DA VERIFICARE. Firmenbuch FN 196751s, LG Steyr. Sede Hermesstraße 7, 4595 Waldneukirchen. Specializzata in imballaggi in cartone ondulato cachierato offset. NOTA ASSETTO: fondata nel 2000 anche con la partecipazione di Dinkhauser Verpackungen (Tirolo). Prokuristen: Karl Ömmer. Membro Fachverband PROPAK.</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Walter Michael Freimüller</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/packit-verpackungen-gmbh</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>office@packit.at</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>https://www.packit.at</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Waldneukirchen, Alta Austria (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.propak.at/mitglieder/item/pack-it-verpackungen-gmbh</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>pratopac GmbH</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Carta/Packaging — cartone ondulato</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 18 Mio. € - ca. 70-75 dipendenti (fonte Wirtschaftszeit.at / VN.at, dato 2020-2021; 15 Mio. € nel 2018). Firmenbuch FN 217837w, LG Feldkirch. Sede Riedstraße 1-5, 6833 Klaus. PERFETTAMENTE IN TARGET 10-20 M€. Produce cartone ondulato, cartonaggi, tubi e barattoli in cartone spiralato. NOTA ASSETTO: socio unico WA Holding GmbH (holding familiare Vorarlberg); esiste inoltre la joint venture pratopac Gmeiner GmbH con Gmeiner nel settore anime/tubi.</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Alexander Abbrederis</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>info@pratopac.at</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pratopac.at</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Klaus, Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pratopac.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Amann Kaffee GmbH</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione e import caffè verde</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Bilancio: totale attivo 10,6 Mio. €, patrimonio netto 6,8 Mio. €, equity ratio 64,1% (esercizio 2025, fonte firmenabc.at/firmenatlas.com). Dipendenti 31-50 (fonte karriere.at). Fatturato puntuale non pubblicato. Firmenbuch FN 185621y, LG Feldkirch; UID ATU47491904. Fondata nel 1993 da Peter e Rupert Amann, oggi guidata da Peter Amann con i figli Johanna e Florian; torrefazione propria nel Bregenzerwald e nuova sede/centro logistico nel Millennium Park di Lustenau. Acquista caffè verde all'origine per la propria tostatura = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Peter Amann</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/amann-kaffee-gmbh</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>info@amann-kaffee.at</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amann-kaffee.at</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Lustenau (torrefazione a Schwarzenberg), Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amann-kaffee.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>EZA Fairer Handel GmbH</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — import caffè verde e cacao</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 16 Mio. € - 51-200 dipendenti (fonte eza.cc Geschäftsbericht / wlw.at, dati 2022-2024). Firmenbuch FN 69275a, LG Salzburg. Pioniere del commercio equo in Austria (dal 1975): importa direttamente caffè verde (44% del fatturato) e cacao/cioccolato dai Paesi produttori, senza intermediari - quindi IMPORTATORE DIRETTO di due commodity Allegato I EUDR. IN TARGET 10-20 M€. Doppia filiera caffè + cacao.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Michael Scherndl</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/eza-fairer-handel</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>office@eza.at</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eza.cc</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Köstendorf bei Salzburg, Salisburgo (Salzburg)</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.eza.cc/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Helmut Sachers Kaffee GmbH</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import/export</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 5,2 Mio. € - ca. 26 dipendenti (ultimo dato pubblico 2016/2017, fonte faq-genuss.com / firmenabc.at). Firmenbuch FN 105466y, HG Wien. AZIENDA DI CONFINE (limite inferiore ~5 M€ della forbice tollerabile). Fondata nel 1929 a Vienna; ha attraversato un Sanierungsverfahren (2017) ed è oggi risanata e ATTIVA sotto nuova proprietà: SAWE Holding GmbH 80% + COFFEETREE S.r.l. 20%, GF dal 14.07.2020. Circa 450 t di caffè lavorate/anno, quota export ~20%; oggetto sociale include esplicitamente import/export di prodotti alimentari. Considerata la maggiore torrefazione bio dell'Austria.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Hannes Schlögl</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>office@helmutsachers.at</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>https://www.helmutsachers.at</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Oeynhausen, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.helmutsachers.at/en/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>J. Hornig GmbH</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione + import caffè verde</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato 18,2 Mio. € - ca. 51 dipendenti (fonte wirtschaftszeit.at / austria-forum.org, dato 2022-2023). Firmenbuch FN 91930p, LG für ZRS Graz. Torrefazione familiare fondata nel 1912, 4a generazione (Johannes Hornig, titolare/CEO di famiglia); importa caffè verde direttamente dai Paesi d'origine e rifornisce oltre 5.000 clienti out-of-home. PERFETTAMENTE IN TARGET 10-20 M€. Importatore di Rohkaffee = operatore EUDR in senso stretto.</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Thomas Schusteritsch</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/j-hornig</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>online@jhornig.at</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jhornig.com</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Kalsdorf bei Graz, Stiria (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jhornig.com/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Naber Kaffee Manufaktur GmbH</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione e commercio caffè verde</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 3,5 Mio. € - ca. 15 dipendenti (fonte cash.at / cafeplusco.com, 2023-2024): AZIENDA SOTTO IL TARGET, segnalata come tale ma inserita perché commercia esplicitamente CAFFÈ VERDE (Rohkaffee). Firmenbuch FN 441118d, HG Wien; UID ATU69904712. Torrefazione viennese storica fondata nel 1908 da Georg Naber, dal 2015 controllata al 95% da café+co International Holding GmbH; tosta fino a 2 t di caffè al giorno, forte quota di private label; nel 2024-2025 ha rilevato una torrefazione tradizionale carinziana e aperto la sede di Klagenfurt. Oggetto sociale: produzione, tostatura e confezionamento di caffè in grani e commercio di caffè tostato E CRUDO.</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Marco Salvatori</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (con Bernd Nitschmann)</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>office@naberkaffee.com</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>https://naberkaffee.com</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Vienna (Wien), Strebersdorf; seconda sede Klagenfurt</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>https://naberkaffee.com/en/legal/imprint/</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Testa Rossa Caffe GmbH</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Caffè — torrefazione propria e franchising</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato e dipendenti non pubblicati sui portali gratuiti (firmenabc.at/KSV1870 espongono solo i dati anagrafici) - VERIFICARE. Firmenbuch FN 100910y, LG Innsbruck; UID ATU24581405; costituita il 04.02.1993; socio unico Leopold Wedl (100%), gruppo Wedl (Handelshaus Wedl, Mils). Gestisce il sistema di franchising internazionale TESTA ROSSA caffèbar (dal 1999, oltre 100 locali in Europa e Medio Oriente) e la torrefazione interna: la miscela di caffè verde viene tostata in proprio = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>KR Leopold Wedl</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>franchise@testarossacaffe.com</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.testarossacaffe.com</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Mils bei Hall in Tirol, Tirolo (Tirol)</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.testarossacaffe.com/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Berger Feinste Confiserie GmbH</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — confiserie e praline</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Ca. 100 dipendenti, 8 punti vendita propri in Salisburghese, Tirolo e Stiria, export mondiale (fonte confiserie-berger.at / chocolats-de-luxe.de, dati 2023-2025). Fatturato non pubblicato: firmenabc.at non espone il dato (Jahresabschluss non integralmente accessibile) - VERIFICARE. Firmenbuch FN 254861x, capitale 35.000 €, soci Hubert Berger 50% e Christine Berger 50%. Fondata nel 1994 a Lofer. Lavora couverture/cacao certificato Fairtrade (partner Fairtrade Austria): trasformatore di cacao = operatore/commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Hubert Berger</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (con Christine Berger)</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>schokolade@confiserie-berger.at</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>https://www.confiserie-berger.at</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Lofer, Salisburgo (Salzburg)</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.confiserie-berger.at/en/imprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Confiserie Wenschitz GmbH</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Ca. 30 dipendenti; totale attivo di bilancio 4,4 Mio. €, patrimonio netto 2,0 Mio. € (esercizio 2025, fonte firmenabc.at / firmenatlas.com). Fatturato non pubblicato: stimabile SOTTO la forbice target (probabile 5-8 Mio. €) - AZIENDA PICCOLA, segnalata come tale. Firmenbuch FN 273013s, LG Linz; UID ATU62268101. Maître Chocolatier con 'Pralinenwelt' ad Allhaming; produce praline, figure di cioccolato e marzapane in lavorazione artigianale assistita. Trasformatore di cacao/couverture = operatore o commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Helmut Wenschitz</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführender Gesellschafter</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>office@wenschitz.at</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wenschitz.at</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Allhaming, Alta Austria (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wenschitz.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Fürst GmbH</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — praline e Mozartkugeln</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Ca. 65-70 dipendenti, di cui 35 nella nuova manifattura di Elsbethen; produzione ca. 3,7 milioni di Original Salzburger Mozartkugel all'anno; investimento di 'diversi milioni di euro' nel nuovo stabilimento aperto a febbraio 2024 (fonte SN.at / wko.at / salzburgwiki, 2024-2026). Fatturato non pubblicato - VERIFICARE. Firmenbuch FN 257955x, LG Salzburg; UID ATU61451413. Café-Konditorei fondata nel 1884, 5a generazione (Martin Fürst dal 2015), inventrice della Mozartkugel (1890); 4 punti vendita a Salisburgo. Grande utilizzatore di cioccolato/cacao = operatore o commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Martin Fürst</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>versand@fuerst.cc</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>https://www.original-mozartkugel.com</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Salisburgo (Salzburg), produzione a Elsbethen</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.original-mozartkugel.com/en/imprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Heidi Chocolat AG</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — dolciumi al cioccolato</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 18 Mio. € - ca. 180 dipendenti (fonte Wikipedia/dati aziendali, ultimo dato pubblico 2018; ordine di grandezza confermato da cash.at). Firmenbuch FN 397683d, LG Wiener Neustadt; UID ATU67943648. Titolare del marchio storico viennese Niemetz Schwedenbomben (dal 1926) rilevato nel 2013; produzione trasferita a Wiener Neudorf. IN TARGET 10-20 M€. Grande utilizzatore di cioccolato/cacao per il rivestimento dei prodotti = operatore/commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Alexander Grund</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/heidi-chocolat-ag-niemetz-schwedenbomben%C2%AE</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>office@schwedenbomben.at</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>https://niemetz.at</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Wiener Neudorf, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>https://niemetz.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Landgarten GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Cacao/Cioccolato — snack bio ricoperti + cioccolato</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato non pubblicato (Jahresabschluss non integralmente accessibile su firmenabc.at) - VERIFICARE. Ordine di grandezza del gruppo stimabile in fascia 20-35 Mio. € dopo l'acquisizione: nel marzo 2025 Landgarten ha rilevato il 100% della cioccolateria Franz Hauswirth Ges.m.b.H. di Kittsee (14,6 Mio. € di fatturato 2022/23, ca. 70 dipendenti mantenuti), uscita dall'insolvenza di fine 2024. Firmenbuch FN 128998d, LG Korneuburg; 3 soci (2 accomandanti + 1 accomandatario Landgarten GmbH). Produttore di snack bio dal 1989, ricoperti di cioccolato Fairtrade: acquirente diretto di cacao/cioccolato = operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Herbert Stava</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>office@landgarten.at</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://landgarten.at</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Bruck an der Leitha, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>https://landgarten.at/en/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Deisenhammer Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — articoli tecnici in elastomero</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>100-199 dipendenti (firmenabc.at, 2025); fatturato non pubblicato. Fondata 1989, sedi Gunskirchen e Linz. Firmenbuch FN 100139p</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Hartmut Hermann Lauer</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>anfrage@deisenhammer.at</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.deisenhammer.at/</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Gunskirchen, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/deisenhammer-gesellschaft-m-b-h_How</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Gummiwerk Czermak &amp; Feger, Gesellschaft m.b.H. &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — lattice di caucciù naturale</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>21-50 dipendenti (herold.at/firmenabc.at, 2025); fatturato non pubblicato — PMI sotto la soglia target. Fondata 1949; palloni e articoli senza saldature in lattice di gomma naturale, mescole di gomma. Firmenbuch FN 18060i (KG) / FN 45245m (GmbH)</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Ing. Dominik Czermak</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>office@gummiwerk.at</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gummiwerk.at/</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Imst (Brennbichl), Tirol</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/gummiwerk-czermak-feger-gesellschaft-m-b-h-co-kg_Pho</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Persicaner &amp; Co. Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Gomma — commercio articoli tecnici in gomma</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>2 Geschäftsführer e 2 soci (firmenabc.at, 2025); fatturato e organico non pubblicati — grossista di O-ring, lastre di gomma, cinghie, tubi. Fondata 1875, familiare dal 1960. Firmenbuch FN 129338d</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Martin Winkelhöfer</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>office@persicaner.at</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.persicaner.at/</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Wien (Favoriten, 10. Bezirk), Wien</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/persicaner-co-gesellschaft-m-b-h_fFv</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Zrunek Gummiwaren Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Gomma — articoli tecnici in gomma ed elastomeri</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>10-19 dipendenti, classe di fatturato 0-10 Mio. €, Bilanzsumme 1,74 Mio. € al 31.12.2024 (firmenabc.at / northdata). NOTA: sotto la soglia target — produttore austriaco di articoli in gomma dal 1947. Altri GF: Mag. Dr. Ulrich Zrunek, Dipl.-Ing. Helena Zrunek Marja</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Max Zrunek</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Gewerberechtlicher Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>office@zrunek.at</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>https://www.zrunek.at/</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Wien (Döbling, 19. Bezirk), Wien</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/zrunek-gummiwaren-gesellschaft-m-b-h_plo</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>"Sojarei" Vollwertkost-Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — lavorazione soia bio (tofu)</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Ca. 50 dipendenti (fonte advantageaustria.org / sito aziendale, dato 2023-2024); fatturato non pubblicato. Firmenbuch FN 118580h. Fondata nel 1984, è il più grande e antico produttore di tofu dell'Austria e leader nazionale nei prodotti biologici a base di soia; fornisce tutte le principali catene retail austriache, il canale Reformhaus/bio e la ristorazione. Co-Geschäftsführung/tecnica: Andreas Eschner e Ing. Gerhard Eschner. Operatore EUDR sulla soia (Allegato I) anche se acquistata in UE.</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Ernst Ternon</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/sojarei-vollwertkost-gmbh</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>info@sojarei.at</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sojarei.at</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Traiskirchen, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.northdata.com/Sojarei%20Vollwertkost-GmbH,%20Traiskirchen/118580h</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Gsellmann Mischfuttererzeugung GmbH</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi composti e materie prime</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Bilancio: totale attivo 28,5 Mio. € e patrimonio netto 8,9 Mio. € (esercizio 2025, fonte firmeninfo.at / firmenatlas.com); ca. 60 dipendenti (fonte firmenabc.at). Firmenbuch FN 317883a. ATTENZIONE TAGLIA: il fatturato non è pubblicato e con capacità fino a 600 t/giorno potrebbe superare i 40 M€ per effetto del costo materia prima; resta però PMI familiare indipendente (3ª/4ª generazione, mulino dal 1890, ca. 3.000 clienti abituali). Altri Geschäftsführer: Josef Gsellmann, Maria Gsellmann.</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Andreas Gsellmann</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>office@gsellmann.com</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.gsellmann.com</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Kohlberg / Gnas, Stiria (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gsellmann.com/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Ignaz Göweil GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimi biologici, soia bio</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>22 dipendenti (fonte OÖ Nachrichten / nachrichten.at, articolo 2023); fatturato non divulgato dall'azienda (l'articolo precisa che Göweil non comunica il fatturato; quota di capitale proprio 15% da Firmenbuch). Mulino e mangimificio familiare, dal 1985 focalizzato sui mangimi e dal 2002 interamente convertito al biologico: specialista di mangimi composti bio (pollame, bovini, suini, cavalli, alpaca) con impiego di panello/soia biologica. PMI piccola, sotto la fascia target ma perfettamente in perimetro EUDR.</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>Karin Göweil</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>office@goeweil-muehle.at</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.goeweil-muehle.at</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Engerwitzdorf (Engerwitzberg), Alta Austria (Oberösterreich)</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goeweil-muehle.at/kontakt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Königshofer GmbH</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimificio e commercio mangimi</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Ca. 65 dipendenti (fonte sito aziendale 'Über uns' e firmenabc.at, dato 2024); fatturato non pubblicato nelle fonti aperte — per un mangimificio di questa scala si colloca indicativamente nella fascia 15-40 M€. Firmenbuch FN 442776t, UID ATU69978367. Stabilimento di Ebergassing (Franzensthalstraße 25) con silo cereali da 7.000 t, 53 celle materie prime e 44 celle prodotto finito; produce mangimi per cavalli e zootecnia con certificazione NON-GMO e pastus+ (impiego di soia/estratto di soia). Seconda Geschäftsführerin: Sarina Feurer.</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Mag. Astrid Pieler</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>ebergassing@koenigshofer.at</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>https://www.koenigshofer-futtermittel.at</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Ebergassing, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>https://www.koenigshofer-futtermittel.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Mischfutterwerk Großschedl GmbH</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimificio e commercio soia</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 8,5 Mio. € - ca. 15 dipendenti (fonte firmenabc.at / firmeninfo.at, dato 2023-2024). Firmenbuch FN 268698w. Azienda familiare al sito di Hofing dal 1780, produzione di mangimi composti dal 1964; oltre al mangimificio gestisce mulino e commercio di cereali, sementi e mangimi (Sojaschrot). Secondo Geschäftsführer: Mag. Dagmar Großschedl. IN TARGET (parte bassa della forbice tollerata 5-40 M€).</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>Herbert Großschedl</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>office@grosschedl-futter.at</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>http://www.grosschedl-futter.at</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>Blaindorf / Feistritztal (Hofing), Stiria (Steiermark)</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>http://www.grosschedl-futter.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Reitbauer Betriebs- u. Handels GmbH</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimificio e commercio agricolo</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Oltre 55-60 dipendenti (fonte sito aziendale 'Firma' e meinbezirk.at, 2023-2024); fatturato non pubblicato nelle fonti aperte. Firmenbuch FN 73386x, LG St. Pölten. Azienda familiare dal 1897, descritta come uno dei maggiori mangimifici privati d'Austria: mulino cereali, mangimificio (Mischfutter per bovini, suini, pollame) e Landhandel; utilizza componenti proteiche a base di soia. Ha anche una segheria, ma il core mangimi/cereali è l'attività in perimetro EUDR (soia).</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Stefan Reitbauer</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>office@reitbauer.co.at</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>https://www.reitbauer.co.at</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Vestenthal / Haidershofen, Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>https://www.reitbauer.co.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Rickl - Mühle GmbH</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — commercio cereali e Sojaschrot</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>PMI familiare fondata nel 1894, gestita da 3 responsabili (2 Geschäftsführer + 1 procuratore); fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at / firmeninfo.at / evi.gv.at, 2024-2025). Firmenbuch FN 162039v, LG Korneuburg, UID ATU43171303. Mulino e Landhandel a 35 km da Vienna: commercio di cereali convenzionali e bio, mangimi, sementi, concimi; a catalogo Sojaschrot (farina di estrazione di soia) come mangime proteico — attività di immissione sul mercato di soia = perimetro EUDR. TAGLIA DA VERIFICARE: probabile fascia bassa (5-15 M€).</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Josef Rickl</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>office@rickl.at</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rickl.at</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>Groß-Schweinbarth (Bezirk Gänserndorf), Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rickl.at/produkt/sojaschrot/</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Vorarlberger Mühlen und Mischfutterwerke GmbH</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mangimificio regionale</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Fatturato ca. 20 Mio. € - PMI industriale (fonte firmenabc.at / rassegna Raiffeisen Vorarlberg, dato 2022-2024). Firmenbuch FN 70012i, LG Feldkirch. Marchio 'Ländle Futter'; dal 2021 tornata azienda a controllo puramente familiare (uscita della Raiffeisenlandesbank Vorarlberg). Nuovo stabilimento mangimi a Dornbirn, Stöckenstraße 8. Utilizza panelli/estratto di soia nelle miscele. PERFETTAMENTE IN TARGET 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Bernd Hagen</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>office@laendlefutter.at</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>https://www.laendlefutter.at</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>Dornbirn (sede legale Feldkirch), Vorarlberg</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>https://www.laendlefutter.at/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Wieshofermühle Betriebs GmbH</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>Mangimi/Soia — mulino e mangimificio</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>PMI familiare alla 6ª generazione, sede a St. Johann da oltre 500 anni; fatturato e organico non pubblicati nelle fonti aperte (fonte sito aziendale / Impressum, 2024-2025). Firmenbuch FN 651815b, LG Innsbruck, UID ATU82121605. Iscritta WKO Tirol come 'Futtermittelerzeuger', 'Handel mit Futtermitteln' e 'Großhandel mit Lebensmitteln'. Uno dei pochi mulini + mangimifici austriaci ancora totalmente in mani private; il Futterwerk produce mangimi per bovini, pollame, suini, cavalli, ovicaprini e selvaggina (componenti proteiche a base di soia). Prokuristin: Mag. Caroline Krainz-Gasteiger.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Mag. Lukas Krainz</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer und 100%iger Anteilseigner</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>info@wieshofermuehle.at</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wieshofermuehle.at</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>St. Johann in Tirol, Tirolo (Tirol)</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wieshofermuehle.at/de/impressum</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>BIOSERVICE Zach Ges.m.b.H.</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Olio di palma — grossista ingredienti bio</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>PMI con oltre 25-30 anni di attività; fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at, WKO Firmen A-Z, advantageaustria.org, 2024-2025). Sedi/operatività a Schrems, Gmünd e St. Pölten (Bassa Austria). Grossista austriaco leader di ingredienti alimentari biologici certificati per trasformatori industriali e artigianali: a catalogo BIO-Palmfett/olio di palma in Großgebinde (fusti/grandi formati), oltre a cacao e caffè — tre commodity dell'Allegato I EUDR nello stesso portafoglio, quindi lead multi-commodity.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Ing. Mag. Robert Zach</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (alleinvertretungsberechtigt) e proprietario</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>zach@bioservice.at</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>https://www.bioservice.at</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Schrems (Wirtschaftspark 1), Bassa Austria (Niederösterreich)</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bioservice.at/en/products/organic-palm-fat-oil/</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Natural Products &amp; Drugs GmbH</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Olio di palma — commercio oli e grassi vegetali</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>PMI attiva a livello internazionale dal 2003, guidata da 2 Geschäftsführer (nomi non pubblicati nelle fonti consultate); fatturato e organico non pubblicati (fonti firmenabc.at, WKO Firmen A-Z, Creditreform, 2024-2025). Firmenbuch FN 283007m, LG Klagenfurt. Sede Neuer Platz 1, 9800 Spittal an der Drau; tel. +43 4762 44340. Società di produzione e commercio certificata ISO/Bio/Demeter con oltre 120 oli vegetali e grassi, oli essenziali, idrolati e materie prime per cosmetica e alimentare; compare tra i fornitori austriaci di Palmöl nella directory B2B wlw.at. NB: portafoglio in larga parte di oli NON Allegato I — il perimetro EUDR riguarda solo la linea olio di palma/palmisto: da qualificare in fase di contatto.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/natural-products-drugs-gmbh</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>http://www.np-d.com</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Spittal an der Drau, Carinzia (Kärnten)</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wlw.at/de/firma/natural-products-drugs-gmbh-958203</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Andrä Hörtnagl Produktion und Handel GmbH</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — carni e salumi, filiale proprie</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>ca. 24-25 Mio. € fatturato, ca. 200-230 dipendenti, 2.700 t/anno (top.tirol / agrarexportfoerderung.de, 2020-2023); Bilanzsumme 14,15 Mio. € al 31.12.2024 (firmenabc.at)</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Fabian Peter Kolozs, B.A. M.A.</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>office@hoertnagl.at</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>https://www.hoertnagl.at/</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Hall in Tirol, Tirol</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/andrae-hoertnagl-produktion-und-handel-gmbh_Cgt</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Fleischwaren Höllerschmid GmbH</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — lavorazione carne bovina, dry-aged</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Bilanzsumme 6,2 Mio. € al 31.03.2025 (firmenabc.at); fatturato non pubblicato — lavora ca. 20 t di carne bovina e 5 t di suino a settimana; azienda familiare di media dimensione, ampliamento 2025 (+2.500 m²). Firmenbuch FN 254597h</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Manfred Höllerschmid</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/fleischwaren-h%C3%B6llerschmid-gmbh</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>office@hoellerschmid.at</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hoellerschmid.at/</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Walkersdorf am Kamp (Grafenegg), Niederösterreich</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/fleischwaren-hoellerschmid-gmbh_HbCr</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>M. Feköhrer GmbH &amp; Co KG</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — macello UE e commercio bestiame</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>ca. 40 Mio. € fatturato, 30 dipendenti (+4 veterinari, 3 classificatori); ca. 11.500 bovini e 54.000 suini macellati/anno — fonte sito aziendale (fekoehrer.at, 2025). NOTA: fatturato gonfiato dal costo materia prima, PMI con soli 30 addetti. Firmenbuch FN 663491y</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Michael Feköhrer</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr"/>
+      <c r="G92" s="6" t="inlineStr">
+        <is>
+          <t>office@fekoehrer.at</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>https://www.fekoehrer.at/</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Mühlheim am Inn, Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>https://www.fekoehrer.at/impressum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Rudolf Frierss &amp; Söhne Fleisch- und Wurstspezialitäten Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — lavorazione carni e salumi</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>ca. 110-120 dipendenti su due stabilimenti a Villach (frierss.at / feines-haus.at, 2025); fatturato non pubblicato. Azienda familiare dal 1898, 5ª generazione. Firmenbuch FN 114403 (LG Klagenfurt)</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Rudolf Frierss</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr"/>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>office@frierss.at</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.frierss.at/</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>Villach, Kärnten</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/rudolf-frierss-soehne-fleisch-und-wurstspezialitaeten-gmbh_BAtZF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>Schwaninger Vieh Export GmbH</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — commercio ed export bestiame</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>12 Mio. € fatturato netto 2021 e 11 Mio. € 2022, 5 dipendenti (firmenabc.at / unternehmen24.info). NOTA: fatturato gonfiato dal costo del bestiame, micro-impresa per addetti. Firmenbuch FN 37288k</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Erwin Schwaninger</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr"/>
+      <c r="G94" s="6" t="inlineStr">
+        <is>
+          <t>office@schwaninger.co.at</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>https://www.viehexport.com/</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>Weer, Tirol</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/schwaninger-vieh-export-gmbh_EBAU</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>WIESTRADING Gesellschaft m.b.H.</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Bovini/Carne — commercio ed export bovini</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>ca. 15.000-20.000 capi commercializzati/anno (wiestrading.at, 2025); fatturato e organico non pubblicati — azienda familiare alla 3ª generazione. Firmenbuch FN 143186v</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Kurt Wiesinger</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>wiesingerviehhandel@aon.at</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiestrading.at/</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>Steegen (Peuerbach), Oberösterreich</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>https://www.firmenabc.at/wiestrading-ges-m-b-h_KDpS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:J95"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId208"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Applicate 27 correzioni certe: tassonomia filiera (FI 21, IT 2) e refusi formali (DK 4)
Tassonomia: le varianti storiche del foglio Finlandia (Legno/Compensato-Prodotti,
Legno/Segheria-Piallatura, Legno/CLT, Legno/Commercio-export) sono ricondotte alle
macro Legno/Arredo e Legno/Segheria, secondo la convenzione unanime degli altri 7 fogli.
Italia: «Caffè (import caffè verde)» -> «Caffè — import caffè verde».

Refusi formali Danimarca, verificati a fonte:
- FREDERICIA FURNITURE: «6,5 M€ DKK» mescolava le due valute -> «6,5 M DKK (≈0,87 M€)»
- Just Coffee -> Just Coffee I/S (interessentskab, CVR 35492380) e riserva sciolta
- INNOVATION LIVING: prefisso LinkedIn de. -> dk.

742 righe invariate, ordine dei fogli ripristinato.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -3090,7 +3090,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Caffè (import caffè verde)</t>
+          <t>Caffè — import caffè verde</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Caffè (import caffè verde)</t>
+          <t>Caffè — import caffè verde</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — finestre/porte in legno</t>
+          <t>Legno/Arredo — finestre/porte in legno</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -9797,7 +9797,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Legno/Segheria e trasformazione</t>
+          <t>Legno/Segheria — trasformazione</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -9845,7 +9845,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — impiallacciatura betulla colorata</t>
+          <t>Legno/Arredo — impiallacciatura betulla colorata</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -10141,7 +10141,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — CLT</t>
+          <t>Legno/Arredo — CLT</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -10193,7 +10193,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — impiallacciatura/laminati</t>
+          <t>Legno/Arredo — impiallacciatura/laminati</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Legno/Segheria-Piallatura</t>
+          <t>Legno/Segheria — piallatura</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -10441,7 +10441,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — compensato betulla/lamellare</t>
+          <t>Legno/Arredo — compensato betulla/lamellare</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Legno/Segheria-Piallatura</t>
+          <t>Legno/Segheria — piallatura</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -10637,7 +10637,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — finestre/porte in legno-alluminio</t>
+          <t>Legno/Arredo — finestre/porte in legno-alluminio</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -10685,7 +10685,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — scale in legno</t>
+          <t>Legno/Arredo — scale in legno</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -10773,7 +10773,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — legno lamellare/glulam</t>
+          <t>Legno/Arredo — legno lamellare/glulam</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — impiallacciatura ed erikoisvaneri</t>
+          <t>Legno/Arredo — impiallacciatura ed erikoisvaneri</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — hirsi/lamellare (glulam)</t>
+          <t>Legno/Arredo — hirsi/lamellare (glulam)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Legno/Commercio-export sahatavara</t>
+          <t>Legno/Segheria — commercio/export sahatavara</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11101,7 +11101,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Legno/CLT (trasformazione)</t>
+          <t>Legno/Arredo — CLT</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Legno/Segheria (betulla)</t>
+          <t>Legno/Segheria — betulla</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -11297,7 +11297,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — finestre/porte in legno-alluminio</t>
+          <t>Legno/Arredo — finestre/porte in legno-alluminio</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -11485,7 +11485,7 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — capriate/prodotti strutturali</t>
+          <t>Legno/Arredo — capriate/prodotti strutturali</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -11537,7 +11537,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Legno/Piallatura (pannelli/paneelit)</t>
+          <t>Legno/Segheria — piallatura (pannelli/paneelit)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — finestre/porte in legno</t>
+          <t>Legno/Arredo — finestre/porte in legno</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Legno/Compensato-Prodotti — parquet/pavimenti in legno</t>
+          <t>Legno/Arredo — parquet/pavimenti in legno</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -14367,7 +14367,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Utile lordo 60,4 M DKK ≈ 8,1 M€ nel 2024 (60,4 M DKK anche nel 2023) / 47 dip. nella sede di Fredericia (lasso.dk/proff.dk 2024); risultato ante imposte 6,5 M€ DKK; fatturato non pubblicato. Stima ricavi ~18-27 M€: da verificare. Capogruppo Thomas Graversen Holding ApS (gruppo indipendente danese)</t>
+          <t>Utile lordo 60,4 M DKK ≈ 8,1 M€ nel 2024 (60,4 M DKK anche nel 2023) / 47 dip. nella sede di Fredericia (lasso.dk/proff.dk 2024); risultato ante imposte 6,5 M DKK (≈0,87 M€); fatturato non pubblicato. Stima ricavi ~18-27 M€: da verificare. Capogruppo Thomas Graversen Holding ApS (gruppo indipendente danese)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/innovation-living-a-s</t>
+          <t>https://dk.linkedin.com/company/innovation-living-a-s</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -16741,7 +16741,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Just Coffee</t>
+          <t>Just Coffee I/S</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Applicate 22 correzioni formali al foglio Italia (forme giuridiche)
Accertate al Registro Imprese in Fase B (con P.IVA):
- Fonpelli S.p.A. -> Fonpelli S.r.l. (P.IVA 01705980249: la forma era errata)
- Conceria Cilp -> Conceria CILP S.r.l. (P.IVA 00190610501)
- Conceria Emmedue -> Conceria Emmedue S.r.l. (P.IVA 00793250242)
- 3C Lavorazione Pelli -> 3 C - Lavorazione Pelli S.r.l.

Normalizzazione ortografica (18): «Srl»/«SpA» -> «S.r.l.»/«S.p.A.», lo stile
maggioritario del foglio (41 record su 59 lo usavano gia').

Lasciate NON corrette, perche' ambigue: Conceria Beschin e Conceria Daniela
corrispondono ciascuna a due entita' omonime distinte al Registro (S.n.c. e S.r.l.
nello stesso comune): va prima identificato quale sia l'operatore EUDR.

742 righe invariate, ordine dei fogli ripristinato.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -565,7 +565,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>3C Lavorazione Pelli S.r.l.</t>
+          <t>3 C - Lavorazione Pelli S.r.l.</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -765,7 +765,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Conceria Cilp</t>
+          <t>Conceria CILP S.r.l.</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -845,7 +845,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Conceria Emmedue</t>
+          <t>Conceria Emmedue S.r.l.</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1261,7 +1261,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Fonpelli S.p.A.</t>
+          <t>Fonpelli S.r.l.</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1301,7 +1301,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>A. Brivio Compensati SpA</t>
+          <t>A. Brivio Compensati S.p.A.</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,7 +1341,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Arko SpA</t>
+          <t>Arko S.p.A.</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1377,7 +1377,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Aster Cucine SpA</t>
+          <t>Aster Cucine S.p.A.</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Basso Legnami Srl</t>
+          <t>Basso Legnami S.r.l.</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Bedogna F.lli Srl</t>
+          <t>Bedogna F.lli S.r.l.</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>C.I.M.A. Srl (Compensati Impiallacciature Materiali Affini)</t>
+          <t>C.I.M.A. S.r.l. (Compensati Impiallacciature Materiali Affini)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Caccaro Srl</t>
+          <t>Caccaro S.r.l.</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1581,7 +1581,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Cadorin Group Srl</t>
+          <t>Cadorin Group S.r.l.</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Compensati Toro SpA</t>
+          <t>Compensati Toro S.p.A.</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1661,7 +1661,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Fratelli Berti Legnami Srl</t>
+          <t>Fratelli Berti Legnami S.r.l.</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1701,7 +1701,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Holzland Fuchs Srl</t>
+          <t>Holzland Fuchs S.r.l.</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1737,7 +1737,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Itlas Srl Società Benefit</t>
+          <t>Itlas S.r.l. Società Benefit</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1777,7 +1777,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Nord Legnami Group Srl</t>
+          <t>Nord Legnami Group S.r.l.</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Nuova River Srl</t>
+          <t>Nuova River S.r.l.</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1857,7 +1857,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Original Parquet SpA</t>
+          <t>Original Parquet S.p.A.</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1897,7 +1897,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>PALM SpA SB</t>
+          <t>PALM S.p.A. SB</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -1937,7 +1937,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Segheria Saccavini Srl</t>
+          <t>Segheria Saccavini S.r.l.</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1977,7 +1977,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Zalf SpA (Zalf Industria Mobili Componibili)</t>
+          <t>Zalf S.p.A. (Zalf Industria Mobili Componibili)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Applicate 5 correzioni di denominazione accertate ai registri
- Danimarca: NPI (Nordic Panel Import) -> NPI A/S (CVR 37418730)
- Olanda: Rompa Tanneries B.V. -> Vitelco Leather B.V. (sciolta la JV, Vitelco socio unico)
- Austria: Karnische Massiv Moebel GmbH -> Karnische-Massiv-Moebel Gesellschaft m.b.H. (FN 094638z)
- Belgio: Confiserie Vandenbulcke NV -> Vandenbulcke Confiserie NV (ordine registrale KBO)
- Germania: Paletten Meyer -> Josef Meyer Palettenbau Inh. Julian Meyer (impresa individuale)

Non applicate le espansioni di ragioni sociali abbreviate ma corrette (Goebel,
Fuhlrott) ne' AB -> Aktiebolag in Svezia, dove il foglio non ha uno stile
maggioritario (47 AB contro 42 Aktiebolag).

742 righe invariate, ordine dei fogli ripristinato.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -5391,7 +5391,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Paletten Meyer</t>
+          <t>Josef Meyer Palettenbau Inh. Julian Meyer (Paletten Meyer)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -15229,7 +15229,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>NPI (Nordic Panel Import)</t>
+          <t>NPI A/S (Nordic Panel Import)</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -23473,7 +23473,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Rompa Tanneries B.V.</t>
+          <t>Vitelco Leather B.V. (già Rompa Tanneries B.V.)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -31456,70 +31456,74 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Confiserie Vandenbulcke NV</t>
+          <t>Corné Port-Royal Chocolatier SA</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e tavolette</t>
+          <t>Cacao/Cioccolato — praline artigianali</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 13.332.120 € e 31,5 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-12-2024). N. impresa BE 0417.738.319. Fondata 1949; export in oltre 50 paesi. In pieno target 10-20 M€.</t>
+          <t>Fatturato 8.796.906 € (ultimo bilancio depositato NBB, deposito 26-06-2025; 8.421.952 € e 54° posto di settore su trendstop.knack.be). N. impresa BE 0433.283.558. Sede Avenue Vésale 12, 1300 Wavre; maison storica (marchio dal 1932), rete di ~20 boutique in Belgio e 15 in Francia. Sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr"/>
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/chocolatiervandenbulcke</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="inlineStr">
-        <is>
-          <t>info@vandenbulcke.com</t>
+          <t>https://be.linkedin.com/company/corn-port-royal</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>https://www.vandenbulcke.com/</t>
+          <t>https://www.corneportroyal.com/</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Heule, Kortrijk (West-Vlaanderen) — Fiandre</t>
+          <t>Wavre (Brabant wallon) — Vallonia</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0417738319/confiserie-vandenbulcke</t>
+          <t>https://www.companyweb.be/en/0433283558/corne-port-royal-chocolatier</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Corné Port-Royal Chocolatier SA</t>
+          <t>Delafaille NV</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline artigianali</t>
+          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 8.796.906 € (ultimo bilancio depositato NBB, deposito 26-06-2025; 8.421.952 € e 54° posto di settore su trendstop.knack.be). N. impresa BE 0433.283.558. Sede Avenue Vésale 12, 1300 Wavre; maison storica (marchio dal 1932), rete di ~20 boutique in Belgio e 15 in Francia. Sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr"/>
-      <c r="E66" s="5" t="inlineStr"/>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/corn-port-royal</t>
-        </is>
-      </c>
+          <t>Fatturato 14.244.468 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB, deposito 17-06-2025); 43° nel settore cioccolato e dolciumi. N. impresa BE 0467.502.683. In pieno target 10-20 M€. Legame di gruppo: acquisita dallo svizzero Maestrani Schweizer Schokoladen (con la controllata Ostrapack); resta però PMI belga autonoma con obblighi EUDR propri.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Paul Daems</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>CEO / gedelegeerd bestuurder (uscente, transizione dopo l'acquisizione Maestrani 2025)</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31527,47 +31531,43 @@
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>https://www.corneportroyal.com/</t>
+          <t>https://www.delafaille.be/</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Wavre (Brabant wallon) — Vallonia</t>
+          <t>Melsele, Beveren-Kruibeke-Zwijndrecht (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0433283558/corne-port-royal-chocolatier</t>
+          <t>https://trendstop.knack.be/nl/detail/467502683/delafaille.aspx</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Delafaille NV</t>
+          <t>Dolfin SA</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
+          <t>Cacao/Cioccolato — tavolette premium</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 14.244.468 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB, deposito 17-06-2025); 43° nel settore cioccolato e dolciumi. N. impresa BE 0467.502.683. In pieno target 10-20 M€. Legame di gruppo: acquisita dallo svizzero Maestrani Schweizer Schokoladen (con la controllata Ostrapack); resta però PMI belga autonoma con obblighi EUDR propri.</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Paul Daems</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>CEO / gedelegeerd bestuurder (uscente, transizione dopo l'acquisizione Maestrani 2025)</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr"/>
+          <t>33,2 FTE da ultimo bilancio depositato NBB (deposito 20-01-2026, cifra d'affari non pubblicata); fatturato ~6 M€ secondo la stampa economica (L'Avenir/RTBF, ~385 t di cioccolato/anno). N. impresa BE 0437.332.220. Sede Avenue Robert Schuman 172, 1401 Baulers (Nivelles). Prima cioccolateria belga certificata carbon neutral (2008); programma di sostenibilità cacao proprio 'Cocoa Act 4'. Taglia sotto la fascia ottimale, nel range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr"/>
+      <c r="E67" s="3" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/dolfin-sa</t>
+        </is>
+      </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31575,311 +31575,311 @@
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>https://www.delafaille.be/</t>
+          <t>https://www.dolfin.be/</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Melsele, Beveren-Kruibeke-Zwijndrecht (Oost-Vlaanderen) — Fiandre</t>
+          <t>Baulers, Nivelles (Brabant wallon) — Vallonia</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/467502683/delafaille.aspx</t>
+          <t>https://www.companyweb.be/en/0437332220/dolfin</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Dolfin SA</t>
+          <t>Gudrun Commercial NV</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — tavolette premium</t>
+          <t>Cacao/Cioccolato — praline e tartufi</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>33,2 FTE da ultimo bilancio depositato NBB (deposito 20-01-2026, cifra d'affari non pubblicata); fatturato ~6 M€ secondo la stampa economica (L'Avenir/RTBF, ~385 t di cioccolato/anno). N. impresa BE 0437.332.220. Sede Avenue Robert Schuman 172, 1401 Baulers (Nivelles). Prima cioccolateria belga certificata carbon neutral (2008); programma di sostenibilità cacao proprio 'Cocoa Act 4'. Taglia sotto la fascia ottimale, nel range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr"/>
-      <c r="E68" s="5" t="inlineStr"/>
+          <t>Fatturato 43.457.280 € e 138,6 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 15-07-2026). N. impresa BE 0476.530.118. Sede Industriestraat 18, 2500 Lier. Firmataria di Beyond Chocolate. AZIENDA DI CONFINE: fatturato sopra la fascia tollerabile 5-40 M€ (ma sotto la soglia di esclusione ~50 M€). Legame di gruppo: acquisita dal gruppo spagnolo Natra (che controlla anche Natra Chocolate Belgium NV, ~93 M€, fuori target).</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Sofie De Lathouwer</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/dolfin-sa</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>https://be.linkedin.com/company/gudrun-commercial-nv</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>info@chocolates.be</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>https://www.dolfin.be/</t>
+          <t>https://gudrungroup.be/</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Baulers, Nivelles (Brabant wallon) — Vallonia</t>
+          <t>Lier (Anversa) — Fiandre</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0437332220/dolfin</t>
+          <t>https://www.companyweb.be/en/0476530118/gudrun-commercial</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Gudrun Commercial NV</t>
+          <t>La Chocolaterie Galler SA</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e tartufi</t>
+          <t>Cacao/Cioccolato — tavolette e praline</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 43.457.280 € e 138,6 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 15-07-2026). N. impresa BE 0476.530.118. Sede Industriestraat 18, 2500 Lier. Firmataria di Beyond Chocolate. AZIENDA DI CONFINE: fatturato sopra la fascia tollerabile 5-40 M€ (ma sotto la soglia di esclusione ~50 M€). Legame di gruppo: acquisita dal gruppo spagnolo Natra (che controlla anche Natra Chocolate Belgium NV, ~93 M€, fuori target).</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Sofie De Lathouwer</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/gudrun-commercial-nv</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>info@chocolates.be</t>
+          <t>Fatturato 29.502.986 € (fonte: pappers.be/trendstop, bilancio NBB); dato più recente ~32 M€ con perdita netta 1,7 M€ nel 2024; 194 dipendenti. N. impresa BE 0416.169.689. Azienda di confine nella parte alta del range tollerabile (5-40 M€). Nota: nell'aprile 2026 rilevata da un consorzio vallone con piano di ristrutturazione (~70 licenziamenti su 170).</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr"/>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>https://gudrungroup.be/</t>
+          <t>https://www.galler.com/</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Lier (Anversa) — Fiandre</t>
+          <t>Vaux-sous-Chèvremont (Chaudfontaine), Liegi — Vallonia</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0476530118/gudrun-commercial</t>
+          <t>https://www.pappers.be/fr/company/la-chocolaterie-galler-0416169689</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>La Chocolaterie Galler SA</t>
+          <t>Libeert NV</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — tavolette e praline</t>
+          <t>Cacao/Cioccolato — figure e tavolette di cioccolato</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 29.502.986 € (fonte: pappers.be/trendstop, bilancio NBB); dato più recente ~32 M€ con perdita netta 1,7 M€ nel 2024; 194 dipendenti. N. impresa BE 0416.169.689. Azienda di confine nella parte alta del range tollerabile (5-40 M€). Nota: nell'aprile 2026 rilevata da un consorzio vallone con piano di ristrutturazione (~70 licenziamenti su 170).</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr"/>
-      <c r="E70" s="5" t="inlineStr"/>
+          <t>Fatturato ~35 M€ e 136,8 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 13-11-2025). N. impresa BE 0407.026.747. Azienda familiare, oltre 5.000 t di cioccolato all'anno, gamma bio. Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Lily Libeert</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Co-directrice (4a generazione della famiglia Libeert)</t>
+        </is>
+      </c>
       <c r="F70" s="5" t="inlineStr"/>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>contact@libeert.com</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>https://www.galler.com/</t>
+          <t>https://www.libeert.com/</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Vaux-sous-Chèvremont (Chaudfontaine), Liegi — Vallonia</t>
+          <t>Comines-Warneton (Komen-Waasten), Hainaut — Vallonia</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/fr/company/la-chocolaterie-galler-0416169689</t>
+          <t>https://www.companyweb.be/en/0407026747/libeert</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Libeert NV</t>
+          <t>Manufacture Belge de Chocolats SRL</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — figure e tavolette di cioccolato</t>
+          <t>Cacao/Cioccolato — praline e private label</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ~35 M€ e 136,8 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 13-11-2025). N. impresa BE 0407.026.747. Azienda familiare, oltre 5.000 t di cioccolato all'anno, gamma bio. Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI familiare indipendente.</t>
+          <t>Fatturato 25.731.148 € e 175,1 FTE (fonte: trendstop.levif.be / companyweb.be, ultimo bilancio depositato NBB, deposito 08-07-2025); 30° posto nel settore cioccolato e dolciumi. N. impresa BE 0722.764.519. Firmataria di Beyond Chocolate (impegni su deforestazione e tracciabilità del cacao). Nella parte alta del range tollerabile 5-40 M€.</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Lily Libeert</t>
+          <t>Arnaud Verwilghen</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Co-directrice (4a generazione della famiglia Libeert)</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr"/>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>contact@libeert.com</t>
+          <t>info@mbcchocolates.be</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>https://www.libeert.com/</t>
+          <t>https://www.mbcchocolates.be/</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Comines-Warneton (Komen-Waasten), Hainaut — Vallonia</t>
+          <t>Koekelberg, Bruxelles (1081) — Regione di Bruxelles-Capitale</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0407026747/libeert</t>
+          <t>https://trendstop.levif.be/fr/detail/722764519/manufacture-belge-de-chocolats.aspx</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Manufacture Belge de Chocolats SRL</t>
+          <t>Oxfam Fair Trade CV</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e private label</t>
+          <t>Cacao/Cioccolato — import equosolidale cacao</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 25.731.148 € e 175,1 FTE (fonte: trendstop.levif.be / companyweb.be, ultimo bilancio depositato NBB, deposito 08-07-2025); 30° posto nel settore cioccolato e dolciumi. N. impresa BE 0722.764.519. Firmataria di Beyond Chocolate (impegni su deforestazione e tracciabilità del cacao). Nella parte alta del range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Arnaud Verwilghen</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
+          <t>Fatturato 17.446.343 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB); 81° posto nel settore alimentare/commercio. N. impresa BE 0453.066.016. Importatore equosolidale: acquista cacao (e caffè) direttamente dalle cooperative dei paesi produttori e immette i prodotti sul mercato UE — operatore EUDR in senso stretto. Firmataria di Beyond Chocolate. In pieno target 10-20 M€. Nota: struttura cooperativa legata a Oxfam-Wereldwinkels.</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr"/>
       <c r="F72" s="5" t="inlineStr"/>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>info@mbcchocolates.be</t>
+          <t>info@oft.be</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>https://www.mbcchocolates.be/</t>
+          <t>https://www.oxfamfairtrade.be/</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Koekelberg, Bruxelles (1081) — Regione di Bruxelles-Capitale</t>
+          <t>Gent (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/722764519/manufacture-belge-de-chocolats.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/453066016/oxfam-fairtrade.aspx</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Oxfam Fair Trade CV</t>
+          <t>Pierre Marcolini Group SA</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — import equosolidale cacao</t>
+          <t>Cacao/Cioccolato — bean-to-bar e praline</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 17.446.343 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB); 81° posto nel settore alimentare/commercio. N. impresa BE 0453.066.016. Importatore equosolidale: acquista cacao (e caffè) direttamente dalle cooperative dei paesi produttori e immette i prodotti sul mercato UE — operatore EUDR in senso stretto. Firmataria di Beyond Chocolate. In pieno target 10-20 M€. Nota: struttura cooperativa legata a Oxfam-Wereldwinkels.</t>
+          <t>Fatturato 19.300.806 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0461.740.982. Maison bean-to-bar: acquista e importa direttamente fave di cacao dai paesi d'origine (Vietnam, Madagascar, Ecuador, Perù) — operatore EUDR in senso stretto. In pieno target 10-20 M€. Legame di gruppo: entità collegata Pierre Marcolini Belgium SA (BE 0460.046.551, ~11,3 M€, rete retail).</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr"/>
       <c r="E73" s="3" t="inlineStr"/>
       <c r="F73" s="3" t="inlineStr"/>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>info@oft.be</t>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>https://www.oxfamfairtrade.be/</t>
+          <t>https://eu.marcolini.com/</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Gent (Oost-Vlaanderen) — Fiandre</t>
+          <t>Bruxelles (Haren, 1130) — Regione di Bruxelles-Capitale</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/453066016/oxfam-fairtrade.aspx</t>
+          <t>https://www.pappers.be/fr/company/pierre-marcolini-group-0461740982</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Pierre Marcolini Group SA</t>
+          <t>Pralinart NV</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — bean-to-bar e praline</t>
+          <t>Cacao/Cioccolato — praline</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 19.300.806 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0461.740.982. Maison bean-to-bar: acquista e importa direttamente fave di cacao dai paesi d'origine (Vietnam, Madagascar, Ecuador, Perù) — operatore EUDR in senso stretto. In pieno target 10-20 M€. Legame di gruppo: entità collegata Pierre Marcolini Belgium SA (BE 0460.046.551, ~11,3 M€, rete retail).</t>
+          <t>Fatturato 18.427.020 € e 34 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 02-11-2023). N. impresa BE 0450.589.051. Sede Waaslandlaan 32, 9160 Lokeren; fino a 10 t di praline al giorno. In pieno target 10-20 M€. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), consociata di A &amp; A Chocolaterie NV.</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr"/>
       <c r="E74" s="5" t="inlineStr"/>
-      <c r="F74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
+        </is>
+      </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31887,61 +31887,61 @@
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>https://eu.marcolini.com/</t>
+          <t>https://www.hamlet.be/</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Bruxelles (Haren, 1130) — Regione di Bruxelles-Capitale</t>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/fr/company/pierre-marcolini-group-0461740982</t>
+          <t>https://www.companyweb.be/en/0450589051/pralinart</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Pralinart NV</t>
+          <t>Vandenbulcke Confiserie NV</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline</t>
+          <t>Cacao/Cioccolato — praline e tavolette</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 18.427.020 € e 34 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 02-11-2023). N. impresa BE 0450.589.051. Sede Waaslandlaan 32, 9160 Lokeren; fino a 10 t di praline al giorno. In pieno target 10-20 M€. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), consociata di A &amp; A Chocolaterie NV.</t>
+          <t>Fatturato 13.332.120 € e 31,5 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-12-2024). N. impresa BE 0417.738.319. Fondata 1949; export in oltre 50 paesi. In pieno target 10-20 M€.</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr"/>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
-        </is>
-      </c>
-      <c r="G75" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>https://be.linkedin.com/company/chocolatiervandenbulcke</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>info@vandenbulcke.com</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>https://www.hamlet.be/</t>
+          <t>https://www.vandenbulcke.com/</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+          <t>Heule, Kortrijk (West-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0450589051/pralinart</t>
+          <t>https://www.companyweb.be/en/0417738319/confiserie-vandenbulcke</t>
         </is>
       </c>
     </row>
@@ -33070,25 +33070,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId145"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId153"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId167"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId169"/>
@@ -33953,7 +33953,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Karnische Massiv Möbel GmbH</t>
+          <t>Karnische-Massiv-Möbel Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Belgio: rimossa Covera Packaging (vetro e plastica, non cartone); belgio_03 e austria_03 completi
Covera Packaging NV era censita come «Carta/Packaging - imballaggi cartone ondulato»,
ma si presenta sul proprio sito come grossista di imballaggi in vetro e plastica
rigida: il record era nel censimento su un presupposto falso. Vetro e plastica non
sono commodity dell'Allegato I. Stesso criterio di Immobra, RICO Elastomere e k-tec.

Varia-Pack resta invece nel foglio come rilievo alta aperto: il cartone E' commodity
dell'Allegato I e l'argomento e' solo che l'azienda commercia invece di immettere per
prima: e' la distinzione operatore/commerciante, non un errore di perimetro.

Censimento da 738 a 737 aziende (Belgio 94->93).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28346,7 +28346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -30239,634 +30239,634 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Covera Packaging NV</t>
+          <t>Desmedt Labels BV</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — imballaggi cartone ondulato</t>
+          <t>Carta/Packaging — etichette</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Fatturato nella fascia 10.000.000-25.000.000 € - 9,3 FTE (fonte companyweb.be / fincheck.be, ultimo bilancio depositato NBB; l'azienda deposita in schema abbreviato e non pubblica la cifra d'affari esatta). N. impresa BE 0462.810.754. Produzione e distribuzione di imballaggi in cartone ondulato e materiali d'imballaggio; sede Smallandlaan 37, 2660 Hoboken (Antwerpen). Origine familiare come Comptoir Verrier Anversois. IN TARGET stimato ma verificare il fatturato esatto.</t>
+          <t>Fatturato 6.500.000 € con 32 dipendenti secondo l'ultimo dato pubblicato (fonte made-in.be / Voka Ondernemers); organico più recente indicato in ca. 21 persone a Bornem. Azienda familiare fondata nel 1889 da François Desmedt, oggi alla quinta generazione (Henri Kökler); trasferita da Bruxelles a Bornem nel 2012. Etichette autoadesive prodotte in modo CO2-neutro. SOTTO il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€; dato di fatturato non recentissimo, da riverificare sul bilancio NBB.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Johan Stouten</t>
+          <t>Henri Kökler</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>Zaakvoerder</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/covera-packaging</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>sales@covera.be</t>
+          <t>https://be.linkedin.com/company/desmedt</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>https://covera.be</t>
+          <t>https://www.desmedt.be</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Hoboken (Anversa), Provincia di Anversa (Fiandre)</t>
+          <t>Bornem, Provincia di Anversa (Fiandre)</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>https://fincheck.be/nl/covera-packaging/0462.810.754/Antwerpen/overzicht</t>
+          <t>https://www.made-in.be/antwerpen/desmedt-labels-neemt-nieuwe-start/</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Desmedt Labels BV</t>
+          <t>Emballages Gruselle SRL</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — etichette</t>
+          <t>Carta/Packaging — imballaggi cartone</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 6.500.000 € con 32 dipendenti secondo l'ultimo dato pubblicato (fonte made-in.be / Voka Ondernemers); organico più recente indicato in ca. 21 persone a Bornem. Azienda familiare fondata nel 1889 da François Desmedt, oggi alla quinta generazione (Henri Kökler); trasferita da Bruxelles a Bornem nel 2012. Etichette autoadesive prodotte in modo CO2-neutro. SOTTO il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€; dato di fatturato non recentissimo, da riverificare sul bilancio NBB.</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Henri Kökler</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Zaakvoerder</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/desmedt</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>DATO DI FATTURATO NON PUBBLICATO sulle fonti accessibili (companyweb/fincheck/pappers riportano la scheda ma non la cifra d'affari; l'azienda deposita in schema abbreviato). N. impresa BE 0448.350.331, costituita nel 1992. Azienda familiare, fabbricazione di scatole in cartone e articoli d'imballaggio e protezione; officina nel parco industriale di Martinrou, Rue de Rabiseau 12, 6220 Fleurus. AZIENDA DI CONFINE: taglia stimata SOTTO i 5 M€ — inserita per copertura della filiera in Vallonia, da qualificare prima del contatto.</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>gruselle@skynet.be</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>https://www.desmedt.be</t>
+          <t>https://www.emballagesgruselle.eu</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Bornem, Provincia di Anversa (Fiandre)</t>
+          <t>Fleurus, Provincia di Hainaut (Vallonia)</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>https://www.made-in.be/antwerpen/desmedt-labels-neemt-nieuwe-start/</t>
+          <t>https://trendstop.levif.be/fr/detail/448350331/gruselle-emballages.aspx</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Emballages Gruselle SRL</t>
+          <t>Etilux SA</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — imballaggi cartone</t>
+          <t>Carta/Packaging — etichette</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>DATO DI FATTURATO NON PUBBLICATO sulle fonti accessibili (companyweb/fincheck/pappers riportano la scheda ma non la cifra d'affari; l'azienda deposita in schema abbreviato). N. impresa BE 0448.350.331, costituita nel 1992. Azienda familiare, fabbricazione di scatole in cartone e articoli d'imballaggio e protezione; officina nel parco industriale di Martinrou, Rue de Rabiseau 12, 6220 Fleurus. AZIENDA DI CONFINE: taglia stimata SOTTO i 5 M€ — inserita per copertura della filiera in Vallonia, da qualificare prima del contatto.</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
+          <t>Fatturato consolidato ca. 16.000.000 € e 50 dipendenti (fonte ccimag.be, gennaio 2024; l'articolo ccimag di giugno 2023 indicava ca. 18 M€). 42 FTE nell'ultimo bilancio depositato NBB; la società deposita in schema abbreviato e non pubblica la cifra d'affari (fonte pappers.be / companyweb.be). N. impresa BE 0412.681.550. Sede Rue de l'Espérance 42, 4000 Liegi. Azienda familiare fondata nel 1972: etichette adesive, tracciabilità/RFID, adesivi tecnici e imballaggi; filiale in Lussemburgo. IN TARGET 10-20 M€. Secondo amministratore delegato: Olivier Bronne.</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Quentin Gemoets</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
       <c r="F43" s="3" t="inlineStr"/>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>gruselle@skynet.be</t>
+          <t>info@etilux.be</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>https://www.emballagesgruselle.eu</t>
+          <t>https://www.etilux.com</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Fleurus, Provincia di Hainaut (Vallonia)</t>
+          <t>Liegi, Provincia di Liegi (Vallonia)</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/448350331/gruselle-emballages.aspx</t>
+          <t>https://ccimag.be/2024/01/05/la-transition-generationnelle-se-finalise-chez-etilux/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Etilux SA</t>
+          <t>Imprimerie Bietlot SA</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — etichette</t>
+          <t>Carta/Packaging — stampa</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Fatturato consolidato ca. 16.000.000 € e 50 dipendenti (fonte ccimag.be, gennaio 2024; l'articolo ccimag di giugno 2023 indicava ca. 18 M€). 42 FTE nell'ultimo bilancio depositato NBB; la società deposita in schema abbreviato e non pubblica la cifra d'affari (fonte pappers.be / companyweb.be). N. impresa BE 0412.681.550. Sede Rue de l'Espérance 42, 4000 Liegi. Azienda familiare fondata nel 1972: etichette adesive, tracciabilità/RFID, adesivi tecnici e imballaggi; filiale in Lussemburgo. IN TARGET 10-20 M€. Secondo amministratore delegato: Olivier Bronne.</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Quentin Gemoets</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Administrateur délégué</t>
-        </is>
-      </c>
+          <t>Fatturato 6.970.646 € - 33,5 FTE (fonte companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0473.613.485. Imprimerie industriale offset (magazine, edizione, stampati amministrativi), sede Rue du Rond-Point 185, 6060 Gilly (Charleroi). SOTTO IL TARGET 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Partecipata storica di Sambrinvest.</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="inlineStr"/>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>info@etilux.be</t>
+          <t>info@bietlot.be</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>https://www.etilux.com</t>
+          <t>https://www.bietlot.be</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Liegi, Provincia di Liegi (Vallonia)</t>
+          <t>Gilly (Charleroi), Provincia di Hainaut (Vallonia)</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>https://ccimag.be/2024/01/05/la-transition-generationnelle-se-finalise-chez-etilux/</t>
+          <t>https://www.companyweb.be/fr/0473613485/imprimerie-bietlot</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Imprimerie Bietlot SA</t>
+          <t>Kartonnage Lefevere-Beel NV</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 6.970.646 € - 33,5 FTE (fonte companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0473.613.485. Imprimerie industriale offset (magazine, edizione, stampati amministrativi), sede Rue du Rond-Point 185, 6060 Gilly (Charleroi). SOTTO IL TARGET 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. Partecipata storica di Sambrinvest.</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="3" t="inlineStr"/>
+          <t>Fatturato 26.865.930 € - 69,2 FTE (fonte pappers.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0413.759.339. Trasformazione di cartone ondulato in imballaggi su misura, sede Driekoningenstraat 7, 8710 Wielsbeke. Amministratori: Didier Lefevere, Marieke Lannoo e la società BellRock. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Didier Lefevere</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>CEO / Bestuurder</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/kartonnage-lefevere-beel</t>
+        </is>
+      </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>info@bietlot.be</t>
+          <t>info@lefeverebeel.be</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>https://www.bietlot.be</t>
+          <t>https://www.lefeverebeel.be</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Gilly (Charleroi), Provincia di Hainaut (Vallonia)</t>
+          <t>Wielsbeke, Provincia di Fiandre Occidentali (Fiandre)</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/fr/0473613485/imprimerie-bietlot</t>
+          <t>https://www.pappers.be/nl/company/kartonnage-lefevere-beel-0413759339</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Kartonnage Lefevere-Beel NV</t>
+          <t>Label-Pak-Int'l Co SA</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Carta/Packaging — etichette</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 26.865.930 € - 69,2 FTE (fonte pappers.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0413.759.339. Trasformazione di cartone ondulato in imballaggi su misura, sede Driekoningenstraat 7, 8710 Wielsbeke. Amministratori: Didier Lefevere, Marieke Lannoo e la società BellRock. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Didier Lefevere</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>CEO / Bestuurder</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/kartonnage-lefevere-beel</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>info@lefeverebeel.be</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="inlineStr">
-        <is>
-          <t>https://www.lefeverebeel.be</t>
+          <t>Fatturato NON pubblicato nell'ultimo bilancio depositato NBB (schema abbreviato, deposito 01-07-2023); margine lordo 1.920.400 € e 27,2 FTE (fonte companyweb.be / fincheck.be). N. impresa BE 0402.690.550. Sede Avenue Galilée 8, 1300 Wavre. Azienda familiare fondata nel 1968, oltre 50 anni di stampa di etichette personalizzate in carta. AZIENDA DI CONFINE: dimensione stimata SOTTO il target 10-20 M€ e probabilmente sotto i 5 M€ — da verificare sul bilancio integrale NBB.</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Wielsbeke, Provincia di Fiandre Occidentali (Fiandre)</t>
+          <t>Wavre, Provincia del Brabante Vallone (Vallonia)</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/nl/company/kartonnage-lefevere-beel-0413759339</t>
+          <t>https://www.companyweb.be/en/0402690550/label-pak-int-l-co</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Label-Pak-Int'l Co SA</t>
+          <t>Snel Grafics SA</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — etichette</t>
+          <t>Carta/Packaging — stampa</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato nell'ultimo bilancio depositato NBB (schema abbreviato, deposito 01-07-2023); margine lordo 1.920.400 € e 27,2 FTE (fonte companyweb.be / fincheck.be). N. impresa BE 0402.690.550. Sede Avenue Galilée 8, 1300 Wavre. Azienda familiare fondata nel 1968, oltre 50 anni di stampa di etichette personalizzate in carta. AZIENDA DI CONFINE: dimensione stimata SOTTO il target 10-20 M€ e probabilmente sotto i 5 M€ — da verificare sul bilancio integrale NBB.</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato 11.822.115 € (fonte trendstop.levif.be / companyweb, ultimo bilancio depositato NBB). Ca. 65 dipendenti (fonte ccimag.be / RTBF). N. impresa BE 0440.957.842. Imprimerie offset e digitale (libri, brochure) rilevata in MBO nel 1995 da Roland Soubras e Flavio De Beni. Sede Rue du Fond des Fourches 21, 4041 Vottem. IN TARGET.</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Roland Soubras</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/in/roland-soubras-63aa1560</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>info@snel.be</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.snel.be</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Wavre, Provincia del Brabante Vallone (Vallonia)</t>
+          <t>Vottem (Herstal), Provincia di Liegi (Vallonia)</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0402690550/label-pak-int-l-co</t>
+          <t>https://trendstop.levif.be/fr/detail/440957842/snel-grafics.aspx</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Snel Grafics SA</t>
+          <t>Van de Velde Packaging NV</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 11.822.115 € (fonte trendstop.levif.be / companyweb, ultimo bilancio depositato NBB). Ca. 65 dipendenti (fonte ccimag.be / RTBF). N. impresa BE 0440.957.842. Imprimerie offset e digitale (libri, brochure) rilevata in MBO nel 1995 da Roland Soubras e Flavio De Beni. Sede Rue du Fond des Fourches 21, 4041 Vottem. IN TARGET.</t>
+          <t>Fatturato 15.032.194 € - 52,3 FTE (fonte fincheck.be / pappers.be, ultimo bilancio depositato NBB). N. impresa BE 0444.255.050. Produzione di imballaggi in carta e cartone ondulato, sede Industrielaan 22, 8810 Lichtervelde. PERFETTAMENTE IN TARGET 10-20 M€. LEGAME DI GRUPPO: società del gruppo belga P. Van de Velde / Van de Velde Packaging (quartier generale a Wetteren, ca. 1.300 addetti e 309 M€ di fatturato di gruppo nel 2023, sedi in 8 paesi europei; aumento di capitale 2025 sottoscritto da Kartesia); il gedelegeerd bestuurder iscritto in KBO è la persona giuridica P. Van de Velde NV.</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Roland Soubras</t>
+          <t>Carl Mourisse</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Administrateur délégué</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/in/roland-soubras-63aa1560</t>
-        </is>
-      </c>
+          <t>Bestuurder</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>info@snel.be</t>
+          <t>info.lichtervelde@vandeveldepackaging.com</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>https://www.snel.be</t>
+          <t>https://www.vandeveldepackaging.com</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Vottem (Herstal), Provincia di Liegi (Vallonia)</t>
+          <t>Lichtervelde, Provincia di Fiandre Occidentali (Fiandre)</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/440957842/snel-grafics.aspx</t>
+          <t>https://fincheck.be/en/van-de-velde-packaging/0444.255.050/Lichtervelde/overview</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Van de Velde Packaging NV</t>
+          <t>Varia-Pack NV</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Carta/Packaging — commercio imballaggi carta</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 15.032.194 € - 52,3 FTE (fonte fincheck.be / pappers.be, ultimo bilancio depositato NBB). N. impresa BE 0444.255.050. Produzione di imballaggi in carta e cartone ondulato, sede Industrielaan 22, 8810 Lichtervelde. PERFETTAMENTE IN TARGET 10-20 M€. LEGAME DI GRUPPO: società del gruppo belga P. Van de Velde / Van de Velde Packaging (quartier generale a Wetteren, ca. 1.300 addetti e 309 M€ di fatturato di gruppo nel 2023, sedi in 8 paesi europei; aumento di capitale 2025 sottoscritto da Kartesia); il gedelegeerd bestuurder iscritto in KBO è la persona giuridica P. Van de Velde NV.</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Carl Mourisse</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Bestuurder</t>
-        </is>
-      </c>
+          <t>Fatturato 23.056.460 € - 36,1 FTE (fonte fincheck.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0407.977.446. Grossista/distributore di articoli di carta e cartone e materiali d'imballaggio (NACE commercio all'ingrosso di carta e cartone), sede Aarschotsesteenweg 114, 3012 Wilsele-Leuven. Fondata il 18-01-1971. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. LEGAME DI GRUPPO: appartiene al gruppo britannico Bunzl.</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="3" t="inlineStr"/>
       <c r="F49" s="3" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>info.lichtervelde@vandeveldepackaging.com</t>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>https://www.vandeveldepackaging.com</t>
+          <t>https://www.variapack.com</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Lichtervelde, Provincia di Fiandre Occidentali (Fiandre)</t>
+          <t>Wilsele (Leuven), Provincia del Brabante Fiammingo (Fiandre)</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>https://fincheck.be/en/van-de-velde-packaging/0444.255.050/Lichtervelde/overview</t>
+          <t>https://fincheck.be/nl/varia-pack/0407.977.446/Leuven/overzicht</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Varia-Pack NV</t>
+          <t>Belmoca NV</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — commercio imballaggi carta</t>
+          <t>Caffè — capsule e private label</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 23.056.460 € - 36,1 FTE (fonte fincheck.be / companyweb.be, ultimo bilancio depositato NBB). N. impresa BE 0407.977.446. Grossista/distributore di articoli di carta e cartone e materiali d'imballaggio (NACE commercio all'ingrosso di carta e cartone), sede Aarschotsesteenweg 114, 3012 Wilsele-Leuven. Fondata il 18-01-1971. SOPRA il target 10-20 M€ ma dentro la fascia tollerabile 5-40 M€. LEGAME DI GRUPPO: appartiene al gruppo britannico Bunzl.</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr"/>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato € 13.137.013 (ultimo bilancio depositato NBB; fonte trendstop, 19ª nel settore 'koffie en thee'). Impresa BE 0842.626.627. Sede: Weversstraat 24, 1840 Londerzeel. Produttore di capsule di caffè compatibili (marchio proprio Belmio, lanciato nel 2016) e private label per terzi: acquista e immette caffè sul mercato UE = operatore EUDR. Fatturato in pieno target 10-20 M€. Altro dirigente pubblicato: Alain Adler, Managing Director. Contatto pubblicato sul sito: contact@belmoca.com, tel. 052 73 08 20; sede operativa Weversstraat 24 / Technologielaan 7B, 1840 Londerzeel.</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Bruno van Den Branden</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/belmoca---belmio</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>contact@belmoca.com</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>https://www.variapack.com</t>
+          <t>https://belmoca.com/</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Wilsele (Leuven), Provincia del Brabante Fiammingo (Fiandre)</t>
+          <t>Londerzeel (Fiandre, prov. Vlaams-Brabant)</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>https://fincheck.be/nl/varia-pack/0407.977.446/Leuven/overzicht</t>
+          <t>https://trendstop.knack.be/nl/detail/842626627/belmoca.aspx</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Belmoca NV</t>
+          <t>Cafés Delahaut SRL</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Caffè — capsule e private label</t>
+          <t>Caffè — torrefazione</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Fatturato € 13.137.013 (ultimo bilancio depositato NBB; fonte trendstop, 19ª nel settore 'koffie en thee'). Impresa BE 0842.626.627. Sede: Weversstraat 24, 1840 Londerzeel. Produttore di capsule di caffè compatibili (marchio proprio Belmio, lanciato nel 2016) e private label per terzi: acquista e immette caffè sul mercato UE = operatore EUDR. Fatturato in pieno target 10-20 M€. Altro dirigente pubblicato: Alain Adler, Managing Director. Contatto pubblicato sul sito: contact@belmoca.com, tel. 052 73 08 20; sede operativa Weversstraat 24 / Technologielaan 7B, 1840 Londerzeel.</t>
+          <t>Impresa BE 0418.920.135. Sede: 5020 Namur (Rhisnes), attività a Suarlée; negozio storico Rue de l'Ange 21, 5000 Namur. Tel. +32 81 22 11 58. Margine lordo € 1.648.475 e 22,3 FTE (ultimo bilancio depositato NBB, deposito 02-09-2025; fonte trendstop, 25ª nel settore 'koffie en thee'); NON pubblica il fatturato (schema abbreviato). TAGLIA DA VERIFICARE: in un'intervista del 2022 (Degroof Petercam) il fatturato è indicato intorno ai 5 M€ = soglia minima tollerabile, quindi sotto il target ideale 10-20 M€. Torrefazione familiare dal 1864, importa anche tè artigianali: acquista caffè verde e lo immette sul mercato UE = operatore EUDR. François Delahaut è membro del CdA della federazione Koffiecafé; il fratello Frédéric Delahaut è co-gestore. Unico record vallone della filiera caffè.</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Bruno van Den Branden</t>
+          <t>François Delahaut</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/belmoca---belmio</t>
-        </is>
-      </c>
+          <t>Dirigente (4ª generazione)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>contact@belmoca.com</t>
+          <t>info@cafesdelahaut.be</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>https://belmoca.com/</t>
+          <t>https://www.cafesdelahaut.be/</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Londerzeel (Fiandre, prov. Vlaams-Brabant)</t>
+          <t>Rhisnes-Suarlée / Namur (Vallonia, prov. Namur)</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/842626627/belmoca.aspx</t>
+          <t>https://trendstop.levif.be/fr/detail/418920135/cafes-delahaut.aspx</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Cafés Delahaut SRL</t>
+          <t>Koffie St.-Michel NV</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione</t>
+          <t>Caffè — torrefazione e private label</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Impresa BE 0418.920.135. Sede: 5020 Namur (Rhisnes), attività a Suarlée; negozio storico Rue de l'Ange 21, 5000 Namur. Tel. +32 81 22 11 58. Margine lordo € 1.648.475 e 22,3 FTE (ultimo bilancio depositato NBB, deposito 02-09-2025; fonte trendstop, 25ª nel settore 'koffie en thee'); NON pubblica il fatturato (schema abbreviato). TAGLIA DA VERIFICARE: in un'intervista del 2022 (Degroof Petercam) il fatturato è indicato intorno ai 5 M€ = soglia minima tollerabile, quindi sotto il target ideale 10-20 M€. Torrefazione familiare dal 1864, importa anche tè artigianali: acquista caffè verde e lo immette sul mercato UE = operatore EUDR. François Delahaut è membro del CdA della federazione Koffiecafé; il fratello Frédéric Delahaut è co-gestore. Unico record vallone della filiera caffè.</t>
+          <t>Impresa BE 0406.919.552, fondata nel 1880. Sede: Asiadok 28A, 2030 Antwerpen (porto di Anversa). Margine lordo € 686.005 e 43ª posizione nel settore 'koffie en thee' (trendstop); NON pubblica il fatturato nell'ultimo bilancio depositato (schema abbreviato NBB → ricavi presumibilmente sotto la soglia delle piccole società, ~11 M€): TAGLIA DA VERIFICARE, possibile sotto i 5 M€. Torrefazione familiare, indicata come la più antica e la più grande di Anversa (fornisce ~60% del mercato locale) e private-label roaster per marchi terzi. Contatto alternativo pubblicato: stmichel@skynet.be. Tel. 03 234 34 70.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>François Delahaut</t>
+          <t>Hendrik Hanssens</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Dirigente (4ª generazione)</t>
+          <t>Bedrijfsleider (5ª generazione)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>info@cafesdelahaut.be</t>
+          <t>info@stmichel.be</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>https://www.cafesdelahaut.be/</t>
+          <t>https://stmichel.be/</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Rhisnes-Suarlée / Namur (Vallonia, prov. Namur)</t>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/418920135/cafes-delahaut.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/406919552/koffie-st-michel.aspx</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Koffie St.-Michel NV</t>
+          <t>Mokafina NV</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione e private label</t>
+          <t>Caffè — torrefazione</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Impresa BE 0406.919.552, fondata nel 1880. Sede: Asiadok 28A, 2030 Antwerpen (porto di Anversa). Margine lordo € 686.005 e 43ª posizione nel settore 'koffie en thee' (trendstop); NON pubblica il fatturato nell'ultimo bilancio depositato (schema abbreviato NBB → ricavi presumibilmente sotto la soglia delle piccole società, ~11 M€): TAGLIA DA VERIFICARE, possibile sotto i 5 M€. Torrefazione familiare, indicata come la più antica e la più grande di Anversa (fornisce ~60% del mercato locale) e private-label roaster per marchi terzi. Contatto alternativo pubblicato: stmichel@skynet.be. Tel. 03 234 34 70.</t>
+          <t>Fatturato € 7.967.731 e 11,9 FTE (ultimo bilancio depositato NBB, deposito 27-06-2024; fonte trendstop, 21ª nel settore 'koffie en thee'). Impresa BE 0443.804.001. Sede: Simon De Heuvellaan 2, 2110 Wijnegem. Tel. +32 3 353 10 80. Torrefazione familiare dal 1955 (Mokafina Coffee Roasters), vendita a horeca, retail e B2B. SOTTO IL TARGET IDEALE (8,0 M€, entro il minimo tollerabile di 5 M€). Altri amministratori pubblicati: Olivier Loots, Sofie Verboven. Torrefattore = acquista caffè verde e lo immette sul mercato UE, operatore EUDR.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Hendrik Hanssens</t>
+          <t>Anthony Loots</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Bedrijfsleider (5ª generazione)</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr"/>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/mokafina</t>
+        </is>
+      </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>info@stmichel.be</t>
+          <t>info@mokafina.be</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>https://stmichel.be/</t>
+          <t>https://mokafina.be/</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+          <t>Wijnegem (Fiandre, prov. Antwerpen)</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/406919552/koffie-st-michel.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/443804001/mokafina.aspx</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Mokafina NV</t>
+          <t>Rucquoy Frères NV</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione</t>
+          <t>Caffè — import caffè verde</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Fatturato € 7.967.731 e 11,9 FTE (ultimo bilancio depositato NBB, deposito 27-06-2024; fonte trendstop, 21ª nel settore 'koffie en thee'). Impresa BE 0443.804.001. Sede: Simon De Heuvellaan 2, 2110 Wijnegem. Tel. +32 3 353 10 80. Torrefazione familiare dal 1955 (Mokafina Coffee Roasters), vendita a horeca, retail e B2B. SOTTO IL TARGET IDEALE (8,0 M€, entro il minimo tollerabile di 5 M€). Altri amministratori pubblicati: Olivier Loots, Sofie Verboven. Torrefattore = acquista caffè verde e lo immette sul mercato UE, operatore EUDR.</t>
+          <t>Fatturato € 17.021.444 (ultimo bilancio depositato NBB, deposito 04-06-2025; fonte companyweb/trendstop). Impresa BE 0404.850.383. Sede: Van Meterenkaai 4 bus 14, 2000 Antwerpen (sede sociale registrata anche a Brasschaat). Azienda familiare dal 1919, import/export di caffè verde. TARGET IDEALE: importatore = operatore EUDR in senso stretto, fatturato in pieno range.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Anthony Loots</t>
+          <t>Steven De Punt</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -30876,49 +30876,49 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/mokafina</t>
+          <t>https://be.linkedin.com/company/rucquoy-fr%C3%A8res</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>info@mokafina.be</t>
+          <t>trade@rucquoy.com</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>https://mokafina.be/</t>
+          <t>https://rucquoy.com/</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Wijnegem (Fiandre, prov. Antwerpen)</t>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/443804001/mokafina.aspx</t>
+          <t>https://www.companyweb.be/en/0404850383/rucquoy-freres</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Rucquoy Frères NV</t>
+          <t>Sas NV (Sas Coffee)</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Caffè — import caffè verde</t>
+          <t>Caffè — torrefazione e private label</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Fatturato € 17.021.444 (ultimo bilancio depositato NBB, deposito 04-06-2025; fonte companyweb/trendstop). Impresa BE 0404.850.383. Sede: Van Meterenkaai 4 bus 14, 2000 Antwerpen (sede sociale registrata anche a Brasschaat). Azienda familiare dal 1919, import/export di caffè verde. TARGET IDEALE: importatore = operatore EUDR in senso stretto, fatturato in pieno range.</t>
+          <t>Fatturato € 37.126.839 (ultimo bilancio depositato NBB; fonte trendstop, 14ª nel settore 'koffie en thee'). Impresa BE 0404.190.783. Sede: Dennenlaan 10, 2340 Beerse. Azienda familiare dal 1947, torrefazione + confezionamento private label; fatturato triplicato in 10 anni. BORDERLINE ALTO: 37 M€, entro il range tollerabile (max 40) ma sopra il target ideale 10-20 M€. Torrefattore = importa/immette caffè sul mercato UE, operatore EUDR. ATTENZIONE PROPRIETÀ: non è più un'azienda familiare indipendente — Miko NV ha acquisito Sas nel novembre 2021 (11,4 M€) e l'ha rivenduta il 24-05-2024 al fondo olandese Nimbus Investments (12 M€, svalutazione di 20 M€ per Miko). Il referente indicato (Herman Sas, famiglia fondatrice) risale al periodo pre-cessione: DA RIVERIFICARE prima del contatto; nessun nuovo amministratore delegato risulta pubblicato dopo il 2024. Dirigente pubblicato su LinkedIn: Dominic Sas, Director Sales &amp; Marketing.</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Steven De Punt</t>
+          <t>Herman Sas</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -30926,324 +30926,312 @@
           <t>Gedelegeerd bestuurder</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/rucquoy-fr%C3%A8res</t>
-        </is>
-      </c>
+      <c r="F55" s="3" t="inlineStr"/>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>trade@rucquoy.com</t>
+          <t>info@sas-koffie.be</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>https://rucquoy.com/</t>
+          <t>https://sas-coffee.com/</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+          <t>Beerse (Fiandre, prov. Antwerpen)</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0404850383/rucquoy-freres</t>
+          <t>https://trendstop.knack.be/nl/detail/404190783/sas.aspx</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Sas NV (Sas Coffee)</t>
+          <t>Silco NV</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione e private label</t>
+          <t>Caffè — commercio caffè verde</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Fatturato € 37.126.839 (ultimo bilancio depositato NBB; fonte trendstop, 14ª nel settore 'koffie en thee'). Impresa BE 0404.190.783. Sede: Dennenlaan 10, 2340 Beerse. Azienda familiare dal 1947, torrefazione + confezionamento private label; fatturato triplicato in 10 anni. BORDERLINE ALTO: 37 M€, entro il range tollerabile (max 40) ma sopra il target ideale 10-20 M€. Torrefattore = importa/immette caffè sul mercato UE, operatore EUDR. ATTENZIONE PROPRIETÀ: non è più un'azienda familiare indipendente — Miko NV ha acquisito Sas nel novembre 2021 (11,4 M€) e l'ha rivenduta il 24-05-2024 al fondo olandese Nimbus Investments (12 M€, svalutazione di 20 M€ per Miko). Il referente indicato (Herman Sas, famiglia fondatrice) risale al periodo pre-cessione: DA RIVERIFICARE prima del contatto; nessun nuovo amministratore delegato risulta pubblicato dopo il 2024. Dirigente pubblicato su LinkedIn: Dominic Sas, Director Sales &amp; Marketing.</t>
+          <t>Fatturato € 8.358.215 (ultimo bilancio depositato NBB, deposito 14-06-2024; fonte trendstop, 23ª nel settore 'koffie en thee'). Impresa BE 0715.792.692. Sede: Italiëlei 181, 2000 Antwerpen. Attività principale: groothandel in koffie, thee, cacao en specerijen (NACE 46370). SOTTO IL TARGET IDEALE (8,4 M€, entro il minimo tollerabile) e struttura molto snella (1 FTE dichiarato): tipica trading house di caffè verde. Da verificare la sostanza operativa prima del contatto. Amministratori pubblicati: Philip Van Gestel e Katrien Delaet (fonte northdata/fincheck su dati KBO). Attenzione: fincheck riporta per lo stesso bilancio un fatturato di € 4.843.986 (sotto la soglia minima) contro gli € 8.358.215 di trendstop: cifra da verificare sul deposito NBB. Fondata il 13-12-2018.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Herman Sas</t>
+          <t>Philip Van Gestel e Katrien Delaet</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Gedelegeerd bestuurder</t>
+          <t>Bestuurders</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>info@sas-koffie.be</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>https://sas-coffee.com/</t>
-        </is>
-      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Beerse (Fiandre, prov. Antwerpen)</t>
+          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/404190783/sas.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/715792692/silco.aspx</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Silco NV</t>
+          <t>The Java Coffee Company NV</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Caffè — commercio caffè verde</t>
+          <t>Caffè — torrefazione</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Fatturato € 8.358.215 (ultimo bilancio depositato NBB, deposito 14-06-2024; fonte trendstop, 23ª nel settore 'koffie en thee'). Impresa BE 0715.792.692. Sede: Italiëlei 181, 2000 Antwerpen. Attività principale: groothandel in koffie, thee, cacao en specerijen (NACE 46370). SOTTO IL TARGET IDEALE (8,4 M€, entro il minimo tollerabile) e struttura molto snella (1 FTE dichiarato): tipica trading house di caffè verde. Da verificare la sostanza operativa prima del contatto. Amministratori pubblicati: Philip Van Gestel e Katrien Delaet (fonte northdata/fincheck su dati KBO). Attenzione: fincheck riporta per lo stesso bilancio un fatturato di € 4.843.986 (sotto la soglia minima) contro gli € 8.358.215 di trendstop: cifra da verificare sul deposito NBB. Fondata il 13-12-2018.</t>
+          <t>Fatturato € 12.321.215 (ultimo bilancio depositato NBB; fonte companyweb) e 27,5 FTE; 16ª nel settore 'koffie en thee' per margine lordo (€ 2.726.684, trendstop). Impresa BE 0406.874.220, fondata 29-09-1969 (attività di torrefazione dal 1935). Sede: Wingepark 20, 3110 Rotselaar. Tel. +32 16 30 04 00. Torrefazione familiare Claes di 4ª generazione, CO2-neutrale: acquista caffè verde e lo immette sul mercato UE = operatore EUDR. Fatturato in pieno target 10-20 M€. Wim Claes (3ª gen.) resta amministratore ed è nel CdA della federazione Koffiecafé.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Philip Van Gestel e Katrien Delaet</t>
+          <t>Kathleen Claes</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Bestuurders</t>
-        </is>
-      </c>
-      <c r="F57" s="3" t="inlineStr"/>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
+          <t>CEO (4ª generazione)</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/the-java-coffee-company</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>info@javacoffee.be</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.javacoffee.be/</t>
+        </is>
+      </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Anversa / Antwerpen (Fiandre, prov. Antwerpen)</t>
+          <t>Rotselaar (Fiandre, prov. Vlaams-Brabant)</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/715792692/silco.aspx</t>
+          <t>https://www.companyweb.be/en/0406874220/the-java-coffee-company</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>The Java Coffee Company NV</t>
+          <t>coffeeRoots NV</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione</t>
+          <t>Caffè — torrefazione private label</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Fatturato € 12.321.215 (ultimo bilancio depositato NBB; fonte companyweb) e 27,5 FTE; 16ª nel settore 'koffie en thee' per margine lordo (€ 2.726.684, trendstop). Impresa BE 0406.874.220, fondata 29-09-1969 (attività di torrefazione dal 1935). Sede: Wingepark 20, 3110 Rotselaar. Tel. +32 16 30 04 00. Torrefazione familiare Claes di 4ª generazione, CO2-neutrale: acquista caffè verde e lo immette sul mercato UE = operatore EUDR. Fatturato in pieno target 10-20 M€. Wim Claes (3ª gen.) resta amministratore ed è nel CdA della federazione Koffiecafé.</t>
+          <t>Fatturato € 12.585.973 (ultimo bilancio depositato NBB, deposito 24-07-2024; fonte companyweb). Impresa BE 0429.473.636. Sede sociale: Breeveldse Masten 5, 2970 Schilde; stabilimento di torrefazione a Kruibeke (capannone di 5.000 m² dal 2016). Gruppo coffeeRoots Cantata: torrefazione private label per partner in oltre 30 paesi + retail (marchio Cantata, ~350 punti vendita in 6 paesi). Radici nel 1907 ad Anversa ('t Koffiemoleken / De Verenigde Koffiebranders). Acquista caffè verde e lo trasforma = operatore EUDR. Fatturato in pieno target 10-20 M€. Co-guida citata nelle fonti: Camille Willems. E-mail non pubblicata in fonti verificabili: contatto via modulo su coffeeroots.com/contact-us. Contatto commerciale pubblicato: sales@coffeeroots.com, tel. +32 3 253 18 00 (sito coffeeroots.com/contact-us; ripreso da D&amp;B/RocketReach): verificare prima dell'invio. Sede produttiva: Kasteleinsstraat 19, 9150 Kruibeke.</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Kathleen Claes</t>
+          <t>Chantal Hoorens</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>CEO (4ª generazione)</t>
+          <t>Bedrijfsleider (CEO, famiglia Hoorens)</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/the-java-coffee-company</t>
+          <t>https://fr.linkedin.com/company/coffeeroots</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>info@javacoffee.be</t>
+          <t>sales@coffeeroots.com</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>https://www.javacoffee.be/</t>
+          <t>https://www.coffeeroots.com/</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Rotselaar (Fiandre, prov. Vlaams-Brabant)</t>
+          <t>Schilde (sede sociale) / Kruibeke (torrefazione) (Fiandre, prov. Antwerpen e Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0406874220/the-java-coffee-company</t>
+          <t>https://www.companyweb.be/en/0429473636/coffee-roots</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>coffeeRoots NV</t>
+          <t>A &amp; A Chocolaterie NV</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione private label</t>
+          <t>Cacao/Cioccolato — figure stagionali e tavolette</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Fatturato € 12.585.973 (ultimo bilancio depositato NBB, deposito 24-07-2024; fonte companyweb). Impresa BE 0429.473.636. Sede sociale: Breeveldse Masten 5, 2970 Schilde; stabilimento di torrefazione a Kruibeke (capannone di 5.000 m² dal 2016). Gruppo coffeeRoots Cantata: torrefazione private label per partner in oltre 30 paesi + retail (marchio Cantata, ~350 punti vendita in 6 paesi). Radici nel 1907 ad Anversa ('t Koffiemoleken / De Verenigde Koffiebranders). Acquista caffè verde e lo trasforma = operatore EUDR. Fatturato in pieno target 10-20 M€. Co-guida citata nelle fonti: Camille Willems. E-mail non pubblicata in fonti verificabili: contatto via modulo su coffeeroots.com/contact-us. Contatto commerciale pubblicato: sales@coffeeroots.com, tel. +32 3 253 18 00 (sito coffeeroots.com/contact-us; ripreso da D&amp;B/RocketReach): verificare prima dell'invio. Sede produttiva: Kasteleinsstraat 19, 9150 Kruibeke.</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Chantal Hoorens</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Bedrijfsleider (CEO, famiglia Hoorens)</t>
-        </is>
-      </c>
+          <t>Fatturato 22.087.972 € (ultimo bilancio depositato NBB, deposito 22-10-2025; 25.604.502 € e 31° posto di settore su trendstop.knack.be). N. impresa BE 0892.388.320. Sede Mosten 16, 9160 Lokeren; lavora ~15 t di cioccolato al giorno. Nella parte alta del target ma dentro il range. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), insieme alla consociata Pralinart NV.</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr"/>
+      <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/company/coffeeroots</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>sales@coffeeroots.com</t>
+          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>https://www.coffeeroots.com/</t>
+          <t>https://www.hamlet.be/</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Schilde (sede sociale) / Kruibeke (torrefazione) (Fiandre, prov. Antwerpen e Oost-Vlaanderen)</t>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0429473636/coffee-roots</t>
+          <t>https://www.companyweb.be/en/0892388320/a-a-chocolaterie</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>A &amp; A Chocolaterie NV</t>
+          <t>Belvas SA</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — figure stagionali e tavolette</t>
+          <t>Cacao/Cioccolato — praline bio equosolidali</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 22.087.972 € (ultimo bilancio depositato NBB, deposito 22-10-2025; 25.604.502 € e 31° posto di settore su trendstop.knack.be). N. impresa BE 0892.388.320. Sede Mosten 16, 9160 Lokeren; lavora ~15 t di cioccolato al giorno. Nella parte alta del target ma dentro il range. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), insieme alla consociata Pralinart NV.</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr"/>
-      <c r="E60" s="5" t="inlineStr"/>
-      <c r="F60" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato 10.258.810 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0472.516.692. Cioccolateria industriale bio e Fairtrade: importa fave/semilavorati di cacao certificati — operatore EUDR. Perfettamente in target 10-20 M€.</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Thierry Noesen</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Fondatore / Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>info@belvas.be</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>https://www.hamlet.be/</t>
+          <t>https://www.chocolaterie-belvas.be/</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+          <t>Ghislenghien / Meslin-l'Évêque (Ath), Hainaut — Vallonia</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0892388320/a-a-chocolaterie</t>
+          <t>https://www.pappers.be/fr/company/belvas-0472516692</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Belvas SA</t>
+          <t>Bruyerre Chocolates SA</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline bio equosolidali</t>
+          <t>Cacao/Cioccolato — praline</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 10.258.810 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0472.516.692. Cioccolateria industriale bio e Fairtrade: importa fave/semilavorati di cacao certificati — operatore EUDR. Perfettamente in target 10-20 M€.</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>Thierry Noesen</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>Fondatore / Administrateur délégué</t>
-        </is>
-      </c>
+          <t>Fatturato 6.140.610 € (fonte: trendstop.levif.be, ultimo bilancio depositato NBB). N. impresa BE 0688.794.525. Cioccolatiere dal 1909, oltre 80 varietà di praline. Sotto la fascia ottimale ma nel range tollerabile 5-40 M€. Legame di gruppo: entità distinta da Bruyerre SA (BE 0431.703.151, distribuzione alimentare, ~179,6 M€ — quest'ultima fuori target).</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
       <c r="F61" s="3" t="inlineStr"/>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>info@belvas.be</t>
+          <t>contact@bruyerre.eu</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>https://www.chocolaterie-belvas.be/</t>
+          <t>https://bruyerre.eu/</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Ghislenghien / Meslin-l'Évêque (Ath), Hainaut — Vallonia</t>
+          <t>Gosselies (Charleroi), Hainaut — Vallonia</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/fr/company/belvas-0472516692</t>
+          <t>https://trendstop.levif.be/fr/detail/688794525/bruyerre-chocolates.aspx</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Bruyerre Chocolates SA</t>
+          <t>Chocolaterie Ickx NV</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -31253,140 +31241,148 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 6.140.610 € (fonte: trendstop.levif.be, ultimo bilancio depositato NBB). N. impresa BE 0688.794.525. Cioccolatiere dal 1909, oltre 80 varietà di praline. Sotto la fascia ottimale ma nel range tollerabile 5-40 M€. Legame di gruppo: entità distinta da Bruyerre SA (BE 0431.703.151, distribuzione alimentare, ~179,6 M€ — quest'ultima fuori target).</t>
+          <t>Fatturato 32.746.626 € e 139,7 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-03-2026). N. impresa BE 0421.359.189. Fondata 1981; forte export (Cina, Asia). Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI indipendente.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr"/>
       <c r="E62" s="5" t="inlineStr"/>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/chocolaterie-ickx</t>
+        </is>
+      </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>contact@bruyerre.eu</t>
+          <t>avangastel@choc-ickx.be</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>https://bruyerre.eu/</t>
+          <t>https://www.ickx.be/</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Gosselies (Charleroi), Hainaut — Vallonia</t>
+          <t>Essen (Anversa) — Fiandre</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/688794525/bruyerre-chocolates.aspx</t>
+          <t>https://www.companyweb.be/en/0421359189/chocolaterie-ickx</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Chocolaterie Ickx NV</t>
+          <t>Confiserie De Bie - L'Abeille - Trefin NV</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline</t>
+          <t>Cacao/Cioccolato — cioccolato e confetteria</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 32.746.626 € e 139,7 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-03-2026). N. impresa BE 0421.359.189. Fondata 1981; forte export (Cina, Asia). Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI indipendente.</t>
+          <t>Fatturato 11.404.101 € e 34,4 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 08-06-2026). N. impresa BE 0400.120.050. Sede Waaslandlaan 5, 9160 Lokeren. Produttore di cioccolato e caramelle (marchio Trefin). In pieno target 10-20 M€.</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr"/>
       <c r="E63" s="3" t="inlineStr"/>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/chocolaterie-ickx</t>
-        </is>
-      </c>
+      <c r="F63" s="3" t="inlineStr"/>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>avangastel@choc-ickx.be</t>
+          <t>info@trefin.com</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>https://www.ickx.be/</t>
+          <t>https://www.trefin.com/</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Essen (Anversa) — Fiandre</t>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0421359189/chocolaterie-ickx</t>
+          <t>https://www.companyweb.be/en/0400120050/confiserie-de-bie-l-abeille-trefin</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Confiserie De Bie - L'Abeille - Trefin NV</t>
+          <t>Corné Port-Royal Chocolatier SA</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — cioccolato e confetteria</t>
+          <t>Cacao/Cioccolato — praline artigianali</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 11.404.101 € e 34,4 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 08-06-2026). N. impresa BE 0400.120.050. Sede Waaslandlaan 5, 9160 Lokeren. Produttore di cioccolato e caramelle (marchio Trefin). In pieno target 10-20 M€.</t>
+          <t>Fatturato 8.796.906 € (ultimo bilancio depositato NBB, deposito 26-06-2025; 8.421.952 € e 54° posto di settore su trendstop.knack.be). N. impresa BE 0433.283.558. Sede Avenue Vésale 12, 1300 Wavre; maison storica (marchio dal 1932), rete di ~20 boutique in Belgio e 15 in Francia. Sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr"/>
       <c r="E64" s="5" t="inlineStr"/>
-      <c r="F64" s="5" t="inlineStr"/>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>info@trefin.com</t>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/corn-port-royal</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>https://www.trefin.com/</t>
+          <t>https://www.corneportroyal.com/</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+          <t>Wavre (Brabant wallon) — Vallonia</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0400120050/confiserie-de-bie-l-abeille-trefin</t>
+          <t>https://www.companyweb.be/en/0433283558/corne-port-royal-chocolatier</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Corné Port-Royal Chocolatier SA</t>
+          <t>Delafaille NV</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline artigianali</t>
+          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 8.796.906 € (ultimo bilancio depositato NBB, deposito 26-06-2025; 8.421.952 € e 54° posto di settore su trendstop.knack.be). N. impresa BE 0433.283.558. Sede Avenue Vésale 12, 1300 Wavre; maison storica (marchio dal 1932), rete di ~20 boutique in Belgio e 15 in Francia. Sotto la fascia ottimale ma dentro il range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr"/>
-      <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/corn-port-royal</t>
-        </is>
-      </c>
+          <t>Fatturato 14.244.468 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB, deposito 17-06-2025); 43° nel settore cioccolato e dolciumi. N. impresa BE 0467.502.683. In pieno target 10-20 M€. Legame di gruppo: acquisita dallo svizzero Maestrani Schweizer Schokoladen (con la controllata Ostrapack); resta però PMI belga autonoma con obblighi EUDR propri.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Paul Daems</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>CEO / gedelegeerd bestuurder (uscente, transizione dopo l'acquisizione Maestrani 2025)</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr"/>
       <c r="G65" s="3" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31394,47 +31390,43 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>https://www.corneportroyal.com/</t>
+          <t>https://www.delafaille.be/</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Wavre (Brabant wallon) — Vallonia</t>
+          <t>Melsele, Beveren-Kruibeke-Zwijndrecht (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0433283558/corne-port-royal-chocolatier</t>
+          <t>https://trendstop.knack.be/nl/detail/467502683/delafaille.aspx</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Delafaille NV</t>
+          <t>Dolfin SA</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
+          <t>Cacao/Cioccolato — tavolette premium</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 14.244.468 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB, deposito 17-06-2025); 43° nel settore cioccolato e dolciumi. N. impresa BE 0467.502.683. In pieno target 10-20 M€. Legame di gruppo: acquisita dallo svizzero Maestrani Schweizer Schokoladen (con la controllata Ostrapack); resta però PMI belga autonoma con obblighi EUDR propri.</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>Paul Daems</t>
-        </is>
-      </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>CEO / gedelegeerd bestuurder (uscente, transizione dopo l'acquisizione Maestrani 2025)</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr"/>
+          <t>33,2 FTE da ultimo bilancio depositato NBB (deposito 20-01-2026, cifra d'affari non pubblicata); fatturato ~6 M€ secondo la stampa economica (L'Avenir/RTBF, ~385 t di cioccolato/anno). N. impresa BE 0437.332.220. Sede Avenue Robert Schuman 172, 1401 Baulers (Nivelles). Prima cioccolateria belga certificata carbon neutral (2008); programma di sostenibilità cacao proprio 'Cocoa Act 4'. Taglia sotto la fascia ottimale, nel range tollerabile 5-40 M€.</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr"/>
+      <c r="E66" s="5" t="inlineStr"/>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/dolfin-sa</t>
+        </is>
+      </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31442,311 +31434,311 @@
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>https://www.delafaille.be/</t>
+          <t>https://www.dolfin.be/</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Melsele, Beveren-Kruibeke-Zwijndrecht (Oost-Vlaanderen) — Fiandre</t>
+          <t>Baulers, Nivelles (Brabant wallon) — Vallonia</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/467502683/delafaille.aspx</t>
+          <t>https://www.companyweb.be/en/0437332220/dolfin</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Dolfin SA</t>
+          <t>Gudrun Commercial NV</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — tavolette premium</t>
+          <t>Cacao/Cioccolato — praline e tartufi</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>33,2 FTE da ultimo bilancio depositato NBB (deposito 20-01-2026, cifra d'affari non pubblicata); fatturato ~6 M€ secondo la stampa economica (L'Avenir/RTBF, ~385 t di cioccolato/anno). N. impresa BE 0437.332.220. Sede Avenue Robert Schuman 172, 1401 Baulers (Nivelles). Prima cioccolateria belga certificata carbon neutral (2008); programma di sostenibilità cacao proprio 'Cocoa Act 4'. Taglia sotto la fascia ottimale, nel range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr"/>
-      <c r="E67" s="3" t="inlineStr"/>
+          <t>Fatturato 43.457.280 € e 138,6 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 15-07-2026). N. impresa BE 0476.530.118. Sede Industriestraat 18, 2500 Lier. Firmataria di Beyond Chocolate. AZIENDA DI CONFINE: fatturato sopra la fascia tollerabile 5-40 M€ (ma sotto la soglia di esclusione ~50 M€). Legame di gruppo: acquisita dal gruppo spagnolo Natra (che controlla anche Natra Chocolate Belgium NV, ~93 M€, fuori target).</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Sofie De Lathouwer</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/dolfin-sa</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>https://be.linkedin.com/company/gudrun-commercial-nv</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>info@chocolates.be</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>https://www.dolfin.be/</t>
+          <t>https://gudrungroup.be/</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Baulers, Nivelles (Brabant wallon) — Vallonia</t>
+          <t>Lier (Anversa) — Fiandre</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0437332220/dolfin</t>
+          <t>https://www.companyweb.be/en/0476530118/gudrun-commercial</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Gudrun Commercial NV</t>
+          <t>La Chocolaterie Galler SA</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e tartufi</t>
+          <t>Cacao/Cioccolato — tavolette e praline</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 43.457.280 € e 138,6 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 15-07-2026). N. impresa BE 0476.530.118. Sede Industriestraat 18, 2500 Lier. Firmataria di Beyond Chocolate. AZIENDA DI CONFINE: fatturato sopra la fascia tollerabile 5-40 M€ (ma sotto la soglia di esclusione ~50 M€). Legame di gruppo: acquisita dal gruppo spagnolo Natra (che controlla anche Natra Chocolate Belgium NV, ~93 M€, fuori target).</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>Sofie De Lathouwer</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/gudrun-commercial-nv</t>
-        </is>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>info@chocolates.be</t>
+          <t>Fatturato 29.502.986 € (fonte: pappers.be/trendstop, bilancio NBB); dato più recente ~32 M€ con perdita netta 1,7 M€ nel 2024; 194 dipendenti. N. impresa BE 0416.169.689. Azienda di confine nella parte alta del range tollerabile (5-40 M€). Nota: nell'aprile 2026 rilevata da un consorzio vallone con piano di ristrutturazione (~70 licenziamenti su 170).</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>https://gudrungroup.be/</t>
+          <t>https://www.galler.com/</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Lier (Anversa) — Fiandre</t>
+          <t>Vaux-sous-Chèvremont (Chaudfontaine), Liegi — Vallonia</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0476530118/gudrun-commercial</t>
+          <t>https://www.pappers.be/fr/company/la-chocolaterie-galler-0416169689</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>La Chocolaterie Galler SA</t>
+          <t>Libeert NV</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — tavolette e praline</t>
+          <t>Cacao/Cioccolato — figure e tavolette di cioccolato</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 29.502.986 € (fonte: pappers.be/trendstop, bilancio NBB); dato più recente ~32 M€ con perdita netta 1,7 M€ nel 2024; 194 dipendenti. N. impresa BE 0416.169.689. Azienda di confine nella parte alta del range tollerabile (5-40 M€). Nota: nell'aprile 2026 rilevata da un consorzio vallone con piano di ristrutturazione (~70 licenziamenti su 170).</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="3" t="inlineStr"/>
+          <t>Fatturato ~35 M€ e 136,8 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 13-11-2025). N. impresa BE 0407.026.747. Azienda familiare, oltre 5.000 t di cioccolato all'anno, gamma bio. Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Lily Libeert</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Co-directrice (4a generazione della famiglia Libeert)</t>
+        </is>
+      </c>
       <c r="F69" s="3" t="inlineStr"/>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>contact@libeert.com</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>https://www.galler.com/</t>
+          <t>https://www.libeert.com/</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Vaux-sous-Chèvremont (Chaudfontaine), Liegi — Vallonia</t>
+          <t>Comines-Warneton (Komen-Waasten), Hainaut — Vallonia</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/fr/company/la-chocolaterie-galler-0416169689</t>
+          <t>https://www.companyweb.be/en/0407026747/libeert</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Libeert NV</t>
+          <t>Manufacture Belge de Chocolats SRL</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — figure e tavolette di cioccolato</t>
+          <t>Cacao/Cioccolato — praline e private label</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ~35 M€ e 136,8 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 13-11-2025). N. impresa BE 0407.026.747. Azienda familiare, oltre 5.000 t di cioccolato all'anno, gamma bio. Azienda di confine nella parte alta del range tollerabile (5-40 M€), ma resta PMI familiare indipendente.</t>
+          <t>Fatturato 25.731.148 € e 175,1 FTE (fonte: trendstop.levif.be / companyweb.be, ultimo bilancio depositato NBB, deposito 08-07-2025); 30° posto nel settore cioccolato e dolciumi. N. impresa BE 0722.764.519. Firmataria di Beyond Chocolate (impegni su deforestazione e tracciabilità del cacao). Nella parte alta del range tollerabile 5-40 M€.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Lily Libeert</t>
+          <t>Arnaud Verwilghen</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Co-directrice (4a generazione della famiglia Libeert)</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>contact@libeert.com</t>
+          <t>info@mbcchocolates.be</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>https://www.libeert.com/</t>
+          <t>https://www.mbcchocolates.be/</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Comines-Warneton (Komen-Waasten), Hainaut — Vallonia</t>
+          <t>Koekelberg, Bruxelles (1081) — Regione di Bruxelles-Capitale</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0407026747/libeert</t>
+          <t>https://trendstop.levif.be/fr/detail/722764519/manufacture-belge-de-chocolats.aspx</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Manufacture Belge de Chocolats SRL</t>
+          <t>Oxfam Fair Trade CV</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e private label</t>
+          <t>Cacao/Cioccolato — import equosolidale cacao</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 25.731.148 € e 175,1 FTE (fonte: trendstop.levif.be / companyweb.be, ultimo bilancio depositato NBB, deposito 08-07-2025); 30° posto nel settore cioccolato e dolciumi. N. impresa BE 0722.764.519. Firmataria di Beyond Chocolate (impegni su deforestazione e tracciabilità del cacao). Nella parte alta del range tollerabile 5-40 M€.</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>Arnaud Verwilghen</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
+          <t>Fatturato 17.446.343 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB); 81° posto nel settore alimentare/commercio. N. impresa BE 0453.066.016. Importatore equosolidale: acquista cacao (e caffè) direttamente dalle cooperative dei paesi produttori e immette i prodotti sul mercato UE — operatore EUDR in senso stretto. Firmataria di Beyond Chocolate. In pieno target 10-20 M€. Nota: struttura cooperativa legata a Oxfam-Wereldwinkels.</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr"/>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>info@mbcchocolates.be</t>
+          <t>info@oft.be</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>https://www.mbcchocolates.be/</t>
+          <t>https://www.oxfamfairtrade.be/</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Koekelberg, Bruxelles (1081) — Regione di Bruxelles-Capitale</t>
+          <t>Gent (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/722764519/manufacture-belge-de-chocolats.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/453066016/oxfam-fairtrade.aspx</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Oxfam Fair Trade CV</t>
+          <t>Pierre Marcolini Group SA</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — import equosolidale cacao</t>
+          <t>Cacao/Cioccolato — bean-to-bar e praline</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 17.446.343 € (fonte: trendstop.knack.be, ultimo bilancio depositato NBB); 81° posto nel settore alimentare/commercio. N. impresa BE 0453.066.016. Importatore equosolidale: acquista cacao (e caffè) direttamente dalle cooperative dei paesi produttori e immette i prodotti sul mercato UE — operatore EUDR in senso stretto. Firmataria di Beyond Chocolate. In pieno target 10-20 M€. Nota: struttura cooperativa legata a Oxfam-Wereldwinkels.</t>
+          <t>Fatturato 19.300.806 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0461.740.982. Maison bean-to-bar: acquista e importa direttamente fave di cacao dai paesi d'origine (Vietnam, Madagascar, Ecuador, Perù) — operatore EUDR in senso stretto. In pieno target 10-20 M€. Legame di gruppo: entità collegata Pierre Marcolini Belgium SA (BE 0460.046.551, ~11,3 M€, rete retail).</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr"/>
       <c r="E72" s="5" t="inlineStr"/>
       <c r="F72" s="5" t="inlineStr"/>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>info@oft.be</t>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>https://www.oxfamfairtrade.be/</t>
+          <t>https://eu.marcolini.com/</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Gent (Oost-Vlaanderen) — Fiandre</t>
+          <t>Bruxelles (Haren, 1130) — Regione di Bruxelles-Capitale</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/453066016/oxfam-fairtrade.aspx</t>
+          <t>https://www.pappers.be/fr/company/pierre-marcolini-group-0461740982</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Pierre Marcolini Group SA</t>
+          <t>Pralinart NV</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — bean-to-bar e praline</t>
+          <t>Cacao/Cioccolato — praline</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 19.300.806 € (fonte: pappers.be / trendstop, ultimo bilancio depositato NBB). N. impresa BE 0461.740.982. Maison bean-to-bar: acquista e importa direttamente fave di cacao dai paesi d'origine (Vietnam, Madagascar, Ecuador, Perù) — operatore EUDR in senso stretto. In pieno target 10-20 M€. Legame di gruppo: entità collegata Pierre Marcolini Belgium SA (BE 0460.046.551, ~11,3 M€, rete retail).</t>
+          <t>Fatturato 18.427.020 € e 34 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 02-11-2023). N. impresa BE 0450.589.051. Sede Waaslandlaan 32, 9160 Lokeren; fino a 10 t di praline al giorno. In pieno target 10-20 M€. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), consociata di A &amp; A Chocolaterie NV.</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr"/>
       <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
+        </is>
+      </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
           <t>n.d.</t>
@@ -31754,762 +31746,766 @@
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>https://eu.marcolini.com/</t>
+          <t>https://www.hamlet.be/</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Bruxelles (Haren, 1130) — Regione di Bruxelles-Capitale</t>
+          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>https://www.pappers.be/fr/company/pierre-marcolini-group-0461740982</t>
+          <t>https://www.companyweb.be/en/0450589051/pralinart</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Pralinart NV</t>
+          <t>Vandenbulcke Confiserie NV</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline</t>
+          <t>Cacao/Cioccolato — praline e tavolette</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 18.427.020 € e 34 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 02-11-2023). N. impresa BE 0450.589.051. Sede Waaslandlaan 32, 9160 Lokeren; fino a 10 t di praline al giorno. In pieno target 10-20 M€. Legame di gruppo: controllata al 100% da Hamlet (gruppo familiare belga Geltmeyer), consociata di A &amp; A Chocolaterie NV.</t>
+          <t>Fatturato 13.332.120 € e 31,5 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-12-2024). N. impresa BE 0417.738.319. Fondata 1949; export in oltre 50 paesi. In pieno target 10-20 M€.</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr"/>
       <c r="E74" s="5" t="inlineStr"/>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/a&amp;a-chocolaterie-pralin'art</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>https://be.linkedin.com/company/chocolatiervandenbulcke</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>info@vandenbulcke.com</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>https://www.hamlet.be/</t>
+          <t>https://www.vandenbulcke.com/</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Lokeren (Oost-Vlaanderen) — Fiandre</t>
+          <t>Heule, Kortrijk (West-Vlaanderen) — Fiandre</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0450589051/pralinart</t>
+          <t>https://www.companyweb.be/en/0417738319/confiserie-vandenbulcke</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Vandenbulcke Confiserie NV</t>
+          <t>Hannecard Benelux NV</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e tavolette</t>
+          <t>Gomma — rivestimenti in gomma per rulli</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 13.332.120 € e 31,5 FTE (fonte: companyweb.be, ultimo bilancio depositato NBB, deposito 26-12-2024). N. impresa BE 0417.738.319. Fondata 1949; export in oltre 50 paesi. In pieno target 10-20 M€.</t>
+          <t>Fatturato 16.954.714 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 83,3 FTE; n. impresa BE 0694.906.812</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr"/>
       <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/chocolatiervandenbulcke</t>
+          <t>https://www.linkedin.com/company/hannecard-nv</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>info@vandenbulcke.com</t>
+          <t>contact@hannecard.com</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>https://www.vandenbulcke.com/</t>
+          <t>https://www.hannecard.com/</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Heule, Kortrijk (West-Vlaanderen) — Fiandre</t>
+          <t>Ronse / Renaix (Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0417738319/confiserie-vandenbulcke</t>
+          <t>https://trendstop.knack.be/nl/detail/694906812/hannecard-benelux.aspx</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Hannecard Benelux NV</t>
+          <t>Hercorub NV</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Gomma — rivestimenti in gomma per rulli</t>
+          <t>Gomma — rubbercompounds, technische rubberartikelen</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 16.954.714 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 83,3 FTE; n. impresa BE 0694.906.812</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr"/>
-      <c r="E76" s="5" t="inlineStr"/>
+          <t>Fatturato 15.240.806 EUR (Trends Top/NBB, ultimo esercizio pubblicato); ca. 67-95 dipendenti (fonte aziendale); n. impresa BE 0421.767.381</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Patrick Lenaerts</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Afgevaardigd bestuurder (gedelegeerd bestuurder)</t>
+        </is>
+      </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/hannecard-nv</t>
+          <t>https://be.linkedin.com/company/hercorub-nv</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>contact@hannecard.com</t>
+          <t>info@hercorub.com</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>https://www.hannecard.com/</t>
+          <t>https://www.hercorub.be/</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Ronse / Renaix (Oost-Vlaanderen)</t>
+          <t>Lanaken (Limburg, Vlaanderen)</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/694906812/hannecard-benelux.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/421767381/hercorub.aspx</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Hercorub NV</t>
+          <t>Hexpol Compounding BV</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Gomma — rubbercompounds, technische rubberartikelen</t>
+          <t>Gomma — mescole di gomma (rubber compounding)</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 15.240.806 EUR (Trends Top/NBB, ultimo esercizio pubblicato); ca. 67-95 dipendenti (fonte aziendale); n. impresa BE 0421.767.381</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Patrick Lenaerts</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>Afgevaardigd bestuurder (gedelegeerd bestuurder)</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/hercorub-nv</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>info@hercorub.com</t>
+          <t>Fatturato 31.327.285 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0430.105.126</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr"/>
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>https://www.hercorub.be/</t>
+          <t>https://www.hexpol.com/rubber/plant-locations/hexpol-compounding-sprl/</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Lanaken (Limburg, Vlaanderen)</t>
+          <t>Eupen (Liège, Wallonie – Ostbelgien)</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/421767381/hercorub.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/430105126/hexpol-compounding.aspx</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Hexpol Compounding BV</t>
+          <t>Baert Mengvoeders NV</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Gomma — mescole di gomma (rubber compounding)</t>
+          <t>Mangimi/Soia — mangimi composti bovini, suini, pollame</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 31.327.285 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0430.105.126</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr"/>
-      <c r="E78" s="5" t="inlineStr"/>
-      <c r="F78" s="5" t="inlineStr"/>
-      <c r="G78" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato 38.875.690 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti — taglia gonfiata dal costo materia prima; n. impresa BE 0455.400.845</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Eric Baert</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/baert-mengvoeders</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>info@baertmengvoeders.be</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>https://www.hexpol.com/rubber/plant-locations/hexpol-compounding-sprl/</t>
+          <t>https://www.baertmengvoeders.be/</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Eupen (Liège, Wallonie – Ostbelgien)</t>
+          <t>Zele (Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/430105126/hexpol-compounding.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/455400845/baert-mengvoeders.aspx</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Baert Mengvoeders NV</t>
+          <t>Vanrobaeys Granen &amp; Zaden NV</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi composti bovini, suini, pollame</t>
+          <t>Mangimi/Soia — granaglie e semi per mangimi</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 38.875.690 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti — taglia gonfiata dal costo materia prima; n. impresa BE 0455.400.845</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Eric Baert</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>Gedelegeerd bestuurder</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/baert-mengvoeders</t>
-        </is>
-      </c>
+          <t>Fatturato 19.714.376 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti; n. impresa BE 0452.220.037</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>info@baertmengvoeders.be</t>
+          <t>info@vanrobaeysbelgium.com</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>https://www.baertmengvoeders.be/</t>
+          <t>https://www.vanrobaeysbelgium.com/</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Zele (Oost-Vlaanderen)</t>
+          <t>Menen-Rekkem (West-Vlaanderen)</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/455400845/baert-mengvoeders.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/452220037/vanrobaeys-granen-zaden.aspx</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Vanrobaeys Granen &amp; Zaden NV</t>
+          <t>Voeders Debaillie NV</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — granaglie e semi per mangimi</t>
+          <t>Mangimi/Soia — mangimi composti per bestiame</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 19.714.376 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 10-19 dipendenti; n. impresa BE 0452.220.037</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr"/>
-      <c r="E80" s="5" t="inlineStr"/>
-      <c r="F80" s="5" t="inlineStr"/>
+          <t>Fatturato 11.114.628 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0405.174.839</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Philippe Debaillie</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/voeders-debaillie---aliments-debaillie</t>
+        </is>
+      </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>info@vanrobaeysbelgium.com</t>
+          <t>info@debaillie.be</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>https://www.vanrobaeysbelgium.com/</t>
+          <t>https://debaillie.be/</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Menen-Rekkem (West-Vlaanderen)</t>
+          <t>Roeselare (West-Vlaanderen)</t>
         </is>
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/452220037/vanrobaeys-granen-zaden.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/405174839/voeders-debaillie.aspx</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Voeders Debaillie NV</t>
+          <t>Voeders Mellaerts NV</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi composti per bestiame</t>
+          <t>Mangimi/Soia — mangimi e materie prime</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 11.114.628 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0405.174.839</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>Philippe Debaillie</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>Gedelegeerd bestuurder</t>
-        </is>
-      </c>
+          <t>Fatturato 33.531.211 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 11,5 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0455.669.079</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr"/>
+      <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/voeders-debaillie---aliments-debaillie</t>
+          <t>https://be.linkedin.com/company/voeders-mellaerts</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>info@debaillie.be</t>
+          <t>order@voedersmellaerts.eu</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>https://debaillie.be/</t>
+          <t>https://voedersmellaerts.eu/</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Roeselare (West-Vlaanderen)</t>
+          <t>Tielt-Winge (Sint-Joris-Winge, Vlaams-Brabant)</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/405174839/voeders-debaillie.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/455669079/voeders-mellaerts.aspx</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Voeders Mellaerts NV</t>
+          <t>Voeders Scherrens NV</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi e materie prime</t>
+          <t>Mangimi/Soia — mangimi composti su misura</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 33.531.211 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 11,5 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0455.669.079</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr"/>
-      <c r="E82" s="5" t="inlineStr"/>
+          <t>Fatturato 36.374.114 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0421.626.732</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Geert Scherrens</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Gedelegeerd bestuurder</t>
+        </is>
+      </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>https://be.linkedin.com/company/voeders-mellaerts</t>
+          <t>https://be.linkedin.com/company/scherrensvoeders</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>order@voedersmellaerts.eu</t>
+          <t>info@scherrensvoeders.be</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>https://voedersmellaerts.eu/</t>
+          <t>https://www.scherrensvoeders.be/</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Tielt-Winge (Sint-Joris-Winge, Vlaams-Brabant)</t>
+          <t>Wingene (West-Vlaanderen)</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/455669079/voeders-mellaerts.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/421626732/voeders-scherrens.aspx</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Voeders Scherrens NV</t>
+          <t>Vandeputte Oleochemicals SA</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi composti su misura</t>
+          <t>Olio di palma — raffinazione oli vegetali (soia, lino)</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 36.374.114 EUR (Trends Top/NBB, ultimo esercizio pubblicato); n. impresa BE 0421.626.732</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>Geert Scherrens</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>Gedelegeerd bestuurder</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/scherrensvoeders</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>info@scherrensvoeders.be</t>
+          <t>Fatturato 34.266.885 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 18 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0471.546.593</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr"/>
+      <c r="E83" s="3" t="inlineStr"/>
+      <c r="F83" s="3" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>https://www.scherrensvoeders.be/</t>
+          <t>https://www.vandeputte.com/en/oleochemicals/</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Wingene (West-Vlaanderen)</t>
+          <t>Mouscron (Hainaut, Wallonie)</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/421626732/voeders-scherrens.aspx</t>
+          <t>https://trendstop.levif.be/fr/detail/471546593/vandeputte-oleochemicals.aspx</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Vandeputte Oleochemicals SA</t>
+          <t>Baeten &amp; Co NV</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli vegetali (soia, lino)</t>
+          <t>Olio di palma — raffinazione oli e grassi vegetali/animali</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 34.266.885 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 18 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0471.546.593</t>
+          <t>Fatturato 42.810.588 EUR (bilancio NBB depositato 15-07-2025) — taglia gonfiata dal costo materia prima: solo 13,7 FTE; n. impresa BE 0447.081.908</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr"/>
       <c r="E84" s="5" t="inlineStr"/>
       <c r="F84" s="5" t="inlineStr"/>
-      <c r="G84" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>info@baetennv.be</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>https://www.vandeputte.com/en/oleochemicals/</t>
+          <t>https://baetennv.be/</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Mouscron (Hainaut, Wallonie)</t>
+          <t>Berlare (Overmere, Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/471546593/vandeputte-oleochemicals.aspx</t>
+          <t>https://www.companyweb.be/en/0447081908/baeten-co</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Baeten &amp; Co NV</t>
+          <t>Repro NV</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli e grassi vegetali/animali</t>
+          <t>Olio di palma — raffinazione oli e grassi vegetali</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 42.810.588 EUR (bilancio NBB depositato 15-07-2025) — taglia gonfiata dal costo materia prima: solo 13,7 FTE; n. impresa BE 0447.081.908</t>
+          <t>Fatturato 14.157.353 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 1-5 dipendenti (societa' di raffinazione del Group Vandamme); n. impresa BE 0439.000.818</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr"/>
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr"/>
-      <c r="G85" s="4" t="inlineStr">
-        <is>
-          <t>info@baetennv.be</t>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>https://baetennv.be/</t>
+          <t>https://www.groupvandamme.com/</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Berlare (Overmere, Oost-Vlaanderen)</t>
+          <t>Deinze (Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0447081908/baeten-co</t>
+          <t>https://trendstop.knack.be/nl/detail/439000818/repro.aspx</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Repro NV</t>
+          <t>Royale Lacroix SA</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli e grassi vegetali</t>
+          <t>Olio di palma — margarine e grassi alimentari</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 14.157.353 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 1-5 dipendenti (societa' di raffinazione del Group Vandamme); n. impresa BE 0439.000.818</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr"/>
-      <c r="E86" s="5" t="inlineStr"/>
-      <c r="F86" s="5" t="inlineStr"/>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato 49.349.520 EUR (bilancio NBB, ultimo esercizio pubblicato) — taglia gonfiata dal costo materia prima: solo 18,6 FTE; n. impresa BE 0404.423.583</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Patrice Lacroix</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/royale-lacroix</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>info@royalelacroix.be</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>https://www.groupvandamme.com/</t>
+          <t>https://www.royalelacroix.com/</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Deinze (Oost-Vlaanderen)</t>
+          <t>Flémalle (Liège, Wallonie)</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/439000818/repro.aspx</t>
+          <t>https://www.companyweb.be/en/0404423583/royale-lacroix</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Royale Lacroix SA</t>
+          <t>Ameloot BV</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — margarine e grassi alimentari</t>
+          <t>Bovini/Carne — macellazione e ingrosso</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 49.349.520 EUR (bilancio NBB, ultimo esercizio pubblicato) — taglia gonfiata dal costo materia prima: solo 18,6 FTE; n. impresa BE 0404.423.583</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>Patrice Lacroix</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>Administrateur délégué</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/royale-lacroix</t>
-        </is>
-      </c>
+          <t>Fatturato 49.298.205 EUR (Trends Top/NBB, ultimo esercizio); n. impresa BE 0413.029.562. AZIENDA DI CONFINE: sopra i 40 M€ ma PMI familiare indipendente (3a generazione) con macello integrato SGL; dal 2024 controlla Slachtgroep Leieland BV; fatturato gonfiato dal costo materia prima.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>info@royalelacroix.be</t>
+          <t>petra@ameloot.org</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>https://www.royalelacroix.com/</t>
+          <t>https://omerameloot.com/nl</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Flémalle (Liège, Wallonie)</t>
+          <t>Harelbeke (West-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0404423583/royale-lacroix</t>
+          <t>https://trendstop.knack.be/nl/detail/413029562/ameloot.aspx</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Ameloot BV</t>
+          <t>Dierickx NV</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione e ingrosso</t>
+          <t>Bovini/Carne — sezionamento carne bovina</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 49.298.205 EUR (Trends Top/NBB, ultimo esercizio); n. impresa BE 0413.029.562. AZIENDA DI CONFINE: sopra i 40 M€ ma PMI familiare indipendente (3a generazione) con macello integrato SGL; dal 2024 controlla Slachtgroep Leieland BV; fatturato gonfiato dal costo materia prima.</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr"/>
-      <c r="E88" s="5" t="inlineStr"/>
+          <t>Fatturato 40.843.828 EUR (ultimo bilancio depositato NBB, via Trends Top/Companyweb); azienda familiare indipendente alla 5a generazione; n. impresa BE 0422.204.673. Al limite alto della fascia: nella carne il fatturato e' gonfiato dal costo della materia prima.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Cis van den Broeck</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Zaakvoerder</t>
+        </is>
+      </c>
       <c r="F88" s="5" t="inlineStr"/>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>petra@ameloot.org</t>
+          <t>info@dierickxnv.be</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>https://omerameloot.com/nl</t>
+          <t>https://dierickxnv.be/</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Harelbeke (West-Vlaanderen, Fiandre)</t>
+          <t>Zele (Oost-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/413029562/ameloot.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/422204673/dierickx.aspx</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Dierickx NV</t>
+          <t>Euro Meat Group NV</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — sezionamento carne bovina</t>
+          <t>Bovini/Carne — macellazione bovini</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 40.843.828 EUR (ultimo bilancio depositato NBB, via Trends Top/Companyweb); azienda familiare indipendente alla 5a generazione; n. impresa BE 0422.204.673. Al limite alto della fascia: nella carne il fatturato e' gonfiato dal costo della materia prima.</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>Cis van den Broeck</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>Zaakvoerder</t>
-        </is>
-      </c>
+          <t>Fatturato ca. 11 milioni EUR (VILT, stampa settoriale agroalimentare belga); organico ca. 50 persone (40 operai + 10 impiegati); capacita' 75.000 bovini ed equini/anno, ca. 125.000 bovini macellati per conto terzi. Numero d'impresa BE non verificato su fonte pubblica. Fa parte del gruppo Cadus NV (macelli in Belgio) ed e' socio Febev.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr"/>
-      <c r="G89" s="4" t="inlineStr">
-        <is>
-          <t>info@dierickxnv.be</t>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>https://dierickxnv.be/</t>
+          <t>http://www.euromeatgroup.be/nl/home/</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Zele (Oost-Vlaanderen, Fiandre)</t>
+          <t>Moeskroen / Mouscron (Hainaut, Vallonia)</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/422204673/dierickx.aspx</t>
+          <t>https://vilt.be/nl/nieuws/vijf-vleesspecialisten-nemen-familiebedrijf-derwa-over</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Euro Meat Group NV</t>
+          <t>Jos Leemput BV</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione bovini</t>
+          <t>Bovini/Carne — commercio all'ingrosso e sezionamento</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 11 milioni EUR (VILT, stampa settoriale agroalimentare belga); organico ca. 50 persone (40 operai + 10 impiegati); capacita' 75.000 bovini ed equini/anno, ca. 125.000 bovini macellati per conto terzi. Numero d'impresa BE non verificato su fonte pubblica. Fa parte del gruppo Cadus NV (macelli in Belgio) ed e' socio Febev.</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr"/>
-      <c r="E90" s="5" t="inlineStr"/>
+          <t>Fatturato 44.954.796 EUR e 16,2 FTE (ultimo bilancio depositato NBB, via Companyweb/FinCheck); n. impresa BE 0424.110.724. AZIENDA DI CONFINE: sopra 40 M€ ma con soli 16 dipendenti - caso tipico di fatturato gonfiato dal costo della materia prima; PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Jos Leemput</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Titolare, responsabile acquisto e selezione bestiame (sito aziendale)</t>
+        </is>
+      </c>
       <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="5" t="inlineStr">
         <is>
@@ -32518,170 +32514,162 @@
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>http://www.euromeatgroup.be/nl/home/</t>
+          <t>https://www.leemput.be/</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Moeskroen / Mouscron (Hainaut, Vallonia)</t>
+          <t>Tienen / Hakendover (Vlaams-Brabant, Fiandre)</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>https://vilt.be/nl/nieuws/vijf-vleesspecialisten-nemen-familiebedrijf-derwa-over</t>
+          <t>https://trendstop.knack.be/nl/detail/424110724/leemput-jos.aspx</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Jos Leemput BV</t>
+          <t>Slachthuis Swaegers NV</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — commercio all'ingrosso e sezionamento</t>
+          <t>Bovini/Carne — macellazione e sezionamento bovini</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 44.954.796 EUR e 16,2 FTE (ultimo bilancio depositato NBB, via Companyweb/FinCheck); n. impresa BE 0424.110.724. AZIENDA DI CONFINE: sopra 40 M€ ma con soli 16 dipendenti - caso tipico di fatturato gonfiato dal costo della materia prima; PMI familiare indipendente.</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Jos Leemput</t>
-        </is>
-      </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>Titolare, responsabile acquisto e selezione bestiame (sito aziendale)</t>
-        </is>
-      </c>
+          <t>Fatturato 4.287.787 EUR e 4,8 FTE nella societa' di macellazione (ultimo bilancio NBB, via Companyweb/Trends Top); n. impresa BE 0436.764.571. SOTTO LA SOGLIA dei 5 M€ come singola entita': il fatturato riflette solo i servizi di macellazione: il gruppo familiare Swaegers &amp; Co dichiara 70.000 bovini/anno e 22.000 t di capacita' annua, quindi volumi EUDR molto superiori al fatturato contabile.</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr"/>
       <c r="F91" s="3" t="inlineStr"/>
-      <c r="G91" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>info@swaegers.be</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>https://www.leemput.be/</t>
+          <t>https://www.swaegers.be/</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Tienen / Hakendover (Vlaams-Brabant, Fiandre)</t>
+          <t>Hoogstraten (Antwerpen, Fiandre)</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/424110724/leemput-jos.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/436764571/swaegers-slachthuis.aspx</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Slachthuis Swaegers NV</t>
+          <t>Slachthuis Velzeke BV</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione e sezionamento bovini</t>
+          <t>Bovini/Carne — macellazione bovini</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 4.287.787 EUR e 4,8 FTE nella societa' di macellazione (ultimo bilancio NBB, via Companyweb/Trends Top); n. impresa BE 0436.764.571. SOTTO LA SOGLIA dei 5 M€ come singola entita': il fatturato riflette solo i servizi di macellazione: il gruppo familiare Swaegers &amp; Co dichiara 70.000 bovini/anno e 22.000 t di capacita' annua, quindi volumi EUDR molto superiori al fatturato contabile.</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr"/>
-      <c r="E92" s="5" t="inlineStr"/>
+          <t>50-99 dipendenti (Companyweb, dati piu' recenti); capacita' 2.000 bovini/settimana, uno dei maggiori macelli bovini del Belgio; n. impresa BE 1018.071.121. Fatturato NON disponibile: entita' costituita il 30/12/2024 (cambio di proprieta' nel 2025), nessun bilancio con cifra d'affari ancora depositato. Altri amministratori indicati: Guy De Bruycker, Johan Castelein.</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Wouter Cokelaere</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Bestuurder</t>
+        </is>
+      </c>
       <c r="F92" s="5" t="inlineStr"/>
-      <c r="G92" s="6" t="inlineStr">
-        <is>
-          <t>info@swaegers.be</t>
-        </is>
-      </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>https://www.swaegers.be/</t>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Hoogstraten (Antwerpen, Fiandre)</t>
+          <t>Velzeke-Ruddershove, Zottegem (Oost-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/436764571/swaegers-slachthuis.aspx</t>
+          <t>https://www.companyweb.be/nl/1018071121/slachthuis-velzeke</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Slachthuis Velzeke BV</t>
+          <t>Sopraco NV</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione bovini</t>
+          <t>Bovini/Carne — fornitura e ingrosso carni</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>50-99 dipendenti (Companyweb, dati piu' recenti); capacita' 2.000 bovini/settimana, uno dei maggiori macelli bovini del Belgio; n. impresa BE 1018.071.121. Fatturato NON disponibile: entita' costituita il 30/12/2024 (cambio di proprieta' nel 2025), nessun bilancio con cifra d'affari ancora depositato. Altri amministratori indicati: Guy De Bruycker, Johan Castelein.</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>Wouter Cokelaere</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>Bestuurder</t>
-        </is>
-      </c>
+          <t>Fatturato 8.889.508 EUR e 45,5 FTE (ultimo bilancio depositato NBB, via Companyweb/Trends Top); n. impresa BE 0507.988.901. Nella fascia bassa tollerata (5-40 M€). Capofila del gruppo familiare Sopraco, che dal 2017 controlla anche Rompa Leder (filiera pelle): doppia esposizione EUDR bovini + pelle.</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr"/>
       <c r="F93" s="3" t="inlineStr"/>
-      <c r="G93" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>info@sopraco.eu</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sopraco.eu/</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>Velzeke-Ruddershove, Zottegem (Oost-Vlaanderen, Fiandre)</t>
+          <t>Geel (Antwerpen, Fiandre)</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/nl/1018071121/slachthuis-velzeke</t>
+          <t>https://trendstop.knack.be/en/detail/507988901/sopraco.aspx</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Sopraco NV</t>
+          <t>Van De Walle SRL</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — fornitura e ingrosso carni</t>
+          <t>Bovini/Carne — commercio all'ingrosso</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 8.889.508 EUR e 45,5 FTE (ultimo bilancio depositato NBB, via Companyweb/Trends Top); n. impresa BE 0507.988.901. Nella fascia bassa tollerata (5-40 M€). Capofila del gruppo familiare Sopraco, che dal 2017 controlla anche Rompa Leder (filiera pelle): doppia esposizione EUDR bovini + pelle.</t>
+          <t>n. impresa BE 0893.625.564 (Trends Top). Fatturato e organico NON pubblicati in forma accessibile (schema abbreviato NBB): azienda familiare fondata nel 1954, filiera verticalizzata dall'allevamento alla consegna con flotta frigo propria, clientela di macellerie e GDO. Dimensione stimabile come PMI, da verificare sul bilancio NBB.</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr"/>
@@ -32689,107 +32677,67 @@
       <c r="F94" s="5" t="inlineStr"/>
       <c r="G94" s="6" t="inlineStr">
         <is>
-          <t>info@sopraco.eu</t>
+          <t>info@vdw-grossisteenviande.be</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>https://www.sopraco.eu/</t>
+          <t>https://vdw-grossisteenviande.be/</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Geel (Antwerpen, Fiandre)</t>
+          <t>Wayaux / Villers-Perwin, Les Bons Villers (Hainaut, Vallonia)</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/en/detail/507988901/sopraco.aspx</t>
+          <t>https://trendstop.levif.be/fr/detail/893625564/van-de-walle.aspx</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>Van De Walle SRL</t>
+          <t>Vleeshandel Vens NV</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — commercio all'ingrosso</t>
+          <t>Bovini/Carne — ingrosso e sezionamento</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>n. impresa BE 0893.625.564 (Trends Top). Fatturato e organico NON pubblicati in forma accessibile (schema abbreviato NBB): azienda familiare fondata nel 1954, filiera verticalizzata dall'allevamento alla consegna con flotta frigo propria, clientela di macellerie e GDO. Dimensione stimabile come PMI, da verificare sul bilancio NBB.</t>
+          <t>32 FTE in bilancio (oltre 40 collaboratori secondo il sito aziendale); fatturato NON pubblicato (schema abbreviato NBB), margine lordo dichiarato 1.950.416 EUR; n. impresa BE 0468.329.064. Azienda familiare dal 1975; tratta rundsvlees, kalfsvlees, varkensvlees e lamsvlees.</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr"/>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="3" t="inlineStr"/>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>info@vdw-grossisteenviande.be</t>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>https://vdw-grossisteenviande.be/</t>
+          <t>https://vleeshandelvens.be/</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>Wayaux / Villers-Perwin, Les Bons Villers (Hainaut, Vallonia)</t>
+          <t>Lendelede (West-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/893625564/van-de-walle.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Vleeshandel Vens NV</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>Bovini/Carne — ingrosso e sezionamento</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>32 FTE in bilancio (oltre 40 collaboratori secondo il sito aziendale); fatturato NON pubblicato (schema abbreviato NBB), margine lordo dichiarato 1.950.416 EUR; n. impresa BE 0468.329.064. Azienda familiare dal 1975; tratta rundsvlees, kalfsvlees, varkensvlees e lamsvlees.</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr"/>
-      <c r="E96" s="5" t="inlineStr"/>
-      <c r="F96" s="5" t="inlineStr"/>
-      <c r="G96" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H96" s="6" t="inlineStr">
-        <is>
-          <t>https://vleeshandelvens.be/</t>
-        </is>
-      </c>
-      <c r="I96" s="5" t="inlineStr">
-        <is>
-          <t>Lendelede (West-Vlaanderen, Fiandre)</t>
-        </is>
-      </c>
-      <c r="J96" s="5" t="inlineStr">
-        <is>
           <t>https://www.companyweb.be/en/0468329064/vleeshandel-vens</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J96"/>
+  <autoFilter ref="A2:J95"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -32889,74 +32837,74 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId121"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId123"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId131"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId166"/>
@@ -32964,13 +32912,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId177"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId180"/>
@@ -32979,29 +32927,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId191"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Austria: rimossa Bayer Kartonagen (asset deal, non piu' un produttore)
A gennaio 2025 Schwarzach Packaging ha rilevato macchine e portafoglio prodotti con
un asset deal; la produzione e' stata trasferita da Lustenau a Schwarzach e il
titolare si e' ritirato. Precedente identico gia' applicato dal progetto: Getama
Danmark, rimossa perche' «non e' piu' un produttore, quindi non e' un operatore EUDR».

TEGUM resta invece nel foglio: l'argomento di perimetro e' inferenza («gli articoli
tecnici sono tipicamente in elastomeri sintetici»), non evidenza come per Helvoet,
dove era l'azienda stessa a pubblicare una gamma di soli polimeri sintetici.

Censimento da 737 a 736 aziende (Austria 92->91).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$95</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32958,7 +32958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -35143,122 +35143,122 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Bayer Kartonagen GmbH</t>
+          <t>Bösmüller Print Management GesmbH &amp; Co KG</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartotecnica</t>
+          <t>Carta/Packaging — stampa e imballaggi</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 12 Mio. € con 80 dipendenti (fonte Vorarlberger Nachrichten VN.at, intervista 08.11.2019); stima successiva 27,3 Mio. € (die-deutsche-wirtschaft.de ranking, dato stimato). Firmenbuch FN 388412w. Impresa familiare di 3a generazione, Schillerstraße 16. IN TARGET 10-20 M€ secondo il dato pubblicato. ATTENZIONE LEGAME DI GRUPPO: la produzione è stata rilevata da Schwarzach Packaging (Schwarzach, Vorarlberg) con effetto retroattivo dal 1° gennaio - verificare l'assetto attuale prima del contatto.</t>
+          <t>Ca. 65 dipendenti su 3 sedi (Wien, Stockerau, Krems), di cui ca. 50 nello stabilimento di Stockerau (fonte sito aziendale/lehrlingsportal.at, dato 2023-2024). Fatturato non pubblicato: n.d. Firmenbuch FN 276051h, HG Wien. Sede legale Obere Augartenstraße 32, 1020 Wien; stabilimento Josef-Sandhofer-Straße 3, 2000 Stockerau. STIMA SOTTO LA FASCIA IDEALE: con ~65 addetti il fatturato è verosimilmente vicino o inferiore alla soglia dei 10 M€ - da verificare. Impresa familiare (2a generazione); secondo Geschäftsführer: Markus Purker. Attiva anche nel Verpackungsdruck (astucci e packaging in cartoncino).</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Josef Andreas Bayer</t>
+          <t>Ing. Doris Wallner-Bösmüller</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/bayer-kartonagen-gmbh</t>
-        </is>
-      </c>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>office@bayer-kartonagen.com</t>
+          <t>office@boesmueller.at</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>https://www.bayer-kartonagen.com</t>
+          <t>https://boesmueller.at</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Lustenau, Vorarlberg</t>
+          <t>Stockerau, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/bayer-kartonagen-gmbh_IPzn</t>
+          <t>https://boesmueller.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Bösmüller Print Management GesmbH &amp; Co KG</t>
+          <t>CARINI GmbH</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa e imballaggi</t>
+          <t>Carta/Packaging — etichette</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Ca. 65 dipendenti su 3 sedi (Wien, Stockerau, Krems), di cui ca. 50 nello stabilimento di Stockerau (fonte sito aziendale/lehrlingsportal.at, dato 2023-2024). Fatturato non pubblicato: n.d. Firmenbuch FN 276051h, HG Wien. Sede legale Obere Augartenstraße 32, 1020 Wien; stabilimento Josef-Sandhofer-Straße 3, 2000 Stockerau. STIMA SOTTO LA FASCIA IDEALE: con ~65 addetti il fatturato è verosimilmente vicino o inferiore alla soglia dei 10 M€ - da verificare. Impresa familiare (2a generazione); secondo Geschäftsführer: Markus Purker. Attiva anche nel Verpackungsdruck (astucci e packaging in cartoncino).</t>
+          <t>Fatturato ca. 5,2 Mio. USD (~4,8 Mio. €) - 33 dipendenti (fonte profilo RocketReach, dato stimato). Firmenbuch FN 205435k. Sede Industrie Nord, Bildgasse 42, 6890 Lustenau. AZIENDA SOTTO LA SOGLIA MINIMA 5 M€ secondo la stima disponibile: dimensione DA VERIFICARE prima del contatto (l'azienda si presenta come una delle principali etichettifici dell'area di lingua tedesca, quindi il dato stimato potrebbe essere sottostimato). Impresa familiare fondata nel 1939, 4a generazione (Simon Sohm in direzione, tecnica applicativa e vendite).</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Ing. Doris Wallner-Bösmüller</t>
+          <t>Edgar Sohm</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführerin</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr"/>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/carini-gmbh</t>
+        </is>
+      </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>office@boesmueller.at</t>
+          <t>welcome@carini.at</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>https://boesmueller.at</t>
+          <t>https://www.carini.at</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Stockerau, Bassa Austria (Niederösterreich)</t>
+          <t>Lustenau, Vorarlberg</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>https://boesmueller.at/impressum/</t>
+          <t>https://www.carini.at/unternehmen-karriere/impressum/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>CARINI GmbH</t>
+          <t>Flatz GmbH</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — etichette</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 5,2 Mio. USD (~4,8 Mio. €) - 33 dipendenti (fonte profilo RocketReach, dato stimato). Firmenbuch FN 205435k. Sede Industrie Nord, Bildgasse 42, 6890 Lustenau. AZIENDA SOTTO LA SOGLIA MINIMA 5 M€ secondo la stima disponibile: dimensione DA VERIFICARE prima del contatto (l'azienda si presenta come una delle principali etichettifici dell'area di lingua tedesca, quindi il dato stimato potrebbe essere sottostimato). Impresa familiare fondata nel 1939, 4a generazione (Simon Sohm in direzione, tecnica applicativa e vendite).</t>
+          <t>Fatturato stimato ca. 18,4 Mio. USD (~17 Mio. €) - 96 dipendenti (fonte profilo RocketReach, dato stimato); azienda attiva dal 1935, uno dei principali produttori austriaci di imballaggi in cartone ondulato. Firmenbuch FN 136639s, LG Feldkirch. IN TARGET 10-20 M€. 4 stabilimenti a Lauterach (Funkenstraße 6/11, Scheibenstraße 20). Impresa familiare indipendente; Hans-Peter Flatz indicato come co-Geschäftsführer in fonti di stampa.</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Edgar Sohm</t>
+          <t>Mag. Stefan Flatz</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -35268,149 +35268,145 @@
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>https://at.linkedin.com/company/carini-gmbh</t>
+          <t>https://at.linkedin.com/company/flatz-gmbh</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>welcome@carini.at</t>
+          <t>office@flatz.com</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>https://www.carini.at</t>
+          <t>https://www.flatz.com</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Lustenau, Vorarlberg</t>
+          <t>Lauterach, Vorarlberg</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>https://www.carini.at/unternehmen-karriere/impressum/</t>
+          <t>https://www.flatz.com/de/karriere/kontakt/</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Flatz GmbH</t>
+          <t>Gruber Karton Kreativ GmbH</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Carta/Packaging — cartotecnica e imballaggi</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Fatturato stimato ca. 18,4 Mio. USD (~17 Mio. €) - 96 dipendenti (fonte profilo RocketReach, dato stimato); azienda attiva dal 1935, uno dei principali produttori austriaci di imballaggi in cartone ondulato. Firmenbuch FN 136639s, LG Feldkirch. IN TARGET 10-20 M€. 4 stabilimenti a Lauterach (Funkenstraße 6/11, Scheibenstraße 20). Impresa familiare indipendente; Hans-Peter Flatz indicato come co-Geschäftsführer in fonti di stampa.</t>
+          <t>Fatturato e numero di dipendenti non pubblicati nelle fonti consultate: n.d. (fonte WKO Firmen A-Z / firmennetzwerk.at, 2025). Firmenbuch FN 643739a, Ried im Innkreis. Sede Frankenburger Straße 17, 4910 Ried im Innkreis. Impresa familiare con oltre 120 anni di attività, produce cartonaggi, imballaggi in cartone teso e ondulato, scatole per spedizione. DIMENSIONE DA VERIFICARE: probabilmente sotto la fascia ideale 10-20 M€. Gewerberechtlicher Geschäftsführer: Christian Magoč. Società collegata: Gruber Immo GmbH.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Mag. Stefan Flatz</t>
+          <t>Dipl.-Ing. Janin Simader, BSc</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/flatz-gmbh</t>
-        </is>
-      </c>
+          <t>Geschäftsführerin</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr"/>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>office@flatz.com</t>
+          <t>office@gruber-karton-kreativ.at</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>https://www.flatz.com</t>
+          <t>https://gruber-kartonagen.at</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Lauterach, Vorarlberg</t>
+          <t>Ried im Innkreis, Alta Austria (Oberösterreich)</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>https://www.flatz.com/de/karriere/kontakt/</t>
+          <t>https://firmen.wko.at/gruber-karton-kreativ-gmbh-hersteller-von-kartonagen-karton-und-wellpappverpackungen/ober%C3%B6sterreich/?firmaid=d38297c8-65cd-4957-b852-3e53194f9fbd</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Gruber Karton Kreativ GmbH</t>
+          <t>Kliemstein Papierverarbeitungs GmbH</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartotecnica e imballaggi</t>
+          <t>Carta/Packaging — lavorazione carta</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Fatturato e numero di dipendenti non pubblicati nelle fonti consultate: n.d. (fonte WKO Firmen A-Z / firmennetzwerk.at, 2025). Firmenbuch FN 643739a, Ried im Innkreis. Sede Frankenburger Straße 17, 4910 Ried im Innkreis. Impresa familiare con oltre 120 anni di attività, produce cartonaggi, imballaggi in cartone teso e ondulato, scatole per spedizione. DIMENSIONE DA VERIFICARE: probabilmente sotto la fascia ideale 10-20 M€. Gewerberechtlicher Geschäftsführer: Christian Magoč. Società collegata: Gruber Immo GmbH.</t>
+          <t>Fatturato ca. 7 Mio. USD (~6,5 Mio. €) - 24 dipendenti nella sede (fonte Dun &amp; Bradstreet business directory, dato stimato). Firmenbuch FN 229062g. Sede Bahnhofstraße 6, 8330 Feldbach. AZIENDA SOTTO LA FASCIA IDEALE 10-20 M€: rientra solo nel margine basso del range tollerabile 5-40 M€. Impresa familiare che lavora industrialmente carta e cartone (quaderni, blocchi, rilegature, cartelline, blocchi flipchart). Membro del Fachverband PROPAK.</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Dipl.-Ing. Janin Simader, BSc</t>
+          <t>Mag. Thomas Kliemstein</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführerin</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>office@gruber-karton-kreativ.at</t>
+          <t>office@kliemstein.co.at</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>https://gruber-kartonagen.at</t>
+          <t>https://www.kliemstein.co.at</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Ried im Innkreis, Alta Austria (Oberösterreich)</t>
+          <t>Feldbach, Stiria (Steiermark)</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>https://firmen.wko.at/gruber-karton-kreativ-gmbh-hersteller-von-kartonagen-karton-und-wellpappverpackungen/ober%C3%B6sterreich/?firmaid=d38297c8-65cd-4957-b852-3e53194f9fbd</t>
+          <t>https://www.kliemstein.co.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Kliemstein Papierverarbeitungs GmbH</t>
+          <t>Margarethner Verpackungsgesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — lavorazione carta</t>
+          <t>Carta/Packaging — cartone ondulato e display</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 7 Mio. USD (~6,5 Mio. €) - 24 dipendenti nella sede (fonte Dun &amp; Bradstreet business directory, dato stimato). Firmenbuch FN 229062g. Sede Bahnhofstraße 6, 8330 Feldbach. AZIENDA SOTTO LA FASCIA IDEALE 10-20 M€: rientra solo nel margine basso del range tollerabile 5-40 M€. Impresa familiare che lavora industrialmente carta e cartone (quaderni, blocchi, rilegature, cartelline, blocchi flipchart). Membro del Fachverband PROPAK.</t>
+          <t>Oltre 30 dipendenti (fonte WKO Firmen A-Z / karriere.at, dato 2024-2025). Fatturato non pubblicato: n.d.; con ~30 addetti la stima è verosimilmente sotto i 10 M€ - DA VERIFICARE. Firmenbuch FN 39371z, BG Korneuburg. Sede Heidestraße 17, 2433 Margarethen am Moos. Produce imballaggi speciali e display in cartone ondulato e teso (POS). Membro del Forum Wellpappe Austria. ATTENZIONE LEGAME DI GRUPPO: 100% Inter Carton Gesellschaft m.b.H. (Wien), che detiene anche il 34% di DONAUWELL Wellpappe.</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Mag. Thomas Kliemstein</t>
+          <t>DI Richard Höfer</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -35421,44 +35417,44 @@
       <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>office@kliemstein.co.at</t>
+          <t>office@mvg.co.at</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>https://www.kliemstein.co.at</t>
+          <t>https://mvg.co.at</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Feldbach, Stiria (Steiermark)</t>
+          <t>Margarethen am Moos, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>https://www.kliemstein.co.at/impressum/</t>
+          <t>https://mvg.co.at/impressum</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Margarethner Verpackungsgesellschaft m.b.H.</t>
+          <t>MÜROLL GmbH</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato e display</t>
+          <t>Carta/Packaging — rotoli carta ed etichette</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Oltre 30 dipendenti (fonte WKO Firmen A-Z / karriere.at, dato 2024-2025). Fatturato non pubblicato: n.d.; con ~30 addetti la stima è verosimilmente sotto i 10 M€ - DA VERIFICARE. Firmenbuch FN 39371z, BG Korneuburg. Sede Heidestraße 17, 2433 Margarethen am Moos. Produce imballaggi speciali e display in cartone ondulato e teso (POS). Membro del Forum Wellpappe Austria. ATTENZIONE LEGAME DI GRUPPO: 100% Inter Carton Gesellschaft m.b.H. (Wien), che detiene anche il 34% di DONAUWELL Wellpappe.</t>
+          <t>Ca. 140 dipendenti (fonte sito aziendale / WKO Firmen A-Z, dato 2024). Fatturato non pubblicato: n.d.; con 140 addetti la fascia stimata è ~25-40 M€, quindi al limite superiore del range tollerabile - DA VERIFICARE. Firmenbuch FN 68918a, LG Feldkirch. Sede Satteinser Straße 12, 6820 Frastanz. Produce rotoli di carta, banderole, etichette stampate e nastri adesivi (unico produttore austriaco di nastri adesivi): quota rilevante ma non esclusiva di prodotti a base carta. ASSETTO: 99,5% Johann und Oswald Müller Privatstiftung. Altri Geschäftsführer: Uwe Müller, Kurt Pichler.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>DI Richard Höfer</t>
+          <t>Michael Müller</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -35469,44 +35465,44 @@
       <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>office@mvg.co.at</t>
+          <t>office@mueroll.com</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>https://mvg.co.at</t>
+          <t>https://www.mueroll.com</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Margarethen am Moos, Bassa Austria (Niederösterreich)</t>
+          <t>Frastanz, Vorarlberg</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>https://mvg.co.at/impressum</t>
+          <t>https://www.mueroll.com/en/imprint</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>MÜROLL GmbH</t>
+          <t>Print Alliance HAV Produktions GmbH</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — rotoli carta ed etichette</t>
+          <t>Carta/Packaging — stampa offset</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Ca. 140 dipendenti (fonte sito aziendale / WKO Firmen A-Z, dato 2024). Fatturato non pubblicato: n.d.; con 140 addetti la fascia stimata è ~25-40 M€, quindi al limite superiore del range tollerabile - DA VERIFICARE. Firmenbuch FN 68918a, LG Feldkirch. Sede Satteinser Straße 12, 6820 Frastanz. Produce rotoli di carta, banderole, etichette stampate e nastri adesivi (unico produttore austriaco di nastri adesivi): quota rilevante ma non esclusiva di prodotti a base carta. ASSETTO: 99,5% Johann und Oswald Müller Privatstiftung. Altri Geschäftsführer: Uwe Müller, Kurt Pichler.</t>
+          <t>Oltre 180 dipendenti (fonte sito aziendale / leitbetriebe.at, dato 2024). Fatturato non pubblicato: n.d.; con oltre 180 addetti la stima si colloca nella fascia alta del range tollerabile (~30-40 M€) - DA VERIFICARE prima del contatto. Firmenbuch FN 426711t, LG Wiener Neustadt. Sede Druckhausstraße 1, 2540 Bad Vöslau. Definita la più grande tipografia offset a foglio dell'Austria, attiva 24h; forte consumo di carta e cartoncino (rilevanza EUDR Allegato I). Membro Leitbetriebe Austria.</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Michael Müller</t>
+          <t>Christoph Preitler</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
@@ -35517,44 +35513,44 @@
       <c r="F53" s="3" t="inlineStr"/>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>office@mueroll.com</t>
+          <t>office@printalliance.at</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>https://www.mueroll.com</t>
+          <t>https://printalliance.at</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Frastanz, Vorarlberg</t>
+          <t>Bad Vöslau, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>https://www.mueroll.com/en/imprint</t>
+          <t>https://printalliance.at/impressum</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Print Alliance HAV Produktions GmbH</t>
+          <t>Salzer Papier GmbH</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa offset</t>
+          <t>Carta/Packaging — cartiera</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Oltre 180 dipendenti (fonte sito aziendale / leitbetriebe.at, dato 2024). Fatturato non pubblicato: n.d.; con oltre 180 addetti la stima si colloca nella fascia alta del range tollerabile (~30-40 M€) - DA VERIFICARE prima del contatto. Firmenbuch FN 426711t, LG Wiener Neustadt. Sede Druckhausstraße 1, 2540 Bad Vöslau. Definita la più grande tipografia offset a foglio dell'Austria, attiva 24h; forte consumo di carta e cartoncino (rilevanza EUDR Allegato I). Membro Leitbetriebe Austria.</t>
+          <t>Fatturato stimato ca. 42 Mio. € (fonte die-deutsche-wirtschaft.de, stima su dati 2023) - 51-200 dipendenti (fonte LinkedIn/firmenabc); nel 2007 24,5 Mio. € con 95 dipendenti (noe.ORF.at). Produzione ca. 30.000 t di carta/anno. Firmenbuch FN 312367p, LG St. Pölten. AZIENDA DI CONFINE: la stima 42 Mio. € supera di poco la fascia tollerabile 5-40 M€ ma resta ben sotto la soglia di esclusione ~50 M€. Impresa familiare all'8a generazione, parte della Salzer Gruppe (Papier, Industrie-Service, Holz). Co-Geschäftsführer citato in stampa: Dr. Harald Egger. Membro Austropapier.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Christoph Preitler</t>
+          <t>Thomas Salzer</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -35562,47 +35558,51 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/salzer-papier-gmbh</t>
+        </is>
+      </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>office@printalliance.at</t>
+          <t>office@salzer.at</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>https://printalliance.at</t>
+          <t>https://www.salzer.at</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Bad Vöslau, Bassa Austria (Niederösterreich)</t>
+          <t>St. Pölten (Stattersdorf), Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>https://printalliance.at/impressum</t>
+          <t>https://www.salzer.at/en/gruppe/kontakt/impressum/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Salzer Papier GmbH</t>
+          <t>Samson-Druck Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartiera</t>
+          <t>Carta/Packaging — stampa</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Fatturato stimato ca. 42 Mio. € (fonte die-deutsche-wirtschaft.de, stima su dati 2023) - 51-200 dipendenti (fonte LinkedIn/firmenabc); nel 2007 24,5 Mio. € con 95 dipendenti (noe.ORF.at). Produzione ca. 30.000 t di carta/anno. Firmenbuch FN 312367p, LG St. Pölten. AZIENDA DI CONFINE: la stima 42 Mio. € supera di poco la fascia tollerabile 5-40 M€ ma resta ben sotto la soglia di esclusione ~50 M€. Impresa familiare all'8a generazione, parte della Salzer Gruppe (Papier, Industrie-Service, Holz). Co-Geschäftsführer citato in stampa: Dr. Harald Egger. Membro Austropapier.</t>
+          <t>Fatturato oltre 18 Mio. € - ca. 120 dipendenti (fonte salzburg.wirtschaftszeit.at / die-salzburger-industrie.at, dato pubblicato 2023-2024). Firmenbuch FN 66316z, LG Salzburg. Azienda familiare di 3a generazione (Ramsbacher/Valentin/Frost), una delle maggiori tipografie offset austriache. PERFETTAMENTE IN TARGET 10-20 M€. Secondo Geschäftsführer: Tibor Valentin. Nota: 100% detenuta da Aichhorn Beteiligungs GmbH (holding familiare, non gruppo multinazionale).</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Thomas Salzer</t>
+          <t>Markus Ramsbacher</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -35612,49 +35612,49 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>https://at.linkedin.com/company/salzer-papier-gmbh</t>
+          <t>https://at.linkedin.com/company/samson-druck</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>office@salzer.at</t>
+          <t>office@samsondruck.at</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>https://www.salzer.at</t>
+          <t>https://www.samsondruck.at</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>St. Pölten (Stattersdorf), Bassa Austria (Niederösterreich)</t>
+          <t>St. Margarethen im Lungau, Salisburgo (Salzburg)</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>https://www.salzer.at/en/gruppe/kontakt/impressum/</t>
+          <t>https://www.samsondruck.at/impressum</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Samson-Druck Gesellschaft m.b.H.</t>
+          <t>Steirerpack GmbH</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Fatturato oltre 18 Mio. € - ca. 120 dipendenti (fonte salzburg.wirtschaftszeit.at / die-salzburger-industrie.at, dato pubblicato 2023-2024). Firmenbuch FN 66316z, LG Salzburg. Azienda familiare di 3a generazione (Ramsbacher/Valentin/Frost), una delle maggiori tipografie offset austriache. PERFETTAMENTE IN TARGET 10-20 M€. Secondo Geschäftsführer: Tibor Valentin. Nota: 100% detenuta da Aichhorn Beteiligungs GmbH (holding familiare, non gruppo multinazionale).</t>
+          <t>Fatturato non pubblicato: n.d. Dipendenti non pubblicati nelle fonti consultate (fonte firmenabc.at / WKO Firmen A-Z / propak.at). Firmenbuch FN 79280p, LG Leoben (Handelsgericht). Sede Hauptstraße 21, 8763 Pölstal. Azienda fondata nel 1902, produce cartone ondulato, astucci, imballaggi fustellati, display e cartoni per vino. Membro del Forum Wellpappe Austria: i 7 produttori del forum occupano complessivamente ca. 1.600 addetti, il che colloca Steirerpack tra le realtà medie del settore. DIMENSIONE DA VERIFICARE. Co-Geschäftsführer: Franz Grafendorfer.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Markus Ramsbacher</t>
+          <t>Mag. Wolfgang Habenberger</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -35664,49 +35664,49 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>https://at.linkedin.com/company/samson-druck</t>
+          <t>https://de.linkedin.com/company/steirerpack</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>office@samsondruck.at</t>
+          <t>office@steirerpack.at</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>https://www.samsondruck.at</t>
+          <t>https://steirerpack.at</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>St. Margarethen im Lungau, Salisburgo (Salzburg)</t>
+          <t>Pölstal (Möderbrugg), Stiria (Steiermark)</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>https://www.samsondruck.at/impressum</t>
+          <t>https://steirerpack.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Steirerpack GmbH</t>
+          <t>Ulrich Etiketten Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Carta/Packaging — etichette</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato: n.d. Dipendenti non pubblicati nelle fonti consultate (fonte firmenabc.at / WKO Firmen A-Z / propak.at). Firmenbuch FN 79280p, LG Leoben (Handelsgericht). Sede Hauptstraße 21, 8763 Pölstal. Azienda fondata nel 1902, produce cartone ondulato, astucci, imballaggi fustellati, display e cartoni per vino. Membro del Forum Wellpappe Austria: i 7 produttori del forum occupano complessivamente ca. 1.600 addetti, il che colloca Steirerpack tra le realtà medie del settore. DIMENSIONE DA VERIFICARE. Co-Geschäftsführer: Franz Grafendorfer.</t>
+          <t>Fatturato ca. 33 Mio. € (+4% sull'anno precedente) - ca. 200 dipendenti (fonte labelpack.de / profili aziendali, 2023). Firmenbuch FN 89306h, BG Korneuburg. Sede produttiva Betriebsstraße 3, 2011 Höbersdorf; 3 uffici vendita in Germania. Azienda familiare indipendente. SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€. Co-Geschäftsführer: Florian Ulrich.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Mag. Wolfgang Habenberger</t>
+          <t>Dr. Rainer Ulrich</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -35714,51 +35714,47 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>https://de.linkedin.com/company/steirerpack</t>
-        </is>
-      </c>
+      <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>office@steirerpack.at</t>
+          <t>ulrich@ulrich.at</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>https://steirerpack.at</t>
+          <t>https://ulrich.at</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Pölstal (Möderbrugg), Stiria (Steiermark)</t>
+          <t>Höbersdorf (Sierndorf), Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>https://steirerpack.at/impressum/</t>
+          <t>https://ulrich.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Ulrich Etiketten Gesellschaft m.b.H.</t>
+          <t>Wellpappenfabrik TEWA Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — etichette</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 33 Mio. € (+4% sull'anno precedente) - ca. 200 dipendenti (fonte labelpack.de / profili aziendali, 2023). Firmenbuch FN 89306h, BG Korneuburg. Sede produttiva Betriebsstraße 3, 2011 Höbersdorf; 3 uffici vendita in Germania. Azienda familiare indipendente. SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€. Co-Geschäftsführer: Florian Ulrich.</t>
+          <t>Fatturato 12,5 Mio. € - ca. 50 dipendenti (fonte meinbezirk.at, articolo sulla successione familiare; fatturato riferito al 2012, organico aggiornato). IN TARGET 10-20 M€ secondo il dato pubblicato, ma il fatturato è un dato datato - DA VERIFICARE. Sede Buscheiden 9, 9560 Feldkirchen. Sito produttivo attivo dal 1846, impresa familiare. Membro del Forum Wellpappe Austria (7 produttori austriaci di cartone ondulato). Geschäftsführender Gesellschafter: KommR Franz Ronge.</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Dr. Rainer Ulrich</t>
+          <t>Felix Ronge</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -35769,44 +35765,44 @@
       <c r="F58" s="5" t="inlineStr"/>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>ulrich@ulrich.at</t>
+          <t>wirmachendas@tewa.com</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>https://ulrich.at</t>
+          <t>https://www.tewa.com</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Höbersdorf (Sierndorf), Bassa Austria (Niederösterreich)</t>
+          <t>Feldkirchen in Kärnten, Carinzia (Kärnten)</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>https://ulrich.at/impressum/</t>
+          <t>https://www.tewa.com/team-1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Wellpappenfabrik TEWA Gesellschaft m.b.H.</t>
+          <t>Wograndl Druck GmbH</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Carta/Packaging — stampa</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 12,5 Mio. € - ca. 50 dipendenti (fonte meinbezirk.at, articolo sulla successione familiare; fatturato riferito al 2012, organico aggiornato). IN TARGET 10-20 M€ secondo il dato pubblicato, ma il fatturato è un dato datato - DA VERIFICARE. Sede Buscheiden 9, 9560 Feldkirchen. Sito produttivo attivo dal 1846, impresa familiare. Membro del Forum Wellpappe Austria (7 produttori austriaci di cartone ondulato). Geschäftsführender Gesellschafter: KommR Franz Ronge.</t>
+          <t>Ca. 48 dipendenti (fonte meinbezirk.at, articolo 2020-2021); descritta come la maggiore tipografia del Burgenland e tra le prime dieci in Austria; 26 gruppi stampa/verniciatura su tre turni. Fatturato non pubblicato: n.d. Firmenbuch FN 272989f, LG Eisenstadt. Sede Druckweg 1, 7210 Walbersdorf/Mattersburg. STIMA SOTTO LA FASCIA IDEALE: con ~48 addetti il fatturato è verosimilmente sotto i 10 M€ - da verificare. Impresa familiare fondata nel 1956 da Josef Wograndl.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Felix Ronge</t>
+          <t>Jochen Wograndl</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -35814,47 +35810,51 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F59" s="3" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/wograndl-druck-gmbh</t>
+        </is>
+      </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>wirmachendas@tewa.com</t>
+          <t>print@wograndl.com</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>https://www.tewa.com</t>
+          <t>https://www.wograndl.com</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Feldkirchen in Kärnten, Carinzia (Kärnten)</t>
+          <t>Mattersburg (Walbersdorf), Burgenland</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>https://www.tewa.com/team-1</t>
+          <t>https://www.wograndl.com/kontakt</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Wograndl Druck GmbH</t>
+          <t>pack it! Verpackungen GmbH</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — stampa</t>
+          <t>Carta/Packaging — cartone ondulato offset</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Ca. 48 dipendenti (fonte meinbezirk.at, articolo 2020-2021); descritta come la maggiore tipografia del Burgenland e tra le prime dieci in Austria; 26 gruppi stampa/verniciatura su tre turni. Fatturato non pubblicato: n.d. Firmenbuch FN 272989f, LG Eisenstadt. Sede Druckweg 1, 7210 Walbersdorf/Mattersburg. STIMA SOTTO LA FASCIA IDEALE: con ~48 addetti il fatturato è verosimilmente sotto i 10 M€ - da verificare. Impresa familiare fondata nel 1956 da Josef Wograndl.</t>
+          <t>Fatturato 25,5 Mio. € (+15% sui ca. 23 Mio. € dell'anno precedente) - 63 dipendenti su produzione a quattro turni (fonte meinbezirk.at / packreport.de, dato riferito al bilancio successivo al 2011; investimento di 15 Mio. € nel nuovo impianto di cartone ondulato). SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€; dato non recente, DA VERIFICARE. Firmenbuch FN 196751s, LG Steyr. Sede Hermesstraße 7, 4595 Waldneukirchen. Specializzata in imballaggi in cartone ondulato cachierato offset. NOTA ASSETTO: fondata nel 2000 anche con la partecipazione di Dinkhauser Verpackungen (Tirolo). Prokuristen: Karl Ömmer. Membro Fachverband PROPAK.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Jochen Wograndl</t>
+          <t>Dipl.-Ing. Walter Michael Freimüller</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -35864,49 +35864,49 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/wograndl-druck-gmbh</t>
+          <t>https://at.linkedin.com/company/packit-verpackungen-gmbh</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>print@wograndl.com</t>
+          <t>office@packit.at</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>https://www.wograndl.com</t>
+          <t>https://www.packit.at</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Mattersburg (Walbersdorf), Burgenland</t>
+          <t>Waldneukirchen, Alta Austria (Oberösterreich)</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>https://www.wograndl.com/kontakt</t>
+          <t>https://www.propak.at/mitglieder/item/pack-it-verpackungen-gmbh</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>pack it! Verpackungen GmbH</t>
+          <t>pratopac GmbH</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato offset</t>
+          <t>Carta/Packaging — cartone ondulato</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 25,5 Mio. € (+15% sui ca. 23 Mio. € dell'anno precedente) - 63 dipendenti su produzione a quattro turni (fonte meinbezirk.at / packreport.de, dato riferito al bilancio successivo al 2011; investimento di 15 Mio. € nel nuovo impianto di cartone ondulato). SOPRA la fascia ideale 10-20 M€ ma dentro il range tollerabile 5-40 M€; dato non recente, DA VERIFICARE. Firmenbuch FN 196751s, LG Steyr. Sede Hermesstraße 7, 4595 Waldneukirchen. Specializzata in imballaggi in cartone ondulato cachierato offset. NOTA ASSETTO: fondata nel 2000 anche con la partecipazione di Dinkhauser Verpackungen (Tirolo). Prokuristen: Karl Ömmer. Membro Fachverband PROPAK.</t>
+          <t>Fatturato 18 Mio. € - ca. 70-75 dipendenti (fonte Wirtschaftszeit.at / VN.at, dato 2020-2021; 15 Mio. € nel 2018). Firmenbuch FN 217837w, LG Feldkirch. Sede Riedstraße 1-5, 6833 Klaus. PERFETTAMENTE IN TARGET 10-20 M€. Produce cartone ondulato, cartonaggi, tubi e barattoli in cartone spiralato. NOTA ASSETTO: socio unico WA Holding GmbH (holding familiare Vorarlberg); esiste inoltre la joint venture pratopac Gmeiner GmbH con Gmeiner nel settore anime/tubi.</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Dipl.-Ing. Walter Michael Freimüller</t>
+          <t>Alexander Abbrederis</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -35914,51 +35914,47 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/packit-verpackungen-gmbh</t>
-        </is>
-      </c>
+      <c r="F61" s="3" t="inlineStr"/>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>office@packit.at</t>
+          <t>info@pratopac.at</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>https://www.packit.at</t>
+          <t>https://www.pratopac.at</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Waldneukirchen, Alta Austria (Oberösterreich)</t>
+          <t>Klaus, Vorarlberg</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>https://www.propak.at/mitglieder/item/pack-it-verpackungen-gmbh</t>
+          <t>https://www.pratopac.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>pratopac GmbH</t>
+          <t>Amann Kaffee GmbH</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Carta/Packaging — cartone ondulato</t>
+          <t>Caffè — torrefazione e import caffè verde</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 18 Mio. € - ca. 70-75 dipendenti (fonte Wirtschaftszeit.at / VN.at, dato 2020-2021; 15 Mio. € nel 2018). Firmenbuch FN 217837w, LG Feldkirch. Sede Riedstraße 1-5, 6833 Klaus. PERFETTAMENTE IN TARGET 10-20 M€. Produce cartone ondulato, cartonaggi, tubi e barattoli in cartone spiralato. NOTA ASSETTO: socio unico WA Holding GmbH (holding familiare Vorarlberg); esiste inoltre la joint venture pratopac Gmeiner GmbH con Gmeiner nel settore anime/tubi.</t>
+          <t>Bilancio: totale attivo 10,6 Mio. €, patrimonio netto 6,8 Mio. €, equity ratio 64,1% (esercizio 2025, fonte firmenabc.at/firmenatlas.com). Dipendenti 31-50 (fonte karriere.at). Fatturato puntuale non pubblicato. Firmenbuch FN 185621y, LG Feldkirch; UID ATU47491904. Fondata nel 1993 da Peter e Rupert Amann, oggi guidata da Peter Amann con i figli Johanna e Florian; torrefazione propria nel Bregenzerwald e nuova sede/centro logistico nel Millennium Park di Lustenau. Acquista caffè verde all'origine per la propria tostatura = operatore EUDR.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Alexander Abbrederis</t>
+          <t>Peter Amann</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -35966,47 +35962,51 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>https://de.linkedin.com/company/amann-kaffee-gmbh</t>
+        </is>
+      </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>info@pratopac.at</t>
+          <t>info@amann-kaffee.at</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>https://www.pratopac.at</t>
+          <t>https://www.amann-kaffee.at</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Klaus, Vorarlberg</t>
+          <t>Lustenau (torrefazione a Schwarzenberg), Vorarlberg</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>https://www.pratopac.at/impressum/</t>
+          <t>https://www.amann-kaffee.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Amann Kaffee GmbH</t>
+          <t>EZA Fairer Handel GmbH</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione e import caffè verde</t>
+          <t>Caffè — import caffè verde e cacao</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Bilancio: totale attivo 10,6 Mio. €, patrimonio netto 6,8 Mio. €, equity ratio 64,1% (esercizio 2025, fonte firmenabc.at/firmenatlas.com). Dipendenti 31-50 (fonte karriere.at). Fatturato puntuale non pubblicato. Firmenbuch FN 185621y, LG Feldkirch; UID ATU47491904. Fondata nel 1993 da Peter e Rupert Amann, oggi guidata da Peter Amann con i figli Johanna e Florian; torrefazione propria nel Bregenzerwald e nuova sede/centro logistico nel Millennium Park di Lustenau. Acquista caffè verde all'origine per la propria tostatura = operatore EUDR.</t>
+          <t>Fatturato ca. 16 Mio. € - 51-200 dipendenti (fonte eza.cc Geschäftsbericht / wlw.at, dati 2022-2024). Firmenbuch FN 69275a, LG Salzburg. Pioniere del commercio equo in Austria (dal 1975): importa direttamente caffè verde (44% del fatturato) e cacao/cioccolato dai Paesi produttori, senza intermediari - quindi IMPORTATORE DIRETTO di due commodity Allegato I EUDR. IN TARGET 10-20 M€. Doppia filiera caffè + cacao.</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Peter Amann</t>
+          <t>Michael Scherndl</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -36016,49 +36016,49 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/amann-kaffee-gmbh</t>
+          <t>https://at.linkedin.com/company/eza-fairer-handel</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>info@amann-kaffee.at</t>
+          <t>office@eza.at</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>https://www.amann-kaffee.at</t>
+          <t>https://www.eza.cc</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Lustenau (torrefazione a Schwarzenberg), Vorarlberg</t>
+          <t>Köstendorf bei Salzburg, Salisburgo (Salzburg)</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>https://www.amann-kaffee.at/impressum/</t>
+          <t>https://www.eza.cc/impressum</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>EZA Fairer Handel GmbH</t>
+          <t>Helmut Sachers Kaffee GmbH</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Caffè — import caffè verde e cacao</t>
+          <t>Caffè — torrefazione + import/export</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 16 Mio. € - 51-200 dipendenti (fonte eza.cc Geschäftsbericht / wlw.at, dati 2022-2024). Firmenbuch FN 69275a, LG Salzburg. Pioniere del commercio equo in Austria (dal 1975): importa direttamente caffè verde (44% del fatturato) e cacao/cioccolato dai Paesi produttori, senza intermediari - quindi IMPORTATORE DIRETTO di due commodity Allegato I EUDR. IN TARGET 10-20 M€. Doppia filiera caffè + cacao.</t>
+          <t>Fatturato ca. 5,2 Mio. € - ca. 26 dipendenti (ultimo dato pubblico 2016/2017, fonte faq-genuss.com / firmenabc.at). Firmenbuch FN 105466y, HG Wien. AZIENDA DI CONFINE (limite inferiore ~5 M€ della forbice tollerabile). Fondata nel 1929 a Vienna; ha attraversato un Sanierungsverfahren (2017) ed è oggi risanata e ATTIVA sotto nuova proprietà: SAWE Holding GmbH 80% + COFFEETREE S.r.l. 20%, GF dal 14.07.2020. Circa 450 t di caffè lavorate/anno, quota export ~20%; oggetto sociale include esplicitamente import/export di prodotti alimentari. Considerata la maggiore torrefazione bio dell'Austria.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Michael Scherndl</t>
+          <t>Hannes Schlögl</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -36066,51 +36066,47 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F64" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/eza-fairer-handel</t>
-        </is>
-      </c>
+      <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>office@eza.at</t>
+          <t>office@helmutsachers.at</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>https://www.eza.cc</t>
+          <t>https://www.helmutsachers.at</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Köstendorf bei Salzburg, Salisburgo (Salzburg)</t>
+          <t>Oeynhausen, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>https://www.eza.cc/impressum</t>
+          <t>https://www.helmutsachers.at/en/impressum/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Helmut Sachers Kaffee GmbH</t>
+          <t>J. Hornig GmbH</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione + import/export</t>
+          <t>Caffè — torrefazione + import caffè verde</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 5,2 Mio. € - ca. 26 dipendenti (ultimo dato pubblico 2016/2017, fonte faq-genuss.com / firmenabc.at). Firmenbuch FN 105466y, HG Wien. AZIENDA DI CONFINE (limite inferiore ~5 M€ della forbice tollerabile). Fondata nel 1929 a Vienna; ha attraversato un Sanierungsverfahren (2017) ed è oggi risanata e ATTIVA sotto nuova proprietà: SAWE Holding GmbH 80% + COFFEETREE S.r.l. 20%, GF dal 14.07.2020. Circa 450 t di caffè lavorate/anno, quota export ~20%; oggetto sociale include esplicitamente import/export di prodotti alimentari. Considerata la maggiore torrefazione bio dell'Austria.</t>
+          <t>Fatturato 18,2 Mio. € - ca. 51 dipendenti (fonte wirtschaftszeit.at / austria-forum.org, dato 2022-2023). Firmenbuch FN 91930p, LG für ZRS Graz. Torrefazione familiare fondata nel 1912, 4a generazione (Johannes Hornig, titolare/CEO di famiglia); importa caffè verde direttamente dai Paesi d'origine e rifornisce oltre 5.000 clienti out-of-home. PERFETTAMENTE IN TARGET 10-20 M€. Importatore di Rohkaffee = operatore EUDR in senso stretto.</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Hannes Schlögl</t>
+          <t>Mag. Thomas Schusteritsch</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -36118,291 +36114,291 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/j-hornig</t>
+        </is>
+      </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>office@helmutsachers.at</t>
+          <t>online@jhornig.at</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>https://www.helmutsachers.at</t>
+          <t>https://www.jhornig.com</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Oeynhausen, Bassa Austria (Niederösterreich)</t>
+          <t>Kalsdorf bei Graz, Stiria (Steiermark)</t>
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>https://www.helmutsachers.at/en/impressum/</t>
+          <t>https://www.jhornig.com/impressum/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>J. Hornig GmbH</t>
+          <t>Naber Kaffee Manufaktur GmbH</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione + import caffè verde</t>
+          <t>Caffè — torrefazione e commercio caffè verde</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 18,2 Mio. € - ca. 51 dipendenti (fonte wirtschaftszeit.at / austria-forum.org, dato 2022-2023). Firmenbuch FN 91930p, LG für ZRS Graz. Torrefazione familiare fondata nel 1912, 4a generazione (Johannes Hornig, titolare/CEO di famiglia); importa caffè verde direttamente dai Paesi d'origine e rifornisce oltre 5.000 clienti out-of-home. PERFETTAMENTE IN TARGET 10-20 M€. Importatore di Rohkaffee = operatore EUDR in senso stretto.</t>
+          <t>Fatturato ca. 3,5 Mio. € - ca. 15 dipendenti (fonte cash.at / cafeplusco.com, 2023-2024): AZIENDA SOTTO IL TARGET, segnalata come tale ma inserita perché commercia esplicitamente CAFFÈ VERDE (Rohkaffee). Firmenbuch FN 441118d, HG Wien; UID ATU69904712. Torrefazione viennese storica fondata nel 1908 da Georg Naber, dal 2015 controllata al 95% da café+co International Holding GmbH; tosta fino a 2 t di caffè al giorno, forte quota di private label; nel 2024-2025 ha rilevato una torrefazione tradizionale carinziana e aperto la sede di Klagenfurt. Oggetto sociale: produzione, tostatura e confezionamento di caffè in grani e commercio di caffè tostato E CRUDO.</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Mag. Thomas Schusteritsch</t>
+          <t>Marco Salvatori</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/j-hornig</t>
-        </is>
-      </c>
+          <t>Geschäftsführer (con Bernd Nitschmann)</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>online@jhornig.at</t>
+          <t>office@naberkaffee.com</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>https://www.jhornig.com</t>
+          <t>https://naberkaffee.com</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>Kalsdorf bei Graz, Stiria (Steiermark)</t>
+          <t>Vienna (Wien), Strebersdorf; seconda sede Klagenfurt</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>https://www.jhornig.com/impressum/</t>
+          <t>https://naberkaffee.com/en/legal/imprint/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Naber Kaffee Manufaktur GmbH</t>
+          <t>Testa Rossa Caffe GmbH</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione e commercio caffè verde</t>
+          <t>Caffè — torrefazione propria e franchising</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 3,5 Mio. € - ca. 15 dipendenti (fonte cash.at / cafeplusco.com, 2023-2024): AZIENDA SOTTO IL TARGET, segnalata come tale ma inserita perché commercia esplicitamente CAFFÈ VERDE (Rohkaffee). Firmenbuch FN 441118d, HG Wien; UID ATU69904712. Torrefazione viennese storica fondata nel 1908 da Georg Naber, dal 2015 controllata al 95% da café+co International Holding GmbH; tosta fino a 2 t di caffè al giorno, forte quota di private label; nel 2024-2025 ha rilevato una torrefazione tradizionale carinziana e aperto la sede di Klagenfurt. Oggetto sociale: produzione, tostatura e confezionamento di caffè in grani e commercio di caffè tostato E CRUDO.</t>
+          <t>Fatturato e dipendenti non pubblicati sui portali gratuiti (firmenabc.at/KSV1870 espongono solo i dati anagrafici) - VERIFICARE. Firmenbuch FN 100910y, LG Innsbruck; UID ATU24581405; costituita il 04.02.1993; socio unico Leopold Wedl (100%), gruppo Wedl (Handelshaus Wedl, Mils). Gestisce il sistema di franchising internazionale TESTA ROSSA caffèbar (dal 1999, oltre 100 locali in Europa e Medio Oriente) e la torrefazione interna: la miscela di caffè verde viene tostata in proprio = operatore EUDR.</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Marco Salvatori</t>
+          <t>KR Leopold Wedl</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer (con Bernd Nitschmann)</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr"/>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>office@naberkaffee.com</t>
+          <t>franchise@testarossacaffe.com</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
         <is>
-          <t>https://naberkaffee.com</t>
+          <t>https://www.testarossacaffe.com</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Vienna (Wien), Strebersdorf; seconda sede Klagenfurt</t>
+          <t>Mils bei Hall in Tirol, Tirolo (Tirol)</t>
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>https://naberkaffee.com/en/legal/imprint/</t>
+          <t>https://www.testarossacaffe.com/impressum</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Testa Rossa Caffe GmbH</t>
+          <t>Berger Feinste Confiserie GmbH</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Caffè — torrefazione propria e franchising</t>
+          <t>Cacao/Cioccolato — confiserie e praline</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Fatturato e dipendenti non pubblicati sui portali gratuiti (firmenabc.at/KSV1870 espongono solo i dati anagrafici) - VERIFICARE. Firmenbuch FN 100910y, LG Innsbruck; UID ATU24581405; costituita il 04.02.1993; socio unico Leopold Wedl (100%), gruppo Wedl (Handelshaus Wedl, Mils). Gestisce il sistema di franchising internazionale TESTA ROSSA caffèbar (dal 1999, oltre 100 locali in Europa e Medio Oriente) e la torrefazione interna: la miscela di caffè verde viene tostata in proprio = operatore EUDR.</t>
+          <t>Ca. 100 dipendenti, 8 punti vendita propri in Salisburghese, Tirolo e Stiria, export mondiale (fonte confiserie-berger.at / chocolats-de-luxe.de, dati 2023-2025). Fatturato non pubblicato: firmenabc.at non espone il dato (Jahresabschluss non integralmente accessibile) - VERIFICARE. Firmenbuch FN 254861x, capitale 35.000 €, soci Hubert Berger 50% e Christine Berger 50%. Fondata nel 1994 a Lofer. Lavora couverture/cacao certificato Fairtrade (partner Fairtrade Austria): trasformatore di cacao = operatore/commerciante EUDR.</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>KR Leopold Wedl</t>
+          <t>Hubert Berger</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführer (con Christine Berger)</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>franchise@testarossacaffe.com</t>
+          <t>schokolade@confiserie-berger.at</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>https://www.testarossacaffe.com</t>
+          <t>https://www.confiserie-berger.at</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Mils bei Hall in Tirol, Tirolo (Tirol)</t>
+          <t>Lofer, Salisburgo (Salzburg)</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>https://www.testarossacaffe.com/impressum</t>
+          <t>https://www.confiserie-berger.at/en/imprint</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Berger Feinste Confiserie GmbH</t>
+          <t>Confiserie Wenschitz GmbH</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — confiserie e praline</t>
+          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Ca. 100 dipendenti, 8 punti vendita propri in Salisburghese, Tirolo e Stiria, export mondiale (fonte confiserie-berger.at / chocolats-de-luxe.de, dati 2023-2025). Fatturato non pubblicato: firmenabc.at non espone il dato (Jahresabschluss non integralmente accessibile) - VERIFICARE. Firmenbuch FN 254861x, capitale 35.000 €, soci Hubert Berger 50% e Christine Berger 50%. Fondata nel 1994 a Lofer. Lavora couverture/cacao certificato Fairtrade (partner Fairtrade Austria): trasformatore di cacao = operatore/commerciante EUDR.</t>
+          <t>Ca. 30 dipendenti; totale attivo di bilancio 4,4 Mio. €, patrimonio netto 2,0 Mio. € (esercizio 2025, fonte firmenabc.at / firmenatlas.com). Fatturato non pubblicato: stimabile SOTTO la forbice target (probabile 5-8 Mio. €) - AZIENDA PICCOLA, segnalata come tale. Firmenbuch FN 273013s, LG Linz; UID ATU62268101. Maître Chocolatier con 'Pralinenwelt' ad Allhaming; produce praline, figure di cioccolato e marzapane in lavorazione artigianale assistita. Trasformatore di cacao/couverture = operatore o commerciante EUDR.</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Hubert Berger</t>
+          <t>Helmut Wenschitz</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer (con Christine Berger)</t>
+          <t>Geschäftsführender Gesellschafter</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr"/>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>schokolade@confiserie-berger.at</t>
+          <t>office@wenschitz.at</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>https://www.confiserie-berger.at</t>
+          <t>https://www.wenschitz.at</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Lofer, Salisburgo (Salzburg)</t>
+          <t>Allhaming, Alta Austria (Oberösterreich)</t>
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>https://www.confiserie-berger.at/en/imprint</t>
+          <t>https://www.wenschitz.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Confiserie Wenschitz GmbH</t>
+          <t>Fürst GmbH</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e figure di cioccolato</t>
+          <t>Cacao/Cioccolato — praline e Mozartkugeln</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Ca. 30 dipendenti; totale attivo di bilancio 4,4 Mio. €, patrimonio netto 2,0 Mio. € (esercizio 2025, fonte firmenabc.at / firmenatlas.com). Fatturato non pubblicato: stimabile SOTTO la forbice target (probabile 5-8 Mio. €) - AZIENDA PICCOLA, segnalata come tale. Firmenbuch FN 273013s, LG Linz; UID ATU62268101. Maître Chocolatier con 'Pralinenwelt' ad Allhaming; produce praline, figure di cioccolato e marzapane in lavorazione artigianale assistita. Trasformatore di cacao/couverture = operatore o commerciante EUDR.</t>
+          <t>Ca. 65-70 dipendenti, di cui 35 nella nuova manifattura di Elsbethen; produzione ca. 3,7 milioni di Original Salzburger Mozartkugel all'anno; investimento di 'diversi milioni di euro' nel nuovo stabilimento aperto a febbraio 2024 (fonte SN.at / wko.at / salzburgwiki, 2024-2026). Fatturato non pubblicato - VERIFICARE. Firmenbuch FN 257955x, LG Salzburg; UID ATU61451413. Café-Konditorei fondata nel 1884, 5a generazione (Martin Fürst dal 2015), inventrice della Mozartkugel (1890); 4 punti vendita a Salisburgo. Grande utilizzatore di cioccolato/cacao = operatore o commerciante EUDR.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Helmut Wenschitz</t>
+          <t>Martin Fürst</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführender Gesellschafter</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>office@wenschitz.at</t>
+          <t>versand@fuerst.cc</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>https://www.wenschitz.at</t>
+          <t>https://www.original-mozartkugel.com</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Allhaming, Alta Austria (Oberösterreich)</t>
+          <t>Salisburgo (Salzburg), produzione a Elsbethen</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>https://www.wenschitz.at/impressum/</t>
+          <t>https://www.original-mozartkugel.com/en/imprint</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Fürst GmbH</t>
+          <t>Heidi Chocolat AG</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — praline e Mozartkugeln</t>
+          <t>Cacao/Cioccolato — dolciumi al cioccolato</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Ca. 65-70 dipendenti, di cui 35 nella nuova manifattura di Elsbethen; produzione ca. 3,7 milioni di Original Salzburger Mozartkugel all'anno; investimento di 'diversi milioni di euro' nel nuovo stabilimento aperto a febbraio 2024 (fonte SN.at / wko.at / salzburgwiki, 2024-2026). Fatturato non pubblicato - VERIFICARE. Firmenbuch FN 257955x, LG Salzburg; UID ATU61451413. Café-Konditorei fondata nel 1884, 5a generazione (Martin Fürst dal 2015), inventrice della Mozartkugel (1890); 4 punti vendita a Salisburgo. Grande utilizzatore di cioccolato/cacao = operatore o commerciante EUDR.</t>
+          <t>Fatturato ca. 18 Mio. € - ca. 180 dipendenti (fonte Wikipedia/dati aziendali, ultimo dato pubblico 2018; ordine di grandezza confermato da cash.at). Firmenbuch FN 397683d, LG Wiener Neustadt; UID ATU67943648. Titolare del marchio storico viennese Niemetz Schwedenbomben (dal 1926) rilevato nel 2013; produzione trasferita a Wiener Neudorf. IN TARGET 10-20 M€. Grande utilizzatore di cioccolato/cacao per il rivestimento dei prodotti = operatore/commerciante EUDR.</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Martin Fürst</t>
+          <t>Alexander Grund</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -36410,47 +36406,51 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F71" s="3" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/heidi-chocolat-ag-niemetz-schwedenbomben%C2%AE</t>
+        </is>
+      </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>versand@fuerst.cc</t>
+          <t>office@schwedenbomben.at</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>https://www.original-mozartkugel.com</t>
+          <t>https://niemetz.at</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Salisburgo (Salzburg), produzione a Elsbethen</t>
+          <t>Wiener Neudorf, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>https://www.original-mozartkugel.com/en/imprint</t>
+          <t>https://niemetz.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Heidi Chocolat AG</t>
+          <t>Landgarten GmbH &amp; Co KG</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — dolciumi al cioccolato</t>
+          <t>Cacao/Cioccolato — snack bio ricoperti + cioccolato</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 18 Mio. € - ca. 180 dipendenti (fonte Wikipedia/dati aziendali, ultimo dato pubblico 2018; ordine di grandezza confermato da cash.at). Firmenbuch FN 397683d, LG Wiener Neustadt; UID ATU67943648. Titolare del marchio storico viennese Niemetz Schwedenbomben (dal 1926) rilevato nel 2013; produzione trasferita a Wiener Neudorf. IN TARGET 10-20 M€. Grande utilizzatore di cioccolato/cacao per il rivestimento dei prodotti = operatore/commerciante EUDR.</t>
+          <t>Fatturato non pubblicato (Jahresabschluss non integralmente accessibile su firmenabc.at) - VERIFICARE. Ordine di grandezza del gruppo stimabile in fascia 20-35 Mio. € dopo l'acquisizione: nel marzo 2025 Landgarten ha rilevato il 100% della cioccolateria Franz Hauswirth Ges.m.b.H. di Kittsee (14,6 Mio. € di fatturato 2022/23, ca. 70 dipendenti mantenuti), uscita dall'insolvenza di fine 2024. Firmenbuch FN 128998d, LG Korneuburg; 3 soci (2 accomandanti + 1 accomandatario Landgarten GmbH). Produttore di snack bio dal 1989, ricoperti di cioccolato Fairtrade: acquirente diretto di cacao/cioccolato = operatore EUDR.</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Alexander Grund</t>
+          <t>Herbert Stava</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -36458,195 +36458,191 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/heidi-chocolat-ag-niemetz-schwedenbomben%C2%AE</t>
-        </is>
-      </c>
+      <c r="F72" s="5" t="inlineStr"/>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>office@schwedenbomben.at</t>
+          <t>office@landgarten.at</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>https://niemetz.at</t>
+          <t>https://landgarten.at</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Wiener Neudorf, Bassa Austria (Niederösterreich)</t>
+          <t>Bruck an der Leitha, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>https://niemetz.at/impressum/</t>
+          <t>https://landgarten.at/en/impressum/</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Landgarten GmbH &amp; Co KG</t>
+          <t>Deisenhammer Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — snack bio ricoperti + cioccolato</t>
+          <t>Gomma — articoli tecnici in elastomero</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (Jahresabschluss non integralmente accessibile su firmenabc.at) - VERIFICARE. Ordine di grandezza del gruppo stimabile in fascia 20-35 Mio. € dopo l'acquisizione: nel marzo 2025 Landgarten ha rilevato il 100% della cioccolateria Franz Hauswirth Ges.m.b.H. di Kittsee (14,6 Mio. € di fatturato 2022/23, ca. 70 dipendenti mantenuti), uscita dall'insolvenza di fine 2024. Firmenbuch FN 128998d, LG Korneuburg; 3 soci (2 accomandanti + 1 accomandatario Landgarten GmbH). Produttore di snack bio dal 1989, ricoperti di cioccolato Fairtrade: acquirente diretto di cacao/cioccolato = operatore EUDR.</t>
+          <t>100-199 dipendenti (firmenabc.at, 2025); fatturato non pubblicato. Fondata 1989, sedi Gunskirchen e Linz. Firmenbuch FN 100139p</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Herbert Stava</t>
+          <t>Hartmut Hermann Lauer</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Gewerberechtlicher Geschäftsführer</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr"/>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>office@landgarten.at</t>
+          <t>anfrage@deisenhammer.at</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>https://landgarten.at</t>
+          <t>https://www.deisenhammer.at/</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Bruck an der Leitha, Bassa Austria (Niederösterreich)</t>
+          <t>Gunskirchen, Oberösterreich</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>https://landgarten.at/en/impressum/</t>
+          <t>https://www.firmenabc.at/deisenhammer-gesellschaft-m-b-h_How</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Deisenhammer Gesellschaft m.b.H.</t>
+          <t>Gummiwerk Czermak &amp; Feger, Gesellschaft m.b.H. &amp; Co KG</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Gomma — articoli tecnici in elastomero</t>
+          <t>Gomma — lattice di caucciù naturale</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>100-199 dipendenti (firmenabc.at, 2025); fatturato non pubblicato. Fondata 1989, sedi Gunskirchen e Linz. Firmenbuch FN 100139p</t>
+          <t>21-50 dipendenti (herold.at/firmenabc.at, 2025); fatturato non pubblicato — PMI sotto la soglia target. Fondata 1949; palloni e articoli senza saldature in lattice di gomma naturale, mescole di gomma. Firmenbuch FN 18060i (KG) / FN 45245m (GmbH)</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Hartmut Hermann Lauer</t>
+          <t>Ing. Dominik Czermak</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Gewerberechtlicher Geschäftsführer</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr"/>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>anfrage@deisenhammer.at</t>
+          <t>office@gummiwerk.at</t>
         </is>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>https://www.deisenhammer.at/</t>
+          <t>https://www.gummiwerk.at/</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Gunskirchen, Oberösterreich</t>
+          <t>Imst (Brennbichl), Tirol</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/deisenhammer-gesellschaft-m-b-h_How</t>
+          <t>https://www.firmenabc.at/gummiwerk-czermak-feger-gesellschaft-m-b-h-co-kg_Pho</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Gummiwerk Czermak &amp; Feger, Gesellschaft m.b.H. &amp; Co KG</t>
+          <t>Persicaner &amp; Co. Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Gomma — lattice di caucciù naturale</t>
+          <t>Gomma — commercio articoli tecnici in gomma</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>21-50 dipendenti (herold.at/firmenabc.at, 2025); fatturato non pubblicato — PMI sotto la soglia target. Fondata 1949; palloni e articoli senza saldature in lattice di gomma naturale, mescole di gomma. Firmenbuch FN 18060i (KG) / FN 45245m (GmbH)</t>
+          <t>2 Geschäftsführer e 2 soci (firmenabc.at, 2025); fatturato e organico non pubblicati — grossista di O-ring, lastre di gomma, cinghie, tubi. Fondata 1875, familiare dal 1960. Firmenbuch FN 129338d</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Ing. Dominik Czermak</t>
+          <t>Martin Winkelhöfer</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Gewerberechtlicher Geschäftsführer</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr"/>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>office@gummiwerk.at</t>
+          <t>office@persicaner.at</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>https://www.gummiwerk.at/</t>
+          <t>https://www.persicaner.at/</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Imst (Brennbichl), Tirol</t>
+          <t>Wien (Favoriten, 10. Bezirk), Wien</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/gummiwerk-czermak-feger-gesellschaft-m-b-h-co-kg_Pho</t>
+          <t>https://www.firmenabc.at/persicaner-co-gesellschaft-m-b-h_fFv</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Persicaner &amp; Co. Gesellschaft m.b.H.</t>
+          <t>Zrunek Gummiwaren Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Gomma — commercio articoli tecnici in gomma</t>
+          <t>Gomma — articoli tecnici in gomma ed elastomeri</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>2 Geschäftsführer e 2 soci (firmenabc.at, 2025); fatturato e organico non pubblicati — grossista di O-ring, lastre di gomma, cinghie, tubi. Fondata 1875, familiare dal 1960. Firmenbuch FN 129338d</t>
+          <t>10-19 dipendenti, classe di fatturato 0-10 Mio. €, Bilanzsumme 1,74 Mio. € al 31.12.2024 (firmenabc.at / northdata). NOTA: sotto la soglia target — produttore austriaco di articoli in gomma dal 1947. Altri GF: Mag. Dr. Ulrich Zrunek, Dipl.-Ing. Helena Zrunek Marja</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Martin Winkelhöfer</t>
+          <t>Dipl.-Ing. Max Zrunek</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -36657,92 +36653,96 @@
       <c r="F76" s="5" t="inlineStr"/>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>office@persicaner.at</t>
+          <t>office@zrunek.at</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>https://www.persicaner.at/</t>
+          <t>https://www.zrunek.at/</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Wien (Favoriten, 10. Bezirk), Wien</t>
+          <t>Wien (Döbling, 19. Bezirk), Wien</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/persicaner-co-gesellschaft-m-b-h_fFv</t>
+          <t>https://www.firmenabc.at/zrunek-gummiwaren-gesellschaft-m-b-h_plo</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Zrunek Gummiwaren Gesellschaft m.b.H.</t>
+          <t>"Sojarei" Vollwertkost-Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Gomma — articoli tecnici in gomma ed elastomeri</t>
+          <t>Mangimi/Soia — lavorazione soia bio (tofu)</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>10-19 dipendenti, classe di fatturato 0-10 Mio. €, Bilanzsumme 1,74 Mio. € al 31.12.2024 (firmenabc.at / northdata). NOTA: sotto la soglia target — produttore austriaco di articoli in gomma dal 1947. Altri GF: Mag. Dr. Ulrich Zrunek, Dipl.-Ing. Helena Zrunek Marja</t>
+          <t>Ca. 50 dipendenti (fonte advantageaustria.org / sito aziendale, dato 2023-2024); fatturato non pubblicato. Firmenbuch FN 118580h. Fondata nel 1984, è il più grande e antico produttore di tofu dell'Austria e leader nazionale nei prodotti biologici a base di soia; fornisce tutte le principali catene retail austriache, il canale Reformhaus/bio e la ristorazione. Co-Geschäftsführung/tecnica: Andreas Eschner e Ing. Gerhard Eschner. Operatore EUDR sulla soia (Allegato I) anche se acquistata in UE.</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Dipl.-Ing. Max Zrunek</t>
+          <t>Mag. Ernst Ternon</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Gewerberechtlicher Geschäftsführer</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr"/>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/sojarei-vollwertkost-gmbh</t>
+        </is>
+      </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>office@zrunek.at</t>
+          <t>info@sojarei.at</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>https://www.zrunek.at/</t>
+          <t>https://www.sojarei.at</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Wien (Döbling, 19. Bezirk), Wien</t>
+          <t>Traiskirchen, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/zrunek-gummiwaren-gesellschaft-m-b-h_plo</t>
+          <t>https://www.northdata.com/Sojarei%20Vollwertkost-GmbH,%20Traiskirchen/118580h</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>"Sojarei" Vollwertkost-Gesellschaft m.b.H.</t>
+          <t>Gsellmann Mischfuttererzeugung GmbH</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — lavorazione soia bio (tofu)</t>
+          <t>Mangimi/Soia — mangimi composti e materie prime</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Ca. 50 dipendenti (fonte advantageaustria.org / sito aziendale, dato 2023-2024); fatturato non pubblicato. Firmenbuch FN 118580h. Fondata nel 1984, è il più grande e antico produttore di tofu dell'Austria e leader nazionale nei prodotti biologici a base di soia; fornisce tutte le principali catene retail austriache, il canale Reformhaus/bio e la ristorazione. Co-Geschäftsführung/tecnica: Andreas Eschner e Ing. Gerhard Eschner. Operatore EUDR sulla soia (Allegato I) anche se acquistata in UE.</t>
+          <t>Bilancio: totale attivo 28,5 Mio. € e patrimonio netto 8,9 Mio. € (esercizio 2025, fonte firmeninfo.at / firmenatlas.com); ca. 60 dipendenti (fonte firmenabc.at). Firmenbuch FN 317883a. ATTENZIONE TAGLIA: il fatturato non è pubblicato e con capacità fino a 600 t/giorno potrebbe superare i 40 M€ per effetto del costo materia prima; resta però PMI familiare indipendente (3ª/4ª generazione, mulino dal 1890, ca. 3.000 clienti abituali). Altri Geschäftsführer: Josef Gsellmann, Maria Gsellmann.</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Mag. Ernst Ternon</t>
+          <t>Andreas Gsellmann</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -36750,99 +36750,95 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/sojarei-vollwertkost-gmbh</t>
-        </is>
-      </c>
+      <c r="F78" s="5" t="inlineStr"/>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>info@sojarei.at</t>
+          <t>office@gsellmann.com</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>https://www.sojarei.at</t>
+          <t>https://www.gsellmann.com</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Traiskirchen, Bassa Austria (Niederösterreich)</t>
+          <t>Kohlberg / Gnas, Stiria (Steiermark)</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>https://www.northdata.com/Sojarei%20Vollwertkost-GmbH,%20Traiskirchen/118580h</t>
+          <t>https://www.gsellmann.com/impressum/</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Gsellmann Mischfuttererzeugung GmbH</t>
+          <t>Ignaz Göweil GmbH &amp; Co KG</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi composti e materie prime</t>
+          <t>Mangimi/Soia — mangimi biologici, soia bio</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Bilancio: totale attivo 28,5 Mio. € e patrimonio netto 8,9 Mio. € (esercizio 2025, fonte firmeninfo.at / firmenatlas.com); ca. 60 dipendenti (fonte firmenabc.at). Firmenbuch FN 317883a. ATTENZIONE TAGLIA: il fatturato non è pubblicato e con capacità fino a 600 t/giorno potrebbe superare i 40 M€ per effetto del costo materia prima; resta però PMI familiare indipendente (3ª/4ª generazione, mulino dal 1890, ca. 3.000 clienti abituali). Altri Geschäftsführer: Josef Gsellmann, Maria Gsellmann.</t>
+          <t>22 dipendenti (fonte OÖ Nachrichten / nachrichten.at, articolo 2023); fatturato non divulgato dall'azienda (l'articolo precisa che Göweil non comunica il fatturato; quota di capitale proprio 15% da Firmenbuch). Mulino e mangimificio familiare, dal 1985 focalizzato sui mangimi e dal 2002 interamente convertito al biologico: specialista di mangimi composti bio (pollame, bovini, suini, cavalli, alpaca) con impiego di panello/soia biologica. PMI piccola, sotto la fascia target ma perfettamente in perimetro EUDR.</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Andreas Gsellmann</t>
+          <t>Karin Göweil</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführerin</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>office@gsellmann.com</t>
+          <t>office@goeweil-muehle.at</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>https://www.gsellmann.com</t>
+          <t>https://www.goeweil-muehle.at</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Kohlberg / Gnas, Stiria (Steiermark)</t>
+          <t>Engerwitzdorf (Engerwitzberg), Alta Austria (Oberösterreich)</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>https://www.gsellmann.com/impressum/</t>
+          <t>https://www.goeweil-muehle.at/kontakt/</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Ignaz Göweil GmbH &amp; Co KG</t>
+          <t>Königshofer GmbH</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimi biologici, soia bio</t>
+          <t>Mangimi/Soia — mangimificio e commercio mangimi</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>22 dipendenti (fonte OÖ Nachrichten / nachrichten.at, articolo 2023); fatturato non divulgato dall'azienda (l'articolo precisa che Göweil non comunica il fatturato; quota di capitale proprio 15% da Firmenbuch). Mulino e mangimificio familiare, dal 1985 focalizzato sui mangimi e dal 2002 interamente convertito al biologico: specialista di mangimi composti bio (pollame, bovini, suini, cavalli, alpaca) con impiego di panello/soia biologica. PMI piccola, sotto la fascia target ma perfettamente in perimetro EUDR.</t>
+          <t>Ca. 65 dipendenti (fonte sito aziendale 'Über uns' e firmenabc.at, dato 2024); fatturato non pubblicato nelle fonti aperte — per un mangimificio di questa scala si colloca indicativamente nella fascia 15-40 M€. Firmenbuch FN 442776t, UID ATU69978367. Stabilimento di Ebergassing (Franzensthalstraße 25) con silo cereali da 7.000 t, 53 celle materie prime e 44 celle prodotto finito; produce mangimi per cavalli e zootecnia con certificazione NON-GMO e pastus+ (impiego di soia/estratto di soia). Seconda Geschäftsführerin: Sarina Feurer.</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Karin Göweil</t>
+          <t>Mag. Astrid Pieler</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -36853,188 +36849,188 @@
       <c r="F80" s="5" t="inlineStr"/>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>office@goeweil-muehle.at</t>
+          <t>ebergassing@koenigshofer.at</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>https://www.goeweil-muehle.at</t>
+          <t>https://www.koenigshofer-futtermittel.at</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Engerwitzdorf (Engerwitzberg), Alta Austria (Oberösterreich)</t>
+          <t>Ebergassing, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>https://www.goeweil-muehle.at/kontakt/</t>
+          <t>https://www.koenigshofer-futtermittel.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Königshofer GmbH</t>
+          <t>Mischfutterwerk Großschedl GmbH</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio e commercio mangimi</t>
+          <t>Mangimi/Soia — mangimificio e commercio soia</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Ca. 65 dipendenti (fonte sito aziendale 'Über uns' e firmenabc.at, dato 2024); fatturato non pubblicato nelle fonti aperte — per un mangimificio di questa scala si colloca indicativamente nella fascia 15-40 M€. Firmenbuch FN 442776t, UID ATU69978367. Stabilimento di Ebergassing (Franzensthalstraße 25) con silo cereali da 7.000 t, 53 celle materie prime e 44 celle prodotto finito; produce mangimi per cavalli e zootecnia con certificazione NON-GMO e pastus+ (impiego di soia/estratto di soia). Seconda Geschäftsführerin: Sarina Feurer.</t>
+          <t>Fatturato ca. 8,5 Mio. € - ca. 15 dipendenti (fonte firmenabc.at / firmeninfo.at, dato 2023-2024). Firmenbuch FN 268698w. Azienda familiare al sito di Hofing dal 1780, produzione di mangimi composti dal 1964; oltre al mangimificio gestisce mulino e commercio di cereali, sementi e mangimi (Sojaschrot). Secondo Geschäftsführer: Mag. Dagmar Großschedl. IN TARGET (parte bassa della forbice tollerata 5-40 M€).</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Mag. Astrid Pieler</t>
+          <t>Herbert Großschedl</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführerin</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr"/>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>ebergassing@koenigshofer.at</t>
+          <t>office@grosschedl-futter.at</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>https://www.koenigshofer-futtermittel.at</t>
+          <t>http://www.grosschedl-futter.at</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Ebergassing, Bassa Austria (Niederösterreich)</t>
+          <t>Blaindorf / Feistritztal (Hofing), Stiria (Steiermark)</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>https://www.koenigshofer-futtermittel.at/impressum/</t>
+          <t>http://www.grosschedl-futter.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Mischfutterwerk Großschedl GmbH</t>
+          <t>Reitbauer Betriebs- u. Handels GmbH</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio e commercio soia</t>
+          <t>Mangimi/Soia — mangimificio e commercio agricolo</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Fatturato ca. 8,5 Mio. € - ca. 15 dipendenti (fonte firmenabc.at / firmeninfo.at, dato 2023-2024). Firmenbuch FN 268698w. Azienda familiare al sito di Hofing dal 1780, produzione di mangimi composti dal 1964; oltre al mangimificio gestisce mulino e commercio di cereali, sementi e mangimi (Sojaschrot). Secondo Geschäftsführer: Mag. Dagmar Großschedl. IN TARGET (parte bassa della forbice tollerata 5-40 M€).</t>
+          <t>Oltre 55-60 dipendenti (fonte sito aziendale 'Firma' e meinbezirk.at, 2023-2024); fatturato non pubblicato nelle fonti aperte. Firmenbuch FN 73386x, LG St. Pölten. Azienda familiare dal 1897, descritta come uno dei maggiori mangimifici privati d'Austria: mulino cereali, mangimificio (Mischfutter per bovini, suini, pollame) e Landhandel; utilizza componenti proteiche a base di soia. Ha anche una segheria, ma il core mangimi/cereali è l'attività in perimetro EUDR (soia).</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Herbert Großschedl</t>
+          <t>Stefan Reitbauer</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr"/>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>office@grosschedl-futter.at</t>
+          <t>office@reitbauer.co.at</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>http://www.grosschedl-futter.at</t>
+          <t>https://www.reitbauer.co.at</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Blaindorf / Feistritztal (Hofing), Stiria (Steiermark)</t>
+          <t>Vestenthal / Haidershofen, Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>http://www.grosschedl-futter.at/impressum/</t>
+          <t>https://www.reitbauer.co.at/impressum</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Reitbauer Betriebs- u. Handels GmbH</t>
+          <t>Rickl - Mühle GmbH</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio e commercio agricolo</t>
+          <t>Mangimi/Soia — commercio cereali e Sojaschrot</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Oltre 55-60 dipendenti (fonte sito aziendale 'Firma' e meinbezirk.at, 2023-2024); fatturato non pubblicato nelle fonti aperte. Firmenbuch FN 73386x, LG St. Pölten. Azienda familiare dal 1897, descritta come uno dei maggiori mangimifici privati d'Austria: mulino cereali, mangimificio (Mischfutter per bovini, suini, pollame) e Landhandel; utilizza componenti proteiche a base di soia. Ha anche una segheria, ma il core mangimi/cereali è l'attività in perimetro EUDR (soia).</t>
+          <t>PMI familiare fondata nel 1894, gestita da 3 responsabili (2 Geschäftsführer + 1 procuratore); fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at / firmeninfo.at / evi.gv.at, 2024-2025). Firmenbuch FN 162039v, LG Korneuburg, UID ATU43171303. Mulino e Landhandel a 35 km da Vienna: commercio di cereali convenzionali e bio, mangimi, sementi, concimi; a catalogo Sojaschrot (farina di estrazione di soia) come mangime proteico — attività di immissione sul mercato di soia = perimetro EUDR. TAGLIA DA VERIFICARE: probabile fascia bassa (5-15 M€).</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Stefan Reitbauer</t>
+          <t>Josef Rickl</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
+          <t>Geschäftsführer</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr"/>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>office@reitbauer.co.at</t>
+          <t>office@rickl.at</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>https://www.reitbauer.co.at</t>
+          <t>https://www.rickl.at</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Vestenthal / Haidershofen, Bassa Austria (Niederösterreich)</t>
+          <t>Groß-Schweinbarth (Bezirk Gänserndorf), Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>https://www.reitbauer.co.at/impressum</t>
+          <t>https://www.rickl.at/produkt/sojaschrot/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Rickl - Mühle GmbH</t>
+          <t>Vorarlberger Mühlen und Mischfutterwerke GmbH</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — commercio cereali e Sojaschrot</t>
+          <t>Mangimi/Soia — mangimificio regionale</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>PMI familiare fondata nel 1894, gestita da 3 responsabili (2 Geschäftsführer + 1 procuratore); fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at / firmeninfo.at / evi.gv.at, 2024-2025). Firmenbuch FN 162039v, LG Korneuburg, UID ATU43171303. Mulino e Landhandel a 35 km da Vienna: commercio di cereali convenzionali e bio, mangimi, sementi, concimi; a catalogo Sojaschrot (farina di estrazione di soia) come mangime proteico — attività di immissione sul mercato di soia = perimetro EUDR. TAGLIA DA VERIFICARE: probabile fascia bassa (5-15 M€).</t>
+          <t>Fatturato ca. 20 Mio. € - PMI industriale (fonte firmenabc.at / rassegna Raiffeisen Vorarlberg, dato 2022-2024). Firmenbuch FN 70012i, LG Feldkirch. Marchio 'Ländle Futter'; dal 2021 tornata azienda a controllo puramente familiare (uscita della Raiffeisenlandesbank Vorarlberg). Nuovo stabilimento mangimi a Dornbirn, Stöckenstraße 8. Utilizza panelli/estratto di soia nelle miscele. PERFETTAMENTE IN TARGET 10-20 M€.</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Josef Rickl</t>
+          <t>Bernd Hagen</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -37045,232 +37041,232 @@
       <c r="F84" s="5" t="inlineStr"/>
       <c r="G84" s="6" t="inlineStr">
         <is>
-          <t>office@rickl.at</t>
+          <t>office@laendlefutter.at</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>https://www.rickl.at</t>
+          <t>https://www.laendlefutter.at</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Groß-Schweinbarth (Bezirk Gänserndorf), Bassa Austria (Niederösterreich)</t>
+          <t>Dornbirn (sede legale Feldkirch), Vorarlberg</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>https://www.rickl.at/produkt/sojaschrot/</t>
+          <t>https://www.laendlefutter.at/impressum</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Vorarlberger Mühlen und Mischfutterwerke GmbH</t>
+          <t>Wieshofermühle Betriebs GmbH</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio regionale</t>
+          <t>Mangimi/Soia — mulino e mangimificio</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 20 Mio. € - PMI industriale (fonte firmenabc.at / rassegna Raiffeisen Vorarlberg, dato 2022-2024). Firmenbuch FN 70012i, LG Feldkirch. Marchio 'Ländle Futter'; dal 2021 tornata azienda a controllo puramente familiare (uscita della Raiffeisenlandesbank Vorarlberg). Nuovo stabilimento mangimi a Dornbirn, Stöckenstraße 8. Utilizza panelli/estratto di soia nelle miscele. PERFETTAMENTE IN TARGET 10-20 M€.</t>
+          <t>PMI familiare alla 6ª generazione, sede a St. Johann da oltre 500 anni; fatturato e organico non pubblicati nelle fonti aperte (fonte sito aziendale / Impressum, 2024-2025). Firmenbuch FN 651815b, LG Innsbruck, UID ATU82121605. Iscritta WKO Tirol come 'Futtermittelerzeuger', 'Handel mit Futtermitteln' e 'Großhandel mit Lebensmitteln'. Uno dei pochi mulini + mangimifici austriaci ancora totalmente in mani private; il Futterwerk produce mangimi per bovini, pollame, suini, cavalli, ovicaprini e selvaggina (componenti proteiche a base di soia). Prokuristin: Mag. Caroline Krainz-Gasteiger.</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Bernd Hagen</t>
+          <t>Mag. Lukas Krainz</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführer und 100%iger Anteilseigner</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr"/>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>office@laendlefutter.at</t>
+          <t>info@wieshofermuehle.at</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>https://www.laendlefutter.at</t>
+          <t>https://www.wieshofermuehle.at</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Dornbirn (sede legale Feldkirch), Vorarlberg</t>
+          <t>St. Johann in Tirol, Tirolo (Tirol)</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>https://www.laendlefutter.at/impressum</t>
+          <t>https://www.wieshofermuehle.at/de/impressum</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Wieshofermühle Betriebs GmbH</t>
+          <t>BIOSERVICE Zach Ges.m.b.H.</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mulino e mangimificio</t>
+          <t>Olio di palma — grossista ingredienti bio</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>PMI familiare alla 6ª generazione, sede a St. Johann da oltre 500 anni; fatturato e organico non pubblicati nelle fonti aperte (fonte sito aziendale / Impressum, 2024-2025). Firmenbuch FN 651815b, LG Innsbruck, UID ATU82121605. Iscritta WKO Tirol come 'Futtermittelerzeuger', 'Handel mit Futtermitteln' e 'Großhandel mit Lebensmitteln'. Uno dei pochi mulini + mangimifici austriaci ancora totalmente in mani private; il Futterwerk produce mangimi per bovini, pollame, suini, cavalli, ovicaprini e selvaggina (componenti proteiche a base di soia). Prokuristin: Mag. Caroline Krainz-Gasteiger.</t>
+          <t>PMI con oltre 25-30 anni di attività; fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at, WKO Firmen A-Z, advantageaustria.org, 2024-2025). Sedi/operatività a Schrems, Gmünd e St. Pölten (Bassa Austria). Grossista austriaco leader di ingredienti alimentari biologici certificati per trasformatori industriali e artigianali: a catalogo BIO-Palmfett/olio di palma in Großgebinde (fusti/grandi formati), oltre a cacao e caffè — tre commodity dell'Allegato I EUDR nello stesso portafoglio, quindi lead multi-commodity.</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Mag. Lukas Krainz</t>
+          <t>Ing. Mag. Robert Zach</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Geschäftsführer und 100%iger Anteilseigner</t>
+          <t>Geschäftsführer (alleinvertretungsberechtigt) e proprietario</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr"/>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>info@wieshofermuehle.at</t>
+          <t>zach@bioservice.at</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>https://www.wieshofermuehle.at</t>
+          <t>https://www.bioservice.at</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>St. Johann in Tirol, Tirolo (Tirol)</t>
+          <t>Schrems (Wirtschaftspark 1), Bassa Austria (Niederösterreich)</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>https://www.wieshofermuehle.at/de/impressum</t>
+          <t>https://www.bioservice.at/en/products/organic-palm-fat-oil/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>BIOSERVICE Zach Ges.m.b.H.</t>
+          <t>Natural Products &amp; Drugs GmbH</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — grossista ingredienti bio</t>
+          <t>Olio di palma — commercio oli e grassi vegetali</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>PMI con oltre 25-30 anni di attività; fatturato e organico non pubblicati nelle fonti aperte (fonti firmenabc.at, WKO Firmen A-Z, advantageaustria.org, 2024-2025). Sedi/operatività a Schrems, Gmünd e St. Pölten (Bassa Austria). Grossista austriaco leader di ingredienti alimentari biologici certificati per trasformatori industriali e artigianali: a catalogo BIO-Palmfett/olio di palma in Großgebinde (fusti/grandi formati), oltre a cacao e caffè — tre commodity dell'Allegato I EUDR nello stesso portafoglio, quindi lead multi-commodity.</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>Ing. Mag. Robert Zach</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>Geschäftsführer (alleinvertretungsberechtigt) e proprietario</t>
-        </is>
-      </c>
-      <c r="F87" s="3" t="inlineStr"/>
-      <c r="G87" s="4" t="inlineStr">
-        <is>
-          <t>zach@bioservice.at</t>
+          <t>PMI attiva a livello internazionale dal 2003, guidata da 2 Geschäftsführer (nomi non pubblicati nelle fonti consultate); fatturato e organico non pubblicati (fonti firmenabc.at, WKO Firmen A-Z, Creditreform, 2024-2025). Firmenbuch FN 283007m, LG Klagenfurt. Sede Neuer Platz 1, 9800 Spittal an der Drau; tel. +43 4762 44340. Società di produzione e commercio certificata ISO/Bio/Demeter con oltre 120 oli vegetali e grassi, oli essenziali, idrolati e materie prime per cosmetica e alimentare; compare tra i fornitori austriaci di Palmöl nella directory B2B wlw.at. NB: portafoglio in larga parte di oli NON Allegato I — il perimetro EUDR riguarda solo la linea olio di palma/palmisto: da qualificare in fase di contatto.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/natural-products-drugs-gmbh</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>https://www.bioservice.at</t>
+          <t>http://www.np-d.com</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Schrems (Wirtschaftspark 1), Bassa Austria (Niederösterreich)</t>
+          <t>Spittal an der Drau, Carinzia (Kärnten)</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>https://www.bioservice.at/en/products/organic-palm-fat-oil/</t>
+          <t>https://www.wlw.at/de/firma/natural-products-drugs-gmbh-958203</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Natural Products &amp; Drugs GmbH</t>
+          <t>Andrä Hörtnagl Produktion und Handel GmbH</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — commercio oli e grassi vegetali</t>
+          <t>Bovini/Carne — carni e salumi, filiale proprie</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>PMI attiva a livello internazionale dal 2003, guidata da 2 Geschäftsführer (nomi non pubblicati nelle fonti consultate); fatturato e organico non pubblicati (fonti firmenabc.at, WKO Firmen A-Z, Creditreform, 2024-2025). Firmenbuch FN 283007m, LG Klagenfurt. Sede Neuer Platz 1, 9800 Spittal an der Drau; tel. +43 4762 44340. Società di produzione e commercio certificata ISO/Bio/Demeter con oltre 120 oli vegetali e grassi, oli essenziali, idrolati e materie prime per cosmetica e alimentare; compare tra i fornitori austriaci di Palmöl nella directory B2B wlw.at. NB: portafoglio in larga parte di oli NON Allegato I — il perimetro EUDR riguarda solo la linea olio di palma/palmisto: da qualificare in fase di contatto.</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr"/>
-      <c r="E88" s="5" t="inlineStr"/>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/natural-products-drugs-gmbh</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>ca. 24-25 Mio. € fatturato, ca. 200-230 dipendenti, 2.700 t/anno (top.tirol / agrarexportfoerderung.de, 2020-2023); Bilanzsumme 14,15 Mio. € al 31.12.2024 (firmenabc.at)</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Fabian Peter Kolozs, B.A. M.A.</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Geschäftsführer</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>office@hoertnagl.at</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>http://www.np-d.com</t>
+          <t>https://www.hoertnagl.at/</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Spittal an der Drau, Carinzia (Kärnten)</t>
+          <t>Hall in Tirol, Tirol</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>https://www.wlw.at/de/firma/natural-products-drugs-gmbh-958203</t>
+          <t>https://www.firmenabc.at/andrae-hoertnagl-produktion-und-handel-gmbh_Cgt</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Andrä Hörtnagl Produktion und Handel GmbH</t>
+          <t>Fleischwaren Höllerschmid GmbH</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — carni e salumi, filiale proprie</t>
+          <t>Bovini/Carne — lavorazione carne bovina, dry-aged</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>ca. 24-25 Mio. € fatturato, ca. 200-230 dipendenti, 2.700 t/anno (top.tirol / agrarexportfoerderung.de, 2020-2023); Bilanzsumme 14,15 Mio. € al 31.12.2024 (firmenabc.at)</t>
+          <t>Bilanzsumme 6,2 Mio. € al 31.03.2025 (firmenabc.at); fatturato non pubblicato — lavora ca. 20 t di carne bovina e 5 t di suino a settimana; azienda familiare di media dimensione, ampliamento 2025 (+2.500 m²). Firmenbuch FN 254597h</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Fabian Peter Kolozs, B.A. M.A.</t>
+          <t>Manfred Höllerschmid</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -37278,47 +37274,51 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F89" s="3" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>https://at.linkedin.com/company/fleischwaren-h%C3%B6llerschmid-gmbh</t>
+        </is>
+      </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>office@hoertnagl.at</t>
+          <t>office@hoellerschmid.at</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>https://www.hoertnagl.at/</t>
+          <t>https://www.hoellerschmid.at/</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Hall in Tirol, Tirol</t>
+          <t>Walkersdorf am Kamp (Grafenegg), Niederösterreich</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/andrae-hoertnagl-produktion-und-handel-gmbh_Cgt</t>
+          <t>https://www.firmenabc.at/fleischwaren-hoellerschmid-gmbh_HbCr</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Fleischwaren Höllerschmid GmbH</t>
+          <t>M. Feköhrer GmbH &amp; Co KG</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — lavorazione carne bovina, dry-aged</t>
+          <t>Bovini/Carne — macello UE e commercio bestiame</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Bilanzsumme 6,2 Mio. € al 31.03.2025 (firmenabc.at); fatturato non pubblicato — lavora ca. 20 t di carne bovina e 5 t di suino a settimana; azienda familiare di media dimensione, ampliamento 2025 (+2.500 m²). Firmenbuch FN 254597h</t>
+          <t>ca. 40 Mio. € fatturato, 30 dipendenti (+4 veterinari, 3 classificatori); ca. 11.500 bovini e 54.000 suini macellati/anno — fonte sito aziendale (fekoehrer.at, 2025). NOTA: fatturato gonfiato dal costo materia prima, PMI con soli 30 addetti. Firmenbuch FN 663491y</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Manfred Höllerschmid</t>
+          <t>Michael Feköhrer</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -37326,51 +37326,47 @@
           <t>Geschäftsführer</t>
         </is>
       </c>
-      <c r="F90" s="6" t="inlineStr">
-        <is>
-          <t>https://at.linkedin.com/company/fleischwaren-h%C3%B6llerschmid-gmbh</t>
-        </is>
-      </c>
+      <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>office@hoellerschmid.at</t>
+          <t>office@fekoehrer.at</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>https://www.hoellerschmid.at/</t>
+          <t>https://www.fekoehrer.at/</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Walkersdorf am Kamp (Grafenegg), Niederösterreich</t>
+          <t>Mühlheim am Inn, Oberösterreich</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/fleischwaren-hoellerschmid-gmbh_HbCr</t>
+          <t>https://www.fekoehrer.at/impressum/</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>M. Feköhrer GmbH &amp; Co KG</t>
+          <t>Rudolf Frierss &amp; Söhne Fleisch- und Wurstspezialitäten Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macello UE e commercio bestiame</t>
+          <t>Bovini/Carne — lavorazione carni e salumi</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>ca. 40 Mio. € fatturato, 30 dipendenti (+4 veterinari, 3 classificatori); ca. 11.500 bovini e 54.000 suini macellati/anno — fonte sito aziendale (fekoehrer.at, 2025). NOTA: fatturato gonfiato dal costo materia prima, PMI con soli 30 addetti. Firmenbuch FN 663491y</t>
+          <t>ca. 110-120 dipendenti su due stabilimenti a Villach (frierss.at / feines-haus.at, 2025); fatturato non pubblicato. Azienda familiare dal 1898, 5ª generazione. Firmenbuch FN 114403 (LG Klagenfurt)</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Michael Feköhrer</t>
+          <t>Rudolf Frierss</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
@@ -37381,44 +37377,44 @@
       <c r="F91" s="3" t="inlineStr"/>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>office@fekoehrer.at</t>
+          <t>office@frierss.at</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>https://www.fekoehrer.at/</t>
+          <t>https://www.frierss.at/</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Mühlheim am Inn, Oberösterreich</t>
+          <t>Villach, Kärnten</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>https://www.fekoehrer.at/impressum/</t>
+          <t>https://www.firmenabc.at/rudolf-frierss-soehne-fleisch-und-wurstspezialitaeten-gmbh_BAtZF</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Rudolf Frierss &amp; Söhne Fleisch- und Wurstspezialitäten Gesellschaft m.b.H.</t>
+          <t>Schwaninger Vieh Export GmbH</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — lavorazione carni e salumi</t>
+          <t>Bovini/Carne — commercio ed export bestiame</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>ca. 110-120 dipendenti su due stabilimenti a Villach (frierss.at / feines-haus.at, 2025); fatturato non pubblicato. Azienda familiare dal 1898, 5ª generazione. Firmenbuch FN 114403 (LG Klagenfurt)</t>
+          <t>12 Mio. € fatturato netto 2021 e 11 Mio. € 2022, 5 dipendenti (firmenabc.at / unternehmen24.info). NOTA: fatturato gonfiato dal costo del bestiame, micro-impresa per addetti. Firmenbuch FN 37288k</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Rudolf Frierss</t>
+          <t>Erwin Schwaninger</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -37429,123 +37425,75 @@
       <c r="F92" s="5" t="inlineStr"/>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>office@frierss.at</t>
+          <t>office@schwaninger.co.at</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>https://www.frierss.at/</t>
+          <t>https://www.viehexport.com/</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Villach, Kärnten</t>
+          <t>Weer, Tirol</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/rudolf-frierss-soehne-fleisch-und-wurstspezialitaeten-gmbh_BAtZF</t>
+          <t>https://www.firmenabc.at/schwaninger-vieh-export-gmbh_EBAU</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Schwaninger Vieh Export GmbH</t>
+          <t>WIESTRADING Gesellschaft m.b.H.</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — commercio ed export bestiame</t>
+          <t>Bovini/Carne — commercio ed export bovini</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>12 Mio. € fatturato netto 2021 e 11 Mio. € 2022, 5 dipendenti (firmenabc.at / unternehmen24.info). NOTA: fatturato gonfiato dal costo del bestiame, micro-impresa per addetti. Firmenbuch FN 37288k</t>
+          <t>ca. 15.000-20.000 capi commercializzati/anno (wiestrading.at, 2025); fatturato e organico non pubblicati — azienda familiare alla 3ª generazione. Firmenbuch FN 143186v</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Erwin Schwaninger</t>
+          <t>Kurt Wiesinger</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Geschäftsführer</t>
+          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>office@schwaninger.co.at</t>
+          <t>wiesingerviehhandel@aon.at</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>https://www.viehexport.com/</t>
+          <t>https://www.wiestrading.at/</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>Weer, Tirol</t>
+          <t>Steegen (Peuerbach), Oberösterreich</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>https://www.firmenabc.at/schwaninger-vieh-export-gmbh_EBAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>WIESTRADING Gesellschaft m.b.H.</t>
-        </is>
-      </c>
-      <c r="B94" s="5" t="inlineStr">
-        <is>
-          <t>Bovini/Carne — commercio ed export bovini</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>ca. 15.000-20.000 capi commercializzati/anno (wiestrading.at, 2025); fatturato e organico non pubblicati — azienda familiare alla 3ª generazione. Firmenbuch FN 143186v</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Kurt Wiesinger</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>Geschäftsführer (alleinvertretungsberechtigt)</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr"/>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>wiesingerviehhandel@aon.at</t>
-        </is>
-      </c>
-      <c r="H94" s="6" t="inlineStr">
-        <is>
-          <t>https://www.wiestrading.at/</t>
-        </is>
-      </c>
-      <c r="I94" s="5" t="inlineStr">
-        <is>
-          <t>Steegen (Peuerbach), Oberösterreich</t>
-        </is>
-      </c>
-      <c r="J94" s="5" t="inlineStr">
-        <is>
           <t>https://www.firmenabc.at/wiestrading-ges-m-b-h_KDpS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J94"/>
+  <autoFilter ref="A2:J93"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -37644,25 +37592,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId93"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId115"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId116"/>
@@ -37671,91 +37619,88 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId129"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="rId135"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId137"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="rId143"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId155"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G71" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G77" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G78" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G79" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G80" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId193"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId194"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId203"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Belgio: rimossa Vandeputte Oleochemicals (lino, non olio di palma)
Caso identico a Immobra, gia' scartata dalla raccolta per lo stesso motivo. Il record
la classificava sotto la macro «Olio di palma», ma l'azienda non tratta palma:
«limits its seed-pressing activity to linseed (around 100.000 ton annually)», per
vernici, inchiostri, linoleum, adesivi, resine e trattamento del legno. Il gruppo
Vandeputte e' un riferimento mondiale del lino (>10% della produzione mondiale), che
NON e' commodity dell'Allegato I. La soia compare solo come standolio e olio
emulsionabile, cioe' derivati acquistati e modificati, non spremitura propria.

Trovata proseguendo la verifica direttamente via WebSearch dopo l'esaurimento della
quota per gli agenti.

Censimento da 736 a 735 aziende (Belgio 93->92).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28346,7 +28346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -32183,281 +32183,289 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>Vandeputte Oleochemicals SA</t>
+          <t>Baeten &amp; Co NV</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli vegetali (soia, lino)</t>
+          <t>Olio di palma — raffinazione oli e grassi vegetali/animali</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 34.266.885 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 18 FTE — taglia gonfiata dal costo materia prima; n. impresa BE 0471.546.593</t>
+          <t>Fatturato 42.810.588 EUR (bilancio NBB depositato 15-07-2025) — taglia gonfiata dal costo materia prima: solo 13,7 FTE; n. impresa BE 0447.081.908</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr"/>
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr"/>
-      <c r="G83" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>info@baetennv.be</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>https://www.vandeputte.com/en/oleochemicals/</t>
+          <t>https://baetennv.be/</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Mouscron (Hainaut, Wallonie)</t>
+          <t>Berlare (Overmere, Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/471546593/vandeputte-oleochemicals.aspx</t>
+          <t>https://www.companyweb.be/en/0447081908/baeten-co</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Baeten &amp; Co NV</t>
+          <t>Repro NV</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli e grassi vegetali/animali</t>
+          <t>Olio di palma — raffinazione oli e grassi vegetali</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 42.810.588 EUR (bilancio NBB depositato 15-07-2025) — taglia gonfiata dal costo materia prima: solo 13,7 FTE; n. impresa BE 0447.081.908</t>
+          <t>Fatturato 14.157.353 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 1-5 dipendenti (societa' di raffinazione del Group Vandamme); n. impresa BE 0439.000.818</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr"/>
       <c r="E84" s="5" t="inlineStr"/>
       <c r="F84" s="5" t="inlineStr"/>
-      <c r="G84" s="6" t="inlineStr">
-        <is>
-          <t>info@baetennv.be</t>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>https://baetennv.be/</t>
+          <t>https://www.groupvandamme.com/</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Berlare (Overmere, Oost-Vlaanderen)</t>
+          <t>Deinze (Oost-Vlaanderen)</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0447081908/baeten-co</t>
+          <t>https://trendstop.knack.be/nl/detail/439000818/repro.aspx</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Repro NV</t>
+          <t>Royale Lacroix SA</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione oli e grassi vegetali</t>
+          <t>Olio di palma — margarine e grassi alimentari</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 14.157.353 EUR (Trends Top/NBB, ultimo esercizio pubblicato); 1-5 dipendenti (societa' di raffinazione del Group Vandamme); n. impresa BE 0439.000.818</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr"/>
-      <c r="E85" s="3" t="inlineStr"/>
-      <c r="F85" s="3" t="inlineStr"/>
-      <c r="G85" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Fatturato 49.349.520 EUR (bilancio NBB, ultimo esercizio pubblicato) — taglia gonfiata dal costo materia prima: solo 18,6 FTE; n. impresa BE 0404.423.583</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Patrice Lacroix</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>Administrateur délégué</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>https://be.linkedin.com/company/royale-lacroix</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>info@royalelacroix.be</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>https://www.groupvandamme.com/</t>
+          <t>https://www.royalelacroix.com/</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Deinze (Oost-Vlaanderen)</t>
+          <t>Flémalle (Liège, Wallonie)</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/439000818/repro.aspx</t>
+          <t>https://www.companyweb.be/en/0404423583/royale-lacroix</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Royale Lacroix SA</t>
+          <t>Ameloot BV</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — margarine e grassi alimentari</t>
+          <t>Bovini/Carne — macellazione e ingrosso</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 49.349.520 EUR (bilancio NBB, ultimo esercizio pubblicato) — taglia gonfiata dal costo materia prima: solo 18,6 FTE; n. impresa BE 0404.423.583</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>Patrice Lacroix</t>
-        </is>
-      </c>
-      <c r="E86" s="5" t="inlineStr">
-        <is>
-          <t>Administrateur délégué</t>
-        </is>
-      </c>
-      <c r="F86" s="6" t="inlineStr">
-        <is>
-          <t>https://be.linkedin.com/company/royale-lacroix</t>
-        </is>
-      </c>
+          <t>Fatturato 49.298.205 EUR (Trends Top/NBB, ultimo esercizio); n. impresa BE 0413.029.562. AZIENDA DI CONFINE: sopra i 40 M€ ma PMI familiare indipendente (3a generazione) con macello integrato SGL; dal 2024 controlla Slachtgroep Leieland BV; fatturato gonfiato dal costo materia prima.</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr"/>
+      <c r="E86" s="5" t="inlineStr"/>
+      <c r="F86" s="5" t="inlineStr"/>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>info@royalelacroix.be</t>
+          <t>petra@ameloot.org</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>https://www.royalelacroix.com/</t>
+          <t>https://omerameloot.com/nl</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Flémalle (Liège, Wallonie)</t>
+          <t>Harelbeke (West-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/en/0404423583/royale-lacroix</t>
+          <t>https://trendstop.knack.be/nl/detail/413029562/ameloot.aspx</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Ameloot BV</t>
+          <t>Dierickx NV</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione e ingrosso</t>
+          <t>Bovini/Carne — sezionamento carne bovina</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 49.298.205 EUR (Trends Top/NBB, ultimo esercizio); n. impresa BE 0413.029.562. AZIENDA DI CONFINE: sopra i 40 M€ ma PMI familiare indipendente (3a generazione) con macello integrato SGL; dal 2024 controlla Slachtgroep Leieland BV; fatturato gonfiato dal costo materia prima.</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr"/>
-      <c r="E87" s="3" t="inlineStr"/>
+          <t>Fatturato 40.843.828 EUR (ultimo bilancio depositato NBB, via Trends Top/Companyweb); azienda familiare indipendente alla 5a generazione; n. impresa BE 0422.204.673. Al limite alto della fascia: nella carne il fatturato e' gonfiato dal costo della materia prima.</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Cis van den Broeck</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Zaakvoerder</t>
+        </is>
+      </c>
       <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>petra@ameloot.org</t>
+          <t>info@dierickxnv.be</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>https://omerameloot.com/nl</t>
+          <t>https://dierickxnv.be/</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Harelbeke (West-Vlaanderen, Fiandre)</t>
+          <t>Zele (Oost-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/413029562/ameloot.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/422204673/dierickx.aspx</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Dierickx NV</t>
+          <t>Euro Meat Group NV</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — sezionamento carne bovina</t>
+          <t>Bovini/Carne — macellazione bovini</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 40.843.828 EUR (ultimo bilancio depositato NBB, via Trends Top/Companyweb); azienda familiare indipendente alla 5a generazione; n. impresa BE 0422.204.673. Al limite alto della fascia: nella carne il fatturato e' gonfiato dal costo della materia prima.</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>Cis van den Broeck</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Zaakvoerder</t>
-        </is>
-      </c>
+          <t>Fatturato ca. 11 milioni EUR (VILT, stampa settoriale agroalimentare belga); organico ca. 50 persone (40 operai + 10 impiegati); capacita' 75.000 bovini ed equini/anno, ca. 125.000 bovini macellati per conto terzi. Numero d'impresa BE non verificato su fonte pubblica. Fa parte del gruppo Cadus NV (macelli in Belgio) ed e' socio Febev.</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr"/>
+      <c r="E88" s="5" t="inlineStr"/>
       <c r="F88" s="5" t="inlineStr"/>
-      <c r="G88" s="6" t="inlineStr">
-        <is>
-          <t>info@dierickxnv.be</t>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>https://dierickxnv.be/</t>
+          <t>http://www.euromeatgroup.be/nl/home/</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Zele (Oost-Vlaanderen, Fiandre)</t>
+          <t>Moeskroen / Mouscron (Hainaut, Vallonia)</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/422204673/dierickx.aspx</t>
+          <t>https://vilt.be/nl/nieuws/vijf-vleesspecialisten-nemen-familiebedrijf-derwa-over</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Euro Meat Group NV</t>
+          <t>Jos Leemput BV</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione bovini</t>
+          <t>Bovini/Carne — commercio all'ingrosso e sezionamento</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 11 milioni EUR (VILT, stampa settoriale agroalimentare belga); organico ca. 50 persone (40 operai + 10 impiegati); capacita' 75.000 bovini ed equini/anno, ca. 125.000 bovini macellati per conto terzi. Numero d'impresa BE non verificato su fonte pubblica. Fa parte del gruppo Cadus NV (macelli in Belgio) ed e' socio Febev.</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr"/>
-      <c r="E89" s="3" t="inlineStr"/>
+          <t>Fatturato 44.954.796 EUR e 16,2 FTE (ultimo bilancio depositato NBB, via Companyweb/FinCheck); n. impresa BE 0424.110.724. AZIENDA DI CONFINE: sopra 40 M€ ma con soli 16 dipendenti - caso tipico di fatturato gonfiato dal costo della materia prima; PMI familiare indipendente.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Jos Leemput</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>Titolare, responsabile acquisto e selezione bestiame (sito aziendale)</t>
+        </is>
+      </c>
       <c r="F89" s="3" t="inlineStr"/>
       <c r="G89" s="3" t="inlineStr">
         <is>
@@ -32466,170 +32474,162 @@
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>http://www.euromeatgroup.be/nl/home/</t>
+          <t>https://www.leemput.be/</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Moeskroen / Mouscron (Hainaut, Vallonia)</t>
+          <t>Tienen / Hakendover (Vlaams-Brabant, Fiandre)</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>https://vilt.be/nl/nieuws/vijf-vleesspecialisten-nemen-familiebedrijf-derwa-over</t>
+          <t>https://trendstop.knack.be/nl/detail/424110724/leemput-jos.aspx</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Jos Leemput BV</t>
+          <t>Slachthuis Swaegers NV</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — commercio all'ingrosso e sezionamento</t>
+          <t>Bovini/Carne — macellazione e sezionamento bovini</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Fatturato 44.954.796 EUR e 16,2 FTE (ultimo bilancio depositato NBB, via Companyweb/FinCheck); n. impresa BE 0424.110.724. AZIENDA DI CONFINE: sopra 40 M€ ma con soli 16 dipendenti - caso tipico di fatturato gonfiato dal costo della materia prima; PMI familiare indipendente.</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>Jos Leemput</t>
-        </is>
-      </c>
-      <c r="E90" s="5" t="inlineStr">
-        <is>
-          <t>Titolare, responsabile acquisto e selezione bestiame (sito aziendale)</t>
-        </is>
-      </c>
+          <t>Fatturato 4.287.787 EUR e 4,8 FTE nella societa' di macellazione (ultimo bilancio NBB, via Companyweb/Trends Top); n. impresa BE 0436.764.571. SOTTO LA SOGLIA dei 5 M€ come singola entita': il fatturato riflette solo i servizi di macellazione: il gruppo familiare Swaegers &amp; Co dichiara 70.000 bovini/anno e 22.000 t di capacita' annua, quindi volumi EUDR molto superiori al fatturato contabile.</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr"/>
       <c r="F90" s="5" t="inlineStr"/>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>info@swaegers.be</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>https://www.leemput.be/</t>
+          <t>https://www.swaegers.be/</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Tienen / Hakendover (Vlaams-Brabant, Fiandre)</t>
+          <t>Hoogstraten (Antwerpen, Fiandre)</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/424110724/leemput-jos.aspx</t>
+          <t>https://trendstop.knack.be/nl/detail/436764571/swaegers-slachthuis.aspx</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Slachthuis Swaegers NV</t>
+          <t>Slachthuis Velzeke BV</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione e sezionamento bovini</t>
+          <t>Bovini/Carne — macellazione bovini</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 4.287.787 EUR e 4,8 FTE nella societa' di macellazione (ultimo bilancio NBB, via Companyweb/Trends Top); n. impresa BE 0436.764.571. SOTTO LA SOGLIA dei 5 M€ come singola entita': il fatturato riflette solo i servizi di macellazione: il gruppo familiare Swaegers &amp; Co dichiara 70.000 bovini/anno e 22.000 t di capacita' annua, quindi volumi EUDR molto superiori al fatturato contabile.</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr"/>
-      <c r="E91" s="3" t="inlineStr"/>
+          <t>50-99 dipendenti (Companyweb, dati piu' recenti); capacita' 2.000 bovini/settimana, uno dei maggiori macelli bovini del Belgio; n. impresa BE 1018.071.121. Fatturato NON disponibile: entita' costituita il 30/12/2024 (cambio di proprieta' nel 2025), nessun bilancio con cifra d'affari ancora depositato. Altri amministratori indicati: Guy De Bruycker, Johan Castelein.</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Wouter Cokelaere</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Bestuurder</t>
+        </is>
+      </c>
       <c r="F91" s="3" t="inlineStr"/>
-      <c r="G91" s="4" t="inlineStr">
-        <is>
-          <t>info@swaegers.be</t>
-        </is>
-      </c>
-      <c r="H91" s="4" t="inlineStr">
-        <is>
-          <t>https://www.swaegers.be/</t>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Hoogstraten (Antwerpen, Fiandre)</t>
+          <t>Velzeke-Ruddershove, Zottegem (Oost-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/nl/detail/436764571/swaegers-slachthuis.aspx</t>
+          <t>https://www.companyweb.be/nl/1018071121/slachthuis-velzeke</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Slachthuis Velzeke BV</t>
+          <t>Sopraco NV</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macellazione bovini</t>
+          <t>Bovini/Carne — fornitura e ingrosso carni</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>50-99 dipendenti (Companyweb, dati piu' recenti); capacita' 2.000 bovini/settimana, uno dei maggiori macelli bovini del Belgio; n. impresa BE 1018.071.121. Fatturato NON disponibile: entita' costituita il 30/12/2024 (cambio di proprieta' nel 2025), nessun bilancio con cifra d'affari ancora depositato. Altri amministratori indicati: Guy De Bruycker, Johan Castelein.</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>Wouter Cokelaere</t>
-        </is>
-      </c>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>Bestuurder</t>
-        </is>
-      </c>
+          <t>Fatturato 8.889.508 EUR e 45,5 FTE (ultimo bilancio depositato NBB, via Companyweb/Trends Top); n. impresa BE 0507.988.901. Nella fascia bassa tollerata (5-40 M€). Capofila del gruppo familiare Sopraco, che dal 2017 controlla anche Rompa Leder (filiera pelle): doppia esposizione EUDR bovini + pelle.</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr"/>
+      <c r="E92" s="5" t="inlineStr"/>
       <c r="F92" s="5" t="inlineStr"/>
-      <c r="G92" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H92" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G92" s="6" t="inlineStr">
+        <is>
+          <t>info@sopraco.eu</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sopraco.eu/</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Velzeke-Ruddershove, Zottegem (Oost-Vlaanderen, Fiandre)</t>
+          <t>Geel (Antwerpen, Fiandre)</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>https://www.companyweb.be/nl/1018071121/slachthuis-velzeke</t>
+          <t>https://trendstop.knack.be/en/detail/507988901/sopraco.aspx</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Sopraco NV</t>
+          <t>Van De Walle SRL</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — fornitura e ingrosso carni</t>
+          <t>Bovini/Carne — commercio all'ingrosso</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Fatturato 8.889.508 EUR e 45,5 FTE (ultimo bilancio depositato NBB, via Companyweb/Trends Top); n. impresa BE 0507.988.901. Nella fascia bassa tollerata (5-40 M€). Capofila del gruppo familiare Sopraco, che dal 2017 controlla anche Rompa Leder (filiera pelle): doppia esposizione EUDR bovini + pelle.</t>
+          <t>n. impresa BE 0893.625.564 (Trends Top). Fatturato e organico NON pubblicati in forma accessibile (schema abbreviato NBB): azienda familiare fondata nel 1954, filiera verticalizzata dall'allevamento alla consegna con flotta frigo propria, clientela di macellerie e GDO. Dimensione stimabile come PMI, da verificare sul bilancio NBB.</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr"/>
@@ -32637,107 +32637,67 @@
       <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>info@sopraco.eu</t>
+          <t>info@vdw-grossisteenviande.be</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>https://www.sopraco.eu/</t>
+          <t>https://vdw-grossisteenviande.be/</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>Geel (Antwerpen, Fiandre)</t>
+          <t>Wayaux / Villers-Perwin, Les Bons Villers (Hainaut, Vallonia)</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>https://trendstop.knack.be/en/detail/507988901/sopraco.aspx</t>
+          <t>https://trendstop.levif.be/fr/detail/893625564/van-de-walle.aspx</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Van De Walle SRL</t>
+          <t>Vleeshandel Vens NV</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — commercio all'ingrosso</t>
+          <t>Bovini/Carne — ingrosso e sezionamento</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>n. impresa BE 0893.625.564 (Trends Top). Fatturato e organico NON pubblicati in forma accessibile (schema abbreviato NBB): azienda familiare fondata nel 1954, filiera verticalizzata dall'allevamento alla consegna con flotta frigo propria, clientela di macellerie e GDO. Dimensione stimabile come PMI, da verificare sul bilancio NBB.</t>
+          <t>32 FTE in bilancio (oltre 40 collaboratori secondo il sito aziendale); fatturato NON pubblicato (schema abbreviato NBB), margine lordo dichiarato 1.950.416 EUR; n. impresa BE 0468.329.064. Azienda familiare dal 1975; tratta rundsvlees, kalfsvlees, varkensvlees e lamsvlees.</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr"/>
       <c r="E94" s="5" t="inlineStr"/>
       <c r="F94" s="5" t="inlineStr"/>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>info@vdw-grossisteenviande.be</t>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>https://vdw-grossisteenviande.be/</t>
+          <t>https://vleeshandelvens.be/</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Wayaux / Villers-Perwin, Les Bons Villers (Hainaut, Vallonia)</t>
+          <t>Lendelede (West-Vlaanderen, Fiandre)</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>https://trendstop.levif.be/fr/detail/893625564/van-de-walle.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="3" t="inlineStr">
-        <is>
-          <t>Vleeshandel Vens NV</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>Bovini/Carne — ingrosso e sezionamento</t>
-        </is>
-      </c>
-      <c r="C95" s="3" t="inlineStr">
-        <is>
-          <t>32 FTE in bilancio (oltre 40 collaboratori secondo il sito aziendale); fatturato NON pubblicato (schema abbreviato NBB), margine lordo dichiarato 1.950.416 EUR; n. impresa BE 0468.329.064. Azienda familiare dal 1975; tratta rundsvlees, kalfsvlees, varkensvlees e lamsvlees.</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr"/>
-      <c r="E95" s="3" t="inlineStr"/>
-      <c r="F95" s="3" t="inlineStr"/>
-      <c r="G95" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>https://vleeshandelvens.be/</t>
-        </is>
-      </c>
-      <c r="I95" s="3" t="inlineStr">
-        <is>
-          <t>Lendelede (West-Vlaanderen, Fiandre)</t>
-        </is>
-      </c>
-      <c r="J95" s="3" t="inlineStr">
-        <is>
           <t>https://www.companyweb.be/en/0468329064/vleeshandel-vens</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J95"/>
+  <autoFilter ref="A2:J94"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -32927,26 +32887,25 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId187"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId195"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId196"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId203"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId205"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Olanda: rimossa Marandi (produzione cessata nel 2014, fabbrica demolita nel 2022)
Rilevata da Lonka nel 2010, produzione di nougat e cioccolato a Lunteren cessata a
inizio 2014 e trasferita alla capogruppo a Roosendaal. La fabbrica di Klomperweg 69
e' stata demolita nel 2022 e sull'area sorge il complesso residenziale «Marandi
Staete». Il record riportava invece «21-50 dipendenti (2025)» a quell'indirizzo.
Precedente: Getama Danmark, rimossa perche' «non e' piu' un produttore, quindi non
e' un operatore EUDR».

olanda_05 completo: 24 rilievi, 5 alta. Altri due casi rilevanti lasciati come
rilievo aperto: Chocolatemakers (fusione con Hands Off in The Chocolate Impact
Group, annuncio 31/03/2026) e Continental Chocolate (controllata del gruppo belga
Baronie dal 2009, non dichiarato).

Censimento da 731 a 730 aziende.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Finlandia'!$A$2:$J$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danimarca'!$A$2:$J$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Svezia'!$A$2:$J$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Olanda'!$A$2:$J$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Belgio'!$A$2:$J$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Austria'!$A$2:$J$92</definedName>
   </definedNames>
@@ -23170,7 +23170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -26499,313 +26499,313 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>Chocolade- en Suikerwerkfabriek Marandi B.V.</t>
+          <t>Chocoladefabriek "De Beemster" B.V.</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — lavorazione cacao e cioccolato</t>
+          <t>Cacao/Cioccolato — cioccolato e frutta secca ricoperta</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. 21-50 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 09065319. Sede Klomperweg 69, Lunteren. Attività registrata: verwerking van cacao + vervaardiging van chocolade en suikerwerk (lavorazione diretta del cacao, quindi rilevante EUDR).</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr"/>
+          <t>Fatturato non pubblicato; stime terze indicano meno di 5 M$ e 11-50 dipendenti (fonte: ZoomInfo / company.info, 2025). KVK 37109862. Membro VBZ. Nota: sotto la soglia ideale 10-20 M€, tenuta per copertura del segmento produzione cioccolato.</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Jos Klijnsma</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Algemeen directeur (general manager)</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/chocoladefabriek-'de-beemster'-b.v.</t>
+        </is>
+      </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.chocobeemster.nl/</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>Lunteren / Ede (Gelderland)</t>
+          <t>Middenbeemster / Purmerend (Noord-Holland)</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>https://www.oozo.nl/bedrijven/ede/lunteren/centrum-lunteren/365228/chocolade-en-suikerwerkfabriek-marandi-b-v</t>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/chocoladefabriek-de-beemster-b-v-middenbeemster-37109862-000020449763</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Chocoladefabriek "De Beemster" B.V.</t>
+          <t>Chocolatemakers B.V.</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — cioccolato e frutta secca ricoperta</t>
+          <t>Cacao/Cioccolato — cioccolato bean-to-bar</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato; stime terze indicano meno di 5 M$ e 11-50 dipendenti (fonte: ZoomInfo / company.info, 2025). KVK 37109862. Membro VBZ. Nota: sotto la soglia ideale 10-20 M€, tenuta per copertura del segmento produzione cioccolato.</t>
+          <t>Fatturato ~4 M€ (fonte: MT/Sprout, articolo sulla fusione con Hands Off, 2025). KVK 57652066. SBI verwerking van cacao. Fabbrica bean-to-bar nel porto di Amsterdam, importa direttamente fave da Congo, Perù e Rep. Dominicana: operatore EUDR. Nota: sotto la fascia 5-40 M€, tenuta per copertura del segmento bean-to-bar.</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Jos Klijnsma</t>
+          <t>Enver Loke</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Algemeen directeur (general manager)</t>
-        </is>
-      </c>
-      <c r="F72" s="6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/chocoladefabriek-'de-beemster'-b.v.</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Oprichter (co-fondatore)</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>info@chocolatemakers.nl</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>https://www.chocobeemster.nl/</t>
+          <t>https://www.chocolatemakers.com/</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Middenbeemster / Purmerend (Noord-Holland)</t>
+          <t>Amsterdam (Noord-Holland)</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/chocoladefabriek-de-beemster-b-v-middenbeemster-37109862-000020449763</t>
+          <t>https://companyinfo.nl/organisatieprofiel/verwerking-van-cacao/chocolatemakers-b-v-amsterdam-57652066-000022805583</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>Chocolatemakers B.V.</t>
+          <t>Continental Chocolate B.V.</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — cioccolato bean-to-bar</t>
+          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ~4 M€ (fonte: MT/Sprout, articolo sulla fusione con Hands Off, 2025). KVK 57652066. SBI verwerking van cacao. Fabbrica bean-to-bar nel porto di Amsterdam, importa direttamente fave da Congo, Perù e Rep. Dominicana: operatore EUDR. Nota: sotto la fascia 5-40 M€, tenuta per copertura del segmento bean-to-bar.</t>
+          <t>Fatturato non pubblicato. 20-49 dipendenti (fonte: transfirm.nl / Dun &amp; Bradstreet, dati KVK 2025). KVK 34146292. Costituita nel 2000. Sede Galvanistraat 10, Rotterdam. Produzione di cioccolato e prodotti dolciari a base di cacao.</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Enver Loke</t>
+          <t>Johannes M.C.G. van Logtestijn</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Oprichter (co-fondatore)</t>
+          <t>Bestuurder / key principal</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr"/>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>info@chocolatemakers.nl</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>https://www.chocolatemakers.com/</t>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Amsterdam (Noord-Holland)</t>
+          <t>Rotterdam (Zuid-Holland)</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/verwerking-van-cacao/chocolatemakers-b-v-amsterdam-57652066-000022805583</t>
+          <t>https://transfirm.nl/nl/organisatie/341462920000-continental-chocolate-b.v.?lang=en</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Continental Chocolate B.V.</t>
+          <t>De Chocoladefabriek B.V.</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
+          <t>Cacao/Cioccolato — produzione cioccolato retail</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. 20-49 dipendenti (fonte: transfirm.nl / Dun &amp; Bradstreet, dati KVK 2025). KVK 34146292. Costituita nel 2000. Sede Galvanistraat 10, Rotterdam. Produzione di cioccolato e prodotti dolciari a base di cacao.</t>
+          <t>Fatturato non pubblicato; ~30 dipendenti (fonte: Het Ondernemersbelang, articolo sull'emissione NPEX di max 3 M€ in certificati di azioni preferenziali cumulative). KVK 37032938. Produttore di cioccolato per il retail olandese (HEMA, catene di supermercati). Probabilmente sotto la fascia ideale ma rilevante come operatore EUDR sul cioccolato.</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Johannes M.C.G. van Logtestijn</t>
+          <t>Hans Neef</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Bestuurder / key principal</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr"/>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>Directeur / eigenaar</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/dechocoladefabriek</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>info@dechocoladefabriek.nl</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>https://www.dechocoladefabriek.nl/</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Rotterdam (Zuid-Holland)</t>
+          <t>Heerhugowaard / Dijk en Waard (Noord-Holland)</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>https://transfirm.nl/nl/organisatie/341462920000-continental-chocolate-b.v.?lang=en</t>
+          <t>https://www.ondernemersbelang.nl/nieuws/de-chocoladefabriek-naar-npex-beurs-met-certificaten/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>De Chocoladefabriek B.V.</t>
+          <t>De Euforij Chocolade B.V.</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — produzione cioccolato retail</t>
+          <t>Cacao/Cioccolato — cioccolato da semilavorati cacao</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato; ~30 dipendenti (fonte: Het Ondernemersbelang, articolo sull'emissione NPEX di max 3 M€ in certificati di azioni preferenziali cumulative). KVK 37032938. Produttore di cioccolato per il retail olandese (HEMA, catene di supermercati). Probabilmente sotto la fascia ideale ma rilevante come operatore EUDR sul cioccolato.</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>Hans Neef</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>Directeur / eigenaar</t>
-        </is>
-      </c>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 61954578. Costituita nel 2014, sede Zaandijkerweg 1, Wormerveer (cluster cacao Zaanstreek). Produce cioccolato partendo da massa di cacao, burro di cacao e cacao in polvere (semilavorati Allegato I EUDR). Nota: micro/piccola impresa, sotto la fascia 5-40 M€, tenuta per copertura del cluster Zaanstreek.</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/dechocoladefabriek</t>
+          <t>https://nl.linkedin.com/company/de-euforij-chocolade-b-v-</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>info@dechocoladefabriek.nl</t>
+          <t>chocolade@euforij.nl</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>https://www.dechocoladefabriek.nl/</t>
+          <t>https://www.euforij.nl/</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Heerhugowaard / Dijk en Waard (Noord-Holland)</t>
+          <t>Wormerveer / Zaanstad (Noord-Holland)</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>https://www.ondernemersbelang.nl/nieuws/de-chocoladefabriek-naar-npex-beurs-met-certificaten/</t>
+          <t>https://www.bedrijvenregister.nl/wormerveer/de-euforij-chocolade-bv</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>De Euforij Chocolade B.V.</t>
+          <t>Martinez Chocolade B.V.</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — cioccolato da semilavorati cacao</t>
+          <t>Cacao/Cioccolato — bonbon e cioccolato</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 61954578. Costituita nel 2014, sede Zaandijkerweg 1, Wormerveer (cluster cacao Zaanstreek). Produce cioccolato partendo da massa di cacao, burro di cacao e cacao in polvere (semilavorati Allegato I EUDR). Nota: micro/piccola impresa, sotto la fascia 5-40 M€, tenuta per copertura del cluster Zaanstreek.</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr"/>
-      <c r="E76" s="5" t="inlineStr"/>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>https://nl.linkedin.com/company/de-euforij-chocolade-b-v-</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>chocolade@euforij.nl</t>
+          <t>Fatturato non pubblicato. 8 dipendenti (6-10 secondo KVK) (fonte: transfirm.nl / oozo.nl, dati KVK 2025). KVK 34128566. Membro VBZ. Nota: nettamente sotto la fascia 5-40 M€, tenuta per copertura del segmento cioccolateria.</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>X. Stam</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>https://www.euforij.nl/</t>
+          <t>https://www.martinezchocolade.nl/</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Wormerveer / Zaanstad (Noord-Holland)</t>
+          <t>Amstelveen (Noord-Holland)</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>https://www.bedrijvenregister.nl/wormerveer/de-euforij-chocolade-bv</t>
+          <t>https://www.transfirm.nl/nl/organisatie/341285660000-martinez-chocolade-b.v.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Martinez Chocolade B.V.</t>
+          <t>Original Beans B.V.</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — bonbon e cioccolato</t>
+          <t>Cacao/Cioccolato — cacao fine e cioccolato premium</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. 8 dipendenti (6-10 secondo KVK) (fonte: transfirm.nl / oozo.nl, dati KVK 2025). KVK 34128566. Membro VBZ. Nota: nettamente sotto la fascia 5-40 M€, tenuta per copertura del segmento cioccolateria.</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>X. Stam</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>Algemeen directeur</t>
-        </is>
-      </c>
+          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 50770764. Sede Mauritskade 64, Amsterdam. Attività registrata: acquisto di fave di cacao per la produzione di cioccolato (in conto terzi), rivendita e commercio all'ingrosso di cioccolato — quindi operatore EUDR sull'import di cacao. Dimensione presumibilmente sotto la fascia 5-40 M€: tenuta per copertura del segmento cacao fine.</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr"/>
+      <c r="E77" s="3" t="inlineStr"/>
       <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" s="3" t="inlineStr">
         <is>
@@ -26814,34 +26814,34 @@
       </c>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>https://www.martinezchocolade.nl/</t>
+          <t>https://originalbeans.com/</t>
         </is>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
-          <t>Amstelveen (Noord-Holland)</t>
+          <t>Amsterdam (Noord-Holland)</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>https://www.transfirm.nl/nl/organisatie/341285660000-martinez-chocolade-b.v.</t>
+          <t>https://www.bedrijvenregister.nl/amsterdam/original-beans</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Original Beans B.V.</t>
+          <t>Ringers' Import B.V.</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — cacao fine e cioccolato premium</t>
+          <t>Cacao/Cioccolato — import/ingrosso cioccolato</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato; n. dipendenti non pubblicato. KVK 50770764. Sede Mauritskade 64, Amsterdam. Attività registrata: acquisto di fave di cacao per la produzione di cioccolato (in conto terzi), rivendita e commercio all'ingrosso di cioccolato — quindi operatore EUDR sull'import di cacao. Dimensione presumibilmente sotto la fascia 5-40 M€: tenuta per copertura del segmento cacao fine.</t>
+          <t>Fatturato non pubblicato. 11-20 dipendenti (fonte: oozo.nl / graydongo.nl, dati KVK, 2025). KVK 18049029. Sede Ir. Lelyweg 49, Haarlem. Attività: groothandel in suiker, chocolade en suikerwerk — importatore/commerciante di cioccolato, quindi soggetto EUDR come operatore o trader.</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr"/>
@@ -26854,34 +26854,34 @@
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>https://originalbeans.com/</t>
+          <t>http://www.ringersimport.nl/</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Amsterdam (Noord-Holland)</t>
+          <t>Haarlem (Noord-Holland)</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>https://www.bedrijvenregister.nl/amsterdam/original-beans</t>
+          <t>https://www.oozo.nl/bedrijven/haarlem/waarder-en-veerpolder/waarderpolder/171566/ringers-import-b-v</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Ringers' Import B.V.</t>
+          <t>Rousseau Chocolade B.V.</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — import/ingrosso cioccolato</t>
+          <t>Cacao/Cioccolato — produzione cioccolato e praline</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. 11-20 dipendenti (fonte: oozo.nl / graydongo.nl, dati KVK, 2025). KVK 18049029. Sede Ir. Lelyweg 49, Haarlem. Attività: groothandel in suiker, chocolade en suikerwerk — importatore/commerciante di cioccolato, quindi soggetto EUDR come operatore o trader.</t>
+          <t>Fatturato non pubblicato. 54 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 14002870. Costituita nel 1955. SBI vervaardiging van chocolade en suikerwerk. Sede Langs de Heij 11, Sittard. Per organico plausibilmente nella fascia 10-20 M€, ma il fatturato non è depositato pubblicamente.</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr"/>
@@ -26892,365 +26892,377 @@
           <t>n.d.</t>
         </is>
       </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>http://www.ringersimport.nl/</t>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
-          <t>Haarlem (Noord-Holland)</t>
+          <t>Sittard / Sittard-Geleen (Limburg)</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>https://www.oozo.nl/bedrijven/haarlem/waarder-en-veerpolder/waarderpolder/171566/ringers-import-b-v</t>
+          <t>https://www.oozo.nl/bedrijven/sittard-geleen/overhoven/industrieterrein-noord/365188/rousseau-chocolade-b-v</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Rousseau Chocolade B.V.</t>
+          <t>Steenland Chocolate B.V.</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — produzione cioccolato e praline</t>
+          <t>Cacao/Cioccolato — produzione cioccolato (monete/medaglie)</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. 54 dipendenti (fonte: oozo.nl, dati KVK, 2025). KVK 14002870. Costituita nel 1955. SBI vervaardiging van chocolade en suikerwerk. Sede Langs de Heij 11, Sittard. Per organico plausibilmente nella fascia 10-20 M€, ma il fatturato non è depositato pubblicamente.</t>
+          <t>Fatturato non pubblicato (deposito abbreviato). 51-100 dipendenti, indicati 55-67 fissi e fino a ~150 in alta stagione (fonte: oozo.nl / graydongo.nl, dati KVK 2025). KVK 24354029. Produttore leader mondiale di monete e medaglioni di cioccolato personalizzati, export in oltre 50 paesi. Nota gruppo: dal 2017 controllata da Sino-Pacific Trading Co. Ltd. Per organico si colloca nella fascia alta del target.</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr"/>
       <c r="E80" s="5" t="inlineStr"/>
-      <c r="F80" s="5" t="inlineStr"/>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/steenland-chocolate</t>
+        </is>
+      </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
           <t>n.d.</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>https://www.steenland.nl/</t>
         </is>
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Sittard / Sittard-Geleen (Limburg)</t>
+          <t>Gouda (Zuid-Holland)</t>
         </is>
       </c>
       <c r="J80" s="5" t="inlineStr">
         <is>
-          <t>https://www.oozo.nl/bedrijven/sittard-geleen/overhoven/industrieterrein-noord/365188/rousseau-chocolade-b-v</t>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/steenland-chocolate-b-v-gouda-24354029-000018029809</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>Steenland Chocolate B.V.</t>
+          <t>Trianon Chocolatiers B.V.</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — produzione cioccolato (monete/medaglie)</t>
+          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (deposito abbreviato). 51-100 dipendenti, indicati 55-67 fissi e fino a ~150 in alta stagione (fonte: oozo.nl / graydongo.nl, dati KVK 2025). KVK 24354029. Produttore leader mondiale di monete e medaglioni di cioccolato personalizzati, export in oltre 50 paesi. Nota gruppo: dal 2017 controllata da Sino-Pacific Trading Co. Ltd. Per organico si colloca nella fascia alta del target.</t>
+          <t>Fatturato non pubblicato. La consociata operativa Trianon Productie B.V. (KVK 17146078) dichiara 21-50 dipendenti (fonte: oozo.nl, dati KVK). KVK 17198255 (Trianon Chocolatiers B.V.). Legame di gruppo: Trianon Holding B.V., Oss (KVK 17151352). Azienda familiare, fabbrica di cioccolato e caramelle; acquirente di cioccolato e semilavorati di cacao.</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr"/>
       <c r="E81" s="3" t="inlineStr"/>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/steenland-chocolate</t>
-        </is>
-      </c>
-      <c r="G81" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="F81" s="3" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>trianon@trianon.nl</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>https://www.steenland.nl/</t>
+          <t>https://www.trianon.nl/</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Gouda (Zuid-Holland)</t>
+          <t>Oss (Noord-Brabant)</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-chocolade-en-suikerwerk/steenland-chocolate-b-v-gouda-24354029-000018029809</t>
+          <t>https://nl.kompass.com/c/trianon-chocolatiers-b-v/nl196607/</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Trianon Chocolatiers B.V.</t>
+          <t>RIS Rubber N.V.</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Cacao/Cioccolato — produzione cioccolato e confetteria</t>
+          <t>Gomma — articoli tecnici e mescole</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato. La consociata operativa Trianon Productie B.V. (KVK 17146078) dichiara 21-50 dipendenti (fonte: oozo.nl, dati KVK). KVK 17198255 (Trianon Chocolatiers B.V.). Legame di gruppo: Trianon Holding B.V., Oss (KVK 17151352). Azienda familiare, fabbrica di cioccolato e caramelle; acquirente di cioccolato e semilavorati di cacao.</t>
+          <t>Fatturato NON pubblicato. 180 dipendenti (fonte sito aziendale risrubber.com / pagina 'Over RIS', 2025). KVK 39067356. Sede Pekstraat 7, 8211 AB Lelystad. Attiva dal 1955, fabbrica di gomma con laboratorio di R&amp;S e impianti di prova propri. Membro NVR-TRA. Ragione sociale N.V. (non B.V.). Con 180 addetti stima fatturato in fascia alta/di confine del target (indicativamente 25-40 M€). E-mail: contatto commerciale pubblicato (Bianca Westmaas, Sales Manager); non risulta pubblicata una casella info@ generica.</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr"/>
       <c r="E82" s="5" t="inlineStr"/>
-      <c r="F82" s="5" t="inlineStr"/>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/ris-rubber-nv</t>
+        </is>
+      </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>trianon@trianon.nl</t>
+          <t>bwestmaas@risrubber.com</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>https://www.trianon.nl/</t>
+          <t>https://www.risrubber.com</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Oss (Noord-Brabant)</t>
+          <t>Lelystad, Flevoland</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>https://nl.kompass.com/c/trianon-chocolatiers-b-v/nl196607/</t>
+          <t>https://www.risrubber.com/over-ris/</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>RIS Rubber N.V.</t>
+          <t>Rubber Design B.V.</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Gomma — articoli tecnici e mescole</t>
+          <t>Gomma — antivibranti gomma-metallo</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato. 180 dipendenti (fonte sito aziendale risrubber.com / pagina 'Over RIS', 2025). KVK 39067356. Sede Pekstraat 7, 8211 AB Lelystad. Attiva dal 1955, fabbrica di gomma con laboratorio di R&amp;S e impianti di prova propri. Membro NVR-TRA. Ragione sociale N.V. (non B.V.). Con 180 addetti stima fatturato in fascia alta/di confine del target (indicativamente 25-40 M€). E-mail: contatto commerciale pubblicato (Bianca Westmaas, Sales Manager); non risulta pubblicata una casella info@ generica.</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr"/>
-      <c r="E83" s="3" t="inlineStr"/>
+          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 101-200 dipendenti (fonte Drimble.nl / Company.info, 2024-2025). KVK 23044439. Sede Industrieweg 21, 2995 BE Heerjansdam. Fondata 1979-1980; progetta, calcola e produce articoli tecnici in gomma e gomma-metallo antivibranti e antirumore per cantieristica navale, yacht e industria. Con 100-200 addetti il fatturato stimato si colloca nella fascia alta del target (indicativamente 20-40 M€). Directeur M. Klijn dal 2020 (fonte Company.info, KVK 23044439).</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>M. Klijn</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Directeur</t>
+        </is>
+      </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/ris-rubber-nv</t>
+          <t>https://nl.linkedin.com/company/rubber-design</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>bwestmaas@risrubber.com</t>
+          <t>info@rubberdesign.nl</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>https://www.risrubber.com</t>
+          <t>https://www.rubberdesign.nl</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Lelystad, Flevoland</t>
+          <t>Heerjansdam (Zwijndrecht), Zuid-Holland</t>
         </is>
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>https://www.risrubber.com/over-ris/</t>
+          <t>https://drimble.nl/bedrijf/heerjansdam/1084011/rubber-design-bv.html</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Rubber Design B.V.</t>
+          <t>Ruma Rubber B.V.</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Gomma — antivibranti gomma-metallo</t>
+          <t>Gomma — articoli tecnici in elastomeri</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato (BV con bilancio abbreviato). 101-200 dipendenti (fonte Drimble.nl / Company.info, 2024-2025). KVK 23044439. Sede Industrieweg 21, 2995 BE Heerjansdam. Fondata 1979-1980; progetta, calcola e produce articoli tecnici in gomma e gomma-metallo antivibranti e antirumore per cantieristica navale, yacht e industria. Con 100-200 addetti il fatturato stimato si colloca nella fascia alta del target (indicativamente 20-40 M€). Directeur M. Klijn dal 2020 (fonte Company.info, KVK 23044439).</t>
+          <t>Fatturato ca. 15 M$ (~14 M€) e 90 dipendenti (fonte Dun &amp; Bradstreet business directory, profilo aggiornato 2024-2025). KVK 04033678. Sede Lindberghstraat 49, 7903 BM Hoogeveen. Fondata 1937, specialista in tecnologia degli elastomeri; stabilimenti anche a Olkusz (PL) e Dubai (UAE). Membro NVR-TRA (Nederlandse Vereniging van Rubberfabrikanten). Fatturato esatto NON depositato pubblicamente (BV con bilancio abbreviato) - dato D&amp;B stimato. IN TARGET.</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>M. Klijn</t>
+          <t>Johannes C. van Haaren</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>Directeur</t>
+          <t>Key principal / Directeur</t>
         </is>
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/rubber-design</t>
+          <t>https://www.linkedin.com/company/ruma-rubber-bv/</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
         <is>
-          <t>info@rubberdesign.nl</t>
+          <t>info@rumarubber.com</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>https://www.rubberdesign.nl</t>
+          <t>https://rumarubber.com</t>
         </is>
       </c>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>Heerjansdam (Zwijndrecht), Zuid-Holland</t>
+          <t>Hoogeveen, Drenthe</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr">
         <is>
-          <t>https://drimble.nl/bedrijf/heerjansdam/1084011/rubber-design-bv.html</t>
+          <t>https://www.dnb.com/business-directory/company-profiles.ruma_rubber_bv.8b91dcdabf64a6f6e9fbc7005f6b7b30.html</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>Ruma Rubber B.V.</t>
+          <t>Beijer Mengvoeders B.V.</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Gomma — articoli tecnici in elastomeri</t>
+          <t>Mangimi/Soia — mangimificio</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Fatturato ca. 15 M$ (~14 M€) e 90 dipendenti (fonte Dun &amp; Bradstreet business directory, profilo aggiornato 2024-2025). KVK 04033678. Sede Lindberghstraat 49, 7903 BM Hoogeveen. Fondata 1937, specialista in tecnologia degli elastomeri; stabilimenti anche a Olkusz (PL) e Dubai (UAE). Membro NVR-TRA (Nederlandse Vereniging van Rubberfabrikanten). Fatturato esatto NON depositato pubblicamente (BV con bilancio abbreviato) - dato D&amp;B stimato. IN TARGET.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). 6-10 dipendenti (fonte: adhocdata.nl / oozo.nl su dati KVK, 2025). KVK 09009943. Micro-mengvoederbedrijf familiare, membro Nevedi: taglia di confine inferiore (fatturato verosimilmente sotto i 10 M€, gonfiato dal costo delle materie prime). Produttore di mangimi composti con impiego di sojaschroot: operatore EUDR.</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Johannes C. van Haaren</t>
+          <t>Jeroen Beijer</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Key principal / Directeur</t>
+          <t>Eigenaar / directeur</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/ruma-rubber-bv/</t>
+          <t>https://www.linkedin.com/in/jeroen-beijer-22214239/</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>info@rumarubber.com</t>
+          <t>info@beijermengvoeders.nl</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
         <is>
-          <t>https://rumarubber.com</t>
+          <t>https://beijermengvoeders.nl/</t>
         </is>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
-          <t>Hoogeveen, Drenthe</t>
+          <t>Driel / Overbetuwe (Gelderland)</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>https://www.dnb.com/business-directory/company-profiles.ruma_rubber_bv.8b91dcdabf64a6f6e9fbc7005f6b7b30.html</t>
+          <t>https://www.adhocdata.nl/bedrijven/ADH000000CCECEG/Driel/Beijer-Mengvoeders-BV</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Beijer Mengvoeders B.V.</t>
+          <t>Booijink Veevoeders B.V.</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio</t>
+          <t>Mangimi/Soia — mangimificio (bovini/suini/avicoli)</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato). 6-10 dipendenti (fonte: adhocdata.nl / oozo.nl su dati KVK, 2025). KVK 09009943. Micro-mengvoederbedrijf familiare, membro Nevedi: taglia di confine inferiore (fatturato verosimilmente sotto i 10 M€, gonfiato dal costo delle materie prime). Produttore di mangimi composti con impiego di sojaschroot: operatore EUDR.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 40 dipendenti (fonte: GraydonGo/Salland Partners, 2025). KVK 38014671. Mengvoederbedrijf familiare indipendente, membro Nevedi, con tre sedi in Overijssel; utilizzatore di sojaschroot per mangimi composti: operatore EUDR.</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Jeroen Beijer</t>
+          <t>Giel Booijink</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Eigenaar / directeur</t>
+          <t>Directeur</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/jeroen-beijer-22214239/</t>
+          <t>https://nl.linkedin.com/company/booijink-veevoeders-b.v.</t>
         </is>
       </c>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t>info@beijermengvoeders.nl</t>
+          <t>info@booijinkveevoeders.nl</t>
         </is>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>https://beijermengvoeders.nl/</t>
+          <t>https://www.booijinkveevoeders.nl/</t>
         </is>
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>Driel / Overbetuwe (Gelderland)</t>
+          <t>Raalte (Overijssel), sedi anche a Luttenberg e Rijssen</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
         <is>
-          <t>https://www.adhocdata.nl/bedrijven/ADH000000CCECEG/Driel/Beijer-Mengvoeders-BV</t>
+          <t>https://graydongo.nl/nl/voeding-booijink-veevoeders-bv-raalte-38014671</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Booijink Veevoeders B.V.</t>
+          <t>Doens Food Ingredients B.V.</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio (bovini/suini/avicoli)</t>
+          <t>Mangimi/Soia — import/export soia biologica</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 40 dipendenti (fonte: GraydonGo/Salland Partners, 2025). KVK 38014671. Mengvoederbedrijf familiare indipendente, membro Nevedi, con tre sedi in Overijssel; utilizzatore di sojaschroot per mangimi composti: operatore EUDR.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 35-40 dipendenti (fonte: Biojournaal/Omroep Zeeland, con piano di assunzione di altri 20-30 addetti a Sas van Gent); LinkedIn indica 11-50. KVK 22048339. Azienda familiare, tra i maggiori importatori/esportatori europei di ingredienti biologici food &amp; feed alla rinfusa (soia, mais, lino, grano): importatore e commerciante EUDR in senso stretto.</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Giel Booijink</t>
+          <t>Walter Doens</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
@@ -27258,702 +27270,650 @@
           <t>Directeur</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>https://nl.linkedin.com/company/booijink-veevoeders-b.v.</t>
-        </is>
-      </c>
+      <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>info@booijinkveevoeders.nl</t>
+          <t>info@doensfood.com</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>https://www.booijinkveevoeders.nl/</t>
+          <t>https://www.doensfood.com/</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
-          <t>Raalte (Overijssel), sedi anche a Luttenberg e Rijssen</t>
+          <t>IJzendijke / Sluis (Zeeland), impianto a Sas van Gent</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>https://graydongo.nl/nl/voeding-booijink-veevoeders-bv-raalte-38014671</t>
+          <t>https://drimble.nl/bedrijf/ijzendijke/17334179/doens-food-ingredients-bv.html</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Doens Food Ingredients B.V.</t>
+          <t>Garvo B.V.</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — import/export soia biologica</t>
+          <t>Mangimi/Soia — produzione mangimi su base cereali/soia</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 35-40 dipendenti (fonte: Biojournaal/Omroep Zeeland, con piano di assunzione di altri 20-30 addetti a Sas van Gent); LinkedIn indica 11-50. KVK 22048339. Azienda familiare, tra i maggiori importatori/esportatori europei di ingredienti biologici food &amp; feed alla rinfusa (soia, mais, lino, grano): importatore e commerciante EUDR in senso stretto.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 25 dipendenti (fonte: vainu.io/GraydonGo, ultimo esercizio disponibile); LinkedIn indica 11-50 addetti. KVK 09004900. Produttore indipendente di oltre 300 mangimi (cavalli, pollame, colombi, animali da hobby) su base cereali e derivati proteici: utilizzatore/operatore EUDR.</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Walter Doens</t>
+          <t>Henkjan Garretsen</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>Directeur</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr"/>
+          <t>Commercieel directeur / aandeelhouder</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/garvo-bv</t>
+        </is>
+      </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>info@doensfood.com</t>
+          <t>garvo@garvo.nl</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>https://www.doensfood.com/</t>
+          <t>https://www.garvo.nl/</t>
         </is>
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>IJzendijke / Sluis (Zeeland), impianto a Sas van Gent</t>
+          <t>Drempt / Bronckhorst (Gelderland)</t>
         </is>
       </c>
       <c r="J88" s="5" t="inlineStr">
         <is>
-          <t>https://drimble.nl/bedrijf/ijzendijke/17334179/doens-food-ingredients-bv.html</t>
+          <t>https://vainu.io/company/garvo-bv-omzet-en-financiele/16180270/bedrijfsinformatie</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Garvo B.V.</t>
+          <t>Gunnewick Mengvoeders B.V.</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — produzione mangimi su base cereali/soia</t>
+          <t>Mangimi/Soia — mangimificio</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo su banche dati a pagamento). 25 dipendenti (fonte: vainu.io/GraydonGo, ultimo esercizio disponibile); LinkedIn indica 11-50 addetti. KVK 09004900. Produttore indipendente di oltre 300 mangimi (cavalli, pollame, colombi, animali da hobby) su base cereali e derivati proteici: utilizzatore/operatore EUDR.</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr">
-        <is>
-          <t>Henkjan Garretsen</t>
-        </is>
-      </c>
-      <c r="E89" s="3" t="inlineStr">
-        <is>
-          <t>Commercieel directeur / aandeelhouder</t>
-        </is>
-      </c>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). 21-50 dipendenti (fonte: oozo.nl / TransFirm su dati KVK, 2025). KVK 09183960. Mengvoederbedrijf familiare indipendente, membro Nevedi, attivo anche nel commercio di granaglie e materie prime per mangimi (sojaschroot incluso): operatore/commerciante EUDR.</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/garvo-bv</t>
+          <t>https://nl.linkedin.com/company/gunnewickmengvoeders</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>garvo@garvo.nl</t>
+          <t>info@gunnewick.com</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
         <is>
-          <t>https://www.garvo.nl/</t>
+          <t>https://gunnewick.com/</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Drempt / Bronckhorst (Gelderland)</t>
+          <t>Vragender / Oost Gelre (Gelderland)</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>https://vainu.io/company/garvo-bv-omzet-en-financiele/16180270/bedrijfsinformatie</t>
+          <t>https://www.oozo.nl/bedrijven/oost-gelre/vragender/bebouwde-kom-vragender/438727/gunnewick-mengvoeders-b-v</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Gunnewick Mengvoeders B.V.</t>
+          <t>P. Bos Mengvoeder- en Kunstmesthandel B.V.</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio</t>
+          <t>Mangimi/Soia — mangimificio e commercio grondstoffen</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato). 21-50 dipendenti (fonte: oozo.nl / TransFirm su dati KVK, 2025). KVK 09183960. Mengvoederbedrijf familiare indipendente, membro Nevedi, attivo anche nel commercio di granaglie e materie prime per mangimi (sojaschroot incluso): operatore/commerciante EUDR.</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr"/>
-      <c r="E90" s="5" t="inlineStr"/>
-      <c r="F90" s="6" t="inlineStr">
-        <is>
-          <t>https://nl.linkedin.com/company/gunnewickmengvoeders</t>
-        </is>
-      </c>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; company.info espone solo il profilo). Ca. 31 dipendenti (fonte: company.info / drimble.nl, 2025). KVK 09056076. Azienda familiare attiva dal 1894, produttore e fornitore di mengvoeder e concimi, dal 2025 in collaborazione con Van Benthem Diervoeders: PMI utilizzatrice di sojaschroot, operatore EUDR.</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>J. Bos</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Algemeen directeur</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr"/>
       <c r="G90" s="6" t="inlineStr">
         <is>
-          <t>info@gunnewick.com</t>
+          <t>info@pbosveevoeders.nl</t>
         </is>
       </c>
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>https://gunnewick.com/</t>
+          <t>https://www.pbosveevoeders.nl/</t>
         </is>
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Vragender / Oost Gelre (Gelderland)</t>
+          <t>Ederveen / Ede (Gelderland)</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
         <is>
-          <t>https://www.oozo.nl/bedrijven/oost-gelre/vragender/bebouwde-kom-vragender/438727/gunnewick-mengvoeders-b-v</t>
+          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-veevoeders/p-bos-mengvoeder-en-kunstmesthandel-b-v-ederveen-09056076-000016850459</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>P. Bos Mengvoeder- en Kunstmesthandel B.V.</t>
+          <t>Van Benthem Diervoeders Vollenhove B.V.</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio e commercio grondstoffen</t>
+          <t>Mangimi/Soia — mangimificio (rundvee/paarden)</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato; company.info espone solo il profilo). Ca. 31 dipendenti (fonte: company.info / drimble.nl, 2025). KVK 09056076. Azienda familiare attiva dal 1894, produttore e fornitore di mengvoeder e concimi, dal 2025 in collaborazione con Van Benthem Diervoeders: PMI utilizzatrice di sojaschroot, operatore EUDR.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). Ca. 20-21 dipendenti (fonte: vbvoer.nl e drimble.nl, 2025). KVK 05044357. Mangimificio familiare attivo dal 1780, produttore di mengvoeder di taglia medio-piccola; dal 2025 collaborazione con P. Bos Veevoeders. Utilizzatore di sojaschroot: operatore/commerciante EUDR.</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>J. Bos</t>
+          <t>Ed van Benthem</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Algemeen directeur</t>
-        </is>
-      </c>
-      <c r="F91" s="3" t="inlineStr"/>
+          <t>Eigenaar / directeur</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-benthem-veevoeders-en-kunstmest-b.v.</t>
+        </is>
+      </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>info@pbosveevoeders.nl</t>
+          <t>info@vanbenthemvollenhove.nl</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
         <is>
-          <t>https://www.pbosveevoeders.nl/</t>
+          <t>https://www.vbvoer.nl/</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Ederveen / Ede (Gelderland)</t>
+          <t>Vollenhove / Steenwijkerland (Overijssel)</t>
         </is>
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/vervaardiging-van-veevoeders/p-bos-mengvoeder-en-kunstmesthandel-b-v-ederveen-09056076-000016850459</t>
+          <t>https://www.vbvoer.nl/van-benthem/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Van Benthem Diervoeders Vollenhove B.V.</t>
+          <t>Van Gorp Diervoeders B.V.</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio (rundvee/paarden)</t>
+          <t>Mangimi/Soia — mangimificio (hobby e zootecnia)</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato). Ca. 20-21 dipendenti (fonte: vbvoer.nl e drimble.nl, 2025). KVK 05044357. Mangimificio familiare attivo dal 1780, produttore di mengvoeder di taglia medio-piccola; dal 2025 collaborazione con P. Bos Veevoeders. Utilizzatore di sojaschroot: operatore/commerciante EUDR.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato). 11-20 dipendenti (fonte: oozo.nl su dati KVK, 2025). KVK 18083568. Mangimificio familiare indipendente con radici a Waspik dal 1923, stabilimento a Waalwijk dal 2005: PMI di taglia medio-piccola (fatturato verosimilmente 5-15 M€, non pubblicato). Utilizzatore di sojaschroot e derivati proteici: operatore EUDR.</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Ed van Benthem</t>
+          <t>Hans van Gorp</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Eigenaar / directeur</t>
+          <t>Directeur</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/van-benthem-veevoeders-en-kunstmest-b.v.</t>
+          <t>https://www.linkedin.com/company/van-gorp-diervoeders-b.v.</t>
         </is>
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>info@vanbenthemvollenhove.nl</t>
+          <t>info@van-gorp.com</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>https://www.vbvoer.nl/</t>
+          <t>https://www.van-gorp.com/</t>
         </is>
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Vollenhove / Steenwijkerland (Overijssel)</t>
+          <t>Waalwijk (Noord-Brabant)</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>https://www.vbvoer.nl/van-benthem/</t>
+          <t>https://www.oozo.nl/bedrijven/waalwijk/waalwijk/industrieterrein-haven/43305/van-gorp-diervoeders-b-v</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Van Gorp Diervoeders B.V.</t>
+          <t>DO IT Organic Food Ingredients B.V.</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Mangimi/Soia — mangimificio (hobby e zootecnia)</t>
+          <t>Olio di palma — import oli vegetali e soia bio</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato). 11-20 dipendenti (fonte: oozo.nl su dati KVK, 2025). KVK 18083568. Mangimificio familiare indipendente con radici a Waspik dal 1923, stabilimento a Waalwijk dal 2005: PMI di taglia medio-piccola (fatturato verosimilmente 5-15 M€, non pubblicato). Utilizzatore di sojaschroot e derivati proteici: operatore EUDR.</t>
+          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo a pagamento). KVK 75119048 (entita DO IT Organic Food Ingredients B.V., Barneveld; il gruppo DO-IT opera dal 1990 ca.). Trader olandese di ingredienti biologici con rete mondiale di fornitori: soia ca. 15% del giro d'affari e oli/grassi (inclusi palma e cocco) ca. 10% - importatore/operatore EUDR su entrambe le commodity. Numero dipendenti non pubblicato.</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Hans van Gorp</t>
+          <t>Hendrik Wijnen</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Directeur</t>
+          <t>CEO / algemeen directeur</t>
         </is>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/van-gorp-diervoeders-b.v.</t>
+          <t>https://nl.linkedin.com/company/doitorganic</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>info@van-gorp.com</t>
+          <t>sales@organic.nl</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
         <is>
-          <t>https://www.van-gorp.com/</t>
+          <t>https://www.doitorganic.nl/</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>Waalwijk (Noord-Brabant)</t>
+          <t>Barneveld (Gelderland)</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>https://www.oozo.nl/bedrijven/waalwijk/waalwijk/industrieterrein-haven/43305/van-gorp-diervoeders-b-v</t>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-voedingsmiddelen-dranken-en-overige-genotmiddelen-algemeen-assortiment/do-it-organic-food-ingredients-b-v-barneveld-75119048-000043017282</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>DO IT Organic Food Ingredients B.V.</t>
+          <t>S.R.C. (Special Refining Company) B.V.</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — import oli vegetali e soia bio</t>
+          <t>Olio di palma — raffinazione conto terzi oli vegetali</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (BV con deposito abbreviato; dati finanziari solo a pagamento). KVK 75119048 (entita DO IT Organic Food Ingredients B.V., Barneveld; il gruppo DO-IT opera dal 1990 ca.). Trader olandese di ingredienti biologici con rete mondiale di fornitori: soia ca. 15% del giro d'affari e oli/grassi (inclusi palma e cocco) ca. 10% - importatore/operatore EUDR su entrambe le commodity. Numero dipendenti non pubblicato.</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>Hendrik Wijnen</t>
-        </is>
-      </c>
-      <c r="E94" s="5" t="inlineStr">
-        <is>
-          <t>CEO / algemeen directeur</t>
-        </is>
-      </c>
+          <t>Fatturato non pubblicato (toll refiner: non acquista né vende olio, fattura solo il servizio di raffinazione — fatturato strutturalmente sotto la soglia dei trader). Capacità di raffinazione oltre 40.000 t/anno; organico ridotto e specializzato (numero esatto non pubblicato). Fondata nel 1996, parte del gruppo Pieter Bon. Circa 60% degli oli e grassi lavorati è biologico. Membro MVO. Raffinatore di palma e altri oli vegetali sul Noordzeekanaal.</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr"/>
+      <c r="E94" s="5" t="inlineStr"/>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/doitorganic</t>
-        </is>
-      </c>
-      <c r="G94" s="6" t="inlineStr">
-        <is>
-          <t>sales@organic.nl</t>
+          <t>https://nl.linkedin.com/company/src-b-v-</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>https://www.doitorganic.nl/</t>
+          <t>https://refinery.nl/</t>
         </is>
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Barneveld (Gelderland)</t>
+          <t>Zaandam / Zaanstad (Noord-Holland)</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-voedingsmiddelen-dranken-en-overige-genotmiddelen-algemeen-assortiment/do-it-organic-food-ingredients-b-v-barneveld-75119048-000043017282</t>
+          <t>https://mvo.nl/organisatie/leden/src</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>S.R.C. (Special Refining Company) B.V.</t>
+          <t>Spack B.V.</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Olio di palma — raffinazione conto terzi oli vegetali</t>
+          <t>Olio di palma — produzione/confezionamento oli vegetali bio</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (toll refiner: non acquista né vende olio, fattura solo il servizio di raffinazione — fatturato strutturalmente sotto la soglia dei trader). Capacità di raffinazione oltre 40.000 t/anno; organico ridotto e specializzato (numero esatto non pubblicato). Fondata nel 1996, parte del gruppo Pieter Bon. Circa 60% degli oli e grassi lavorati è biologico. Membro MVO. Raffinatore di palma e altri oli vegetali sul Noordzeekanaal.</t>
+          <t>Fatturato non pubblicato (company.info espone solo profilo, dati finanziari a pagamento). 10-24 dipendenti (fonte: regiobedrijf.nl su dati KVK, 2025). KVK 24225423. PMI probabilmente sotto i 10 M€ di fatturato: segnalata come taglia di confine inferiore. Nata a Rotterdam nel 1977 come trading di oli e grassi vegetali, oggi produttore/confezionatore di oli vegetali biologici (incl. palma e cocco): operatore EUDR.</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr"/>
       <c r="E95" s="3" t="inlineStr"/>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/src-b-v-</t>
-        </is>
-      </c>
-      <c r="G95" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+          <t>https://nl.linkedin.com/company/spackbv</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>info@spackbv.com</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>https://refinery.nl/</t>
+          <t>https://www.spack.nl/</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>Zaandam / Zaanstad (Noord-Holland)</t>
+          <t>Nieuwe-Tonge / Goeree-Overflakkee (Zuid-Holland)</t>
         </is>
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>https://mvo.nl/organisatie/leden/src</t>
+          <t>https://regiobedrijf.nl/groothandel-in-ruwe-plantaardige-en-dierlijke-olien-en-vetten-en-oliehoudende-grondstoffen/spack-bv-74891.html</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>Spack B.V.</t>
+          <t>G &amp; A Wennekers Vleesgroothandel B.V.</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>Olio di palma — produzione/confezionamento oli vegetali bio</t>
+          <t>Bovini/Carne — grossista rund- en kalfsvlees</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Fatturato non pubblicato (company.info espone solo profilo, dati finanziari a pagamento). 10-24 dipendenti (fonte: regiobedrijf.nl su dati KVK, 2025). KVK 24225423. PMI probabilmente sotto i 10 M€ di fatturato: segnalata come taglia di confine inferiore. Nata a Rotterdam nel 1977 come trading di oli e grassi vegetali, oggi produttore/confezionatore di oli vegetali biologici (incl. palma e cocco): operatore EUDR.</t>
+          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). 11-20 dipendenti (fonte TransFirm / Kompass, profilo 2024-2025). KVK 24315872. Sede Groothandelsmarkt 209, 3044 HH Rotterdam (Spaanse Polder). Azienda familiare fondata nel 1965 da G. Wennekers sr.; specializzata nella lavorazione e nel commercio di carne bovina, di vitello e ovina. Organico contenuto: il fatturato potrebbe collocarsi sotto la fascia target - da verificare in fase di qualifica. Commodity EUDR: bovini.</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr"/>
       <c r="E96" s="5" t="inlineStr"/>
-      <c r="F96" s="6" t="inlineStr">
-        <is>
-          <t>https://nl.linkedin.com/company/spackbv</t>
-        </is>
-      </c>
+      <c r="F96" s="5" t="inlineStr"/>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>info@spackbv.com</t>
+          <t>info@wennekersvlees.nl</t>
         </is>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>https://www.spack.nl/</t>
+          <t>https://www.wennekersvlees.nl</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Nieuwe-Tonge / Goeree-Overflakkee (Zuid-Holland)</t>
+          <t>Rotterdam, Zuid-Holland</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
         <is>
-          <t>https://regiobedrijf.nl/groothandel-in-ruwe-plantaardige-en-dierlijke-olien-en-vetten-en-oliehoudende-grondstoffen/spack-bv-74891.html</t>
+          <t>https://www.transfirm.nl/nl/organisatie/243158720000-g-&amp;-a-wennekers-vleesgroothandel-b.v</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>G &amp; A Wennekers Vleesgroothandel B.V.</t>
+          <t>Kroon Vlees B.V.</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — grossista rund- en kalfsvlees</t>
+          <t>Bovini/Carne — macello e lavorazione</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). 11-20 dipendenti (fonte TransFirm / Kompass, profilo 2024-2025). KVK 24315872. Sede Groothandelsmarkt 209, 3044 HH Rotterdam (Spaanse Polder). Azienda familiare fondata nel 1965 da G. Wennekers sr.; specializzata nella lavorazione e nel commercio di carne bovina, di vitello e ovina. Organico contenuto: il fatturato potrebbe collocarsi sotto la fascia target - da verificare in fase di qualifica. Commodity EUDR: bovini.</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr"/>
-      <c r="E97" s="3" t="inlineStr"/>
+          <t>Fatturato NON pubblicato. KVK 02023970. Sede Gotenburgweg 30, 9723 TM Groningen. Attiva dal 1870; macello e impianto di sezionamento (slachten, uitbenen, snijden, verpakken sotto un unico tetto) per bovini e suini, con approvvigionamento regionale dalle province del Nord. Certificata SKAL per la linea biologica; indicata dalla NVWA come azienda esemplare. Proprietario dal 2014 Henk Luinge (ingegnere chimico). Numero dipendenti non pubblicato nelle fonti aperte consultate. Commodity EUDR: bovini.</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Henk Luinge</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Eigenaar</t>
+        </is>
+      </c>
       <c r="F97" s="3" t="inlineStr"/>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>info@wennekersvlees.nl</t>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>https://www.wennekersvlees.nl</t>
+          <t>https://www.kroonvlees.nl</t>
         </is>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland</t>
+          <t>Groningen, Groningen</t>
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>https://www.transfirm.nl/nl/organisatie/243158720000-g-&amp;-a-wennekers-vleesgroothandel-b.v</t>
+          <t>https://www.kroonvlees.nl/over-kroon-vlees</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>Kroon Vlees B.V.</t>
+          <t>Randstad Vleesgroothandel B.V.</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macello e lavorazione</t>
+          <t>Bovini/Carne — grossista rundvlees</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato. KVK 02023970. Sede Gotenburgweg 30, 9723 TM Groningen. Attiva dal 1870; macello e impianto di sezionamento (slachten, uitbenen, snijden, verpakken sotto un unico tetto) per bovini e suini, con approvvigionamento regionale dalle province del Nord. Certificata SKAL per la linea biologica; indicata dalla NVWA come azienda esemplare. Proprietario dal 2014 Henk Luinge (ingegnere chimico). Numero dipendenti non pubblicato nelle fonti aperte consultate. Commodity EUDR: bovini.</t>
+          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 50 dipendenti (fonte Creditsafe / Kompass, profilo 2024-2025). KVK 24155381. Sede Barendrechtseweg 300-2E, 2992 SL Barendrecht (in precedenza Hekendorpstraat 4, Rotterdam). Costituita 1984, azienda familiare nata come macelleria ad Amersfoort nel 1954 (fam. Van der Arend). Specializzata in carne bovina, in particolare vacca/manza; lavora ca. 200 tonnellate di rundvlees fresco a settimana - volume coerente con la fascia target. Commodity EUDR: bovini. Contatti pubblicati: info@randstadvlees.nl, tel. +31 10 2921800; nel team compare John van der Arend (Directie, Inkoop/Verkoop).</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>Henk Luinge</t>
+          <t>J.H.M. van der Arend</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Eigenaar</t>
+          <t>Algemeen directrice</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr"/>
-      <c r="G98" s="5" t="inlineStr">
-        <is>
-          <t>n.d.</t>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>info@randstadvlees.nl</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>https://www.kroonvlees.nl</t>
+          <t>http://www.randstadvlees.nl</t>
         </is>
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Groningen, Groningen</t>
+          <t>Barendrecht, Zuid-Holland</t>
         </is>
       </c>
       <c r="J98" s="5" t="inlineStr">
         <is>
-          <t>https://www.kroonvlees.nl/over-kroon-vlees</t>
+          <t>https://www.creditsafe.com/business-index/en-gb/company/randstad-vleesgroothandel-bv-nl01183286</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Randstad Vleesgroothandel B.V.</t>
+          <t>Van Kooten Vleesgroothandel B.V.</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Bovini/Carne — grossista rundvlees</t>
+          <t>Bovini/Carne — macello e grossista</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 50 dipendenti (fonte Creditsafe / Kompass, profilo 2024-2025). KVK 24155381. Sede Barendrechtseweg 300-2E, 2992 SL Barendrecht (in precedenza Hekendorpstraat 4, Rotterdam). Costituita 1984, azienda familiare nata come macelleria ad Amersfoort nel 1954 (fam. Van der Arend). Specializzata in carne bovina, in particolare vacca/manza; lavora ca. 200 tonnellate di rundvlees fresco a settimana - volume coerente con la fascia target. Commodity EUDR: bovini. Contatti pubblicati: info@randstadvlees.nl, tel. +31 10 2921800; nel team compare John van der Arend (Directie, Inkoop/Verkoop).</t>
-        </is>
-      </c>
-      <c r="D99" s="3" t="inlineStr">
-        <is>
-          <t>J.H.M. van der Arend</t>
-        </is>
-      </c>
-      <c r="E99" s="3" t="inlineStr">
-        <is>
-          <t>Algemeen directrice</t>
-        </is>
-      </c>
-      <c r="F99" s="3" t="inlineStr"/>
+          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 20 dipendenti (fonte Company.info / Drimble, profilo 2024-2025). KVK 30112737. Sede Oeverweg 3, 3417 XK Montfoort. Azienda familiare con oltre 30 anni di attività nella distribuzione di carne; lavora con macelli medi e grandi. GRUPPO: collegata a Slachterij van Kooten B.V. (Julianalaan 1, 3417 GJ Montfoort, oltre 110 anni di attività, e-mail info@vankooten.nl), che macella, diseossa, confeziona e distribuisce carne bovina, di vitello e ovina. Fascia dimensionale probabilmente sotto il target sui dipendenti, ma i volumi di commercio carne possono collocare il fatturato nella fascia bassa del range. Commodity EUDR: bovini.</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr"/>
+      <c r="E99" s="3" t="inlineStr"/>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/van-kooten-vleesgroothandel-b.v.</t>
+        </is>
+      </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>info@randstadvlees.nl</t>
+          <t>info@vankootenvlees.nl</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
         <is>
-          <t>http://www.randstadvlees.nl</t>
+          <t>https://vankootenvlees.nl</t>
         </is>
       </c>
       <c r="I99" s="3" t="inlineStr">
         <is>
-          <t>Barendrecht, Zuid-Holland</t>
+          <t>Montfoort, Utrecht</t>
         </is>
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>https://www.creditsafe.com/business-index/en-gb/company/randstad-vleesgroothandel-bv-nl01183286</t>
+          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-vlees-en-vleesproducten/van-kooten-vleesgroothandel-b-v-montfoort-30112737-000018814379</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>Van Kooten Vleesgroothandel B.V.</t>
+          <t>Vleesbedrijf Bolscher B.V.</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Bovini/Carne — macello e grossista</t>
+          <t>Bovini/Carne — macello e lavorazione carni rosse</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 20 dipendenti (fonte Company.info / Drimble, profilo 2024-2025). KVK 30112737. Sede Oeverweg 3, 3417 XK Montfoort. Azienda familiare con oltre 30 anni di attività nella distribuzione di carne; lavora con macelli medi e grandi. GRUPPO: collegata a Slachterij van Kooten B.V. (Julianalaan 1, 3417 GJ Montfoort, oltre 110 anni di attività, e-mail info@vankooten.nl), che macella, diseossa, confeziona e distribuisce carne bovina, di vitello e ovina. Fascia dimensionale probabilmente sotto il target sui dipendenti, ma i volumi di commercio carne possono collocare il fatturato nella fascia bassa del range. Commodity EUDR: bovini.</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr"/>
-      <c r="E100" s="5" t="inlineStr"/>
+          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 80 dipendenti (fonte Stagemarkt.nl / stampa regionale 1Twente e Oost.nl, 2024-2025). Sedi: Strootsweg 40, 7547 RW Enschede e Transportcentrum 40 (fonte Drimble). Slachthuis e vleesbedrijf: macellazione, produzione di prodotti a base di carne e commercio di bestiame, carne e prodotti da macelleria; il core business è la carne rossa (rundvlees). Consegne su quasi tutto il territorio olandese. Con ca. 80 addetti la stima di fatturato si colloca nella fascia alta del target. Commodity EUDR: bovini.</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="inlineStr">
+        <is>
+          <t>Roy Bolscher en Chiel Bolscher</t>
+        </is>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Eigenaren</t>
+        </is>
+      </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/van-kooten-vleesgroothandel-b.v.</t>
-        </is>
-      </c>
-      <c r="G100" s="6" t="inlineStr">
-        <is>
-          <t>info@vankootenvlees.nl</t>
+          <t>https://nl.linkedin.com/company/bolscher</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>https://vankootenvlees.nl</t>
+          <t>https://bolscher.nl</t>
         </is>
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>Montfoort, Utrecht</t>
+          <t>Enschede, Overijssel</t>
         </is>
       </c>
       <c r="J100" s="5" t="inlineStr">
         <is>
-          <t>https://companyinfo.nl/organisatieprofiel/groothandel-in-vlees-en-vleesproducten/van-kooten-vleesgroothandel-b-v-montfoort-30112737-000018814379</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>Vleesbedrijf Bolscher B.V.</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>Bovini/Carne — macello e lavorazione carni rosse</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>Fatturato NON pubblicato (B.V. con bilancio abbreviato). Ca. 80 dipendenti (fonte Stagemarkt.nl / stampa regionale 1Twente e Oost.nl, 2024-2025). Sedi: Strootsweg 40, 7547 RW Enschede e Transportcentrum 40 (fonte Drimble). Slachthuis e vleesbedrijf: macellazione, produzione di prodotti a base di carne e commercio di bestiame, carne e prodotti da macelleria; il core business è la carne rossa (rundvlees). Consegne su quasi tutto il territorio olandese. Con ca. 80 addetti la stima di fatturato si colloca nella fascia alta del target. Commodity EUDR: bovini.</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>Roy Bolscher en Chiel Bolscher</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>Eigenaren</t>
-        </is>
-      </c>
-      <c r="F101" s="4" t="inlineStr">
-        <is>
-          <t>https://nl.linkedin.com/company/bolscher</t>
-        </is>
-      </c>
-      <c r="G101" s="3" t="inlineStr">
-        <is>
-          <t>n.d.</t>
-        </is>
-      </c>
-      <c r="H101" s="4" t="inlineStr">
-        <is>
-          <t>https://bolscher.nl</t>
-        </is>
-      </c>
-      <c r="I101" s="3" t="inlineStr">
-        <is>
-          <t>Enschede, Overijssel</t>
-        </is>
-      </c>
-      <c r="J101" s="3" t="inlineStr">
-        <is>
           <t>https://drimble.nl/bedrijf/enschede/19259131/vleesbedrijf-bolscher-bv.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J101"/>
+  <autoFilter ref="A2:J100"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -28129,72 +28089,72 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G73" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G76" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G94" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G97" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G100" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H101" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G72" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G74" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G75" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G81" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G82" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G83" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G84" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G85" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G86" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G87" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G88" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H88" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G89" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H89" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G90" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H90" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G91" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H91" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G92" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H92" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G93" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H93" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H94" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G95" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H95" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G96" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H96" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H97" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G98" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H98" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G99" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H99" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H100" r:id="rId237"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finlandia: rimossa Sisuwood (fallita, konkurssi agosto 2025)
Dopo un tentativo fallito di yrityssaneeraus, Sisuwood Oy e' stata dichiarata in
konkurssi dal tribunale del Pohjois-Savo nell'agosto 2025; tutti i 38 dipendenti
licenziati, curatore nominato. Oggi esiste solo il «Sisuwood Oy konkurssipesae»,
cioe' la massa fallimentare. Stesso criterio di Helmut Sachers e Weissengruber.

finlandia_03 completo: 18 rilievi, 4 alta. Altri tre lasciati come rilievo aperto:
Siparila (63% al gruppo estone Thermory, non dichiarato, e referente senza
riscontro), Selka (dichiara «liikevaihto non pubblicato» ma e' pubblico: 1,7 M€ e
14 dipendenti, fuori forbice di un ordine di grandezza) e BestPak (2,0 M€).

Trovati anche tre dati sui dipendenti gravemente errati: Havi 22 contro ~106
dichiarati, Sahakuutio ~60 contro ~17, Unico 86 contro >100.

Censimento da 729 a 728 aziende.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GBgWuk6qpQ3JrcwnEL72dg
</commit_message>
<xml_diff>
--- a/MyEUDR_Lead_Mapping.xlsx
+++ b/MyEUDR_Lead_Mapping.xlsx
@@ -11578,11 +11578,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>Sisuwood Oy</t>
-        </is>
-      </c>
+      <c r="A42" s="5" t="n"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Legno/Arredo — falegnameria/collettività</t>

</xml_diff>